<commit_message>
Primeros dos entrenamientos completados
</commit_message>
<xml_diff>
--- a/modelos_tfg/MetricasValidacion.xlsx
+++ b/modelos_tfg/MetricasValidacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\modelos_tfg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{838B6F25-BAFE-4436-923F-8D74FB14310A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87188FEC-59DA-487E-A1BC-94037DF1996E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
   <si>
     <t>ID Train</t>
   </si>
@@ -76,6 +76,39 @@
   </si>
   <si>
     <t>GRU</t>
+  </si>
+  <si>
+    <t>V0</t>
+  </si>
+  <si>
+    <t>V1</t>
+  </si>
+  <si>
+    <t>Look Ahead</t>
+  </si>
+  <si>
+    <t>Bacth Size</t>
+  </si>
+  <si>
+    <t>Dense</t>
+  </si>
+  <si>
+    <t>32, 16, 8, 1</t>
+  </si>
+  <si>
+    <t>OBSERVACIONES</t>
+  </si>
+  <si>
+    <t>22 (ET)</t>
+  </si>
+  <si>
+    <t>Train Time (s)</t>
+  </si>
+  <si>
+    <t>8 (ET)</t>
+  </si>
+  <si>
+    <t>19 (ET)</t>
   </si>
 </sst>
 </file>
@@ -145,7 +178,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -344,55 +377,71 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -403,7 +452,96 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -751,7 +889,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:M11"/>
+  <dimension ref="A2:W26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.42578125" customWidth="1"/>
@@ -759,34 +897,52 @@
     <col min="4" max="4" width="11.28515625" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="13.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" customWidth="1"/>
     <col min="9" max="9" width="12.42578125" customWidth="1"/>
+    <col min="10" max="10" width="13" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.42578125" customWidth="1"/>
+    <col min="13" max="13" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:13" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D3" s="19" t="s">
+    <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D3" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="16" t="s">
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17"/>
-      <c r="M3" s="18"/>
-    </row>
-    <row r="4" spans="1:13" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="27" t="s">
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="28"/>
+      <c r="P3" s="28"/>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="S3" s="35"/>
+      <c r="T3" s="35"/>
+      <c r="U3" s="35"/>
+      <c r="V3" s="35"/>
+      <c r="W3" s="36"/>
+    </row>
+    <row r="4" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="C4" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="15" t="s">
         <v>3</v>
       </c>
       <c r="E4" s="6" t="s">
@@ -801,110 +957,251 @@
       <c r="H4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="J4" s="13" t="s">
+      <c r="J4" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="L4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="K4" s="13" t="s">
+      <c r="M4" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="N4" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="L4" s="13" t="s">
+      <c r="O4" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="P4" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="M4" s="14" t="s">
+      <c r="Q4" s="13" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="9"/>
-      <c r="B5" s="28"/>
+      <c r="R4" s="37"/>
+      <c r="S4" s="38"/>
+      <c r="T4" s="38"/>
+      <c r="U4" s="38"/>
+      <c r="V4" s="38"/>
+      <c r="W4" s="39"/>
+    </row>
+    <row r="5" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="8"/>
+      <c r="B5" s="30" t="s">
+        <v>17</v>
+      </c>
       <c r="C5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
-      <c r="H5" s="24"/>
-      <c r="I5" s="25"/>
-      <c r="J5" s="23"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="23"/>
-      <c r="M5" s="24"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
-      <c r="B6" s="9"/>
+      <c r="D5" s="1">
+        <v>2E-3</v>
+      </c>
+      <c r="E5" s="16">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="F5" s="16">
+        <v>-1.0126999999999999</v>
+      </c>
+      <c r="G5" s="16">
+        <v>-1.0149999999999999</v>
+      </c>
+      <c r="H5" s="17">
+        <v>30</v>
+      </c>
+      <c r="I5" s="18">
+        <v>18</v>
+      </c>
+      <c r="J5" s="40">
+        <v>196.68</v>
+      </c>
+      <c r="K5" s="16">
+        <v>6</v>
+      </c>
+      <c r="L5" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="M5" s="16">
+        <v>32</v>
+      </c>
+      <c r="N5" s="16">
+        <v>64</v>
+      </c>
+      <c r="O5" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="P5" s="16">
+        <v>0.2</v>
+      </c>
+      <c r="Q5" s="17">
+        <v>1E-3</v>
+      </c>
+      <c r="R5" s="41"/>
+      <c r="S5" s="42"/>
+      <c r="T5" s="42"/>
+      <c r="U5" s="42"/>
+      <c r="V5" s="42"/>
+      <c r="W5" s="43"/>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A6" s="8"/>
+      <c r="B6" s="31"/>
       <c r="C6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
-      <c r="M6" s="9"/>
-    </row>
-    <row r="7" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="15" t="s">
+      <c r="D6" s="1">
+        <v>3.4000000000000002E-2</v>
+      </c>
+      <c r="E6">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="F6">
+        <v>-362.46839999999997</v>
+      </c>
+      <c r="G6">
+        <v>-362.88470000000001</v>
+      </c>
+      <c r="H6" s="8">
+        <v>87.8</v>
+      </c>
+      <c r="I6" s="1">
+        <v>18</v>
+      </c>
+      <c r="J6">
+        <v>136.82</v>
+      </c>
+      <c r="K6">
+        <v>6</v>
+      </c>
+      <c r="L6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M6">
+        <v>32</v>
+      </c>
+      <c r="N6">
+        <v>64</v>
+      </c>
+      <c r="O6" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="P6">
+        <v>0.2</v>
+      </c>
+      <c r="Q6" s="8">
+        <v>1E-3</v>
+      </c>
+      <c r="R6" s="44"/>
+      <c r="S6" s="45"/>
+      <c r="T6" s="45"/>
+      <c r="U6" s="45"/>
+      <c r="V6" s="45"/>
+      <c r="W6" s="46"/>
+    </row>
+    <row r="7" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="8"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="4"/>
-    </row>
-    <row r="8" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9"/>
+      <c r="D7" s="2">
+        <v>1E-3</v>
+      </c>
+      <c r="E7" s="3">
+        <v>2E-3</v>
+      </c>
+      <c r="F7" s="3">
+        <v>-0.4486</v>
+      </c>
+      <c r="G7" s="3">
+        <v>-0.45019999999999999</v>
+      </c>
+      <c r="H7" s="4">
+        <v>69.3</v>
+      </c>
+      <c r="I7" s="2">
+        <v>18</v>
+      </c>
+      <c r="J7" s="3">
+        <v>309.79000000000002</v>
+      </c>
+      <c r="K7" s="3">
+        <v>6</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="M7" s="3">
+        <v>32</v>
+      </c>
+      <c r="N7" s="3">
+        <v>64</v>
+      </c>
+      <c r="O7" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="P7" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="Q7" s="4">
+        <v>1E-3</v>
+      </c>
+      <c r="R7" s="47"/>
+      <c r="S7" s="48"/>
+      <c r="T7" s="48"/>
+      <c r="U7" s="48"/>
+      <c r="V7" s="48"/>
+      <c r="W7" s="49"/>
+    </row>
+    <row r="8" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="8"/>
+      <c r="B8" s="33" t="s">
+        <v>18</v>
+      </c>
       <c r="C8" s="5" t="s">
         <v>15</v>
       </c>
       <c r="D8" s="1"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="11"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="10"/>
       <c r="I8" s="1"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
-      <c r="M8" s="9"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="9"/>
-      <c r="B9" s="9"/>
+      <c r="O8" s="22"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="41"/>
+      <c r="S8" s="42"/>
+      <c r="T8" s="42"/>
+      <c r="U8" s="42"/>
+      <c r="V8" s="42"/>
+      <c r="W8" s="43"/>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A9" s="8"/>
+      <c r="B9" s="31"/>
       <c r="C9" s="5" t="s">
         <v>14</v>
       </c>
       <c r="D9" s="1"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="9"/>
+      <c r="H9" s="8"/>
       <c r="I9" s="1"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
-      <c r="L9" s="8"/>
-      <c r="M9" s="9"/>
-    </row>
-    <row r="10" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="9"/>
-      <c r="B10" s="9"/>
+      <c r="O9" s="22"/>
+      <c r="Q9" s="8"/>
+      <c r="R9" s="44"/>
+      <c r="S9" s="50"/>
+      <c r="T9" s="50"/>
+      <c r="U9" s="50"/>
+      <c r="V9" s="50"/>
+      <c r="W9" s="46"/>
+    </row>
+    <row r="10" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="8"/>
+      <c r="B10" s="32"/>
       <c r="C10" s="5" t="s">
         <v>16</v>
       </c>
@@ -917,16 +1214,77 @@
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
-      <c r="M10" s="4"/>
-    </row>
-    <row r="11" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="23"/>
+      <c r="P10" s="3"/>
+      <c r="Q10" s="4"/>
+      <c r="R10" s="47"/>
+      <c r="S10" s="48"/>
+      <c r="T10" s="48"/>
+      <c r="U10" s="48"/>
+      <c r="V10" s="48"/>
+      <c r="W10" s="49"/>
+    </row>
+    <row r="11" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="O11" s="22"/>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="O12" s="22"/>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="O13" s="22"/>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="O14" s="22"/>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="O15" s="22"/>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="O16" s="22"/>
+    </row>
+    <row r="17" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O17" s="22"/>
+    </row>
+    <row r="18" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O18" s="22"/>
+    </row>
+    <row r="19" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O19" s="22"/>
+    </row>
+    <row r="20" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O20" s="22"/>
+    </row>
+    <row r="21" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O21" s="22"/>
+    </row>
+    <row r="22" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O22" s="22"/>
+    </row>
+    <row r="23" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O23" s="22"/>
+    </row>
+    <row r="24" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O24" s="22"/>
+    </row>
+    <row r="25" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O25" s="22"/>
+    </row>
+    <row r="26" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O26" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="7">
     <mergeCell ref="D3:H3"/>
-    <mergeCell ref="I3:M3"/>
+    <mergeCell ref="I3:Q3"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="R3:W4"/>
+    <mergeCell ref="R5:W7"/>
+    <mergeCell ref="R8:W10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Entrenamientos completados. Modificación de código
</commit_message>
<xml_diff>
--- a/modelos_tfg/MetricasValidacion.xlsx
+++ b/modelos_tfg/MetricasValidacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\modelos_tfg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F5011BA-E423-40F3-B2A8-037C9DF1B400}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DF3D416-492D-4D32-AF87-1A425AB32641}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="50">
   <si>
     <t>ID Train</t>
   </si>
@@ -130,6 +130,52 @@
   </si>
   <si>
     <t>V3</t>
+  </si>
+  <si>
+    <t>23 (ES)</t>
+  </si>
+  <si>
+    <t>V4</t>
+  </si>
+  <si>
+    <t>He ampliado el conjunto de datos</t>
+  </si>
+  <si>
+    <t>Limitado entre marzo y septiembre</t>
+  </si>
+  <si>
+    <t>16, 1</t>
+  </si>
+  <si>
+    <t>64, 32</t>
+  </si>
+  <si>
+    <t>38 (ES)</t>
+  </si>
+  <si>
+    <t>20 (ES)</t>
+  </si>
+  <si>
+    <t>He modificado el patience a 20</t>
+  </si>
+  <si>
+    <t>V5</t>
+  </si>
+  <si>
+    <t>He aumentado el patience a 50 y he bajado mucho más el LR.
+Además, he cambiado la arquitectura de los modelos</t>
+  </si>
+  <si>
+    <t>V6</t>
+  </si>
+  <si>
+    <t>65 (ES)</t>
+  </si>
+  <si>
+    <t>32, 16</t>
+  </si>
+  <si>
+    <t>50 (ES)</t>
   </si>
 </sst>
 </file>
@@ -443,7 +489,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -491,6 +537,47 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -512,15 +599,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -539,46 +617,40 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -926,7 +998,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:W26"/>
+  <dimension ref="A2:X26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.42578125" customWidth="1"/>
@@ -945,32 +1017,32 @@
   <sheetData>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="27"/>
-      <c r="I3" s="28" t="s">
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
-      <c r="M3" s="29"/>
-      <c r="N3" s="29"/>
-      <c r="O3" s="29"/>
-      <c r="P3" s="29"/>
-      <c r="Q3" s="30"/>
-      <c r="R3" s="35" t="s">
+      <c r="J3" s="46"/>
+      <c r="K3" s="46"/>
+      <c r="L3" s="46"/>
+      <c r="M3" s="46"/>
+      <c r="N3" s="46"/>
+      <c r="O3" s="46"/>
+      <c r="P3" s="46"/>
+      <c r="Q3" s="47"/>
+      <c r="R3" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="36"/>
-      <c r="T3" s="36"/>
-      <c r="U3" s="36"/>
-      <c r="V3" s="36"/>
-      <c r="W3" s="37"/>
+      <c r="S3" s="50"/>
+      <c r="T3" s="50"/>
+      <c r="U3" s="50"/>
+      <c r="V3" s="50"/>
+      <c r="W3" s="51"/>
     </row>
     <row r="4" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="20" t="s">
@@ -1021,16 +1093,16 @@
       <c r="Q4" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="38"/>
-      <c r="S4" s="39"/>
-      <c r="T4" s="39"/>
-      <c r="U4" s="39"/>
-      <c r="V4" s="39"/>
-      <c r="W4" s="40"/>
+      <c r="R4" s="52"/>
+      <c r="S4" s="53"/>
+      <c r="T4" s="53"/>
+      <c r="U4" s="53"/>
+      <c r="V4" s="53"/>
+      <c r="W4" s="54"/>
     </row>
     <row r="5" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="48" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -1078,16 +1150,18 @@
       <c r="Q5" s="17">
         <v>1E-3</v>
       </c>
-      <c r="R5" s="41"/>
-      <c r="S5" s="42"/>
-      <c r="T5" s="42"/>
-      <c r="U5" s="42"/>
-      <c r="V5" s="42"/>
-      <c r="W5" s="43"/>
+      <c r="R5" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="S5" s="31"/>
+      <c r="T5" s="31"/>
+      <c r="U5" s="31"/>
+      <c r="V5" s="31"/>
+      <c r="W5" s="32"/>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
-      <c r="B6" s="32"/>
+      <c r="B6" s="40"/>
       <c r="C6" s="5" t="s">
         <v>12</v>
       </c>
@@ -1109,7 +1183,7 @@
       <c r="I6" s="1">
         <v>18</v>
       </c>
-      <c r="J6" s="50">
+      <c r="J6">
         <v>128.26</v>
       </c>
       <c r="K6">
@@ -1133,16 +1207,16 @@
       <c r="Q6" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R6" s="44"/>
-      <c r="S6" s="45"/>
-      <c r="T6" s="45"/>
-      <c r="U6" s="45"/>
-      <c r="V6" s="45"/>
-      <c r="W6" s="46"/>
+      <c r="R6" s="33"/>
+      <c r="S6" s="34"/>
+      <c r="T6" s="34"/>
+      <c r="U6" s="34"/>
+      <c r="V6" s="34"/>
+      <c r="W6" s="35"/>
     </row>
     <row r="7" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8"/>
-      <c r="B7" s="33"/>
+      <c r="B7" s="41"/>
       <c r="C7" s="14" t="s">
         <v>14</v>
       </c>
@@ -1188,16 +1262,16 @@
       <c r="Q7" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R7" s="47"/>
-      <c r="S7" s="48"/>
-      <c r="T7" s="48"/>
-      <c r="U7" s="48"/>
-      <c r="V7" s="48"/>
-      <c r="W7" s="49"/>
+      <c r="R7" s="36"/>
+      <c r="S7" s="37"/>
+      <c r="T7" s="37"/>
+      <c r="U7" s="37"/>
+      <c r="V7" s="37"/>
+      <c r="W7" s="38"/>
     </row>
     <row r="8" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="39" t="s">
         <v>24</v>
       </c>
       <c r="C8" s="5" t="s">
@@ -1221,53 +1295,55 @@
       <c r="I8" s="1">
         <v>18</v>
       </c>
-      <c r="J8" s="50">
+      <c r="J8">
         <v>47.31</v>
       </c>
-      <c r="K8" s="50">
+      <c r="K8">
         <v>6</v>
       </c>
-      <c r="L8" s="50" t="s">
+      <c r="L8" t="s">
         <v>29</v>
       </c>
-      <c r="M8" s="50">
+      <c r="M8">
         <v>32</v>
       </c>
-      <c r="N8" s="50">
+      <c r="N8">
         <v>64</v>
       </c>
       <c r="O8" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="P8" s="50">
+      <c r="P8">
         <v>0.2</v>
       </c>
       <c r="Q8" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R8" s="41"/>
-      <c r="S8" s="42"/>
-      <c r="T8" s="42"/>
-      <c r="U8" s="42"/>
-      <c r="V8" s="42"/>
-      <c r="W8" s="43"/>
+      <c r="R8" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="S8" s="31"/>
+      <c r="T8" s="31"/>
+      <c r="U8" s="31"/>
+      <c r="V8" s="31"/>
+      <c r="W8" s="32"/>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
-      <c r="B9" s="32"/>
+      <c r="B9" s="40"/>
       <c r="C9" s="5" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="1">
         <v>169.54</v>
       </c>
-      <c r="E9" s="50">
+      <c r="E9">
         <v>443.73099999999999</v>
       </c>
-      <c r="F9" s="50">
+      <c r="F9">
         <v>0.80089999999999995</v>
       </c>
-      <c r="G9" s="50">
+      <c r="G9">
         <v>0.80049999999999999</v>
       </c>
       <c r="H9" s="8">
@@ -1276,10 +1352,10 @@
       <c r="I9" s="1">
         <v>18</v>
       </c>
-      <c r="J9" s="50">
+      <c r="J9">
         <v>95.75</v>
       </c>
-      <c r="K9" s="50">
+      <c r="K9">
         <v>6</v>
       </c>
       <c r="L9" t="s">
@@ -1300,16 +1376,16 @@
       <c r="Q9" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R9" s="44"/>
-      <c r="S9" s="45"/>
-      <c r="T9" s="45"/>
-      <c r="U9" s="45"/>
-      <c r="V9" s="45"/>
-      <c r="W9" s="46"/>
+      <c r="R9" s="33"/>
+      <c r="S9" s="34"/>
+      <c r="T9" s="34"/>
+      <c r="U9" s="34"/>
+      <c r="V9" s="34"/>
+      <c r="W9" s="35"/>
     </row>
     <row r="10" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8"/>
-      <c r="B10" s="33"/>
+      <c r="B10" s="41"/>
       <c r="C10" s="5" t="s">
         <v>14</v>
       </c>
@@ -1355,219 +1431,704 @@
       <c r="Q10" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R10" s="47"/>
-      <c r="S10" s="48"/>
-      <c r="T10" s="48"/>
-      <c r="U10" s="48"/>
-      <c r="V10" s="48"/>
-      <c r="W10" s="49"/>
+      <c r="R10" s="36"/>
+      <c r="S10" s="37"/>
+      <c r="T10" s="37"/>
+      <c r="U10" s="37"/>
+      <c r="V10" s="37"/>
+      <c r="W10" s="38"/>
     </row>
     <row r="11" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="52">
+      <c r="D11" s="1">
         <v>156.679</v>
       </c>
-      <c r="E11" s="50">
+      <c r="E11">
         <v>439.01499999999999</v>
       </c>
-      <c r="F11" s="50">
+      <c r="F11">
         <v>0.80510000000000004</v>
       </c>
-      <c r="G11" s="50">
+      <c r="G11">
         <v>0.80469999999999997</v>
       </c>
-      <c r="H11" s="53">
+      <c r="H11" s="8">
         <v>30</v>
       </c>
-      <c r="I11" s="52">
+      <c r="I11" s="1">
         <v>18</v>
       </c>
-      <c r="J11" s="50">
+      <c r="J11">
         <v>92.58</v>
       </c>
-      <c r="K11" s="50">
+      <c r="K11">
         <v>6</v>
       </c>
-      <c r="L11" s="50" t="s">
+      <c r="L11" t="s">
         <v>31</v>
       </c>
-      <c r="M11" s="51">
-        <v>64</v>
-      </c>
-      <c r="N11" s="50">
+      <c r="M11" s="25">
+        <v>64</v>
+      </c>
+      <c r="N11">
         <v>64</v>
       </c>
       <c r="O11" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="P11" s="51">
+      <c r="P11" s="25">
         <v>0.3</v>
       </c>
-      <c r="Q11" s="53">
+      <c r="Q11" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R11" s="41"/>
-      <c r="S11" s="42"/>
-      <c r="T11" s="42"/>
-      <c r="U11" s="42"/>
-      <c r="V11" s="42"/>
-      <c r="W11" s="43"/>
+      <c r="R11" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="S11" s="31"/>
+      <c r="T11" s="31"/>
+      <c r="U11" s="31"/>
+      <c r="V11" s="31"/>
+      <c r="W11" s="32"/>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B12" s="32"/>
-      <c r="C12" s="55" t="s">
+      <c r="B12" s="40"/>
+      <c r="C12" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="52">
+      <c r="D12" s="1">
         <v>208.43</v>
       </c>
-      <c r="E12" s="50">
+      <c r="E12">
         <v>527.37</v>
       </c>
-      <c r="F12" s="50">
+      <c r="F12">
         <v>0.71870000000000001</v>
       </c>
-      <c r="G12" s="50">
+      <c r="G12">
         <v>0.71819999999999995</v>
       </c>
-      <c r="H12" s="53">
+      <c r="H12" s="8">
         <v>87.8</v>
       </c>
-      <c r="I12" s="52">
+      <c r="I12" s="1">
         <v>18</v>
       </c>
-      <c r="J12" s="50">
+      <c r="J12">
         <v>55.35</v>
       </c>
-      <c r="K12" s="50">
+      <c r="K12">
         <v>6</v>
       </c>
-      <c r="L12" s="50" t="s">
+      <c r="L12" t="s">
         <v>32</v>
       </c>
-      <c r="M12" s="51">
-        <v>64</v>
-      </c>
-      <c r="N12" s="50">
+      <c r="M12" s="25">
+        <v>64</v>
+      </c>
+      <c r="N12">
         <v>64</v>
       </c>
       <c r="O12" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="P12" s="51">
+      <c r="P12" s="25">
         <v>0.3</v>
       </c>
-      <c r="Q12" s="53">
+      <c r="Q12" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R12" s="44"/>
-      <c r="S12" s="54"/>
-      <c r="T12" s="54"/>
-      <c r="U12" s="54"/>
-      <c r="V12" s="54"/>
-      <c r="W12" s="46"/>
+      <c r="R12" s="33"/>
+      <c r="S12" s="34"/>
+      <c r="T12" s="34"/>
+      <c r="U12" s="34"/>
+      <c r="V12" s="34"/>
+      <c r="W12" s="35"/>
     </row>
     <row r="13" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="32"/>
-      <c r="C13" s="56" t="s">
+      <c r="B13" s="40"/>
+      <c r="C13" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="57">
+      <c r="D13" s="2">
         <v>157.624</v>
       </c>
-      <c r="E13" s="58">
+      <c r="E13" s="3">
         <v>433.28500000000003</v>
       </c>
-      <c r="F13" s="58">
+      <c r="F13" s="3">
         <v>0.81010000000000004</v>
       </c>
-      <c r="G13" s="58">
+      <c r="G13" s="3">
         <v>0.80979999999999996</v>
       </c>
-      <c r="H13" s="59">
+      <c r="H13" s="4">
         <v>69.3</v>
       </c>
-      <c r="I13" s="57">
+      <c r="I13" s="2">
         <v>18</v>
       </c>
-      <c r="J13" s="58">
+      <c r="J13" s="3">
         <v>97.66</v>
       </c>
-      <c r="K13" s="58">
+      <c r="K13" s="3">
         <v>6</v>
       </c>
-      <c r="L13" s="58" t="s">
+      <c r="L13" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="M13" s="60">
-        <v>64</v>
-      </c>
-      <c r="N13" s="58">
+      <c r="M13" s="28">
+        <v>64</v>
+      </c>
+      <c r="N13" s="3">
         <v>64</v>
       </c>
       <c r="O13" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="P13" s="60">
+      <c r="P13" s="28">
         <v>0.3</v>
       </c>
       <c r="Q13" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R13" s="47"/>
-      <c r="S13" s="48"/>
-      <c r="T13" s="48"/>
-      <c r="U13" s="48"/>
-      <c r="V13" s="48"/>
-      <c r="W13" s="49"/>
+      <c r="R13" s="36"/>
+      <c r="S13" s="37"/>
+      <c r="T13" s="37"/>
+      <c r="U13" s="37"/>
+      <c r="V13" s="37"/>
+      <c r="W13" s="38"/>
     </row>
     <row r="14" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="9"/>
-      <c r="O14" s="22"/>
+      <c r="B14" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="1">
+        <v>46.762999999999998</v>
+      </c>
+      <c r="E14">
+        <v>100.31399999999999</v>
+      </c>
+      <c r="F14">
+        <v>0.94040000000000001</v>
+      </c>
+      <c r="G14">
+        <v>0.94030000000000002</v>
+      </c>
+      <c r="H14" s="8">
+        <v>30</v>
+      </c>
+      <c r="I14" s="1">
+        <v>18</v>
+      </c>
+      <c r="J14">
+        <v>90.56</v>
+      </c>
+      <c r="K14">
+        <v>6</v>
+      </c>
+      <c r="L14" t="s">
+        <v>35</v>
+      </c>
+      <c r="M14" s="73">
+        <v>64</v>
+      </c>
+      <c r="N14">
+        <v>64</v>
+      </c>
+      <c r="O14" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="P14" s="73">
+        <v>0.3</v>
+      </c>
+      <c r="Q14" s="8">
+        <v>1E-3</v>
+      </c>
+      <c r="R14" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="S14" s="31"/>
+      <c r="T14" s="31"/>
+      <c r="U14" s="31"/>
+      <c r="V14" s="31"/>
+      <c r="W14" s="32"/>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="O15" s="22"/>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="O16" s="22"/>
-    </row>
-    <row r="17" spans="15:15" x14ac:dyDescent="0.25">
-      <c r="O17" s="22"/>
-    </row>
-    <row r="18" spans="15:15" x14ac:dyDescent="0.25">
-      <c r="O18" s="22"/>
-    </row>
-    <row r="19" spans="15:15" x14ac:dyDescent="0.25">
-      <c r="O19" s="22"/>
-    </row>
-    <row r="20" spans="15:15" x14ac:dyDescent="0.25">
-      <c r="O20" s="22"/>
-    </row>
-    <row r="21" spans="15:15" x14ac:dyDescent="0.25">
-      <c r="O21" s="22"/>
-    </row>
-    <row r="22" spans="15:15" x14ac:dyDescent="0.25">
-      <c r="O22" s="22"/>
-    </row>
-    <row r="23" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="B15" s="40"/>
+      <c r="C15" s="55" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="1">
+        <v>71.069999999999993</v>
+      </c>
+      <c r="E15">
+        <v>127.996</v>
+      </c>
+      <c r="F15">
+        <v>0.90290000000000004</v>
+      </c>
+      <c r="G15">
+        <v>0.90280000000000005</v>
+      </c>
+      <c r="H15" s="8">
+        <v>87.8</v>
+      </c>
+      <c r="I15" s="1">
+        <v>18</v>
+      </c>
+      <c r="J15">
+        <v>116.5</v>
+      </c>
+      <c r="K15">
+        <v>6</v>
+      </c>
+      <c r="L15" t="s">
+        <v>32</v>
+      </c>
+      <c r="M15" s="73">
+        <v>64</v>
+      </c>
+      <c r="N15">
+        <v>64</v>
+      </c>
+      <c r="O15" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="P15" s="73">
+        <v>0.3</v>
+      </c>
+      <c r="Q15" s="8">
+        <v>1E-3</v>
+      </c>
+      <c r="R15" s="33"/>
+      <c r="S15" s="34"/>
+      <c r="T15" s="34"/>
+      <c r="U15" s="34"/>
+      <c r="V15" s="34"/>
+      <c r="W15" s="35"/>
+    </row>
+    <row r="16" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="41"/>
+      <c r="C16" s="56" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="3">
+        <v>77.900000000000006</v>
+      </c>
+      <c r="E16" s="3">
+        <v>136.596</v>
+      </c>
+      <c r="F16" s="3">
+        <v>0.88939999999999997</v>
+      </c>
+      <c r="G16" s="3">
+        <v>0.88929999999999998</v>
+      </c>
+      <c r="H16" s="4">
+        <v>69.3</v>
+      </c>
+      <c r="I16" s="2">
+        <v>18</v>
+      </c>
+      <c r="J16">
+        <v>104.68</v>
+      </c>
+      <c r="K16" s="3">
+        <v>6</v>
+      </c>
+      <c r="L16" t="s">
+        <v>32</v>
+      </c>
+      <c r="M16" s="66">
+        <v>64</v>
+      </c>
+      <c r="N16" s="3">
+        <v>64</v>
+      </c>
+      <c r="O16" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="P16" s="66">
+        <v>0.3</v>
+      </c>
+      <c r="Q16" s="3">
+        <v>1E-3</v>
+      </c>
+      <c r="R16" s="36"/>
+      <c r="S16" s="37"/>
+      <c r="T16" s="37"/>
+      <c r="U16" s="37"/>
+      <c r="V16" s="37"/>
+      <c r="W16" s="38"/>
+    </row>
+    <row r="17" spans="1:24" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="8"/>
+      <c r="B17" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" s="62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="57">
+        <v>48.356000000000002</v>
+      </c>
+      <c r="E17" s="57">
+        <v>103.378</v>
+      </c>
+      <c r="F17" s="57">
+        <v>0.93669999999999998</v>
+      </c>
+      <c r="G17" s="57">
+        <v>0.93659999999999999</v>
+      </c>
+      <c r="H17" s="63">
+        <v>23.1</v>
+      </c>
+      <c r="I17" s="59">
+        <v>18</v>
+      </c>
+      <c r="J17" s="9">
+        <v>142.66</v>
+      </c>
+      <c r="K17" s="57">
+        <v>6</v>
+      </c>
+      <c r="L17" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="M17" s="57">
+        <v>64</v>
+      </c>
+      <c r="N17" s="58">
+        <v>64</v>
+      </c>
+      <c r="O17" s="61" t="s">
+        <v>39</v>
+      </c>
+      <c r="P17" s="58">
+        <v>0.2</v>
+      </c>
+      <c r="Q17" s="70">
+        <v>1E-3</v>
+      </c>
+      <c r="R17" s="31" t="s">
+        <v>43</v>
+      </c>
+      <c r="S17" s="31"/>
+      <c r="T17" s="31"/>
+      <c r="U17" s="31"/>
+      <c r="V17" s="31"/>
+      <c r="W17" s="32"/>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A18" s="8"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="62" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="57">
+        <v>75.974000000000004</v>
+      </c>
+      <c r="E18" s="57">
+        <v>135.078</v>
+      </c>
+      <c r="F18" s="57">
+        <v>0.89190000000000003</v>
+      </c>
+      <c r="G18" s="57">
+        <v>0.80179999999999996</v>
+      </c>
+      <c r="H18" s="63">
+        <v>126.6</v>
+      </c>
+      <c r="I18" s="59">
+        <v>18</v>
+      </c>
+      <c r="J18" s="57">
+        <v>241.72</v>
+      </c>
+      <c r="K18" s="57">
+        <v>6</v>
+      </c>
+      <c r="L18" s="57" t="s">
+        <v>42</v>
+      </c>
+      <c r="M18" s="57">
+        <v>64</v>
+      </c>
+      <c r="N18" s="61" t="s">
+        <v>40</v>
+      </c>
+      <c r="O18" s="61" t="s">
+        <v>39</v>
+      </c>
+      <c r="P18" s="58">
+        <v>0.15</v>
+      </c>
+      <c r="Q18" s="63">
+        <v>1E-3</v>
+      </c>
+      <c r="R18" s="64"/>
+      <c r="S18" s="64"/>
+      <c r="T18" s="64"/>
+      <c r="U18" s="64"/>
+      <c r="V18" s="64"/>
+      <c r="W18" s="35"/>
+      <c r="X18" s="69"/>
+    </row>
+    <row r="19" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="8"/>
+      <c r="B19" s="38"/>
+      <c r="C19" s="65" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="66">
+        <v>86.263000000000005</v>
+      </c>
+      <c r="E19" s="66">
+        <v>136.91300000000001</v>
+      </c>
+      <c r="F19" s="66">
+        <v>0.88890000000000002</v>
+      </c>
+      <c r="G19" s="66">
+        <v>0.88880000000000003</v>
+      </c>
+      <c r="H19" s="67">
+        <v>96.6</v>
+      </c>
+      <c r="I19" s="3">
+        <v>18</v>
+      </c>
+      <c r="J19" s="3">
+        <v>263.45</v>
+      </c>
+      <c r="K19" s="66">
+        <v>6</v>
+      </c>
+      <c r="L19" s="66" t="s">
+        <v>42</v>
+      </c>
+      <c r="M19" s="66">
+        <v>64</v>
+      </c>
+      <c r="N19" s="68" t="s">
+        <v>40</v>
+      </c>
+      <c r="O19" s="68" t="s">
+        <v>39</v>
+      </c>
+      <c r="P19" s="28">
+        <v>0.15</v>
+      </c>
+      <c r="Q19" s="67">
+        <v>1E-3</v>
+      </c>
+      <c r="R19" s="37"/>
+      <c r="S19" s="37"/>
+      <c r="T19" s="37"/>
+      <c r="U19" s="37"/>
+      <c r="V19" s="37"/>
+      <c r="W19" s="38"/>
+    </row>
+    <row r="20" spans="1:24" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="8"/>
+      <c r="B20" s="39" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20" s="62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="57">
+        <v>51.14</v>
+      </c>
+      <c r="E20" s="57">
+        <v>107.42100000000001</v>
+      </c>
+      <c r="F20" s="57">
+        <v>9.9315999999999995</v>
+      </c>
+      <c r="G20" s="57">
+        <v>0.93149999999999999</v>
+      </c>
+      <c r="H20" s="8">
+        <v>23.1</v>
+      </c>
+      <c r="I20" s="57">
+        <v>18</v>
+      </c>
+      <c r="J20" s="57">
+        <v>241.78</v>
+      </c>
+      <c r="K20" s="57">
+        <v>6</v>
+      </c>
+      <c r="L20" s="57" t="s">
+        <v>47</v>
+      </c>
+      <c r="M20" s="57">
+        <v>64</v>
+      </c>
+      <c r="N20" s="60">
+        <v>64</v>
+      </c>
+      <c r="O20" s="60" t="s">
+        <v>39</v>
+      </c>
+      <c r="P20" s="58">
+        <v>0.2</v>
+      </c>
+      <c r="Q20" s="74">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R20" s="71" t="s">
+        <v>45</v>
+      </c>
+      <c r="S20" s="31"/>
+      <c r="T20" s="31"/>
+      <c r="U20" s="31"/>
+      <c r="V20" s="31"/>
+      <c r="W20" s="32"/>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A21" s="8"/>
+      <c r="B21" s="40"/>
+      <c r="C21" s="62" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" s="57">
+        <v>276.649</v>
+      </c>
+      <c r="E21" s="57">
+        <v>495.26499999999999</v>
+      </c>
+      <c r="F21" s="57">
+        <v>-0.45350000000000001</v>
+      </c>
+      <c r="G21" s="57">
+        <v>-0.4551</v>
+      </c>
+      <c r="H21" s="8">
+        <v>35.4</v>
+      </c>
+      <c r="I21" s="57">
+        <v>18</v>
+      </c>
+      <c r="J21" s="57">
+        <v>460.35</v>
+      </c>
+      <c r="K21" s="57">
+        <v>6</v>
+      </c>
+      <c r="L21" s="57" t="s">
+        <v>49</v>
+      </c>
+      <c r="M21" s="57">
+        <v>64</v>
+      </c>
+      <c r="N21" s="61" t="s">
+        <v>48</v>
+      </c>
+      <c r="O21" s="60" t="s">
+        <v>39</v>
+      </c>
+      <c r="P21" s="58">
+        <v>0.1</v>
+      </c>
+      <c r="Q21" s="75">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R21" s="33"/>
+      <c r="S21" s="34"/>
+      <c r="T21" s="34"/>
+      <c r="U21" s="34"/>
+      <c r="V21" s="34"/>
+      <c r="W21" s="35"/>
+    </row>
+    <row r="22" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="8"/>
+      <c r="B22" s="41"/>
+      <c r="C22" s="65" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="3">
+        <v>64.364999999999995</v>
+      </c>
+      <c r="E22" s="3">
+        <v>124.925</v>
+      </c>
+      <c r="F22" s="3">
+        <v>0.90749999999999997</v>
+      </c>
+      <c r="G22" s="3">
+        <v>0.90739999999999998</v>
+      </c>
+      <c r="H22" s="4">
+        <v>27.4</v>
+      </c>
+      <c r="I22" s="3">
+        <v>18</v>
+      </c>
+      <c r="J22" s="3">
+        <v>558.16</v>
+      </c>
+      <c r="K22" s="3">
+        <v>6</v>
+      </c>
+      <c r="L22" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="M22" s="3">
+        <v>64</v>
+      </c>
+      <c r="N22" s="68" t="s">
+        <v>48</v>
+      </c>
+      <c r="O22" s="72" t="s">
+        <v>39</v>
+      </c>
+      <c r="P22" s="28">
+        <v>0.1</v>
+      </c>
+      <c r="Q22" s="76">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R22" s="36"/>
+      <c r="S22" s="37"/>
+      <c r="T22" s="37"/>
+      <c r="U22" s="37"/>
+      <c r="V22" s="37"/>
+      <c r="W22" s="38"/>
+    </row>
+    <row r="23" spans="1:24" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="O23" s="22"/>
     </row>
-    <row r="24" spans="15:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
       <c r="O24" s="22"/>
     </row>
-    <row r="25" spans="15:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
       <c r="O25" s="22"/>
     </row>
-    <row r="26" spans="15:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
       <c r="O26" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="15">
+    <mergeCell ref="R17:W19"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="R20:W22"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="R14:W16"/>
+    <mergeCell ref="B14:B16"/>
     <mergeCell ref="B11:B13"/>
     <mergeCell ref="R11:W13"/>
     <mergeCell ref="D3:H3"/>

</xml_diff>

<commit_message>
Sigo con el entrenamiento
</commit_message>
<xml_diff>
--- a/modelos_tfg/MetricasValidacion.xlsx
+++ b/modelos_tfg/MetricasValidacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\modelos_tfg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DF3D416-492D-4D32-AF87-1A425AB32641}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E20C5A4-E67E-4E78-8DD1-01F4B586676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="62">
   <si>
     <t>ID Train</t>
   </si>
@@ -176,13 +176,51 @@
   </si>
   <si>
     <t>50 (ES)</t>
+  </si>
+  <si>
+    <t>V7</t>
+  </si>
+  <si>
+    <t>51 (ES)</t>
+  </si>
+  <si>
+    <t>84 (ES)</t>
+  </si>
+  <si>
+    <t>He añadido K.clear_session() para que borre los pesos del
+entrenamiento anterior</t>
+  </si>
+  <si>
+    <t>32, 16, 1</t>
+  </si>
+  <si>
+    <t>V8</t>
+  </si>
+  <si>
+    <t>77 (ES)</t>
+  </si>
+  <si>
+    <t>El patience sigue siendo el mismo</t>
+  </si>
+  <si>
+    <t>V9</t>
+  </si>
+  <si>
+    <t>53 (ES)</t>
+  </si>
+  <si>
+    <t>He aplicado un lr distinto a la RNN que a la LSTM y GRU.
+Además, he modificado la estructura de los modelos. Básicamente he combinado la V7 y V8</t>
+  </si>
+  <si>
+    <t>V10</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -202,6 +240,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -489,7 +534,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -542,115 +587,151 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -998,7 +1079,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:X26"/>
+  <dimension ref="A2:W35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.42578125" customWidth="1"/>
@@ -1017,32 +1098,32 @@
   <sheetData>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D3" s="42" t="s">
+      <c r="D3" s="72" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="44"/>
-      <c r="I3" s="45" t="s">
+      <c r="E3" s="73"/>
+      <c r="F3" s="73"/>
+      <c r="G3" s="73"/>
+      <c r="H3" s="74"/>
+      <c r="I3" s="75" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="46"/>
-      <c r="K3" s="46"/>
-      <c r="L3" s="46"/>
-      <c r="M3" s="46"/>
-      <c r="N3" s="46"/>
-      <c r="O3" s="46"/>
-      <c r="P3" s="46"/>
-      <c r="Q3" s="47"/>
-      <c r="R3" s="49" t="s">
+      <c r="J3" s="76"/>
+      <c r="K3" s="76"/>
+      <c r="L3" s="76"/>
+      <c r="M3" s="76"/>
+      <c r="N3" s="76"/>
+      <c r="O3" s="76"/>
+      <c r="P3" s="76"/>
+      <c r="Q3" s="77"/>
+      <c r="R3" s="79" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="50"/>
-      <c r="T3" s="50"/>
-      <c r="U3" s="50"/>
-      <c r="V3" s="50"/>
-      <c r="W3" s="51"/>
+      <c r="S3" s="80"/>
+      <c r="T3" s="80"/>
+      <c r="U3" s="80"/>
+      <c r="V3" s="80"/>
+      <c r="W3" s="81"/>
     </row>
     <row r="4" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="20" t="s">
@@ -1093,16 +1174,16 @@
       <c r="Q4" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="52"/>
-      <c r="S4" s="53"/>
-      <c r="T4" s="53"/>
-      <c r="U4" s="53"/>
-      <c r="V4" s="53"/>
-      <c r="W4" s="54"/>
+      <c r="R4" s="82"/>
+      <c r="S4" s="83"/>
+      <c r="T4" s="83"/>
+      <c r="U4" s="83"/>
+      <c r="V4" s="83"/>
+      <c r="W4" s="84"/>
     </row>
     <row r="5" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
-      <c r="B5" s="48" t="s">
+      <c r="B5" s="78" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -1132,7 +1213,7 @@
       <c r="K5" s="16">
         <v>6</v>
       </c>
-      <c r="L5" s="16" t="s">
+      <c r="L5" s="24" t="s">
         <v>26</v>
       </c>
       <c r="M5" s="16">
@@ -1150,18 +1231,18 @@
       <c r="Q5" s="17">
         <v>1E-3</v>
       </c>
-      <c r="R5" s="30" t="s">
+      <c r="R5" s="85" t="s">
         <v>38</v>
       </c>
-      <c r="S5" s="31"/>
-      <c r="T5" s="31"/>
-      <c r="U5" s="31"/>
-      <c r="V5" s="31"/>
-      <c r="W5" s="32"/>
+      <c r="S5" s="52"/>
+      <c r="T5" s="52"/>
+      <c r="U5" s="52"/>
+      <c r="V5" s="52"/>
+      <c r="W5" s="53"/>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
-      <c r="B6" s="40"/>
+      <c r="B6" s="49"/>
       <c r="C6" s="5" t="s">
         <v>12</v>
       </c>
@@ -1189,7 +1270,7 @@
       <c r="K6">
         <v>6</v>
       </c>
-      <c r="L6" t="s">
+      <c r="L6" s="32" t="s">
         <v>27</v>
       </c>
       <c r="M6">
@@ -1207,16 +1288,16 @@
       <c r="Q6" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R6" s="33"/>
-      <c r="S6" s="34"/>
-      <c r="T6" s="34"/>
-      <c r="U6" s="34"/>
-      <c r="V6" s="34"/>
-      <c r="W6" s="35"/>
+      <c r="R6" s="54"/>
+      <c r="S6" s="55"/>
+      <c r="T6" s="55"/>
+      <c r="U6" s="55"/>
+      <c r="V6" s="55"/>
+      <c r="W6" s="56"/>
     </row>
     <row r="7" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8"/>
-      <c r="B7" s="41"/>
+      <c r="B7" s="50"/>
       <c r="C7" s="14" t="s">
         <v>14</v>
       </c>
@@ -1244,7 +1325,7 @@
       <c r="K7" s="3">
         <v>6</v>
       </c>
-      <c r="L7" s="3" t="s">
+      <c r="L7" s="35" t="s">
         <v>28</v>
       </c>
       <c r="M7" s="3">
@@ -1262,16 +1343,16 @@
       <c r="Q7" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R7" s="36"/>
-      <c r="S7" s="37"/>
-      <c r="T7" s="37"/>
-      <c r="U7" s="37"/>
-      <c r="V7" s="37"/>
-      <c r="W7" s="38"/>
+      <c r="R7" s="57"/>
+      <c r="S7" s="58"/>
+      <c r="T7" s="58"/>
+      <c r="U7" s="58"/>
+      <c r="V7" s="58"/>
+      <c r="W7" s="59"/>
     </row>
     <row r="8" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
-      <c r="B8" s="39" t="s">
+      <c r="B8" s="48" t="s">
         <v>24</v>
       </c>
       <c r="C8" s="5" t="s">
@@ -1301,7 +1382,7 @@
       <c r="K8">
         <v>6</v>
       </c>
-      <c r="L8" t="s">
+      <c r="L8" s="32" t="s">
         <v>29</v>
       </c>
       <c r="M8">
@@ -1319,18 +1400,18 @@
       <c r="Q8" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R8" s="30" t="s">
+      <c r="R8" s="85" t="s">
         <v>38</v>
       </c>
-      <c r="S8" s="31"/>
-      <c r="T8" s="31"/>
-      <c r="U8" s="31"/>
-      <c r="V8" s="31"/>
-      <c r="W8" s="32"/>
+      <c r="S8" s="52"/>
+      <c r="T8" s="52"/>
+      <c r="U8" s="52"/>
+      <c r="V8" s="52"/>
+      <c r="W8" s="53"/>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
-      <c r="B9" s="40"/>
+      <c r="B9" s="49"/>
       <c r="C9" s="5" t="s">
         <v>12</v>
       </c>
@@ -1358,7 +1439,7 @@
       <c r="K9">
         <v>6</v>
       </c>
-      <c r="L9" t="s">
+      <c r="L9" s="32" t="s">
         <v>30</v>
       </c>
       <c r="M9">
@@ -1376,16 +1457,16 @@
       <c r="Q9" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R9" s="33"/>
-      <c r="S9" s="34"/>
-      <c r="T9" s="34"/>
-      <c r="U9" s="34"/>
-      <c r="V9" s="34"/>
-      <c r="W9" s="35"/>
+      <c r="R9" s="54"/>
+      <c r="S9" s="55"/>
+      <c r="T9" s="55"/>
+      <c r="U9" s="55"/>
+      <c r="V9" s="55"/>
+      <c r="W9" s="56"/>
     </row>
     <row r="10" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8"/>
-      <c r="B10" s="41"/>
+      <c r="B10" s="50"/>
       <c r="C10" s="5" t="s">
         <v>14</v>
       </c>
@@ -1413,7 +1494,7 @@
       <c r="K10" s="3">
         <v>6</v>
       </c>
-      <c r="L10" s="3" t="s">
+      <c r="L10" s="35" t="s">
         <v>29</v>
       </c>
       <c r="M10" s="3">
@@ -1431,15 +1512,15 @@
       <c r="Q10" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R10" s="36"/>
-      <c r="S10" s="37"/>
-      <c r="T10" s="37"/>
-      <c r="U10" s="37"/>
-      <c r="V10" s="37"/>
-      <c r="W10" s="38"/>
+      <c r="R10" s="57"/>
+      <c r="S10" s="58"/>
+      <c r="T10" s="58"/>
+      <c r="U10" s="58"/>
+      <c r="V10" s="58"/>
+      <c r="W10" s="59"/>
     </row>
     <row r="11" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="39" t="s">
+      <c r="B11" s="48" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="29" t="s">
@@ -1469,7 +1550,7 @@
       <c r="K11">
         <v>6</v>
       </c>
-      <c r="L11" t="s">
+      <c r="L11" s="32" t="s">
         <v>31</v>
       </c>
       <c r="M11" s="25">
@@ -1487,17 +1568,17 @@
       <c r="Q11" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R11" s="30" t="s">
+      <c r="R11" s="85" t="s">
         <v>38</v>
       </c>
-      <c r="S11" s="31"/>
-      <c r="T11" s="31"/>
-      <c r="U11" s="31"/>
-      <c r="V11" s="31"/>
-      <c r="W11" s="32"/>
+      <c r="S11" s="52"/>
+      <c r="T11" s="52"/>
+      <c r="U11" s="52"/>
+      <c r="V11" s="52"/>
+      <c r="W11" s="53"/>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B12" s="40"/>
+      <c r="B12" s="49"/>
       <c r="C12" s="26" t="s">
         <v>12</v>
       </c>
@@ -1525,7 +1606,7 @@
       <c r="K12">
         <v>6</v>
       </c>
-      <c r="L12" t="s">
+      <c r="L12" s="32" t="s">
         <v>32</v>
       </c>
       <c r="M12" s="25">
@@ -1543,15 +1624,15 @@
       <c r="Q12" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R12" s="33"/>
-      <c r="S12" s="34"/>
-      <c r="T12" s="34"/>
-      <c r="U12" s="34"/>
-      <c r="V12" s="34"/>
-      <c r="W12" s="35"/>
+      <c r="R12" s="54"/>
+      <c r="S12" s="55"/>
+      <c r="T12" s="55"/>
+      <c r="U12" s="55"/>
+      <c r="V12" s="55"/>
+      <c r="W12" s="56"/>
     </row>
     <row r="13" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="40"/>
+      <c r="B13" s="49"/>
       <c r="C13" s="27" t="s">
         <v>14</v>
       </c>
@@ -1579,7 +1660,7 @@
       <c r="K13" s="3">
         <v>6</v>
       </c>
-      <c r="L13" s="3" t="s">
+      <c r="L13" s="35" t="s">
         <v>33</v>
       </c>
       <c r="M13" s="28">
@@ -1597,15 +1678,15 @@
       <c r="Q13" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R13" s="36"/>
-      <c r="S13" s="37"/>
-      <c r="T13" s="37"/>
-      <c r="U13" s="37"/>
-      <c r="V13" s="37"/>
-      <c r="W13" s="38"/>
+      <c r="R13" s="57"/>
+      <c r="S13" s="58"/>
+      <c r="T13" s="58"/>
+      <c r="U13" s="58"/>
+      <c r="V13" s="58"/>
+      <c r="W13" s="59"/>
     </row>
     <row r="14" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="39" t="s">
+      <c r="B14" s="48" t="s">
         <v>36</v>
       </c>
       <c r="C14" s="20" t="s">
@@ -1635,10 +1716,10 @@
       <c r="K14">
         <v>6</v>
       </c>
-      <c r="L14" t="s">
+      <c r="L14" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="M14" s="73">
+      <c r="M14">
         <v>64</v>
       </c>
       <c r="N14">
@@ -1647,24 +1728,24 @@
       <c r="O14" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="P14" s="73">
+      <c r="P14">
         <v>0.3</v>
       </c>
       <c r="Q14" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R14" s="30" t="s">
+      <c r="R14" s="85" t="s">
         <v>37</v>
       </c>
-      <c r="S14" s="31"/>
-      <c r="T14" s="31"/>
-      <c r="U14" s="31"/>
-      <c r="V14" s="31"/>
-      <c r="W14" s="32"/>
+      <c r="S14" s="52"/>
+      <c r="T14" s="52"/>
+      <c r="U14" s="52"/>
+      <c r="V14" s="52"/>
+      <c r="W14" s="53"/>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B15" s="40"/>
-      <c r="C15" s="55" t="s">
+      <c r="B15" s="49"/>
+      <c r="C15" s="30" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="1">
@@ -1691,10 +1772,10 @@
       <c r="K15">
         <v>6</v>
       </c>
-      <c r="L15" t="s">
+      <c r="L15" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="M15" s="73">
+      <c r="M15">
         <v>64</v>
       </c>
       <c r="N15">
@@ -1703,22 +1784,22 @@
       <c r="O15" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="P15" s="73">
+      <c r="P15">
         <v>0.3</v>
       </c>
       <c r="Q15" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R15" s="33"/>
-      <c r="S15" s="34"/>
-      <c r="T15" s="34"/>
-      <c r="U15" s="34"/>
-      <c r="V15" s="34"/>
-      <c r="W15" s="35"/>
+      <c r="R15" s="54"/>
+      <c r="S15" s="55"/>
+      <c r="T15" s="55"/>
+      <c r="U15" s="55"/>
+      <c r="V15" s="55"/>
+      <c r="W15" s="56"/>
     </row>
     <row r="16" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="41"/>
-      <c r="C16" s="56" t="s">
+      <c r="B16" s="50"/>
+      <c r="C16" s="31" t="s">
         <v>14</v>
       </c>
       <c r="D16" s="3">
@@ -1745,10 +1826,10 @@
       <c r="K16" s="3">
         <v>6</v>
       </c>
-      <c r="L16" t="s">
+      <c r="L16" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="M16" s="66">
+      <c r="M16" s="3">
         <v>64</v>
       </c>
       <c r="N16" s="3">
@@ -1757,153 +1838,152 @@
       <c r="O16" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="P16" s="66">
+      <c r="P16" s="3">
         <v>0.3</v>
       </c>
       <c r="Q16" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R16" s="36"/>
-      <c r="S16" s="37"/>
-      <c r="T16" s="37"/>
-      <c r="U16" s="37"/>
-      <c r="V16" s="37"/>
-      <c r="W16" s="38"/>
-    </row>
-    <row r="17" spans="1:24" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="R16" s="57"/>
+      <c r="S16" s="58"/>
+      <c r="T16" s="58"/>
+      <c r="U16" s="58"/>
+      <c r="V16" s="58"/>
+      <c r="W16" s="59"/>
+    </row>
+    <row r="17" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
-      <c r="B17" s="32" t="s">
+      <c r="B17" s="53" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="62" t="s">
+      <c r="C17" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="D17" s="57">
+      <c r="D17">
         <v>48.356000000000002</v>
       </c>
-      <c r="E17" s="57">
+      <c r="E17">
         <v>103.378</v>
       </c>
-      <c r="F17" s="57">
+      <c r="F17">
         <v>0.93669999999999998</v>
       </c>
-      <c r="G17" s="57">
+      <c r="G17">
         <v>0.93659999999999999</v>
       </c>
-      <c r="H17" s="63">
+      <c r="H17" s="8">
         <v>23.1</v>
       </c>
-      <c r="I17" s="59">
+      <c r="I17" s="1">
         <v>18</v>
       </c>
       <c r="J17" s="9">
         <v>142.66</v>
       </c>
-      <c r="K17" s="57">
-        <v>6</v>
-      </c>
-      <c r="L17" s="9" t="s">
+      <c r="K17">
+        <v>6</v>
+      </c>
+      <c r="L17" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="M17" s="57">
-        <v>64</v>
-      </c>
-      <c r="N17" s="58">
-        <v>64</v>
-      </c>
-      <c r="O17" s="61" t="s">
+      <c r="M17">
+        <v>64</v>
+      </c>
+      <c r="N17" s="25">
+        <v>64</v>
+      </c>
+      <c r="O17" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="P17" s="58">
+      <c r="P17" s="25">
         <v>0.2</v>
       </c>
-      <c r="Q17" s="70">
+      <c r="Q17" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R17" s="31" t="s">
+      <c r="R17" s="52" t="s">
         <v>43</v>
       </c>
-      <c r="S17" s="31"/>
-      <c r="T17" s="31"/>
-      <c r="U17" s="31"/>
-      <c r="V17" s="31"/>
-      <c r="W17" s="32"/>
-    </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="S17" s="52"/>
+      <c r="T17" s="52"/>
+      <c r="U17" s="52"/>
+      <c r="V17" s="52"/>
+      <c r="W17" s="53"/>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
-      <c r="B18" s="35"/>
-      <c r="C18" s="62" t="s">
+      <c r="B18" s="56"/>
+      <c r="C18" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="D18" s="57">
+      <c r="D18">
         <v>75.974000000000004</v>
       </c>
-      <c r="E18" s="57">
+      <c r="E18">
         <v>135.078</v>
       </c>
-      <c r="F18" s="57">
+      <c r="F18">
         <v>0.89190000000000003</v>
       </c>
-      <c r="G18" s="57">
+      <c r="G18">
         <v>0.80179999999999996</v>
       </c>
-      <c r="H18" s="63">
+      <c r="H18" s="8">
         <v>126.6</v>
       </c>
-      <c r="I18" s="59">
+      <c r="I18" s="1">
         <v>18</v>
       </c>
-      <c r="J18" s="57">
+      <c r="J18">
         <v>241.72</v>
       </c>
-      <c r="K18" s="57">
-        <v>6</v>
-      </c>
-      <c r="L18" s="57" t="s">
+      <c r="K18">
+        <v>6</v>
+      </c>
+      <c r="L18" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="M18" s="57">
-        <v>64</v>
-      </c>
-      <c r="N18" s="61" t="s">
+      <c r="M18">
+        <v>64</v>
+      </c>
+      <c r="N18" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="O18" s="61" t="s">
+      <c r="O18" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="P18" s="58">
+      <c r="P18" s="25">
         <v>0.15</v>
       </c>
-      <c r="Q18" s="63">
+      <c r="Q18" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R18" s="64"/>
-      <c r="S18" s="64"/>
-      <c r="T18" s="64"/>
-      <c r="U18" s="64"/>
-      <c r="V18" s="64"/>
-      <c r="W18" s="35"/>
-      <c r="X18" s="69"/>
-    </row>
-    <row r="19" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R18" s="55"/>
+      <c r="S18" s="55"/>
+      <c r="T18" s="55"/>
+      <c r="U18" s="55"/>
+      <c r="V18" s="55"/>
+      <c r="W18" s="56"/>
+    </row>
+    <row r="19" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8"/>
-      <c r="B19" s="38"/>
-      <c r="C19" s="65" t="s">
+      <c r="B19" s="59"/>
+      <c r="C19" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="66">
+      <c r="D19" s="3">
         <v>86.263000000000005</v>
       </c>
-      <c r="E19" s="66">
+      <c r="E19" s="3">
         <v>136.91300000000001</v>
       </c>
-      <c r="F19" s="66">
+      <c r="F19" s="3">
         <v>0.88890000000000002</v>
       </c>
-      <c r="G19" s="66">
+      <c r="G19" s="3">
         <v>0.88880000000000003</v>
       </c>
-      <c r="H19" s="67">
+      <c r="H19" s="4">
         <v>96.6</v>
       </c>
       <c r="I19" s="3">
@@ -1912,152 +1992,152 @@
       <c r="J19" s="3">
         <v>263.45</v>
       </c>
-      <c r="K19" s="66">
-        <v>6</v>
-      </c>
-      <c r="L19" s="66" t="s">
+      <c r="K19" s="3">
+        <v>6</v>
+      </c>
+      <c r="L19" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="M19" s="66">
-        <v>64</v>
-      </c>
-      <c r="N19" s="68" t="s">
+      <c r="M19" s="3">
+        <v>64</v>
+      </c>
+      <c r="N19" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="O19" s="68" t="s">
+      <c r="O19" s="34" t="s">
         <v>39</v>
       </c>
       <c r="P19" s="28">
         <v>0.15</v>
       </c>
-      <c r="Q19" s="67">
+      <c r="Q19" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R19" s="37"/>
-      <c r="S19" s="37"/>
-      <c r="T19" s="37"/>
-      <c r="U19" s="37"/>
-      <c r="V19" s="37"/>
-      <c r="W19" s="38"/>
-    </row>
-    <row r="20" spans="1:24" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="R19" s="58"/>
+      <c r="S19" s="58"/>
+      <c r="T19" s="58"/>
+      <c r="U19" s="58"/>
+      <c r="V19" s="58"/>
+      <c r="W19" s="59"/>
+    </row>
+    <row r="20" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8"/>
-      <c r="B20" s="39" t="s">
+      <c r="B20" s="48" t="s">
         <v>46</v>
       </c>
-      <c r="C20" s="62" t="s">
+      <c r="C20" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="D20" s="57">
+      <c r="D20">
         <v>51.14</v>
       </c>
-      <c r="E20" s="57">
+      <c r="E20">
         <v>107.42100000000001</v>
       </c>
-      <c r="F20" s="57">
+      <c r="F20">
         <v>9.9315999999999995</v>
       </c>
-      <c r="G20" s="57">
+      <c r="G20">
         <v>0.93149999999999999</v>
       </c>
       <c r="H20" s="8">
         <v>23.1</v>
       </c>
-      <c r="I20" s="57">
+      <c r="I20">
         <v>18</v>
       </c>
-      <c r="J20" s="57">
+      <c r="J20">
         <v>241.78</v>
       </c>
-      <c r="K20" s="57">
-        <v>6</v>
-      </c>
-      <c r="L20" s="57" t="s">
+      <c r="K20">
+        <v>6</v>
+      </c>
+      <c r="L20" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="M20" s="57">
-        <v>64</v>
-      </c>
-      <c r="N20" s="60">
-        <v>64</v>
-      </c>
-      <c r="O20" s="60" t="s">
+      <c r="M20">
+        <v>64</v>
+      </c>
+      <c r="N20" s="32">
+        <v>64</v>
+      </c>
+      <c r="O20" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P20" s="58">
+      <c r="P20" s="25">
         <v>0.2</v>
       </c>
-      <c r="Q20" s="74">
+      <c r="Q20" s="36">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R20" s="71" t="s">
+      <c r="R20" s="51" t="s">
         <v>45</v>
       </c>
-      <c r="S20" s="31"/>
-      <c r="T20" s="31"/>
-      <c r="U20" s="31"/>
-      <c r="V20" s="31"/>
-      <c r="W20" s="32"/>
-    </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="S20" s="52"/>
+      <c r="T20" s="52"/>
+      <c r="U20" s="52"/>
+      <c r="V20" s="52"/>
+      <c r="W20" s="53"/>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
-      <c r="B21" s="40"/>
-      <c r="C21" s="62" t="s">
+      <c r="B21" s="49"/>
+      <c r="C21" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="57">
+      <c r="D21">
         <v>276.649</v>
       </c>
-      <c r="E21" s="57">
+      <c r="E21">
         <v>495.26499999999999</v>
       </c>
-      <c r="F21" s="57">
+      <c r="F21" s="41">
         <v>-0.45350000000000001</v>
       </c>
-      <c r="G21" s="57">
+      <c r="G21" s="41">
         <v>-0.4551</v>
       </c>
       <c r="H21" s="8">
         <v>35.4</v>
       </c>
-      <c r="I21" s="57">
+      <c r="I21">
         <v>18</v>
       </c>
-      <c r="J21" s="57">
+      <c r="J21">
         <v>460.35</v>
       </c>
-      <c r="K21" s="57">
-        <v>6</v>
-      </c>
-      <c r="L21" s="57" t="s">
+      <c r="K21">
+        <v>6</v>
+      </c>
+      <c r="L21" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="M21" s="57">
-        <v>64</v>
-      </c>
-      <c r="N21" s="61" t="s">
+      <c r="M21">
+        <v>64</v>
+      </c>
+      <c r="N21" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="O21" s="60" t="s">
+      <c r="O21" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P21" s="58">
+      <c r="P21" s="25">
         <v>0.1</v>
       </c>
-      <c r="Q21" s="75">
+      <c r="Q21" s="37">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R21" s="33"/>
-      <c r="S21" s="34"/>
-      <c r="T21" s="34"/>
-      <c r="U21" s="34"/>
-      <c r="V21" s="34"/>
-      <c r="W21" s="35"/>
-    </row>
-    <row r="22" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R21" s="54"/>
+      <c r="S21" s="55"/>
+      <c r="T21" s="55"/>
+      <c r="U21" s="55"/>
+      <c r="V21" s="55"/>
+      <c r="W21" s="56"/>
+    </row>
+    <row r="22" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="8"/>
-      <c r="B22" s="41"/>
-      <c r="C22" s="65" t="s">
+      <c r="B22" s="50"/>
+      <c r="C22" s="31" t="s">
         <v>14</v>
       </c>
       <c r="D22" s="3">
@@ -2084,53 +2164,677 @@
       <c r="K22" s="3">
         <v>6</v>
       </c>
-      <c r="L22" s="3" t="s">
+      <c r="L22" s="35" t="s">
         <v>49</v>
       </c>
       <c r="M22" s="3">
         <v>64</v>
       </c>
-      <c r="N22" s="68" t="s">
+      <c r="N22" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="O22" s="72" t="s">
+      <c r="O22" s="35" t="s">
         <v>39</v>
       </c>
       <c r="P22" s="28">
         <v>0.1</v>
       </c>
-      <c r="Q22" s="76">
+      <c r="Q22" s="38">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R22" s="36"/>
-      <c r="S22" s="37"/>
-      <c r="T22" s="37"/>
-      <c r="U22" s="37"/>
-      <c r="V22" s="37"/>
-      <c r="W22" s="38"/>
-    </row>
-    <row r="23" spans="1:24" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="O23" s="22"/>
-    </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="O24" s="22"/>
-    </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="O25" s="22"/>
-    </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="O26" s="22"/>
-    </row>
+      <c r="R22" s="57"/>
+      <c r="S22" s="58"/>
+      <c r="T22" s="58"/>
+      <c r="U22" s="58"/>
+      <c r="V22" s="58"/>
+      <c r="W22" s="59"/>
+    </row>
+    <row r="23" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="8"/>
+      <c r="B23" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="9">
+        <v>276.649</v>
+      </c>
+      <c r="E23" s="39">
+        <v>495265</v>
+      </c>
+      <c r="F23" s="42">
+        <v>-0.45350000000000001</v>
+      </c>
+      <c r="G23" s="42">
+        <v>-0.4551</v>
+      </c>
+      <c r="H23" s="10">
+        <v>23.1</v>
+      </c>
+      <c r="I23" s="9">
+        <v>18</v>
+      </c>
+      <c r="J23" s="9">
+        <v>219.42</v>
+      </c>
+      <c r="K23" s="9">
+        <v>6</v>
+      </c>
+      <c r="L23" s="40" t="s">
+        <v>51</v>
+      </c>
+      <c r="M23" s="9">
+        <v>64</v>
+      </c>
+      <c r="N23" s="40">
+        <v>64</v>
+      </c>
+      <c r="O23" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="P23" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="Q23" s="10">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R23" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="S23" s="52"/>
+      <c r="T23" s="52"/>
+      <c r="U23" s="52"/>
+      <c r="V23" s="52"/>
+      <c r="W23" s="53"/>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A24" s="8"/>
+      <c r="B24" s="49"/>
+      <c r="C24" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24">
+        <v>51.393000000000001</v>
+      </c>
+      <c r="E24">
+        <v>110.699</v>
+      </c>
+      <c r="F24">
+        <v>0.9274</v>
+      </c>
+      <c r="G24">
+        <v>0.92730000000000001</v>
+      </c>
+      <c r="H24" s="8">
+        <v>35.4</v>
+      </c>
+      <c r="I24">
+        <v>18</v>
+      </c>
+      <c r="J24">
+        <v>1003.15</v>
+      </c>
+      <c r="K24">
+        <v>6</v>
+      </c>
+      <c r="L24" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="M24">
+        <v>64</v>
+      </c>
+      <c r="N24" s="32" t="s">
+        <v>48</v>
+      </c>
+      <c r="O24" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="P24">
+        <v>0.1</v>
+      </c>
+      <c r="Q24" s="8">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R24" s="54"/>
+      <c r="S24" s="55"/>
+      <c r="T24" s="55"/>
+      <c r="U24" s="55"/>
+      <c r="V24" s="55"/>
+      <c r="W24" s="56"/>
+    </row>
+    <row r="25" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="8"/>
+      <c r="B25" s="50"/>
+      <c r="C25" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="3">
+        <v>78.093000000000004</v>
+      </c>
+      <c r="E25" s="3">
+        <v>153.08199999999999</v>
+      </c>
+      <c r="F25" s="3">
+        <v>0.86109999999999998</v>
+      </c>
+      <c r="G25" s="3">
+        <v>0.86099999999999999</v>
+      </c>
+      <c r="H25" s="4">
+        <v>27.4</v>
+      </c>
+      <c r="I25" s="3">
+        <v>18</v>
+      </c>
+      <c r="J25" s="3">
+        <v>657.69</v>
+      </c>
+      <c r="K25" s="3">
+        <v>6</v>
+      </c>
+      <c r="L25" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="M25" s="3">
+        <v>64</v>
+      </c>
+      <c r="N25" s="35" t="s">
+        <v>48</v>
+      </c>
+      <c r="O25" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="P25" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="Q25" s="4">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R25" s="57"/>
+      <c r="S25" s="58"/>
+      <c r="T25" s="58"/>
+      <c r="U25" s="58"/>
+      <c r="V25" s="58"/>
+      <c r="W25" s="59"/>
+    </row>
+    <row r="26" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="8"/>
+      <c r="B26" s="48" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="9">
+        <v>47.706000000000003</v>
+      </c>
+      <c r="E26" s="9">
+        <v>101.812</v>
+      </c>
+      <c r="F26" s="9">
+        <v>0.93859999999999999</v>
+      </c>
+      <c r="G26" s="9">
+        <v>0.9385</v>
+      </c>
+      <c r="H26" s="10">
+        <v>29.3</v>
+      </c>
+      <c r="I26" s="9">
+        <v>18</v>
+      </c>
+      <c r="J26" s="9">
+        <v>360.29</v>
+      </c>
+      <c r="K26" s="9">
+        <v>6</v>
+      </c>
+      <c r="L26" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="M26" s="9">
+        <v>64</v>
+      </c>
+      <c r="N26" s="9">
+        <v>64</v>
+      </c>
+      <c r="O26" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="P26" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="Q26" s="36">
+        <v>1E-3</v>
+      </c>
+      <c r="R26" s="85" t="s">
+        <v>57</v>
+      </c>
+      <c r="S26" s="52"/>
+      <c r="T26" s="52"/>
+      <c r="U26" s="52"/>
+      <c r="V26" s="52"/>
+      <c r="W26" s="53"/>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A27" s="8"/>
+      <c r="B27" s="49"/>
+      <c r="C27" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27">
+        <v>276.649</v>
+      </c>
+      <c r="E27">
+        <v>495.26499999999999</v>
+      </c>
+      <c r="F27" s="41">
+        <v>-0.45350000000000001</v>
+      </c>
+      <c r="G27" s="41">
+        <v>-0.4551</v>
+      </c>
+      <c r="H27" s="8">
+        <v>126.6</v>
+      </c>
+      <c r="I27">
+        <v>18</v>
+      </c>
+      <c r="J27">
+        <v>619.63</v>
+      </c>
+      <c r="K27">
+        <v>6</v>
+      </c>
+      <c r="L27" s="32" t="s">
+        <v>49</v>
+      </c>
+      <c r="M27">
+        <v>64</v>
+      </c>
+      <c r="N27" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="O27" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="P27">
+        <v>0.1</v>
+      </c>
+      <c r="Q27" s="37">
+        <v>1E-3</v>
+      </c>
+      <c r="R27" s="54"/>
+      <c r="S27" s="55"/>
+      <c r="T27" s="55"/>
+      <c r="U27" s="55"/>
+      <c r="V27" s="55"/>
+      <c r="W27" s="56"/>
+    </row>
+    <row r="28" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="8"/>
+      <c r="B28" s="50"/>
+      <c r="C28" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="3">
+        <v>74.569999999999993</v>
+      </c>
+      <c r="E28" s="3">
+        <v>145.054</v>
+      </c>
+      <c r="F28" s="3">
+        <v>0.97529999999999994</v>
+      </c>
+      <c r="G28" s="3">
+        <v>0.87519999999999998</v>
+      </c>
+      <c r="H28" s="4">
+        <v>96.6</v>
+      </c>
+      <c r="I28" s="3">
+        <v>18</v>
+      </c>
+      <c r="J28" s="3">
+        <v>764.03</v>
+      </c>
+      <c r="K28" s="3">
+        <v>6</v>
+      </c>
+      <c r="L28" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="M28" s="3">
+        <v>64</v>
+      </c>
+      <c r="N28" s="34" t="s">
+        <v>40</v>
+      </c>
+      <c r="O28" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="P28" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="Q28" s="38">
+        <v>1E-3</v>
+      </c>
+      <c r="R28" s="57"/>
+      <c r="S28" s="58"/>
+      <c r="T28" s="58"/>
+      <c r="U28" s="58"/>
+      <c r="V28" s="58"/>
+      <c r="W28" s="59"/>
+    </row>
+    <row r="29" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="48" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" s="9">
+        <v>49.481000000000002</v>
+      </c>
+      <c r="E29" s="9">
+        <v>104.151</v>
+      </c>
+      <c r="F29" s="9">
+        <v>0.93569999999999998</v>
+      </c>
+      <c r="G29" s="9">
+        <v>0.93569999999999998</v>
+      </c>
+      <c r="H29" s="10">
+        <v>23.1</v>
+      </c>
+      <c r="I29" s="9">
+        <v>18</v>
+      </c>
+      <c r="J29" s="9">
+        <v>222.14</v>
+      </c>
+      <c r="K29" s="9">
+        <v>6</v>
+      </c>
+      <c r="L29" s="40" t="s">
+        <v>59</v>
+      </c>
+      <c r="M29" s="9">
+        <v>64</v>
+      </c>
+      <c r="N29" s="9">
+        <v>64</v>
+      </c>
+      <c r="O29" s="44" t="s">
+        <v>39</v>
+      </c>
+      <c r="P29" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="Q29" s="10">
+        <v>1E-3</v>
+      </c>
+      <c r="R29" s="51" t="s">
+        <v>60</v>
+      </c>
+      <c r="S29" s="52"/>
+      <c r="T29" s="52"/>
+      <c r="U29" s="52"/>
+      <c r="V29" s="52"/>
+      <c r="W29" s="53"/>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A30" s="8"/>
+      <c r="B30" s="49"/>
+      <c r="C30" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30">
+        <v>80.540999999999997</v>
+      </c>
+      <c r="E30">
+        <v>144.51499999999999</v>
+      </c>
+      <c r="F30">
+        <v>0.87619999999999998</v>
+      </c>
+      <c r="G30">
+        <v>0.87609999999999999</v>
+      </c>
+      <c r="H30" s="8">
+        <v>35.4</v>
+      </c>
+      <c r="I30">
+        <v>18</v>
+      </c>
+      <c r="J30">
+        <v>427.08</v>
+      </c>
+      <c r="K30">
+        <v>6</v>
+      </c>
+      <c r="L30" s="32" t="s">
+        <v>49</v>
+      </c>
+      <c r="M30">
+        <v>64</v>
+      </c>
+      <c r="N30" s="33" t="s">
+        <v>48</v>
+      </c>
+      <c r="O30" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="P30">
+        <v>0.1</v>
+      </c>
+      <c r="Q30" s="8">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R30" s="54"/>
+      <c r="S30" s="55"/>
+      <c r="T30" s="55"/>
+      <c r="U30" s="55"/>
+      <c r="V30" s="55"/>
+      <c r="W30" s="56"/>
+    </row>
+    <row r="31" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="8"/>
+      <c r="B31" s="50"/>
+      <c r="C31" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31" s="3">
+        <v>78.808000000000007</v>
+      </c>
+      <c r="E31" s="3">
+        <v>140.17099999999999</v>
+      </c>
+      <c r="F31" s="3">
+        <v>0.88360000000000005</v>
+      </c>
+      <c r="G31" s="3">
+        <v>0.88339999999999996</v>
+      </c>
+      <c r="H31" s="4">
+        <v>27.4</v>
+      </c>
+      <c r="I31" s="3">
+        <v>18</v>
+      </c>
+      <c r="J31" s="3">
+        <v>460.56</v>
+      </c>
+      <c r="K31" s="3">
+        <v>6</v>
+      </c>
+      <c r="L31" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="M31" s="3">
+        <v>64</v>
+      </c>
+      <c r="N31" s="34" t="s">
+        <v>48</v>
+      </c>
+      <c r="O31" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="P31" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="Q31" s="4">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R31" s="57"/>
+      <c r="S31" s="58"/>
+      <c r="T31" s="58"/>
+      <c r="U31" s="58"/>
+      <c r="V31" s="58"/>
+      <c r="W31" s="59"/>
+    </row>
+    <row r="32" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="60" t="s">
+        <v>61</v>
+      </c>
+      <c r="C32" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="45">
+        <v>30</v>
+      </c>
+      <c r="J32" s="9">
+        <v>260.20999999999998</v>
+      </c>
+      <c r="K32" s="9">
+        <v>6</v>
+      </c>
+      <c r="L32" s="40" t="s">
+        <v>59</v>
+      </c>
+      <c r="M32" s="9">
+        <v>64</v>
+      </c>
+      <c r="N32" s="9">
+        <v>64</v>
+      </c>
+      <c r="O32" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="P32" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="Q32" s="10">
+        <v>1E-3</v>
+      </c>
+      <c r="R32" s="63"/>
+      <c r="S32" s="64"/>
+      <c r="T32" s="64"/>
+      <c r="U32" s="64"/>
+      <c r="V32" s="64"/>
+      <c r="W32" s="65"/>
+    </row>
+    <row r="33" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B33" s="61"/>
+      <c r="C33" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="H33" s="8"/>
+      <c r="I33" s="46">
+        <v>30</v>
+      </c>
+      <c r="J33" s="86">
+        <v>667.58</v>
+      </c>
+      <c r="K33">
+        <v>6</v>
+      </c>
+      <c r="L33" s="32" t="s">
+        <v>49</v>
+      </c>
+      <c r="M33">
+        <v>64</v>
+      </c>
+      <c r="N33" s="32" t="s">
+        <v>48</v>
+      </c>
+      <c r="O33" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="P33">
+        <v>0.1</v>
+      </c>
+      <c r="Q33" s="8">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R33" s="66"/>
+      <c r="S33" s="67"/>
+      <c r="T33" s="67"/>
+      <c r="U33" s="67"/>
+      <c r="V33" s="67"/>
+      <c r="W33" s="68"/>
+    </row>
+    <row r="34" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="62"/>
+      <c r="C34" s="43" t="s">
+        <v>14</v>
+      </c>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="47">
+        <v>30</v>
+      </c>
+      <c r="J34" s="3"/>
+      <c r="K34" s="3">
+        <v>6</v>
+      </c>
+      <c r="L34" s="35"/>
+      <c r="M34" s="3">
+        <v>64</v>
+      </c>
+      <c r="N34" s="35" t="s">
+        <v>48</v>
+      </c>
+      <c r="O34" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="P34" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="Q34" s="4">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R34" s="69"/>
+      <c r="S34" s="70"/>
+      <c r="T34" s="70"/>
+      <c r="U34" s="70"/>
+      <c r="V34" s="70"/>
+      <c r="W34" s="71"/>
+    </row>
+    <row r="35" spans="2:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="23">
+    <mergeCell ref="R11:W13"/>
     <mergeCell ref="R17:W19"/>
     <mergeCell ref="B17:B19"/>
     <mergeCell ref="R20:W22"/>
     <mergeCell ref="B20:B22"/>
     <mergeCell ref="R14:W16"/>
     <mergeCell ref="B14:B16"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="R11:W13"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="R29:W31"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="R32:W34"/>
     <mergeCell ref="D3:H3"/>
     <mergeCell ref="I3:Q3"/>
     <mergeCell ref="B5:B7"/>
@@ -2138,8 +2842,14 @@
     <mergeCell ref="R3:W4"/>
     <mergeCell ref="R5:W7"/>
     <mergeCell ref="R8:W10"/>
+    <mergeCell ref="B23:B25"/>
+    <mergeCell ref="R23:W25"/>
+    <mergeCell ref="B26:B28"/>
+    <mergeCell ref="R26:W28"/>
+    <mergeCell ref="B11:B13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Entrenamiento con 1 día de ventana
</commit_message>
<xml_diff>
--- a/modelos_tfg/MetricasValidacion.xlsx
+++ b/modelos_tfg/MetricasValidacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\modelos_tfg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59343658-D81E-446C-8876-678F04938D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{090B1B97-CCE6-4858-B037-CFC7FB4C4A5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="70">
   <si>
     <t>ID Train</t>
   </si>
@@ -217,6 +217,28 @@
   </si>
   <si>
     <t>Simplemente he modificado el seq_length</t>
+  </si>
+  <si>
+    <t>V11</t>
+  </si>
+  <si>
+    <t>73 (ES)</t>
+  </si>
+  <si>
+    <t>Simplemente he reducido el seq_length a una ventana más
+pequeña, he eliminado Pot_gen de las features y he hecho más simple la LSTM</t>
+  </si>
+  <si>
+    <t>V12</t>
+  </si>
+  <si>
+    <t>66 (ES)</t>
+  </si>
+  <si>
+    <t>78 (ES)</t>
+  </si>
+  <si>
+    <t>75 (ES)</t>
   </si>
 </sst>
 </file>
@@ -255,7 +277,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -298,6 +320,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFB7EC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="21">
     <border>
@@ -537,7 +565,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -620,75 +648,107 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -707,7 +767,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -716,6 +778,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFFB7EC"/>
       <color rgb="FF35D33D"/>
       <color rgb="FF1B7B20"/>
       <color rgb="FF3366FF"/>
@@ -1055,7 +1118,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:W35"/>
+  <dimension ref="A2:W41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.42578125" customWidth="1"/>
@@ -1074,32 +1137,32 @@
   <sheetData>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D3" s="64" t="s">
+      <c r="D3" s="75" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="65"/>
-      <c r="F3" s="65"/>
-      <c r="G3" s="65"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="67" t="s">
+      <c r="E3" s="76"/>
+      <c r="F3" s="76"/>
+      <c r="G3" s="76"/>
+      <c r="H3" s="77"/>
+      <c r="I3" s="78" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="68"/>
-      <c r="K3" s="68"/>
-      <c r="L3" s="68"/>
-      <c r="M3" s="68"/>
-      <c r="N3" s="68"/>
-      <c r="O3" s="68"/>
-      <c r="P3" s="68"/>
-      <c r="Q3" s="69"/>
-      <c r="R3" s="71" t="s">
+      <c r="J3" s="79"/>
+      <c r="K3" s="79"/>
+      <c r="L3" s="79"/>
+      <c r="M3" s="79"/>
+      <c r="N3" s="79"/>
+      <c r="O3" s="79"/>
+      <c r="P3" s="79"/>
+      <c r="Q3" s="80"/>
+      <c r="R3" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="72"/>
-      <c r="T3" s="72"/>
-      <c r="U3" s="72"/>
-      <c r="V3" s="72"/>
-      <c r="W3" s="73"/>
+      <c r="S3" s="86"/>
+      <c r="T3" s="86"/>
+      <c r="U3" s="86"/>
+      <c r="V3" s="86"/>
+      <c r="W3" s="87"/>
     </row>
     <row r="4" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="20" t="s">
@@ -1150,16 +1213,16 @@
       <c r="Q4" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="74"/>
-      <c r="S4" s="75"/>
-      <c r="T4" s="75"/>
-      <c r="U4" s="75"/>
-      <c r="V4" s="75"/>
-      <c r="W4" s="76"/>
-    </row>
-    <row r="5" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="R4" s="88"/>
+      <c r="S4" s="89"/>
+      <c r="T4" s="89"/>
+      <c r="U4" s="89"/>
+      <c r="V4" s="89"/>
+      <c r="W4" s="90"/>
+    </row>
+    <row r="5" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
-      <c r="B5" s="70" t="s">
+      <c r="B5" s="81" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -1207,18 +1270,18 @@
       <c r="Q5" s="17">
         <v>1E-3</v>
       </c>
-      <c r="R5" s="48" t="s">
+      <c r="R5" s="74" t="s">
         <v>38</v>
       </c>
-      <c r="S5" s="49"/>
-      <c r="T5" s="49"/>
-      <c r="U5" s="49"/>
-      <c r="V5" s="49"/>
-      <c r="W5" s="50"/>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="S5" s="66"/>
+      <c r="T5" s="66"/>
+      <c r="U5" s="66"/>
+      <c r="V5" s="66"/>
+      <c r="W5" s="67"/>
+    </row>
+    <row r="6" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
-      <c r="B6" s="59"/>
+      <c r="B6" s="82"/>
       <c r="C6" s="5" t="s">
         <v>12</v>
       </c>
@@ -1264,16 +1327,16 @@
       <c r="Q6" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R6" s="51"/>
-      <c r="S6" s="52"/>
-      <c r="T6" s="52"/>
-      <c r="U6" s="52"/>
-      <c r="V6" s="52"/>
-      <c r="W6" s="53"/>
-    </row>
-    <row r="7" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R6" s="68"/>
+      <c r="S6" s="69"/>
+      <c r="T6" s="69"/>
+      <c r="U6" s="69"/>
+      <c r="V6" s="69"/>
+      <c r="W6" s="70"/>
+    </row>
+    <row r="7" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8"/>
-      <c r="B7" s="60"/>
+      <c r="B7" s="83"/>
       <c r="C7" s="14" t="s">
         <v>14</v>
       </c>
@@ -1319,16 +1382,16 @@
       <c r="Q7" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R7" s="54"/>
-      <c r="S7" s="55"/>
-      <c r="T7" s="55"/>
-      <c r="U7" s="55"/>
-      <c r="V7" s="55"/>
-      <c r="W7" s="56"/>
-    </row>
-    <row r="8" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="R7" s="71"/>
+      <c r="S7" s="72"/>
+      <c r="T7" s="72"/>
+      <c r="U7" s="72"/>
+      <c r="V7" s="72"/>
+      <c r="W7" s="73"/>
+    </row>
+    <row r="8" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
-      <c r="B8" s="58" t="s">
+      <c r="B8" s="84" t="s">
         <v>24</v>
       </c>
       <c r="C8" s="5" t="s">
@@ -1376,18 +1439,18 @@
       <c r="Q8" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R8" s="48" t="s">
+      <c r="R8" s="74" t="s">
         <v>38</v>
       </c>
-      <c r="S8" s="49"/>
-      <c r="T8" s="49"/>
-      <c r="U8" s="49"/>
-      <c r="V8" s="49"/>
-      <c r="W8" s="50"/>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="S8" s="66"/>
+      <c r="T8" s="66"/>
+      <c r="U8" s="66"/>
+      <c r="V8" s="66"/>
+      <c r="W8" s="67"/>
+    </row>
+    <row r="9" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
-      <c r="B9" s="59"/>
+      <c r="B9" s="82"/>
       <c r="C9" s="5" t="s">
         <v>12</v>
       </c>
@@ -1433,16 +1496,16 @@
       <c r="Q9" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R9" s="51"/>
-      <c r="S9" s="52"/>
-      <c r="T9" s="52"/>
-      <c r="U9" s="52"/>
-      <c r="V9" s="52"/>
-      <c r="W9" s="53"/>
-    </row>
-    <row r="10" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R9" s="68"/>
+      <c r="S9" s="69"/>
+      <c r="T9" s="69"/>
+      <c r="U9" s="69"/>
+      <c r="V9" s="69"/>
+      <c r="W9" s="70"/>
+    </row>
+    <row r="10" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8"/>
-      <c r="B10" s="60"/>
+      <c r="B10" s="83"/>
       <c r="C10" s="5" t="s">
         <v>14</v>
       </c>
@@ -1488,15 +1551,15 @@
       <c r="Q10" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R10" s="54"/>
-      <c r="S10" s="55"/>
-      <c r="T10" s="55"/>
-      <c r="U10" s="55"/>
-      <c r="V10" s="55"/>
-      <c r="W10" s="56"/>
-    </row>
-    <row r="11" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="58" t="s">
+      <c r="R10" s="71"/>
+      <c r="S10" s="72"/>
+      <c r="T10" s="72"/>
+      <c r="U10" s="72"/>
+      <c r="V10" s="72"/>
+      <c r="W10" s="73"/>
+    </row>
+    <row r="11" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="84" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="29" t="s">
@@ -1544,17 +1607,17 @@
       <c r="Q11" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R11" s="48" t="s">
+      <c r="R11" s="74" t="s">
         <v>38</v>
       </c>
-      <c r="S11" s="49"/>
-      <c r="T11" s="49"/>
-      <c r="U11" s="49"/>
-      <c r="V11" s="49"/>
-      <c r="W11" s="50"/>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B12" s="59"/>
+      <c r="S11" s="66"/>
+      <c r="T11" s="66"/>
+      <c r="U11" s="66"/>
+      <c r="V11" s="66"/>
+      <c r="W11" s="67"/>
+    </row>
+    <row r="12" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="82"/>
       <c r="C12" s="26" t="s">
         <v>12</v>
       </c>
@@ -1600,15 +1663,15 @@
       <c r="Q12" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R12" s="51"/>
-      <c r="S12" s="52"/>
-      <c r="T12" s="52"/>
-      <c r="U12" s="52"/>
-      <c r="V12" s="52"/>
-      <c r="W12" s="53"/>
-    </row>
-    <row r="13" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="59"/>
+      <c r="R12" s="68"/>
+      <c r="S12" s="69"/>
+      <c r="T12" s="69"/>
+      <c r="U12" s="69"/>
+      <c r="V12" s="69"/>
+      <c r="W12" s="70"/>
+    </row>
+    <row r="13" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="82"/>
       <c r="C13" s="27" t="s">
         <v>14</v>
       </c>
@@ -1654,15 +1717,15 @@
       <c r="Q13" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R13" s="54"/>
-      <c r="S13" s="55"/>
-      <c r="T13" s="55"/>
-      <c r="U13" s="55"/>
-      <c r="V13" s="55"/>
-      <c r="W13" s="56"/>
-    </row>
-    <row r="14" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="58" t="s">
+      <c r="R13" s="71"/>
+      <c r="S13" s="72"/>
+      <c r="T13" s="72"/>
+      <c r="U13" s="72"/>
+      <c r="V13" s="72"/>
+      <c r="W13" s="73"/>
+    </row>
+    <row r="14" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="84" t="s">
         <v>36</v>
       </c>
       <c r="C14" s="20" t="s">
@@ -1710,17 +1773,17 @@
       <c r="Q14" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R14" s="48" t="s">
+      <c r="R14" s="74" t="s">
         <v>37</v>
       </c>
-      <c r="S14" s="49"/>
-      <c r="T14" s="49"/>
-      <c r="U14" s="49"/>
-      <c r="V14" s="49"/>
-      <c r="W14" s="50"/>
-    </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B15" s="59"/>
+      <c r="S14" s="66"/>
+      <c r="T14" s="66"/>
+      <c r="U14" s="66"/>
+      <c r="V14" s="66"/>
+      <c r="W14" s="67"/>
+    </row>
+    <row r="15" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="82"/>
       <c r="C15" s="30" t="s">
         <v>12</v>
       </c>
@@ -1766,15 +1829,15 @@
       <c r="Q15" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R15" s="51"/>
-      <c r="S15" s="52"/>
-      <c r="T15" s="52"/>
-      <c r="U15" s="52"/>
-      <c r="V15" s="52"/>
-      <c r="W15" s="53"/>
-    </row>
-    <row r="16" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="60"/>
+      <c r="R15" s="68"/>
+      <c r="S15" s="69"/>
+      <c r="T15" s="69"/>
+      <c r="U15" s="69"/>
+      <c r="V15" s="69"/>
+      <c r="W15" s="70"/>
+    </row>
+    <row r="16" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="83"/>
       <c r="C16" s="31" t="s">
         <v>14</v>
       </c>
@@ -1820,16 +1883,16 @@
       <c r="Q16" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R16" s="54"/>
-      <c r="S16" s="55"/>
-      <c r="T16" s="55"/>
-      <c r="U16" s="55"/>
-      <c r="V16" s="55"/>
-      <c r="W16" s="56"/>
-    </row>
-    <row r="17" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="R16" s="71"/>
+      <c r="S16" s="72"/>
+      <c r="T16" s="72"/>
+      <c r="U16" s="72"/>
+      <c r="V16" s="72"/>
+      <c r="W16" s="73"/>
+    </row>
+    <row r="17" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
-      <c r="B17" s="50" t="s">
+      <c r="B17" s="87" t="s">
         <v>44</v>
       </c>
       <c r="C17" s="30" t="s">
@@ -1877,18 +1940,18 @@
       <c r="Q17" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R17" s="49" t="s">
+      <c r="R17" s="66" t="s">
         <v>43</v>
       </c>
-      <c r="S17" s="49"/>
-      <c r="T17" s="49"/>
-      <c r="U17" s="49"/>
-      <c r="V17" s="49"/>
-      <c r="W17" s="50"/>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="S17" s="66"/>
+      <c r="T17" s="66"/>
+      <c r="U17" s="66"/>
+      <c r="V17" s="66"/>
+      <c r="W17" s="67"/>
+    </row>
+    <row r="18" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
-      <c r="B18" s="53"/>
+      <c r="B18" s="91"/>
       <c r="C18" s="30" t="s">
         <v>12</v>
       </c>
@@ -1934,16 +1997,16 @@
       <c r="Q18" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R18" s="52"/>
-      <c r="S18" s="52"/>
-      <c r="T18" s="52"/>
-      <c r="U18" s="52"/>
-      <c r="V18" s="52"/>
-      <c r="W18" s="53"/>
-    </row>
-    <row r="19" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R18" s="69"/>
+      <c r="S18" s="69"/>
+      <c r="T18" s="69"/>
+      <c r="U18" s="69"/>
+      <c r="V18" s="69"/>
+      <c r="W18" s="70"/>
+    </row>
+    <row r="19" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8"/>
-      <c r="B19" s="56"/>
+      <c r="B19" s="90"/>
       <c r="C19" s="31" t="s">
         <v>14</v>
       </c>
@@ -1989,16 +2052,16 @@
       <c r="Q19" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R19" s="55"/>
-      <c r="S19" s="55"/>
-      <c r="T19" s="55"/>
-      <c r="U19" s="55"/>
-      <c r="V19" s="55"/>
-      <c r="W19" s="56"/>
-    </row>
-    <row r="20" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="R19" s="72"/>
+      <c r="S19" s="72"/>
+      <c r="T19" s="72"/>
+      <c r="U19" s="72"/>
+      <c r="V19" s="72"/>
+      <c r="W19" s="73"/>
+    </row>
+    <row r="20" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8"/>
-      <c r="B20" s="58" t="s">
+      <c r="B20" s="84" t="s">
         <v>46</v>
       </c>
       <c r="C20" s="30" t="s">
@@ -2046,18 +2109,18 @@
       <c r="Q20" s="36">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R20" s="57" t="s">
+      <c r="R20" s="65" t="s">
         <v>45</v>
       </c>
-      <c r="S20" s="49"/>
-      <c r="T20" s="49"/>
-      <c r="U20" s="49"/>
-      <c r="V20" s="49"/>
-      <c r="W20" s="50"/>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="S20" s="66"/>
+      <c r="T20" s="66"/>
+      <c r="U20" s="66"/>
+      <c r="V20" s="66"/>
+      <c r="W20" s="67"/>
+    </row>
+    <row r="21" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
-      <c r="B21" s="59"/>
+      <c r="B21" s="82"/>
       <c r="C21" s="30" t="s">
         <v>12</v>
       </c>
@@ -2103,16 +2166,16 @@
       <c r="Q21" s="37">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R21" s="51"/>
-      <c r="S21" s="52"/>
-      <c r="T21" s="52"/>
-      <c r="U21" s="52"/>
-      <c r="V21" s="52"/>
-      <c r="W21" s="53"/>
-    </row>
-    <row r="22" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R21" s="68"/>
+      <c r="S21" s="69"/>
+      <c r="T21" s="69"/>
+      <c r="U21" s="69"/>
+      <c r="V21" s="69"/>
+      <c r="W21" s="70"/>
+    </row>
+    <row r="22" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="8"/>
-      <c r="B22" s="60"/>
+      <c r="B22" s="83"/>
       <c r="C22" s="31" t="s">
         <v>14</v>
       </c>
@@ -2158,16 +2221,16 @@
       <c r="Q22" s="38">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R22" s="54"/>
-      <c r="S22" s="55"/>
-      <c r="T22" s="55"/>
-      <c r="U22" s="55"/>
-      <c r="V22" s="55"/>
-      <c r="W22" s="56"/>
+      <c r="R22" s="71"/>
+      <c r="S22" s="72"/>
+      <c r="T22" s="72"/>
+      <c r="U22" s="72"/>
+      <c r="V22" s="72"/>
+      <c r="W22" s="73"/>
     </row>
     <row r="23" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8"/>
-      <c r="B23" s="58" t="s">
+      <c r="B23" s="53" t="s">
         <v>50</v>
       </c>
       <c r="C23" s="20" t="s">
@@ -2215,18 +2278,18 @@
       <c r="Q23" s="10">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R23" s="57" t="s">
+      <c r="R23" s="65" t="s">
         <v>53</v>
       </c>
-      <c r="S23" s="49"/>
-      <c r="T23" s="49"/>
-      <c r="U23" s="49"/>
-      <c r="V23" s="49"/>
-      <c r="W23" s="50"/>
+      <c r="S23" s="66"/>
+      <c r="T23" s="66"/>
+      <c r="U23" s="66"/>
+      <c r="V23" s="66"/>
+      <c r="W23" s="67"/>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A24" s="8"/>
-      <c r="B24" s="59"/>
+      <c r="B24" s="54"/>
       <c r="C24" s="30" t="s">
         <v>12</v>
       </c>
@@ -2272,16 +2335,16 @@
       <c r="Q24" s="8">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R24" s="51"/>
-      <c r="S24" s="52"/>
-      <c r="T24" s="52"/>
-      <c r="U24" s="52"/>
-      <c r="V24" s="52"/>
-      <c r="W24" s="53"/>
+      <c r="R24" s="68"/>
+      <c r="S24" s="69"/>
+      <c r="T24" s="69"/>
+      <c r="U24" s="69"/>
+      <c r="V24" s="69"/>
+      <c r="W24" s="70"/>
     </row>
     <row r="25" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="8"/>
-      <c r="B25" s="60"/>
+      <c r="B25" s="55"/>
       <c r="C25" s="31" t="s">
         <v>14</v>
       </c>
@@ -2327,16 +2390,16 @@
       <c r="Q25" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R25" s="54"/>
-      <c r="S25" s="55"/>
-      <c r="T25" s="55"/>
-      <c r="U25" s="55"/>
-      <c r="V25" s="55"/>
-      <c r="W25" s="56"/>
+      <c r="R25" s="71"/>
+      <c r="S25" s="72"/>
+      <c r="T25" s="72"/>
+      <c r="U25" s="72"/>
+      <c r="V25" s="72"/>
+      <c r="W25" s="73"/>
     </row>
     <row r="26" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8"/>
-      <c r="B26" s="58" t="s">
+      <c r="B26" s="53" t="s">
         <v>55</v>
       </c>
       <c r="C26" s="20" t="s">
@@ -2375,7 +2438,7 @@
       <c r="N26" s="9">
         <v>64</v>
       </c>
-      <c r="O26" s="40" t="s">
+      <c r="O26" s="44" t="s">
         <v>54</v>
       </c>
       <c r="P26" s="9">
@@ -2384,18 +2447,18 @@
       <c r="Q26" s="36">
         <v>1E-3</v>
       </c>
-      <c r="R26" s="48" t="s">
+      <c r="R26" s="74" t="s">
         <v>57</v>
       </c>
-      <c r="S26" s="49"/>
-      <c r="T26" s="49"/>
-      <c r="U26" s="49"/>
-      <c r="V26" s="49"/>
-      <c r="W26" s="50"/>
+      <c r="S26" s="66"/>
+      <c r="T26" s="66"/>
+      <c r="U26" s="66"/>
+      <c r="V26" s="66"/>
+      <c r="W26" s="67"/>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" s="8"/>
-      <c r="B27" s="59"/>
+      <c r="B27" s="54"/>
       <c r="C27" s="30" t="s">
         <v>12</v>
       </c>
@@ -2441,16 +2504,16 @@
       <c r="Q27" s="37">
         <v>1E-3</v>
       </c>
-      <c r="R27" s="51"/>
-      <c r="S27" s="52"/>
-      <c r="T27" s="52"/>
-      <c r="U27" s="52"/>
-      <c r="V27" s="52"/>
-      <c r="W27" s="53"/>
+      <c r="R27" s="68"/>
+      <c r="S27" s="69"/>
+      <c r="T27" s="69"/>
+      <c r="U27" s="69"/>
+      <c r="V27" s="69"/>
+      <c r="W27" s="70"/>
     </row>
     <row r="28" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="8"/>
-      <c r="B28" s="60"/>
+      <c r="B28" s="55"/>
       <c r="C28" s="31" t="s">
         <v>14</v>
       </c>
@@ -2496,15 +2559,15 @@
       <c r="Q28" s="38">
         <v>1E-3</v>
       </c>
-      <c r="R28" s="54"/>
-      <c r="S28" s="55"/>
-      <c r="T28" s="55"/>
-      <c r="U28" s="55"/>
-      <c r="V28" s="55"/>
-      <c r="W28" s="56"/>
+      <c r="R28" s="71"/>
+      <c r="S28" s="72"/>
+      <c r="T28" s="72"/>
+      <c r="U28" s="72"/>
+      <c r="V28" s="72"/>
+      <c r="W28" s="73"/>
     </row>
     <row r="29" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="58" t="s">
+      <c r="B29" s="53" t="s">
         <v>58</v>
       </c>
       <c r="C29" s="29" t="s">
@@ -2552,18 +2615,18 @@
       <c r="Q29" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R29" s="57" t="s">
+      <c r="R29" s="65" t="s">
         <v>60</v>
       </c>
-      <c r="S29" s="49"/>
-      <c r="T29" s="49"/>
-      <c r="U29" s="49"/>
-      <c r="V29" s="49"/>
-      <c r="W29" s="50"/>
+      <c r="S29" s="66"/>
+      <c r="T29" s="66"/>
+      <c r="U29" s="66"/>
+      <c r="V29" s="66"/>
+      <c r="W29" s="67"/>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" s="8"/>
-      <c r="B30" s="59"/>
+      <c r="B30" s="54"/>
       <c r="C30" s="26" t="s">
         <v>12</v>
       </c>
@@ -2609,16 +2672,16 @@
       <c r="Q30" s="8">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R30" s="51"/>
-      <c r="S30" s="52"/>
-      <c r="T30" s="52"/>
-      <c r="U30" s="52"/>
-      <c r="V30" s="52"/>
-      <c r="W30" s="53"/>
+      <c r="R30" s="68"/>
+      <c r="S30" s="69"/>
+      <c r="T30" s="69"/>
+      <c r="U30" s="69"/>
+      <c r="V30" s="69"/>
+      <c r="W30" s="70"/>
     </row>
     <row r="31" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="8"/>
-      <c r="B31" s="60"/>
+      <c r="B31" s="55"/>
       <c r="C31" s="43" t="s">
         <v>14</v>
       </c>
@@ -2664,15 +2727,15 @@
       <c r="Q31" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R31" s="54"/>
-      <c r="S31" s="55"/>
-      <c r="T31" s="55"/>
-      <c r="U31" s="55"/>
-      <c r="V31" s="55"/>
-      <c r="W31" s="56"/>
+      <c r="R31" s="71"/>
+      <c r="S31" s="72"/>
+      <c r="T31" s="72"/>
+      <c r="U31" s="72"/>
+      <c r="V31" s="72"/>
+      <c r="W31" s="73"/>
     </row>
     <row r="32" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="61" t="s">
+      <c r="B32" s="53" t="s">
         <v>61</v>
       </c>
       <c r="C32" s="29" t="s">
@@ -2720,30 +2783,30 @@
       <c r="Q32" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R32" s="48" t="s">
+      <c r="R32" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="S32" s="49"/>
-      <c r="T32" s="49"/>
-      <c r="U32" s="49"/>
-      <c r="V32" s="49"/>
-      <c r="W32" s="50"/>
-    </row>
-    <row r="33" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B33" s="62"/>
+      <c r="S32" s="66"/>
+      <c r="T32" s="66"/>
+      <c r="U32" s="66"/>
+      <c r="V32" s="66"/>
+      <c r="W32" s="67"/>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B33" s="54"/>
       <c r="C33" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="D33" s="77">
+      <c r="D33">
         <v>135.97300000000001</v>
       </c>
-      <c r="E33" s="77">
+      <c r="E33">
         <v>226.589</v>
       </c>
-      <c r="F33" s="77">
+      <c r="F33">
         <v>0.7</v>
       </c>
-      <c r="G33" s="77">
+      <c r="G33">
         <v>0.69969999999999999</v>
       </c>
       <c r="H33" s="8">
@@ -2776,15 +2839,15 @@
       <c r="Q33" s="8">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R33" s="51"/>
-      <c r="S33" s="52"/>
-      <c r="T33" s="52"/>
-      <c r="U33" s="52"/>
-      <c r="V33" s="52"/>
-      <c r="W33" s="53"/>
-    </row>
-    <row r="34" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="63"/>
+      <c r="R33" s="68"/>
+      <c r="S33" s="69"/>
+      <c r="T33" s="69"/>
+      <c r="U33" s="69"/>
+      <c r="V33" s="69"/>
+      <c r="W33" s="70"/>
+    </row>
+    <row r="34" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="55"/>
       <c r="C34" s="43" t="s">
         <v>14</v>
       </c>
@@ -2830,27 +2893,349 @@
       <c r="Q34" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R34" s="54"/>
-      <c r="S34" s="55"/>
-      <c r="T34" s="55"/>
-      <c r="U34" s="55"/>
-      <c r="V34" s="55"/>
-      <c r="W34" s="56"/>
-    </row>
-    <row r="35" spans="2:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+      <c r="R34" s="71"/>
+      <c r="S34" s="72"/>
+      <c r="T34" s="72"/>
+      <c r="U34" s="72"/>
+      <c r="V34" s="72"/>
+      <c r="W34" s="73"/>
+    </row>
+    <row r="35" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="8"/>
+      <c r="B35" s="53" t="s">
+        <v>63</v>
+      </c>
+      <c r="C35" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" s="48">
+        <v>48.41</v>
+      </c>
+      <c r="E35" s="9">
+        <v>101.381</v>
+      </c>
+      <c r="F35" s="9">
+        <v>0.93989999999999996</v>
+      </c>
+      <c r="G35" s="9">
+        <v>0.93979999999999997</v>
+      </c>
+      <c r="H35" s="10">
+        <v>22.9</v>
+      </c>
+      <c r="I35" s="46">
+        <v>9</v>
+      </c>
+      <c r="J35">
+        <v>213.17</v>
+      </c>
+      <c r="K35">
+        <v>6</v>
+      </c>
+      <c r="L35" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="M35">
+        <v>64</v>
+      </c>
+      <c r="N35">
+        <v>64</v>
+      </c>
+      <c r="O35" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="P35">
+        <v>0.2</v>
+      </c>
+      <c r="Q35" s="8">
+        <v>1E-3</v>
+      </c>
+      <c r="R35" s="65" t="s">
+        <v>65</v>
+      </c>
+      <c r="S35" s="66"/>
+      <c r="T35" s="66"/>
+      <c r="U35" s="66"/>
+      <c r="V35" s="66"/>
+      <c r="W35" s="67"/>
+    </row>
+    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A36" s="8"/>
+      <c r="B36" s="54"/>
+      <c r="C36" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="D36" s="1">
+        <v>84.8</v>
+      </c>
+      <c r="E36">
+        <v>152.18299999999999</v>
+      </c>
+      <c r="F36">
+        <v>0.86450000000000005</v>
+      </c>
+      <c r="G36">
+        <v>0.86439999999999995</v>
+      </c>
+      <c r="H36" s="8">
+        <v>23.6</v>
+      </c>
+      <c r="I36" s="46">
+        <v>9</v>
+      </c>
+      <c r="J36">
+        <v>195.09</v>
+      </c>
+      <c r="K36">
+        <v>6</v>
+      </c>
+      <c r="L36" s="32" t="s">
+        <v>49</v>
+      </c>
+      <c r="M36">
+        <v>64</v>
+      </c>
+      <c r="N36" s="25">
+        <v>32</v>
+      </c>
+      <c r="O36" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="P36">
+        <v>0.1</v>
+      </c>
+      <c r="Q36" s="37">
+        <v>1E-3</v>
+      </c>
+      <c r="R36" s="68"/>
+      <c r="S36" s="69"/>
+      <c r="T36" s="69"/>
+      <c r="U36" s="69"/>
+      <c r="V36" s="69"/>
+      <c r="W36" s="70"/>
+    </row>
+    <row r="37" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="8"/>
+      <c r="B37" s="55"/>
+      <c r="C37" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="D37" s="2">
+        <v>277.791</v>
+      </c>
+      <c r="E37" s="3">
+        <v>498.125</v>
+      </c>
+      <c r="F37" s="50">
+        <v>-0.45140000000000002</v>
+      </c>
+      <c r="G37" s="50">
+        <v>-0.45279999999999998</v>
+      </c>
+      <c r="H37" s="4">
+        <v>27</v>
+      </c>
+      <c r="I37" s="49">
+        <v>9</v>
+      </c>
+      <c r="J37" s="3">
+        <v>322.19</v>
+      </c>
+      <c r="K37" s="3">
+        <v>6</v>
+      </c>
+      <c r="L37" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="M37" s="3">
+        <v>64</v>
+      </c>
+      <c r="N37" s="35" t="s">
+        <v>48</v>
+      </c>
+      <c r="O37" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="P37" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="Q37" s="4">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R37" s="71"/>
+      <c r="S37" s="72"/>
+      <c r="T37" s="72"/>
+      <c r="U37" s="72"/>
+      <c r="V37" s="72"/>
+      <c r="W37" s="73"/>
+    </row>
+    <row r="38" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="53" t="s">
+        <v>66</v>
+      </c>
+      <c r="C38" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" s="48">
+        <v>42.213999999999999</v>
+      </c>
+      <c r="E38" s="9">
+        <v>92.585999999999999</v>
+      </c>
+      <c r="F38" s="9">
+        <v>0.94740000000000002</v>
+      </c>
+      <c r="G38" s="9">
+        <v>0.94730000000000003</v>
+      </c>
+      <c r="H38" s="10">
+        <v>22.9</v>
+      </c>
+      <c r="I38" s="52">
+        <v>240</v>
+      </c>
+      <c r="J38" s="9">
+        <v>729.62</v>
+      </c>
+      <c r="K38" s="9">
+        <v>6</v>
+      </c>
+      <c r="L38" s="40" t="s">
+        <v>67</v>
+      </c>
+      <c r="M38" s="9">
+        <v>64</v>
+      </c>
+      <c r="N38" s="9">
+        <v>64</v>
+      </c>
+      <c r="O38" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="P38" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="Q38" s="10">
+        <v>1E-3</v>
+      </c>
+      <c r="R38" s="56"/>
+      <c r="S38" s="57"/>
+      <c r="T38" s="57"/>
+      <c r="U38" s="57"/>
+      <c r="V38" s="57"/>
+      <c r="W38" s="58"/>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B39" s="54"/>
+      <c r="C39" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="D39" s="1">
+        <v>46.45</v>
+      </c>
+      <c r="E39">
+        <v>97.028999999999996</v>
+      </c>
+      <c r="F39">
+        <v>0.94220000000000004</v>
+      </c>
+      <c r="G39">
+        <v>0.94210000000000005</v>
+      </c>
+      <c r="H39" s="8">
+        <v>23.6</v>
+      </c>
+      <c r="I39" s="51">
+        <v>240</v>
+      </c>
+      <c r="J39">
+        <v>1738.86</v>
+      </c>
+      <c r="K39">
+        <v>6</v>
+      </c>
+      <c r="L39" s="32" t="s">
+        <v>68</v>
+      </c>
+      <c r="M39">
+        <v>64</v>
+      </c>
+      <c r="N39">
+        <v>32</v>
+      </c>
+      <c r="O39" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="P39">
+        <v>0.1</v>
+      </c>
+      <c r="Q39" s="8">
+        <v>1E-3</v>
+      </c>
+      <c r="R39" s="59"/>
+      <c r="S39" s="60"/>
+      <c r="T39" s="60"/>
+      <c r="U39" s="60"/>
+      <c r="V39" s="60"/>
+      <c r="W39" s="61"/>
+    </row>
+    <row r="40" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="55"/>
+      <c r="C40" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="D40" s="2">
+        <v>48.531999999999996</v>
+      </c>
+      <c r="E40" s="3">
+        <v>101.703</v>
+      </c>
+      <c r="F40" s="3">
+        <v>0.9365</v>
+      </c>
+      <c r="G40" s="3">
+        <v>0.93640000000000001</v>
+      </c>
+      <c r="H40" s="4">
+        <v>27</v>
+      </c>
+      <c r="I40" s="49">
+        <v>240</v>
+      </c>
+      <c r="J40" s="3">
+        <v>3750.19</v>
+      </c>
+      <c r="K40" s="3">
+        <v>6</v>
+      </c>
+      <c r="L40" s="35" t="s">
+        <v>69</v>
+      </c>
+      <c r="M40" s="3">
+        <v>64</v>
+      </c>
+      <c r="N40" s="35" t="s">
+        <v>48</v>
+      </c>
+      <c r="O40" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="P40" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="Q40" s="4">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R40" s="62"/>
+      <c r="S40" s="63"/>
+      <c r="T40" s="63"/>
+      <c r="U40" s="63"/>
+      <c r="V40" s="63"/>
+      <c r="W40" s="64"/>
+    </row>
+    <row r="41" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="23">
-    <mergeCell ref="B29:B31"/>
-    <mergeCell ref="R29:W31"/>
-    <mergeCell ref="B32:B34"/>
-    <mergeCell ref="R32:W34"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="I3:Q3"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="R3:W4"/>
-    <mergeCell ref="R5:W7"/>
-    <mergeCell ref="R8:W10"/>
+  <mergeCells count="27">
     <mergeCell ref="B23:B25"/>
     <mergeCell ref="R23:W25"/>
     <mergeCell ref="B26:B28"/>
@@ -2863,6 +3248,21 @@
     <mergeCell ref="B20:B22"/>
     <mergeCell ref="R14:W16"/>
     <mergeCell ref="B14:B16"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="I3:Q3"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="R3:W4"/>
+    <mergeCell ref="R5:W7"/>
+    <mergeCell ref="R8:W10"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="R38:W40"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="R35:W37"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="R29:W31"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="R32:W34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>

<commit_message>
Añado red CNN y comparo
</commit_message>
<xml_diff>
--- a/modelos_tfg/MetricasValidacion.xlsx
+++ b/modelos_tfg/MetricasValidacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\modelos_tfg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{090B1B97-CCE6-4858-B037-CFC7FB4C4A5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0763A6D6-C557-46EC-8090-E7332E54B1AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="81">
   <si>
     <t>ID Train</t>
   </si>
@@ -239,6 +239,41 @@
   </si>
   <si>
     <t>75 (ES)</t>
+  </si>
+  <si>
+    <t>CNN</t>
+  </si>
+  <si>
+    <t>NaN</t>
+  </si>
+  <si>
+    <t>99 (ES)</t>
+  </si>
+  <si>
+    <t>64 (ES)</t>
+  </si>
+  <si>
+    <t>V13</t>
+  </si>
+  <si>
+    <t>V14</t>
+  </si>
+  <si>
+    <t>He añadido un modelo CNN</t>
+  </si>
+  <si>
+    <t>Junto con el nuevo modelo CNN, le he dado a la arquitectura
+de cada modelo el mismo número de neuronas, y he puesto
+una ventana temporal de 5 horas</t>
+  </si>
+  <si>
+    <t>57 (ES)</t>
+  </si>
+  <si>
+    <t>56 (ES)</t>
+  </si>
+  <si>
+    <t>V15</t>
   </si>
 </sst>
 </file>
@@ -277,7 +312,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -326,6 +361,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="21">
     <border>
@@ -565,7 +612,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -648,7 +695,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
@@ -770,6 +816,46 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1118,7 +1204,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:W41"/>
+  <dimension ref="A2:W53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.42578125" customWidth="1"/>
@@ -1137,32 +1223,32 @@
   <sheetData>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D3" s="75" t="s">
+      <c r="D3" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="76"/>
-      <c r="F3" s="76"/>
-      <c r="G3" s="76"/>
-      <c r="H3" s="77"/>
-      <c r="I3" s="78" t="s">
+      <c r="E3" s="75"/>
+      <c r="F3" s="75"/>
+      <c r="G3" s="75"/>
+      <c r="H3" s="76"/>
+      <c r="I3" s="77" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="79"/>
-      <c r="K3" s="79"/>
-      <c r="L3" s="79"/>
-      <c r="M3" s="79"/>
-      <c r="N3" s="79"/>
-      <c r="O3" s="79"/>
-      <c r="P3" s="79"/>
-      <c r="Q3" s="80"/>
-      <c r="R3" s="85" t="s">
+      <c r="J3" s="78"/>
+      <c r="K3" s="78"/>
+      <c r="L3" s="78"/>
+      <c r="M3" s="78"/>
+      <c r="N3" s="78"/>
+      <c r="O3" s="78"/>
+      <c r="P3" s="78"/>
+      <c r="Q3" s="79"/>
+      <c r="R3" s="84" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="86"/>
-      <c r="T3" s="86"/>
-      <c r="U3" s="86"/>
-      <c r="V3" s="86"/>
-      <c r="W3" s="87"/>
+      <c r="S3" s="85"/>
+      <c r="T3" s="85"/>
+      <c r="U3" s="85"/>
+      <c r="V3" s="85"/>
+      <c r="W3" s="86"/>
     </row>
     <row r="4" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="20" t="s">
@@ -1213,16 +1299,16 @@
       <c r="Q4" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="88"/>
-      <c r="S4" s="89"/>
-      <c r="T4" s="89"/>
-      <c r="U4" s="89"/>
-      <c r="V4" s="89"/>
-      <c r="W4" s="90"/>
+      <c r="R4" s="87"/>
+      <c r="S4" s="88"/>
+      <c r="T4" s="88"/>
+      <c r="U4" s="88"/>
+      <c r="V4" s="88"/>
+      <c r="W4" s="89"/>
     </row>
     <row r="5" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
-      <c r="B5" s="81" t="s">
+      <c r="B5" s="80" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -1270,18 +1356,18 @@
       <c r="Q5" s="17">
         <v>1E-3</v>
       </c>
-      <c r="R5" s="74" t="s">
+      <c r="R5" s="73" t="s">
         <v>38</v>
       </c>
-      <c r="S5" s="66"/>
-      <c r="T5" s="66"/>
-      <c r="U5" s="66"/>
-      <c r="V5" s="66"/>
-      <c r="W5" s="67"/>
+      <c r="S5" s="65"/>
+      <c r="T5" s="65"/>
+      <c r="U5" s="65"/>
+      <c r="V5" s="65"/>
+      <c r="W5" s="66"/>
     </row>
     <row r="6" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
-      <c r="B6" s="82"/>
+      <c r="B6" s="81"/>
       <c r="C6" s="5" t="s">
         <v>12</v>
       </c>
@@ -1327,16 +1413,16 @@
       <c r="Q6" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R6" s="68"/>
-      <c r="S6" s="69"/>
-      <c r="T6" s="69"/>
-      <c r="U6" s="69"/>
-      <c r="V6" s="69"/>
-      <c r="W6" s="70"/>
+      <c r="R6" s="67"/>
+      <c r="S6" s="68"/>
+      <c r="T6" s="68"/>
+      <c r="U6" s="68"/>
+      <c r="V6" s="68"/>
+      <c r="W6" s="69"/>
     </row>
     <row r="7" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8"/>
-      <c r="B7" s="83"/>
+      <c r="B7" s="82"/>
       <c r="C7" s="14" t="s">
         <v>14</v>
       </c>
@@ -1382,16 +1468,16 @@
       <c r="Q7" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R7" s="71"/>
-      <c r="S7" s="72"/>
-      <c r="T7" s="72"/>
-      <c r="U7" s="72"/>
-      <c r="V7" s="72"/>
-      <c r="W7" s="73"/>
+      <c r="R7" s="70"/>
+      <c r="S7" s="71"/>
+      <c r="T7" s="71"/>
+      <c r="U7" s="71"/>
+      <c r="V7" s="71"/>
+      <c r="W7" s="72"/>
     </row>
     <row r="8" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
-      <c r="B8" s="84" t="s">
+      <c r="B8" s="83" t="s">
         <v>24</v>
       </c>
       <c r="C8" s="5" t="s">
@@ -1439,18 +1525,18 @@
       <c r="Q8" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R8" s="74" t="s">
+      <c r="R8" s="73" t="s">
         <v>38</v>
       </c>
-      <c r="S8" s="66"/>
-      <c r="T8" s="66"/>
-      <c r="U8" s="66"/>
-      <c r="V8" s="66"/>
-      <c r="W8" s="67"/>
+      <c r="S8" s="65"/>
+      <c r="T8" s="65"/>
+      <c r="U8" s="65"/>
+      <c r="V8" s="65"/>
+      <c r="W8" s="66"/>
     </row>
     <row r="9" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
-      <c r="B9" s="82"/>
+      <c r="B9" s="81"/>
       <c r="C9" s="5" t="s">
         <v>12</v>
       </c>
@@ -1496,16 +1582,16 @@
       <c r="Q9" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R9" s="68"/>
-      <c r="S9" s="69"/>
-      <c r="T9" s="69"/>
-      <c r="U9" s="69"/>
-      <c r="V9" s="69"/>
-      <c r="W9" s="70"/>
+      <c r="R9" s="67"/>
+      <c r="S9" s="68"/>
+      <c r="T9" s="68"/>
+      <c r="U9" s="68"/>
+      <c r="V9" s="68"/>
+      <c r="W9" s="69"/>
     </row>
     <row r="10" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8"/>
-      <c r="B10" s="83"/>
+      <c r="B10" s="82"/>
       <c r="C10" s="5" t="s">
         <v>14</v>
       </c>
@@ -1551,15 +1637,15 @@
       <c r="Q10" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R10" s="71"/>
-      <c r="S10" s="72"/>
-      <c r="T10" s="72"/>
-      <c r="U10" s="72"/>
-      <c r="V10" s="72"/>
-      <c r="W10" s="73"/>
+      <c r="R10" s="70"/>
+      <c r="S10" s="71"/>
+      <c r="T10" s="71"/>
+      <c r="U10" s="71"/>
+      <c r="V10" s="71"/>
+      <c r="W10" s="72"/>
     </row>
     <row r="11" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="84" t="s">
+      <c r="B11" s="83" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="29" t="s">
@@ -1607,17 +1693,17 @@
       <c r="Q11" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R11" s="74" t="s">
+      <c r="R11" s="73" t="s">
         <v>38</v>
       </c>
-      <c r="S11" s="66"/>
-      <c r="T11" s="66"/>
-      <c r="U11" s="66"/>
-      <c r="V11" s="66"/>
-      <c r="W11" s="67"/>
+      <c r="S11" s="65"/>
+      <c r="T11" s="65"/>
+      <c r="U11" s="65"/>
+      <c r="V11" s="65"/>
+      <c r="W11" s="66"/>
     </row>
     <row r="12" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="82"/>
+      <c r="B12" s="81"/>
       <c r="C12" s="26" t="s">
         <v>12</v>
       </c>
@@ -1663,15 +1749,15 @@
       <c r="Q12" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R12" s="68"/>
-      <c r="S12" s="69"/>
-      <c r="T12" s="69"/>
-      <c r="U12" s="69"/>
-      <c r="V12" s="69"/>
-      <c r="W12" s="70"/>
+      <c r="R12" s="67"/>
+      <c r="S12" s="68"/>
+      <c r="T12" s="68"/>
+      <c r="U12" s="68"/>
+      <c r="V12" s="68"/>
+      <c r="W12" s="69"/>
     </row>
     <row r="13" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="82"/>
+      <c r="B13" s="81"/>
       <c r="C13" s="27" t="s">
         <v>14</v>
       </c>
@@ -1717,15 +1803,15 @@
       <c r="Q13" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R13" s="71"/>
-      <c r="S13" s="72"/>
-      <c r="T13" s="72"/>
-      <c r="U13" s="72"/>
-      <c r="V13" s="72"/>
-      <c r="W13" s="73"/>
+      <c r="R13" s="70"/>
+      <c r="S13" s="71"/>
+      <c r="T13" s="71"/>
+      <c r="U13" s="71"/>
+      <c r="V13" s="71"/>
+      <c r="W13" s="72"/>
     </row>
     <row r="14" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="84" t="s">
+      <c r="B14" s="83" t="s">
         <v>36</v>
       </c>
       <c r="C14" s="20" t="s">
@@ -1773,17 +1859,17 @@
       <c r="Q14" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R14" s="74" t="s">
+      <c r="R14" s="73" t="s">
         <v>37</v>
       </c>
-      <c r="S14" s="66"/>
-      <c r="T14" s="66"/>
-      <c r="U14" s="66"/>
-      <c r="V14" s="66"/>
-      <c r="W14" s="67"/>
+      <c r="S14" s="65"/>
+      <c r="T14" s="65"/>
+      <c r="U14" s="65"/>
+      <c r="V14" s="65"/>
+      <c r="W14" s="66"/>
     </row>
     <row r="15" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="82"/>
+      <c r="B15" s="81"/>
       <c r="C15" s="30" t="s">
         <v>12</v>
       </c>
@@ -1829,15 +1915,15 @@
       <c r="Q15" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R15" s="68"/>
-      <c r="S15" s="69"/>
-      <c r="T15" s="69"/>
-      <c r="U15" s="69"/>
-      <c r="V15" s="69"/>
-      <c r="W15" s="70"/>
+      <c r="R15" s="67"/>
+      <c r="S15" s="68"/>
+      <c r="T15" s="68"/>
+      <c r="U15" s="68"/>
+      <c r="V15" s="68"/>
+      <c r="W15" s="69"/>
     </row>
     <row r="16" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="83"/>
+      <c r="B16" s="82"/>
       <c r="C16" s="31" t="s">
         <v>14</v>
       </c>
@@ -1883,16 +1969,16 @@
       <c r="Q16" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R16" s="71"/>
-      <c r="S16" s="72"/>
-      <c r="T16" s="72"/>
-      <c r="U16" s="72"/>
-      <c r="V16" s="72"/>
-      <c r="W16" s="73"/>
+      <c r="R16" s="70"/>
+      <c r="S16" s="71"/>
+      <c r="T16" s="71"/>
+      <c r="U16" s="71"/>
+      <c r="V16" s="71"/>
+      <c r="W16" s="72"/>
     </row>
     <row r="17" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
-      <c r="B17" s="87" t="s">
+      <c r="B17" s="86" t="s">
         <v>44</v>
       </c>
       <c r="C17" s="30" t="s">
@@ -1940,18 +2026,18 @@
       <c r="Q17" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R17" s="66" t="s">
+      <c r="R17" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="S17" s="66"/>
-      <c r="T17" s="66"/>
-      <c r="U17" s="66"/>
-      <c r="V17" s="66"/>
-      <c r="W17" s="67"/>
+      <c r="S17" s="65"/>
+      <c r="T17" s="65"/>
+      <c r="U17" s="65"/>
+      <c r="V17" s="65"/>
+      <c r="W17" s="66"/>
     </row>
     <row r="18" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
-      <c r="B18" s="91"/>
+      <c r="B18" s="90"/>
       <c r="C18" s="30" t="s">
         <v>12</v>
       </c>
@@ -1997,16 +2083,16 @@
       <c r="Q18" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R18" s="69"/>
-      <c r="S18" s="69"/>
-      <c r="T18" s="69"/>
-      <c r="U18" s="69"/>
-      <c r="V18" s="69"/>
-      <c r="W18" s="70"/>
+      <c r="R18" s="68"/>
+      <c r="S18" s="68"/>
+      <c r="T18" s="68"/>
+      <c r="U18" s="68"/>
+      <c r="V18" s="68"/>
+      <c r="W18" s="69"/>
     </row>
     <row r="19" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8"/>
-      <c r="B19" s="90"/>
+      <c r="B19" s="89"/>
       <c r="C19" s="31" t="s">
         <v>14</v>
       </c>
@@ -2052,16 +2138,16 @@
       <c r="Q19" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R19" s="72"/>
-      <c r="S19" s="72"/>
-      <c r="T19" s="72"/>
-      <c r="U19" s="72"/>
-      <c r="V19" s="72"/>
-      <c r="W19" s="73"/>
+      <c r="R19" s="71"/>
+      <c r="S19" s="71"/>
+      <c r="T19" s="71"/>
+      <c r="U19" s="71"/>
+      <c r="V19" s="71"/>
+      <c r="W19" s="72"/>
     </row>
     <row r="20" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8"/>
-      <c r="B20" s="84" t="s">
+      <c r="B20" s="83" t="s">
         <v>46</v>
       </c>
       <c r="C20" s="30" t="s">
@@ -2109,18 +2195,18 @@
       <c r="Q20" s="36">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R20" s="65" t="s">
+      <c r="R20" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="S20" s="66"/>
-      <c r="T20" s="66"/>
-      <c r="U20" s="66"/>
-      <c r="V20" s="66"/>
-      <c r="W20" s="67"/>
+      <c r="S20" s="65"/>
+      <c r="T20" s="65"/>
+      <c r="U20" s="65"/>
+      <c r="V20" s="65"/>
+      <c r="W20" s="66"/>
     </row>
     <row r="21" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
-      <c r="B21" s="82"/>
+      <c r="B21" s="81"/>
       <c r="C21" s="30" t="s">
         <v>12</v>
       </c>
@@ -2166,16 +2252,16 @@
       <c r="Q21" s="37">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R21" s="68"/>
-      <c r="S21" s="69"/>
-      <c r="T21" s="69"/>
-      <c r="U21" s="69"/>
-      <c r="V21" s="69"/>
-      <c r="W21" s="70"/>
+      <c r="R21" s="67"/>
+      <c r="S21" s="68"/>
+      <c r="T21" s="68"/>
+      <c r="U21" s="68"/>
+      <c r="V21" s="68"/>
+      <c r="W21" s="69"/>
     </row>
     <row r="22" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="8"/>
-      <c r="B22" s="83"/>
+      <c r="B22" s="82"/>
       <c r="C22" s="31" t="s">
         <v>14</v>
       </c>
@@ -2221,16 +2307,16 @@
       <c r="Q22" s="38">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R22" s="71"/>
-      <c r="S22" s="72"/>
-      <c r="T22" s="72"/>
-      <c r="U22" s="72"/>
-      <c r="V22" s="72"/>
-      <c r="W22" s="73"/>
+      <c r="R22" s="70"/>
+      <c r="S22" s="71"/>
+      <c r="T22" s="71"/>
+      <c r="U22" s="71"/>
+      <c r="V22" s="71"/>
+      <c r="W22" s="72"/>
     </row>
     <row r="23" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="8"/>
-      <c r="B23" s="53" t="s">
+      <c r="A23" s="117"/>
+      <c r="B23" s="52" t="s">
         <v>50</v>
       </c>
       <c r="C23" s="20" t="s">
@@ -2278,34 +2364,34 @@
       <c r="Q23" s="10">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R23" s="65" t="s">
+      <c r="R23" s="64" t="s">
         <v>53</v>
       </c>
-      <c r="S23" s="66"/>
-      <c r="T23" s="66"/>
-      <c r="U23" s="66"/>
-      <c r="V23" s="66"/>
-      <c r="W23" s="67"/>
+      <c r="S23" s="65"/>
+      <c r="T23" s="65"/>
+      <c r="U23" s="65"/>
+      <c r="V23" s="65"/>
+      <c r="W23" s="66"/>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A24" s="8"/>
-      <c r="B24" s="54"/>
+      <c r="A24" s="117"/>
+      <c r="B24" s="53"/>
       <c r="C24" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="D24">
+      <c r="D24" s="91">
         <v>51.393000000000001</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="91">
         <v>110.699</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="91">
         <v>0.9274</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="91">
         <v>0.92730000000000001</v>
       </c>
-      <c r="H24" s="8">
+      <c r="H24" s="92">
         <v>35.4</v>
       </c>
       <c r="I24">
@@ -2335,16 +2421,16 @@
       <c r="Q24" s="8">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R24" s="68"/>
-      <c r="S24" s="69"/>
-      <c r="T24" s="69"/>
-      <c r="U24" s="69"/>
-      <c r="V24" s="69"/>
-      <c r="W24" s="70"/>
+      <c r="R24" s="67"/>
+      <c r="S24" s="68"/>
+      <c r="T24" s="68"/>
+      <c r="U24" s="68"/>
+      <c r="V24" s="68"/>
+      <c r="W24" s="69"/>
     </row>
     <row r="25" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="8"/>
-      <c r="B25" s="55"/>
+      <c r="A25" s="117"/>
+      <c r="B25" s="54"/>
       <c r="C25" s="31" t="s">
         <v>14</v>
       </c>
@@ -2390,34 +2476,34 @@
       <c r="Q25" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R25" s="71"/>
-      <c r="S25" s="72"/>
-      <c r="T25" s="72"/>
-      <c r="U25" s="72"/>
-      <c r="V25" s="72"/>
-      <c r="W25" s="73"/>
+      <c r="R25" s="70"/>
+      <c r="S25" s="71"/>
+      <c r="T25" s="71"/>
+      <c r="U25" s="71"/>
+      <c r="V25" s="71"/>
+      <c r="W25" s="72"/>
     </row>
     <row r="26" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="8"/>
-      <c r="B26" s="53" t="s">
+      <c r="A26" s="117"/>
+      <c r="B26" s="52" t="s">
         <v>55</v>
       </c>
       <c r="C26" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="D26" s="9">
+      <c r="D26" s="93">
         <v>47.706000000000003</v>
       </c>
-      <c r="E26" s="9">
+      <c r="E26" s="93">
         <v>101.812</v>
       </c>
-      <c r="F26" s="9">
+      <c r="F26" s="93">
         <v>0.93859999999999999</v>
       </c>
-      <c r="G26" s="9">
+      <c r="G26" s="93">
         <v>0.9385</v>
       </c>
-      <c r="H26" s="10">
+      <c r="H26" s="94">
         <v>29.3</v>
       </c>
       <c r="I26" s="9">
@@ -2447,18 +2533,18 @@
       <c r="Q26" s="36">
         <v>1E-3</v>
       </c>
-      <c r="R26" s="74" t="s">
+      <c r="R26" s="73" t="s">
         <v>57</v>
       </c>
-      <c r="S26" s="66"/>
-      <c r="T26" s="66"/>
-      <c r="U26" s="66"/>
-      <c r="V26" s="66"/>
-      <c r="W26" s="67"/>
+      <c r="S26" s="65"/>
+      <c r="T26" s="65"/>
+      <c r="U26" s="65"/>
+      <c r="V26" s="65"/>
+      <c r="W26" s="66"/>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A27" s="8"/>
-      <c r="B27" s="54"/>
+      <c r="A27" s="117"/>
+      <c r="B27" s="53"/>
       <c r="C27" s="30" t="s">
         <v>12</v>
       </c>
@@ -2504,16 +2590,16 @@
       <c r="Q27" s="37">
         <v>1E-3</v>
       </c>
-      <c r="R27" s="68"/>
-      <c r="S27" s="69"/>
-      <c r="T27" s="69"/>
-      <c r="U27" s="69"/>
-      <c r="V27" s="69"/>
-      <c r="W27" s="70"/>
+      <c r="R27" s="67"/>
+      <c r="S27" s="68"/>
+      <c r="T27" s="68"/>
+      <c r="U27" s="68"/>
+      <c r="V27" s="68"/>
+      <c r="W27" s="69"/>
     </row>
     <row r="28" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="8"/>
-      <c r="B28" s="55"/>
+      <c r="A28" s="117"/>
+      <c r="B28" s="54"/>
       <c r="C28" s="31" t="s">
         <v>14</v>
       </c>
@@ -2559,33 +2645,34 @@
       <c r="Q28" s="38">
         <v>1E-3</v>
       </c>
-      <c r="R28" s="71"/>
-      <c r="S28" s="72"/>
-      <c r="T28" s="72"/>
-      <c r="U28" s="72"/>
-      <c r="V28" s="72"/>
-      <c r="W28" s="73"/>
+      <c r="R28" s="70"/>
+      <c r="S28" s="71"/>
+      <c r="T28" s="71"/>
+      <c r="U28" s="71"/>
+      <c r="V28" s="71"/>
+      <c r="W28" s="72"/>
     </row>
     <row r="29" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="53" t="s">
+      <c r="A29" s="118"/>
+      <c r="B29" s="52" t="s">
         <v>58</v>
       </c>
       <c r="C29" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="D29" s="9">
+      <c r="D29" s="93">
         <v>49.481000000000002</v>
       </c>
-      <c r="E29" s="9">
+      <c r="E29" s="93">
         <v>104.151</v>
       </c>
-      <c r="F29" s="9">
+      <c r="F29" s="93">
         <v>0.93569999999999998</v>
       </c>
-      <c r="G29" s="9">
+      <c r="G29" s="93">
         <v>0.93569999999999998</v>
       </c>
-      <c r="H29" s="10">
+      <c r="H29" s="94">
         <v>23.1</v>
       </c>
       <c r="I29" s="9">
@@ -2615,18 +2702,18 @@
       <c r="Q29" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R29" s="65" t="s">
+      <c r="R29" s="64" t="s">
         <v>60</v>
       </c>
-      <c r="S29" s="66"/>
-      <c r="T29" s="66"/>
-      <c r="U29" s="66"/>
-      <c r="V29" s="66"/>
-      <c r="W29" s="67"/>
+      <c r="S29" s="65"/>
+      <c r="T29" s="65"/>
+      <c r="U29" s="65"/>
+      <c r="V29" s="65"/>
+      <c r="W29" s="66"/>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A30" s="8"/>
-      <c r="B30" s="54"/>
+      <c r="A30" s="117"/>
+      <c r="B30" s="53"/>
       <c r="C30" s="26" t="s">
         <v>12</v>
       </c>
@@ -2672,16 +2759,16 @@
       <c r="Q30" s="8">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R30" s="68"/>
-      <c r="S30" s="69"/>
-      <c r="T30" s="69"/>
-      <c r="U30" s="69"/>
-      <c r="V30" s="69"/>
-      <c r="W30" s="70"/>
+      <c r="R30" s="67"/>
+      <c r="S30" s="68"/>
+      <c r="T30" s="68"/>
+      <c r="U30" s="68"/>
+      <c r="V30" s="68"/>
+      <c r="W30" s="69"/>
     </row>
     <row r="31" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="8"/>
-      <c r="B31" s="55"/>
+      <c r="A31" s="117"/>
+      <c r="B31" s="54"/>
       <c r="C31" s="43" t="s">
         <v>14</v>
       </c>
@@ -2727,33 +2814,34 @@
       <c r="Q31" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R31" s="71"/>
-      <c r="S31" s="72"/>
-      <c r="T31" s="72"/>
-      <c r="U31" s="72"/>
-      <c r="V31" s="72"/>
-      <c r="W31" s="73"/>
+      <c r="R31" s="70"/>
+      <c r="S31" s="71"/>
+      <c r="T31" s="71"/>
+      <c r="U31" s="71"/>
+      <c r="V31" s="71"/>
+      <c r="W31" s="72"/>
     </row>
     <row r="32" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="53" t="s">
+      <c r="A32" s="118"/>
+      <c r="B32" s="52" t="s">
         <v>61</v>
       </c>
       <c r="C32" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="D32" s="9">
+      <c r="D32" s="93">
         <v>46.76</v>
       </c>
-      <c r="E32" s="9">
+      <c r="E32" s="93">
         <v>95.427999999999997</v>
       </c>
-      <c r="F32" s="9">
+      <c r="F32" s="93">
         <v>0.94679999999999997</v>
       </c>
-      <c r="G32" s="9">
+      <c r="G32" s="93">
         <v>0.94669999999999999</v>
       </c>
-      <c r="H32" s="10">
+      <c r="H32" s="94">
         <v>23.1</v>
       </c>
       <c r="I32" s="45">
@@ -2783,17 +2871,18 @@
       <c r="Q32" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R32" s="74" t="s">
+      <c r="R32" s="73" t="s">
         <v>62</v>
       </c>
-      <c r="S32" s="66"/>
-      <c r="T32" s="66"/>
-      <c r="U32" s="66"/>
-      <c r="V32" s="66"/>
-      <c r="W32" s="67"/>
+      <c r="S32" s="65"/>
+      <c r="T32" s="65"/>
+      <c r="U32" s="65"/>
+      <c r="V32" s="65"/>
+      <c r="W32" s="66"/>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B33" s="54"/>
+      <c r="A33" s="118"/>
+      <c r="B33" s="53"/>
       <c r="C33" s="26" t="s">
         <v>12</v>
       </c>
@@ -2839,15 +2928,16 @@
       <c r="Q33" s="8">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R33" s="68"/>
-      <c r="S33" s="69"/>
-      <c r="T33" s="69"/>
-      <c r="U33" s="69"/>
-      <c r="V33" s="69"/>
-      <c r="W33" s="70"/>
+      <c r="R33" s="67"/>
+      <c r="S33" s="68"/>
+      <c r="T33" s="68"/>
+      <c r="U33" s="68"/>
+      <c r="V33" s="68"/>
+      <c r="W33" s="69"/>
     </row>
     <row r="34" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="55"/>
+      <c r="A34" s="118"/>
+      <c r="B34" s="54"/>
       <c r="C34" s="43" t="s">
         <v>14</v>
       </c>
@@ -2893,34 +2983,34 @@
       <c r="Q34" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R34" s="71"/>
-      <c r="S34" s="72"/>
-      <c r="T34" s="72"/>
-      <c r="U34" s="72"/>
-      <c r="V34" s="72"/>
-      <c r="W34" s="73"/>
+      <c r="R34" s="70"/>
+      <c r="S34" s="71"/>
+      <c r="T34" s="71"/>
+      <c r="U34" s="71"/>
+      <c r="V34" s="71"/>
+      <c r="W34" s="72"/>
     </row>
     <row r="35" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="8"/>
-      <c r="B35" s="53" t="s">
+      <c r="A35" s="117"/>
+      <c r="B35" s="52" t="s">
         <v>63</v>
       </c>
       <c r="C35" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="D35" s="48">
+      <c r="D35" s="95">
         <v>48.41</v>
       </c>
-      <c r="E35" s="9">
+      <c r="E35" s="93">
         <v>101.381</v>
       </c>
-      <c r="F35" s="9">
+      <c r="F35" s="93">
         <v>0.93989999999999996</v>
       </c>
-      <c r="G35" s="9">
+      <c r="G35" s="93">
         <v>0.93979999999999997</v>
       </c>
-      <c r="H35" s="10">
+      <c r="H35" s="94">
         <v>22.9</v>
       </c>
       <c r="I35" s="46">
@@ -2950,18 +3040,18 @@
       <c r="Q35" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R35" s="65" t="s">
+      <c r="R35" s="64" t="s">
         <v>65</v>
       </c>
-      <c r="S35" s="66"/>
-      <c r="T35" s="66"/>
-      <c r="U35" s="66"/>
-      <c r="V35" s="66"/>
-      <c r="W35" s="67"/>
+      <c r="S35" s="65"/>
+      <c r="T35" s="65"/>
+      <c r="U35" s="65"/>
+      <c r="V35" s="65"/>
+      <c r="W35" s="66"/>
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A36" s="8"/>
-      <c r="B36" s="54"/>
+      <c r="A36" s="117"/>
+      <c r="B36" s="53"/>
       <c r="C36" s="26" t="s">
         <v>12</v>
       </c>
@@ -3007,16 +3097,16 @@
       <c r="Q36" s="37">
         <v>1E-3</v>
       </c>
-      <c r="R36" s="68"/>
-      <c r="S36" s="69"/>
-      <c r="T36" s="69"/>
-      <c r="U36" s="69"/>
-      <c r="V36" s="69"/>
-      <c r="W36" s="70"/>
+      <c r="R36" s="67"/>
+      <c r="S36" s="68"/>
+      <c r="T36" s="68"/>
+      <c r="U36" s="68"/>
+      <c r="V36" s="68"/>
+      <c r="W36" s="69"/>
     </row>
     <row r="37" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="8"/>
-      <c r="B37" s="55"/>
+      <c r="A37" s="117"/>
+      <c r="B37" s="54"/>
       <c r="C37" s="31" t="s">
         <v>14</v>
       </c>
@@ -3026,16 +3116,16 @@
       <c r="E37" s="3">
         <v>498.125</v>
       </c>
-      <c r="F37" s="50">
+      <c r="F37" s="49">
         <v>-0.45140000000000002</v>
       </c>
-      <c r="G37" s="50">
+      <c r="G37" s="49">
         <v>-0.45279999999999998</v>
       </c>
       <c r="H37" s="4">
         <v>27</v>
       </c>
-      <c r="I37" s="49">
+      <c r="I37" s="48">
         <v>9</v>
       </c>
       <c r="J37" s="3">
@@ -3062,36 +3152,37 @@
       <c r="Q37" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R37" s="71"/>
-      <c r="S37" s="72"/>
-      <c r="T37" s="72"/>
-      <c r="U37" s="72"/>
-      <c r="V37" s="72"/>
-      <c r="W37" s="73"/>
+      <c r="R37" s="70"/>
+      <c r="S37" s="71"/>
+      <c r="T37" s="71"/>
+      <c r="U37" s="71"/>
+      <c r="V37" s="71"/>
+      <c r="W37" s="72"/>
     </row>
     <row r="38" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="53" t="s">
+      <c r="A38" s="118"/>
+      <c r="B38" s="52" t="s">
         <v>66</v>
       </c>
       <c r="C38" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="D38" s="48">
+      <c r="D38" s="95">
         <v>42.213999999999999</v>
       </c>
-      <c r="E38" s="9">
+      <c r="E38" s="93">
         <v>92.585999999999999</v>
       </c>
-      <c r="F38" s="9">
+      <c r="F38" s="93">
         <v>0.94740000000000002</v>
       </c>
-      <c r="G38" s="9">
+      <c r="G38" s="93">
         <v>0.94730000000000003</v>
       </c>
-      <c r="H38" s="10">
+      <c r="H38" s="94">
         <v>22.9</v>
       </c>
-      <c r="I38" s="52">
+      <c r="I38" s="51">
         <v>240</v>
       </c>
       <c r="J38" s="9">
@@ -3118,15 +3209,16 @@
       <c r="Q38" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R38" s="56"/>
-      <c r="S38" s="57"/>
-      <c r="T38" s="57"/>
-      <c r="U38" s="57"/>
-      <c r="V38" s="57"/>
-      <c r="W38" s="58"/>
+      <c r="R38" s="55"/>
+      <c r="S38" s="56"/>
+      <c r="T38" s="56"/>
+      <c r="U38" s="56"/>
+      <c r="V38" s="56"/>
+      <c r="W38" s="57"/>
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B39" s="54"/>
+      <c r="A39" s="118"/>
+      <c r="B39" s="53"/>
       <c r="C39" s="30" t="s">
         <v>12</v>
       </c>
@@ -3145,7 +3237,7 @@
       <c r="H39" s="8">
         <v>23.6</v>
       </c>
-      <c r="I39" s="51">
+      <c r="I39" s="50">
         <v>240</v>
       </c>
       <c r="J39">
@@ -3172,15 +3264,16 @@
       <c r="Q39" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R39" s="59"/>
-      <c r="S39" s="60"/>
-      <c r="T39" s="60"/>
-      <c r="U39" s="60"/>
-      <c r="V39" s="60"/>
-      <c r="W39" s="61"/>
+      <c r="R39" s="58"/>
+      <c r="S39" s="59"/>
+      <c r="T39" s="59"/>
+      <c r="U39" s="59"/>
+      <c r="V39" s="59"/>
+      <c r="W39" s="60"/>
     </row>
     <row r="40" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="55"/>
+      <c r="A40" s="118"/>
+      <c r="B40" s="54"/>
       <c r="C40" s="31" t="s">
         <v>14</v>
       </c>
@@ -3199,7 +3292,7 @@
       <c r="H40" s="4">
         <v>27</v>
       </c>
-      <c r="I40" s="49">
+      <c r="I40" s="48">
         <v>240</v>
       </c>
       <c r="J40" s="3">
@@ -3226,16 +3319,616 @@
       <c r="Q40" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R40" s="62"/>
-      <c r="S40" s="63"/>
-      <c r="T40" s="63"/>
-      <c r="U40" s="63"/>
-      <c r="V40" s="63"/>
-      <c r="W40" s="64"/>
-    </row>
-    <row r="41" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+      <c r="R40" s="61"/>
+      <c r="S40" s="62"/>
+      <c r="T40" s="62"/>
+      <c r="U40" s="62"/>
+      <c r="V40" s="62"/>
+      <c r="W40" s="63"/>
+    </row>
+    <row r="41" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="118"/>
+      <c r="B41" s="52" t="s">
+        <v>74</v>
+      </c>
+      <c r="C41" s="96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" s="102">
+        <v>48614</v>
+      </c>
+      <c r="E41" s="103">
+        <v>99.918999999999997</v>
+      </c>
+      <c r="F41" s="103">
+        <v>0.94159999999999999</v>
+      </c>
+      <c r="G41" s="103">
+        <v>0.94159999999999999</v>
+      </c>
+      <c r="H41" s="104">
+        <v>22.9</v>
+      </c>
+      <c r="I41" s="51">
+        <v>21</v>
+      </c>
+      <c r="J41" s="103">
+        <v>232.8</v>
+      </c>
+      <c r="K41" s="103">
+        <v>6</v>
+      </c>
+      <c r="L41" s="105" t="s">
+        <v>73</v>
+      </c>
+      <c r="M41" s="103">
+        <v>64</v>
+      </c>
+      <c r="N41" s="103">
+        <v>64</v>
+      </c>
+      <c r="O41" s="105" t="s">
+        <v>39</v>
+      </c>
+      <c r="P41" s="103">
+        <v>0.2</v>
+      </c>
+      <c r="Q41" s="104">
+        <v>1E-3</v>
+      </c>
+      <c r="R41" s="55" t="s">
+        <v>76</v>
+      </c>
+      <c r="S41" s="56"/>
+      <c r="T41" s="56"/>
+      <c r="U41" s="56"/>
+      <c r="V41" s="56"/>
+      <c r="W41" s="57"/>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A42" s="118"/>
+      <c r="B42" s="53"/>
+      <c r="C42" s="96" t="s">
+        <v>12</v>
+      </c>
+      <c r="D42" s="113">
+        <v>45.213999999999999</v>
+      </c>
+      <c r="E42" s="114">
+        <v>93.855999999999995</v>
+      </c>
+      <c r="F42" s="114">
+        <v>0.94850000000000001</v>
+      </c>
+      <c r="G42" s="114">
+        <v>0.94850000000000001</v>
+      </c>
+      <c r="H42" s="92">
+        <v>23.6</v>
+      </c>
+      <c r="I42" s="50">
+        <v>21</v>
+      </c>
+      <c r="J42" s="106">
+        <v>562.19000000000005</v>
+      </c>
+      <c r="K42" s="97">
+        <v>6</v>
+      </c>
+      <c r="L42" s="98" t="s">
+        <v>72</v>
+      </c>
+      <c r="M42" s="97">
+        <v>64</v>
+      </c>
+      <c r="N42" s="97">
+        <v>32</v>
+      </c>
+      <c r="O42" s="98" t="s">
+        <v>39</v>
+      </c>
+      <c r="P42" s="97">
+        <v>0.1</v>
+      </c>
+      <c r="Q42" s="99">
+        <v>1E-3</v>
+      </c>
+      <c r="R42" s="58"/>
+      <c r="S42" s="107"/>
+      <c r="T42" s="107"/>
+      <c r="U42" s="107"/>
+      <c r="V42" s="107"/>
+      <c r="W42" s="60"/>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A43" s="118"/>
+      <c r="B43" s="53"/>
+      <c r="C43" s="96" t="s">
+        <v>14</v>
+      </c>
+      <c r="D43" s="100">
+        <v>73.799000000000007</v>
+      </c>
+      <c r="E43" s="97">
+        <v>132.626</v>
+      </c>
+      <c r="F43" s="97">
+        <v>0.8972</v>
+      </c>
+      <c r="G43" s="97">
+        <v>0.89710000000000001</v>
+      </c>
+      <c r="H43" s="99">
+        <v>27</v>
+      </c>
+      <c r="I43" s="50">
+        <v>21</v>
+      </c>
+      <c r="J43" s="106">
+        <v>690.97</v>
+      </c>
+      <c r="K43" s="97">
+        <v>6</v>
+      </c>
+      <c r="L43" s="98" t="s">
+        <v>49</v>
+      </c>
+      <c r="M43" s="97">
+        <v>64</v>
+      </c>
+      <c r="N43" s="108" t="s">
+        <v>48</v>
+      </c>
+      <c r="O43" s="98" t="s">
+        <v>39</v>
+      </c>
+      <c r="P43" s="97">
+        <v>0.1</v>
+      </c>
+      <c r="Q43" s="99">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R43" s="58"/>
+      <c r="S43" s="107"/>
+      <c r="T43" s="107"/>
+      <c r="U43" s="107"/>
+      <c r="V43" s="107"/>
+      <c r="W43" s="60"/>
+    </row>
+    <row r="44" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="118"/>
+      <c r="B44" s="54"/>
+      <c r="C44" s="101" t="s">
+        <v>70</v>
+      </c>
+      <c r="D44" s="109">
+        <v>71.367000000000004</v>
+      </c>
+      <c r="E44" s="110">
+        <v>142.86600000000001</v>
+      </c>
+      <c r="F44" s="110">
+        <v>0.88070000000000004</v>
+      </c>
+      <c r="G44" s="110">
+        <v>0.88060000000000005</v>
+      </c>
+      <c r="H44" s="111">
+        <v>22</v>
+      </c>
+      <c r="I44" s="48">
+        <v>21</v>
+      </c>
+      <c r="J44" s="3">
+        <v>168.8</v>
+      </c>
+      <c r="K44" s="110">
+        <v>6</v>
+      </c>
+      <c r="L44" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="M44" s="110">
+        <v>64</v>
+      </c>
+      <c r="N44" s="110">
+        <v>32</v>
+      </c>
+      <c r="O44" s="112" t="s">
+        <v>39</v>
+      </c>
+      <c r="P44" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q44" s="111">
+        <v>1E-3</v>
+      </c>
+      <c r="R44" s="61"/>
+      <c r="S44" s="62"/>
+      <c r="T44" s="62"/>
+      <c r="U44" s="62"/>
+      <c r="V44" s="62"/>
+      <c r="W44" s="63"/>
+    </row>
+    <row r="45" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="118"/>
+      <c r="B45" s="52" t="s">
+        <v>75</v>
+      </c>
+      <c r="C45" s="96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D45" s="113">
+        <v>47.497999999999998</v>
+      </c>
+      <c r="E45" s="114">
+        <v>98.091999999999999</v>
+      </c>
+      <c r="F45" s="114">
+        <v>0.94379999999999997</v>
+      </c>
+      <c r="G45" s="114">
+        <v>0.94369999999999998</v>
+      </c>
+      <c r="H45" s="92">
+        <v>22.9</v>
+      </c>
+      <c r="I45" s="50">
+        <v>30</v>
+      </c>
+      <c r="J45" s="97">
+        <v>367.69</v>
+      </c>
+      <c r="K45" s="103">
+        <v>6</v>
+      </c>
+      <c r="L45" s="98" t="s">
+        <v>78</v>
+      </c>
+      <c r="M45" s="103">
+        <v>64</v>
+      </c>
+      <c r="N45" s="116">
+        <v>64</v>
+      </c>
+      <c r="O45" s="98" t="s">
+        <v>39</v>
+      </c>
+      <c r="P45" s="116">
+        <v>0.1</v>
+      </c>
+      <c r="Q45" s="104">
+        <v>1E-3</v>
+      </c>
+      <c r="R45" s="115" t="s">
+        <v>77</v>
+      </c>
+      <c r="S45" s="56"/>
+      <c r="T45" s="56"/>
+      <c r="U45" s="56"/>
+      <c r="V45" s="56"/>
+      <c r="W45" s="57"/>
+    </row>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A46" s="118"/>
+      <c r="B46" s="53"/>
+      <c r="C46" s="96" t="s">
+        <v>12</v>
+      </c>
+      <c r="D46" s="113">
+        <v>47.232999999999997</v>
+      </c>
+      <c r="E46" s="114">
+        <v>96.742000000000004</v>
+      </c>
+      <c r="F46" s="114">
+        <v>0.94530000000000003</v>
+      </c>
+      <c r="G46" s="114">
+        <v>0.94530000000000003</v>
+      </c>
+      <c r="H46" s="92">
+        <v>79.099999999999994</v>
+      </c>
+      <c r="I46" s="50">
+        <v>30</v>
+      </c>
+      <c r="J46" s="97">
+        <v>671.14</v>
+      </c>
+      <c r="K46" s="97">
+        <v>6</v>
+      </c>
+      <c r="L46" s="98" t="s">
+        <v>79</v>
+      </c>
+      <c r="M46" s="97">
+        <v>64</v>
+      </c>
+      <c r="N46" s="116">
+        <v>64</v>
+      </c>
+      <c r="O46" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="P46" s="116">
+        <v>0.1</v>
+      </c>
+      <c r="Q46" s="99">
+        <v>1E-3</v>
+      </c>
+      <c r="R46" s="58"/>
+      <c r="S46" s="107"/>
+      <c r="T46" s="107"/>
+      <c r="U46" s="107"/>
+      <c r="V46" s="107"/>
+      <c r="W46" s="60"/>
+    </row>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A47" s="118"/>
+      <c r="B47" s="53"/>
+      <c r="C47" s="96" t="s">
+        <v>14</v>
+      </c>
+      <c r="D47" s="100">
+        <v>65.77</v>
+      </c>
+      <c r="E47" s="97">
+        <v>126.881</v>
+      </c>
+      <c r="F47" s="97">
+        <v>0.90590000000000004</v>
+      </c>
+      <c r="G47" s="97">
+        <v>0.90580000000000005</v>
+      </c>
+      <c r="H47" s="99">
+        <v>61.1</v>
+      </c>
+      <c r="I47" s="50">
+        <v>30</v>
+      </c>
+      <c r="J47" s="97">
+        <v>698.6</v>
+      </c>
+      <c r="K47" s="97">
+        <v>6</v>
+      </c>
+      <c r="L47" s="98" t="s">
+        <v>49</v>
+      </c>
+      <c r="M47" s="97">
+        <v>64</v>
+      </c>
+      <c r="N47" s="116">
+        <v>64</v>
+      </c>
+      <c r="O47" s="98" t="s">
+        <v>39</v>
+      </c>
+      <c r="P47" s="116">
+        <v>0.1</v>
+      </c>
+      <c r="Q47" s="99">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R47" s="58"/>
+      <c r="S47" s="107"/>
+      <c r="T47" s="107"/>
+      <c r="U47" s="107"/>
+      <c r="V47" s="107"/>
+      <c r="W47" s="60"/>
+    </row>
+    <row r="48" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="118"/>
+      <c r="B48" s="54"/>
+      <c r="C48" s="101" t="s">
+        <v>70</v>
+      </c>
+      <c r="D48" s="2">
+        <v>62.356000000000002</v>
+      </c>
+      <c r="E48" s="3">
+        <v>124.98399999999999</v>
+      </c>
+      <c r="F48" s="3">
+        <v>0.9073</v>
+      </c>
+      <c r="G48" s="3">
+        <v>0.90720000000000001</v>
+      </c>
+      <c r="H48" s="4">
+        <v>63.9</v>
+      </c>
+      <c r="I48" s="48">
+        <v>30</v>
+      </c>
+      <c r="J48" s="3">
+        <v>145.22999999999999</v>
+      </c>
+      <c r="K48" s="110">
+        <v>6</v>
+      </c>
+      <c r="L48" s="98" t="s">
+        <v>49</v>
+      </c>
+      <c r="M48" s="110">
+        <v>64</v>
+      </c>
+      <c r="N48" s="28">
+        <v>64</v>
+      </c>
+      <c r="O48" s="112" t="s">
+        <v>39</v>
+      </c>
+      <c r="P48" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q48" s="111">
+        <v>1E-3</v>
+      </c>
+      <c r="R48" s="61"/>
+      <c r="S48" s="62"/>
+      <c r="T48" s="62"/>
+      <c r="U48" s="62"/>
+      <c r="V48" s="62"/>
+      <c r="W48" s="63"/>
+    </row>
+    <row r="49" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="117"/>
+      <c r="B49" s="52" t="s">
+        <v>80</v>
+      </c>
+      <c r="C49" s="96" t="s">
+        <v>13</v>
+      </c>
+      <c r="I49" s="50">
+        <v>18</v>
+      </c>
+      <c r="K49" s="103">
+        <v>6</v>
+      </c>
+      <c r="L49" s="9"/>
+      <c r="M49" s="103">
+        <v>64</v>
+      </c>
+      <c r="N49" s="97">
+        <v>64</v>
+      </c>
+      <c r="O49" s="98" t="s">
+        <v>39</v>
+      </c>
+      <c r="P49" s="116">
+        <v>0.1</v>
+      </c>
+      <c r="Q49" s="104">
+        <v>1E-3</v>
+      </c>
+      <c r="R49" s="55"/>
+      <c r="S49" s="56"/>
+      <c r="T49" s="56"/>
+      <c r="U49" s="56"/>
+      <c r="V49" s="56"/>
+      <c r="W49" s="57"/>
+    </row>
+    <row r="50" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A50" s="117"/>
+      <c r="B50" s="53"/>
+      <c r="C50" s="96" t="s">
+        <v>12</v>
+      </c>
+      <c r="I50" s="50">
+        <v>18</v>
+      </c>
+      <c r="K50" s="97">
+        <v>6</v>
+      </c>
+      <c r="M50" s="97">
+        <v>64</v>
+      </c>
+      <c r="N50" s="97">
+        <v>64</v>
+      </c>
+      <c r="O50" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="P50" s="116">
+        <v>0.1</v>
+      </c>
+      <c r="Q50" s="99">
+        <v>1E-3</v>
+      </c>
+      <c r="R50" s="58"/>
+      <c r="S50" s="107"/>
+      <c r="T50" s="107"/>
+      <c r="U50" s="107"/>
+      <c r="V50" s="107"/>
+      <c r="W50" s="60"/>
+    </row>
+    <row r="51" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A51" s="117"/>
+      <c r="B51" s="53"/>
+      <c r="C51" s="96" t="s">
+        <v>14</v>
+      </c>
+      <c r="I51" s="50">
+        <v>18</v>
+      </c>
+      <c r="K51" s="97">
+        <v>6</v>
+      </c>
+      <c r="M51" s="97">
+        <v>64</v>
+      </c>
+      <c r="N51" s="97">
+        <v>64</v>
+      </c>
+      <c r="O51" s="98" t="s">
+        <v>39</v>
+      </c>
+      <c r="P51" s="116">
+        <v>0.1</v>
+      </c>
+      <c r="Q51" s="99">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R51" s="58"/>
+      <c r="S51" s="107"/>
+      <c r="T51" s="107"/>
+      <c r="U51" s="107"/>
+      <c r="V51" s="107"/>
+      <c r="W51" s="60"/>
+    </row>
+    <row r="52" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="117"/>
+      <c r="B52" s="54"/>
+      <c r="C52" s="101" t="s">
+        <v>70</v>
+      </c>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="4"/>
+      <c r="I52" s="48">
+        <v>18</v>
+      </c>
+      <c r="J52" s="3"/>
+      <c r="K52" s="110">
+        <v>6</v>
+      </c>
+      <c r="L52" s="3"/>
+      <c r="M52" s="110">
+        <v>64</v>
+      </c>
+      <c r="N52" s="110">
+        <v>64</v>
+      </c>
+      <c r="O52" s="112" t="s">
+        <v>39</v>
+      </c>
+      <c r="P52" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q52" s="111">
+        <v>1E-3</v>
+      </c>
+      <c r="R52" s="61"/>
+      <c r="S52" s="62"/>
+      <c r="T52" s="62"/>
+      <c r="U52" s="62"/>
+      <c r="V52" s="62"/>
+      <c r="W52" s="63"/>
+    </row>
+    <row r="53" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="33">
+    <mergeCell ref="B41:B44"/>
+    <mergeCell ref="R41:W44"/>
+    <mergeCell ref="R45:W48"/>
+    <mergeCell ref="B45:B48"/>
+    <mergeCell ref="R49:W52"/>
+    <mergeCell ref="B49:B52"/>
     <mergeCell ref="B23:B25"/>
     <mergeCell ref="R23:W25"/>
     <mergeCell ref="B26:B28"/>

</xml_diff>

<commit_message>
Entrenamiento con ventana de 3 horas
</commit_message>
<xml_diff>
--- a/modelos_tfg/MetricasValidacion.xlsx
+++ b/modelos_tfg/MetricasValidacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\modelos_tfg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0763A6D6-C557-46EC-8090-E7332E54B1AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A23E8642-E969-4681-8535-F672818A1128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="77">
   <si>
     <t>ID Train</t>
   </si>
@@ -213,13 +213,7 @@
 Además, he modificado la estructura de los modelos. Básicamente he combinado la V7 y V8</t>
   </si>
   <si>
-    <t>V10</t>
-  </si>
-  <si>
     <t>Simplemente he modificado el seq_length</t>
-  </si>
-  <si>
-    <t>V11</t>
   </si>
   <si>
     <t>73 (ES)</t>
@@ -229,9 +223,6 @@
 pequeña, he eliminado Pot_gen de las features y he hecho más simple la LSTM</t>
   </si>
   <si>
-    <t>V12</t>
-  </si>
-  <si>
     <t>66 (ES)</t>
   </si>
   <si>
@@ -251,12 +242,6 @@
   </si>
   <si>
     <t>64 (ES)</t>
-  </si>
-  <si>
-    <t>V13</t>
-  </si>
-  <si>
-    <t>V14</t>
   </si>
   <si>
     <t>He añadido un modelo CNN</t>
@@ -273,7 +258,10 @@
     <t>56 (ES)</t>
   </si>
   <si>
-    <t>V15</t>
+    <t>61 (ES)</t>
+  </si>
+  <si>
+    <t>97 (ES)</t>
   </si>
 </sst>
 </file>
@@ -612,7 +600,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -699,163 +687,139 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1223,31 +1187,31 @@
   <sheetData>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D3" s="74" t="s">
+      <c r="D3" s="90" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="75"/>
-      <c r="F3" s="75"/>
-      <c r="G3" s="75"/>
-      <c r="H3" s="76"/>
-      <c r="I3" s="77" t="s">
+      <c r="E3" s="91"/>
+      <c r="F3" s="91"/>
+      <c r="G3" s="91"/>
+      <c r="H3" s="92"/>
+      <c r="I3" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="78"/>
-      <c r="K3" s="78"/>
-      <c r="L3" s="78"/>
-      <c r="M3" s="78"/>
-      <c r="N3" s="78"/>
-      <c r="O3" s="78"/>
-      <c r="P3" s="78"/>
-      <c r="Q3" s="79"/>
-      <c r="R3" s="84" t="s">
+      <c r="J3" s="94"/>
+      <c r="K3" s="94"/>
+      <c r="L3" s="94"/>
+      <c r="M3" s="94"/>
+      <c r="N3" s="94"/>
+      <c r="O3" s="94"/>
+      <c r="P3" s="94"/>
+      <c r="Q3" s="95"/>
+      <c r="R3" s="97" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="85"/>
-      <c r="T3" s="85"/>
-      <c r="U3" s="85"/>
-      <c r="V3" s="85"/>
+      <c r="S3" s="98"/>
+      <c r="T3" s="98"/>
+      <c r="U3" s="98"/>
+      <c r="V3" s="98"/>
       <c r="W3" s="86"/>
     </row>
     <row r="4" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1299,16 +1263,16 @@
       <c r="Q4" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="87"/>
-      <c r="S4" s="88"/>
-      <c r="T4" s="88"/>
-      <c r="U4" s="88"/>
-      <c r="V4" s="88"/>
-      <c r="W4" s="89"/>
+      <c r="R4" s="99"/>
+      <c r="S4" s="100"/>
+      <c r="T4" s="100"/>
+      <c r="U4" s="100"/>
+      <c r="V4" s="100"/>
+      <c r="W4" s="88"/>
     </row>
     <row r="5" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
-      <c r="B5" s="80" t="s">
+      <c r="B5" s="96" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -1356,18 +1320,18 @@
       <c r="Q5" s="17">
         <v>1E-3</v>
       </c>
-      <c r="R5" s="73" t="s">
+      <c r="R5" s="83" t="s">
         <v>38</v>
       </c>
-      <c r="S5" s="65"/>
-      <c r="T5" s="65"/>
-      <c r="U5" s="65"/>
-      <c r="V5" s="65"/>
-      <c r="W5" s="66"/>
+      <c r="S5" s="75"/>
+      <c r="T5" s="75"/>
+      <c r="U5" s="75"/>
+      <c r="V5" s="75"/>
+      <c r="W5" s="76"/>
     </row>
     <row r="6" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
-      <c r="B6" s="81"/>
+      <c r="B6" s="85"/>
       <c r="C6" s="5" t="s">
         <v>12</v>
       </c>
@@ -1413,16 +1377,16 @@
       <c r="Q6" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R6" s="67"/>
-      <c r="S6" s="68"/>
-      <c r="T6" s="68"/>
-      <c r="U6" s="68"/>
-      <c r="V6" s="68"/>
-      <c r="W6" s="69"/>
+      <c r="R6" s="77"/>
+      <c r="S6" s="78"/>
+      <c r="T6" s="78"/>
+      <c r="U6" s="78"/>
+      <c r="V6" s="78"/>
+      <c r="W6" s="79"/>
     </row>
     <row r="7" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8"/>
-      <c r="B7" s="82"/>
+      <c r="B7" s="89"/>
       <c r="C7" s="14" t="s">
         <v>14</v>
       </c>
@@ -1468,16 +1432,16 @@
       <c r="Q7" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R7" s="70"/>
-      <c r="S7" s="71"/>
-      <c r="T7" s="71"/>
-      <c r="U7" s="71"/>
-      <c r="V7" s="71"/>
-      <c r="W7" s="72"/>
+      <c r="R7" s="80"/>
+      <c r="S7" s="81"/>
+      <c r="T7" s="81"/>
+      <c r="U7" s="81"/>
+      <c r="V7" s="81"/>
+      <c r="W7" s="82"/>
     </row>
     <row r="8" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
-      <c r="B8" s="83" t="s">
+      <c r="B8" s="84" t="s">
         <v>24</v>
       </c>
       <c r="C8" s="5" t="s">
@@ -1525,18 +1489,18 @@
       <c r="Q8" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R8" s="73" t="s">
+      <c r="R8" s="83" t="s">
         <v>38</v>
       </c>
-      <c r="S8" s="65"/>
-      <c r="T8" s="65"/>
-      <c r="U8" s="65"/>
-      <c r="V8" s="65"/>
-      <c r="W8" s="66"/>
+      <c r="S8" s="75"/>
+      <c r="T8" s="75"/>
+      <c r="U8" s="75"/>
+      <c r="V8" s="75"/>
+      <c r="W8" s="76"/>
     </row>
     <row r="9" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
-      <c r="B9" s="81"/>
+      <c r="B9" s="85"/>
       <c r="C9" s="5" t="s">
         <v>12</v>
       </c>
@@ -1582,16 +1546,16 @@
       <c r="Q9" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R9" s="67"/>
-      <c r="S9" s="68"/>
-      <c r="T9" s="68"/>
-      <c r="U9" s="68"/>
-      <c r="V9" s="68"/>
-      <c r="W9" s="69"/>
+      <c r="R9" s="77"/>
+      <c r="S9" s="78"/>
+      <c r="T9" s="78"/>
+      <c r="U9" s="78"/>
+      <c r="V9" s="78"/>
+      <c r="W9" s="79"/>
     </row>
     <row r="10" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8"/>
-      <c r="B10" s="82"/>
+      <c r="B10" s="89"/>
       <c r="C10" s="5" t="s">
         <v>14</v>
       </c>
@@ -1637,15 +1601,15 @@
       <c r="Q10" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R10" s="70"/>
-      <c r="S10" s="71"/>
-      <c r="T10" s="71"/>
-      <c r="U10" s="71"/>
-      <c r="V10" s="71"/>
-      <c r="W10" s="72"/>
+      <c r="R10" s="80"/>
+      <c r="S10" s="81"/>
+      <c r="T10" s="81"/>
+      <c r="U10" s="81"/>
+      <c r="V10" s="81"/>
+      <c r="W10" s="82"/>
     </row>
     <row r="11" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="83" t="s">
+      <c r="B11" s="84" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="29" t="s">
@@ -1693,17 +1657,17 @@
       <c r="Q11" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R11" s="73" t="s">
+      <c r="R11" s="83" t="s">
         <v>38</v>
       </c>
-      <c r="S11" s="65"/>
-      <c r="T11" s="65"/>
-      <c r="U11" s="65"/>
-      <c r="V11" s="65"/>
-      <c r="W11" s="66"/>
+      <c r="S11" s="75"/>
+      <c r="T11" s="75"/>
+      <c r="U11" s="75"/>
+      <c r="V11" s="75"/>
+      <c r="W11" s="76"/>
     </row>
     <row r="12" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="81"/>
+      <c r="B12" s="85"/>
       <c r="C12" s="26" t="s">
         <v>12</v>
       </c>
@@ -1749,15 +1713,15 @@
       <c r="Q12" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R12" s="67"/>
-      <c r="S12" s="68"/>
-      <c r="T12" s="68"/>
-      <c r="U12" s="68"/>
-      <c r="V12" s="68"/>
-      <c r="W12" s="69"/>
+      <c r="R12" s="77"/>
+      <c r="S12" s="78"/>
+      <c r="T12" s="78"/>
+      <c r="U12" s="78"/>
+      <c r="V12" s="78"/>
+      <c r="W12" s="79"/>
     </row>
     <row r="13" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="81"/>
+      <c r="B13" s="85"/>
       <c r="C13" s="27" t="s">
         <v>14</v>
       </c>
@@ -1803,15 +1767,15 @@
       <c r="Q13" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R13" s="70"/>
-      <c r="S13" s="71"/>
-      <c r="T13" s="71"/>
-      <c r="U13" s="71"/>
-      <c r="V13" s="71"/>
-      <c r="W13" s="72"/>
+      <c r="R13" s="80"/>
+      <c r="S13" s="81"/>
+      <c r="T13" s="81"/>
+      <c r="U13" s="81"/>
+      <c r="V13" s="81"/>
+      <c r="W13" s="82"/>
     </row>
     <row r="14" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="83" t="s">
+      <c r="B14" s="84" t="s">
         <v>36</v>
       </c>
       <c r="C14" s="20" t="s">
@@ -1859,17 +1823,17 @@
       <c r="Q14" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R14" s="73" t="s">
+      <c r="R14" s="83" t="s">
         <v>37</v>
       </c>
-      <c r="S14" s="65"/>
-      <c r="T14" s="65"/>
-      <c r="U14" s="65"/>
-      <c r="V14" s="65"/>
-      <c r="W14" s="66"/>
+      <c r="S14" s="75"/>
+      <c r="T14" s="75"/>
+      <c r="U14" s="75"/>
+      <c r="V14" s="75"/>
+      <c r="W14" s="76"/>
     </row>
     <row r="15" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="81"/>
+      <c r="B15" s="85"/>
       <c r="C15" s="30" t="s">
         <v>12</v>
       </c>
@@ -1915,15 +1879,15 @@
       <c r="Q15" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R15" s="67"/>
-      <c r="S15" s="68"/>
-      <c r="T15" s="68"/>
-      <c r="U15" s="68"/>
-      <c r="V15" s="68"/>
-      <c r="W15" s="69"/>
+      <c r="R15" s="77"/>
+      <c r="S15" s="78"/>
+      <c r="T15" s="78"/>
+      <c r="U15" s="78"/>
+      <c r="V15" s="78"/>
+      <c r="W15" s="79"/>
     </row>
     <row r="16" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="82"/>
+      <c r="B16" s="89"/>
       <c r="C16" s="31" t="s">
         <v>14</v>
       </c>
@@ -1969,12 +1933,12 @@
       <c r="Q16" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R16" s="70"/>
-      <c r="S16" s="71"/>
-      <c r="T16" s="71"/>
-      <c r="U16" s="71"/>
-      <c r="V16" s="71"/>
-      <c r="W16" s="72"/>
+      <c r="R16" s="80"/>
+      <c r="S16" s="81"/>
+      <c r="T16" s="81"/>
+      <c r="U16" s="81"/>
+      <c r="V16" s="81"/>
+      <c r="W16" s="82"/>
     </row>
     <row r="17" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
@@ -2026,18 +1990,18 @@
       <c r="Q17" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R17" s="65" t="s">
+      <c r="R17" s="75" t="s">
         <v>43</v>
       </c>
-      <c r="S17" s="65"/>
-      <c r="T17" s="65"/>
-      <c r="U17" s="65"/>
-      <c r="V17" s="65"/>
-      <c r="W17" s="66"/>
+      <c r="S17" s="75"/>
+      <c r="T17" s="75"/>
+      <c r="U17" s="75"/>
+      <c r="V17" s="75"/>
+      <c r="W17" s="76"/>
     </row>
     <row r="18" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
-      <c r="B18" s="90"/>
+      <c r="B18" s="87"/>
       <c r="C18" s="30" t="s">
         <v>12</v>
       </c>
@@ -2083,16 +2047,16 @@
       <c r="Q18" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R18" s="68"/>
-      <c r="S18" s="68"/>
-      <c r="T18" s="68"/>
-      <c r="U18" s="68"/>
-      <c r="V18" s="68"/>
-      <c r="W18" s="69"/>
+      <c r="R18" s="78"/>
+      <c r="S18" s="78"/>
+      <c r="T18" s="78"/>
+      <c r="U18" s="78"/>
+      <c r="V18" s="78"/>
+      <c r="W18" s="79"/>
     </row>
     <row r="19" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8"/>
-      <c r="B19" s="89"/>
+      <c r="B19" s="88"/>
       <c r="C19" s="31" t="s">
         <v>14</v>
       </c>
@@ -2138,16 +2102,16 @@
       <c r="Q19" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R19" s="71"/>
-      <c r="S19" s="71"/>
-      <c r="T19" s="71"/>
-      <c r="U19" s="71"/>
-      <c r="V19" s="71"/>
-      <c r="W19" s="72"/>
+      <c r="R19" s="81"/>
+      <c r="S19" s="81"/>
+      <c r="T19" s="81"/>
+      <c r="U19" s="81"/>
+      <c r="V19" s="81"/>
+      <c r="W19" s="82"/>
     </row>
     <row r="20" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8"/>
-      <c r="B20" s="83" t="s">
+      <c r="B20" s="84" t="s">
         <v>46</v>
       </c>
       <c r="C20" s="30" t="s">
@@ -2195,18 +2159,18 @@
       <c r="Q20" s="36">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R20" s="64" t="s">
+      <c r="R20" s="74" t="s">
         <v>45</v>
       </c>
-      <c r="S20" s="65"/>
-      <c r="T20" s="65"/>
-      <c r="U20" s="65"/>
-      <c r="V20" s="65"/>
-      <c r="W20" s="66"/>
+      <c r="S20" s="75"/>
+      <c r="T20" s="75"/>
+      <c r="U20" s="75"/>
+      <c r="V20" s="75"/>
+      <c r="W20" s="76"/>
     </row>
     <row r="21" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
-      <c r="B21" s="81"/>
+      <c r="B21" s="85"/>
       <c r="C21" s="30" t="s">
         <v>12</v>
       </c>
@@ -2252,16 +2216,16 @@
       <c r="Q21" s="37">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R21" s="67"/>
-      <c r="S21" s="68"/>
-      <c r="T21" s="68"/>
-      <c r="U21" s="68"/>
-      <c r="V21" s="68"/>
-      <c r="W21" s="69"/>
-    </row>
-    <row r="22" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R21" s="77"/>
+      <c r="S21" s="78"/>
+      <c r="T21" s="78"/>
+      <c r="U21" s="78"/>
+      <c r="V21" s="78"/>
+      <c r="W21" s="79"/>
+    </row>
+    <row r="22" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="8"/>
-      <c r="B22" s="82"/>
+      <c r="B22" s="89"/>
       <c r="C22" s="31" t="s">
         <v>14</v>
       </c>
@@ -2307,17 +2271,17 @@
       <c r="Q22" s="38">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R22" s="70"/>
-      <c r="S22" s="71"/>
-      <c r="T22" s="71"/>
-      <c r="U22" s="71"/>
-      <c r="V22" s="71"/>
-      <c r="W22" s="72"/>
+      <c r="R22" s="80"/>
+      <c r="S22" s="81"/>
+      <c r="T22" s="81"/>
+      <c r="U22" s="81"/>
+      <c r="V22" s="81"/>
+      <c r="W22" s="82"/>
     </row>
     <row r="23" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="117"/>
-      <c r="B23" s="52" t="s">
-        <v>50</v>
+      <c r="A23" s="59"/>
+      <c r="B23" s="61" t="s">
+        <v>15</v>
       </c>
       <c r="C23" s="20" t="s">
         <v>13</v>
@@ -2364,34 +2328,34 @@
       <c r="Q23" s="10">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R23" s="64" t="s">
+      <c r="R23" s="74" t="s">
         <v>53</v>
       </c>
-      <c r="S23" s="65"/>
-      <c r="T23" s="65"/>
-      <c r="U23" s="65"/>
-      <c r="V23" s="65"/>
-      <c r="W23" s="66"/>
+      <c r="S23" s="75"/>
+      <c r="T23" s="75"/>
+      <c r="U23" s="75"/>
+      <c r="V23" s="75"/>
+      <c r="W23" s="76"/>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A24" s="117"/>
-      <c r="B24" s="53"/>
+      <c r="A24" s="59"/>
+      <c r="B24" s="62"/>
       <c r="C24" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="91">
+      <c r="D24" s="52">
         <v>51.393000000000001</v>
       </c>
-      <c r="E24" s="91">
+      <c r="E24" s="52">
         <v>110.699</v>
       </c>
-      <c r="F24" s="91">
+      <c r="F24" s="52">
         <v>0.9274</v>
       </c>
-      <c r="G24" s="91">
+      <c r="G24" s="52">
         <v>0.92730000000000001</v>
       </c>
-      <c r="H24" s="92">
+      <c r="H24" s="53">
         <v>35.4</v>
       </c>
       <c r="I24">
@@ -2421,16 +2385,16 @@
       <c r="Q24" s="8">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R24" s="67"/>
-      <c r="S24" s="68"/>
-      <c r="T24" s="68"/>
-      <c r="U24" s="68"/>
-      <c r="V24" s="68"/>
-      <c r="W24" s="69"/>
+      <c r="R24" s="77"/>
+      <c r="S24" s="78"/>
+      <c r="T24" s="78"/>
+      <c r="U24" s="78"/>
+      <c r="V24" s="78"/>
+      <c r="W24" s="79"/>
     </row>
     <row r="25" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="117"/>
-      <c r="B25" s="54"/>
+      <c r="A25" s="59"/>
+      <c r="B25" s="63"/>
       <c r="C25" s="31" t="s">
         <v>14</v>
       </c>
@@ -2476,34 +2440,34 @@
       <c r="Q25" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R25" s="70"/>
-      <c r="S25" s="71"/>
-      <c r="T25" s="71"/>
-      <c r="U25" s="71"/>
-      <c r="V25" s="71"/>
-      <c r="W25" s="72"/>
+      <c r="R25" s="80"/>
+      <c r="S25" s="81"/>
+      <c r="T25" s="81"/>
+      <c r="U25" s="81"/>
+      <c r="V25" s="81"/>
+      <c r="W25" s="82"/>
     </row>
     <row r="26" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="117"/>
-      <c r="B26" s="52" t="s">
-        <v>55</v>
+      <c r="A26" s="59"/>
+      <c r="B26" s="61" t="s">
+        <v>24</v>
       </c>
       <c r="C26" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="D26" s="93">
+      <c r="D26" s="54">
         <v>47.706000000000003</v>
       </c>
-      <c r="E26" s="93">
+      <c r="E26" s="54">
         <v>101.812</v>
       </c>
-      <c r="F26" s="93">
+      <c r="F26" s="54">
         <v>0.93859999999999999</v>
       </c>
-      <c r="G26" s="93">
+      <c r="G26" s="54">
         <v>0.9385</v>
       </c>
-      <c r="H26" s="94">
+      <c r="H26" s="55">
         <v>29.3</v>
       </c>
       <c r="I26" s="9">
@@ -2533,18 +2497,18 @@
       <c r="Q26" s="36">
         <v>1E-3</v>
       </c>
-      <c r="R26" s="73" t="s">
+      <c r="R26" s="83" t="s">
         <v>57</v>
       </c>
-      <c r="S26" s="65"/>
-      <c r="T26" s="65"/>
-      <c r="U26" s="65"/>
-      <c r="V26" s="65"/>
-      <c r="W26" s="66"/>
+      <c r="S26" s="75"/>
+      <c r="T26" s="75"/>
+      <c r="U26" s="75"/>
+      <c r="V26" s="75"/>
+      <c r="W26" s="76"/>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A27" s="117"/>
-      <c r="B27" s="53"/>
+      <c r="A27" s="59"/>
+      <c r="B27" s="62"/>
       <c r="C27" s="30" t="s">
         <v>12</v>
       </c>
@@ -2590,16 +2554,16 @@
       <c r="Q27" s="37">
         <v>1E-3</v>
       </c>
-      <c r="R27" s="67"/>
-      <c r="S27" s="68"/>
-      <c r="T27" s="68"/>
-      <c r="U27" s="68"/>
-      <c r="V27" s="68"/>
-      <c r="W27" s="69"/>
+      <c r="R27" s="77"/>
+      <c r="S27" s="78"/>
+      <c r="T27" s="78"/>
+      <c r="U27" s="78"/>
+      <c r="V27" s="78"/>
+      <c r="W27" s="79"/>
     </row>
     <row r="28" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="117"/>
-      <c r="B28" s="54"/>
+      <c r="A28" s="59"/>
+      <c r="B28" s="63"/>
       <c r="C28" s="31" t="s">
         <v>14</v>
       </c>
@@ -2645,34 +2609,34 @@
       <c r="Q28" s="38">
         <v>1E-3</v>
       </c>
-      <c r="R28" s="70"/>
-      <c r="S28" s="71"/>
-      <c r="T28" s="71"/>
-      <c r="U28" s="71"/>
-      <c r="V28" s="71"/>
-      <c r="W28" s="72"/>
+      <c r="R28" s="80"/>
+      <c r="S28" s="81"/>
+      <c r="T28" s="81"/>
+      <c r="U28" s="81"/>
+      <c r="V28" s="81"/>
+      <c r="W28" s="82"/>
     </row>
     <row r="29" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="118"/>
-      <c r="B29" s="52" t="s">
-        <v>58</v>
+      <c r="A29" s="60"/>
+      <c r="B29" s="61" t="s">
+        <v>34</v>
       </c>
       <c r="C29" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="D29" s="93">
+      <c r="D29" s="54">
         <v>49.481000000000002</v>
       </c>
-      <c r="E29" s="93">
+      <c r="E29" s="54">
         <v>104.151</v>
       </c>
-      <c r="F29" s="93">
+      <c r="F29" s="54">
         <v>0.93569999999999998</v>
       </c>
-      <c r="G29" s="93">
+      <c r="G29" s="54">
         <v>0.93569999999999998</v>
       </c>
-      <c r="H29" s="94">
+      <c r="H29" s="55">
         <v>23.1</v>
       </c>
       <c r="I29" s="9">
@@ -2702,18 +2666,18 @@
       <c r="Q29" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R29" s="64" t="s">
+      <c r="R29" s="74" t="s">
         <v>60</v>
       </c>
-      <c r="S29" s="65"/>
-      <c r="T29" s="65"/>
-      <c r="U29" s="65"/>
-      <c r="V29" s="65"/>
-      <c r="W29" s="66"/>
+      <c r="S29" s="75"/>
+      <c r="T29" s="75"/>
+      <c r="U29" s="75"/>
+      <c r="V29" s="75"/>
+      <c r="W29" s="76"/>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A30" s="117"/>
-      <c r="B30" s="53"/>
+      <c r="A30" s="59"/>
+      <c r="B30" s="62"/>
       <c r="C30" s="26" t="s">
         <v>12</v>
       </c>
@@ -2759,16 +2723,16 @@
       <c r="Q30" s="8">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R30" s="67"/>
-      <c r="S30" s="68"/>
-      <c r="T30" s="68"/>
-      <c r="U30" s="68"/>
-      <c r="V30" s="68"/>
-      <c r="W30" s="69"/>
+      <c r="R30" s="77"/>
+      <c r="S30" s="78"/>
+      <c r="T30" s="78"/>
+      <c r="U30" s="78"/>
+      <c r="V30" s="78"/>
+      <c r="W30" s="79"/>
     </row>
     <row r="31" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="117"/>
-      <c r="B31" s="54"/>
+      <c r="A31" s="59"/>
+      <c r="B31" s="63"/>
       <c r="C31" s="43" t="s">
         <v>14</v>
       </c>
@@ -2814,34 +2778,34 @@
       <c r="Q31" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R31" s="70"/>
-      <c r="S31" s="71"/>
-      <c r="T31" s="71"/>
-      <c r="U31" s="71"/>
-      <c r="V31" s="71"/>
-      <c r="W31" s="72"/>
+      <c r="R31" s="80"/>
+      <c r="S31" s="81"/>
+      <c r="T31" s="81"/>
+      <c r="U31" s="81"/>
+      <c r="V31" s="81"/>
+      <c r="W31" s="82"/>
     </row>
     <row r="32" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="118"/>
-      <c r="B32" s="52" t="s">
-        <v>61</v>
+      <c r="A32" s="60"/>
+      <c r="B32" s="61" t="s">
+        <v>36</v>
       </c>
       <c r="C32" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="D32" s="93">
+      <c r="D32" s="54">
         <v>46.76</v>
       </c>
-      <c r="E32" s="93">
+      <c r="E32" s="54">
         <v>95.427999999999997</v>
       </c>
-      <c r="F32" s="93">
+      <c r="F32" s="54">
         <v>0.94679999999999997</v>
       </c>
-      <c r="G32" s="93">
+      <c r="G32" s="54">
         <v>0.94669999999999999</v>
       </c>
-      <c r="H32" s="94">
+      <c r="H32" s="55">
         <v>23.1</v>
       </c>
       <c r="I32" s="45">
@@ -2871,18 +2835,18 @@
       <c r="Q32" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R32" s="73" t="s">
-        <v>62</v>
-      </c>
-      <c r="S32" s="65"/>
-      <c r="T32" s="65"/>
-      <c r="U32" s="65"/>
-      <c r="V32" s="65"/>
-      <c r="W32" s="66"/>
+      <c r="R32" s="83" t="s">
+        <v>61</v>
+      </c>
+      <c r="S32" s="75"/>
+      <c r="T32" s="75"/>
+      <c r="U32" s="75"/>
+      <c r="V32" s="75"/>
+      <c r="W32" s="76"/>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A33" s="118"/>
-      <c r="B33" s="53"/>
+      <c r="A33" s="60"/>
+      <c r="B33" s="62"/>
       <c r="C33" s="26" t="s">
         <v>12</v>
       </c>
@@ -2928,16 +2892,16 @@
       <c r="Q33" s="8">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R33" s="67"/>
-      <c r="S33" s="68"/>
-      <c r="T33" s="68"/>
-      <c r="U33" s="68"/>
-      <c r="V33" s="68"/>
-      <c r="W33" s="69"/>
+      <c r="R33" s="77"/>
+      <c r="S33" s="78"/>
+      <c r="T33" s="78"/>
+      <c r="U33" s="78"/>
+      <c r="V33" s="78"/>
+      <c r="W33" s="79"/>
     </row>
     <row r="34" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="118"/>
-      <c r="B34" s="54"/>
+      <c r="A34" s="60"/>
+      <c r="B34" s="63"/>
       <c r="C34" s="43" t="s">
         <v>14</v>
       </c>
@@ -2983,34 +2947,34 @@
       <c r="Q34" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R34" s="70"/>
-      <c r="S34" s="71"/>
-      <c r="T34" s="71"/>
-      <c r="U34" s="71"/>
-      <c r="V34" s="71"/>
-      <c r="W34" s="72"/>
+      <c r="R34" s="80"/>
+      <c r="S34" s="81"/>
+      <c r="T34" s="81"/>
+      <c r="U34" s="81"/>
+      <c r="V34" s="81"/>
+      <c r="W34" s="82"/>
     </row>
     <row r="35" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="117"/>
-      <c r="B35" s="52" t="s">
-        <v>63</v>
+      <c r="A35" s="59"/>
+      <c r="B35" s="61" t="s">
+        <v>44</v>
       </c>
       <c r="C35" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="D35" s="95">
+      <c r="D35" s="56">
         <v>48.41</v>
       </c>
-      <c r="E35" s="93">
+      <c r="E35" s="54">
         <v>101.381</v>
       </c>
-      <c r="F35" s="93">
+      <c r="F35" s="54">
         <v>0.93989999999999996</v>
       </c>
-      <c r="G35" s="93">
+      <c r="G35" s="54">
         <v>0.93979999999999997</v>
       </c>
-      <c r="H35" s="94">
+      <c r="H35" s="55">
         <v>22.9</v>
       </c>
       <c r="I35" s="46">
@@ -3023,7 +2987,7 @@
         <v>6</v>
       </c>
       <c r="L35" s="32" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="M35">
         <v>64</v>
@@ -3040,18 +3004,18 @@
       <c r="Q35" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R35" s="64" t="s">
-        <v>65</v>
-      </c>
-      <c r="S35" s="65"/>
-      <c r="T35" s="65"/>
-      <c r="U35" s="65"/>
-      <c r="V35" s="65"/>
-      <c r="W35" s="66"/>
+      <c r="R35" s="74" t="s">
+        <v>63</v>
+      </c>
+      <c r="S35" s="75"/>
+      <c r="T35" s="75"/>
+      <c r="U35" s="75"/>
+      <c r="V35" s="75"/>
+      <c r="W35" s="76"/>
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A36" s="117"/>
-      <c r="B36" s="53"/>
+      <c r="A36" s="59"/>
+      <c r="B36" s="62"/>
       <c r="C36" s="26" t="s">
         <v>12</v>
       </c>
@@ -3097,16 +3061,16 @@
       <c r="Q36" s="37">
         <v>1E-3</v>
       </c>
-      <c r="R36" s="67"/>
-      <c r="S36" s="68"/>
-      <c r="T36" s="68"/>
-      <c r="U36" s="68"/>
-      <c r="V36" s="68"/>
-      <c r="W36" s="69"/>
+      <c r="R36" s="77"/>
+      <c r="S36" s="78"/>
+      <c r="T36" s="78"/>
+      <c r="U36" s="78"/>
+      <c r="V36" s="78"/>
+      <c r="W36" s="79"/>
     </row>
     <row r="37" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="117"/>
-      <c r="B37" s="54"/>
+      <c r="A37" s="59"/>
+      <c r="B37" s="63"/>
       <c r="C37" s="31" t="s">
         <v>14</v>
       </c>
@@ -3152,34 +3116,34 @@
       <c r="Q37" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R37" s="70"/>
-      <c r="S37" s="71"/>
-      <c r="T37" s="71"/>
-      <c r="U37" s="71"/>
-      <c r="V37" s="71"/>
-      <c r="W37" s="72"/>
+      <c r="R37" s="80"/>
+      <c r="S37" s="81"/>
+      <c r="T37" s="81"/>
+      <c r="U37" s="81"/>
+      <c r="V37" s="81"/>
+      <c r="W37" s="82"/>
     </row>
     <row r="38" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="118"/>
-      <c r="B38" s="52" t="s">
-        <v>66</v>
+      <c r="A38" s="60"/>
+      <c r="B38" s="61" t="s">
+        <v>46</v>
       </c>
       <c r="C38" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="D38" s="95">
+      <c r="D38" s="56">
         <v>42.213999999999999</v>
       </c>
-      <c r="E38" s="93">
+      <c r="E38" s="54">
         <v>92.585999999999999</v>
       </c>
-      <c r="F38" s="93">
+      <c r="F38" s="54">
         <v>0.94740000000000002</v>
       </c>
-      <c r="G38" s="93">
+      <c r="G38" s="54">
         <v>0.94730000000000003</v>
       </c>
-      <c r="H38" s="94">
+      <c r="H38" s="55">
         <v>22.9</v>
       </c>
       <c r="I38" s="51">
@@ -3192,7 +3156,7 @@
         <v>6</v>
       </c>
       <c r="L38" s="40" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="M38" s="9">
         <v>64</v>
@@ -3209,16 +3173,16 @@
       <c r="Q38" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R38" s="55"/>
-      <c r="S38" s="56"/>
-      <c r="T38" s="56"/>
-      <c r="U38" s="56"/>
-      <c r="V38" s="56"/>
-      <c r="W38" s="57"/>
+      <c r="R38" s="64"/>
+      <c r="S38" s="65"/>
+      <c r="T38" s="65"/>
+      <c r="U38" s="65"/>
+      <c r="V38" s="65"/>
+      <c r="W38" s="66"/>
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A39" s="118"/>
-      <c r="B39" s="53"/>
+      <c r="A39" s="60"/>
+      <c r="B39" s="62"/>
       <c r="C39" s="30" t="s">
         <v>12</v>
       </c>
@@ -3247,7 +3211,7 @@
         <v>6</v>
       </c>
       <c r="L39" s="32" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="M39">
         <v>64</v>
@@ -3264,16 +3228,16 @@
       <c r="Q39" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R39" s="58"/>
-      <c r="S39" s="59"/>
-      <c r="T39" s="59"/>
-      <c r="U39" s="59"/>
-      <c r="V39" s="59"/>
-      <c r="W39" s="60"/>
+      <c r="R39" s="67"/>
+      <c r="S39" s="68"/>
+      <c r="T39" s="68"/>
+      <c r="U39" s="68"/>
+      <c r="V39" s="68"/>
+      <c r="W39" s="69"/>
     </row>
     <row r="40" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="118"/>
-      <c r="B40" s="54"/>
+      <c r="A40" s="60"/>
+      <c r="B40" s="63"/>
       <c r="C40" s="31" t="s">
         <v>14</v>
       </c>
@@ -3302,7 +3266,7 @@
         <v>6</v>
       </c>
       <c r="L40" s="35" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="M40" s="3">
         <v>64</v>
@@ -3319,201 +3283,201 @@
       <c r="Q40" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R40" s="61"/>
-      <c r="S40" s="62"/>
-      <c r="T40" s="62"/>
-      <c r="U40" s="62"/>
-      <c r="V40" s="62"/>
-      <c r="W40" s="63"/>
+      <c r="R40" s="70"/>
+      <c r="S40" s="71"/>
+      <c r="T40" s="71"/>
+      <c r="U40" s="71"/>
+      <c r="V40" s="71"/>
+      <c r="W40" s="72"/>
     </row>
     <row r="41" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="118"/>
-      <c r="B41" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="C41" s="96" t="s">
+      <c r="A41" s="60"/>
+      <c r="B41" s="61" t="s">
+        <v>50</v>
+      </c>
+      <c r="C41" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="D41" s="102">
+      <c r="D41" s="57">
         <v>48614</v>
       </c>
-      <c r="E41" s="103">
+      <c r="E41" s="9">
         <v>99.918999999999997</v>
       </c>
-      <c r="F41" s="103">
+      <c r="F41" s="9">
         <v>0.94159999999999999</v>
       </c>
-      <c r="G41" s="103">
+      <c r="G41" s="9">
         <v>0.94159999999999999</v>
       </c>
-      <c r="H41" s="104">
+      <c r="H41" s="10">
         <v>22.9</v>
       </c>
       <c r="I41" s="51">
         <v>21</v>
       </c>
-      <c r="J41" s="103">
+      <c r="J41" s="9">
         <v>232.8</v>
       </c>
-      <c r="K41" s="103">
-        <v>6</v>
-      </c>
-      <c r="L41" s="105" t="s">
-        <v>73</v>
-      </c>
-      <c r="M41" s="103">
-        <v>64</v>
-      </c>
-      <c r="N41" s="103">
-        <v>64</v>
-      </c>
-      <c r="O41" s="105" t="s">
+      <c r="K41" s="9">
+        <v>6</v>
+      </c>
+      <c r="L41" s="40" t="s">
+        <v>70</v>
+      </c>
+      <c r="M41" s="9">
+        <v>64</v>
+      </c>
+      <c r="N41" s="9">
+        <v>64</v>
+      </c>
+      <c r="O41" s="40" t="s">
         <v>39</v>
       </c>
-      <c r="P41" s="103">
+      <c r="P41" s="9">
         <v>0.2</v>
       </c>
-      <c r="Q41" s="104">
+      <c r="Q41" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R41" s="55" t="s">
-        <v>76</v>
-      </c>
-      <c r="S41" s="56"/>
-      <c r="T41" s="56"/>
-      <c r="U41" s="56"/>
-      <c r="V41" s="56"/>
-      <c r="W41" s="57"/>
+      <c r="R41" s="64" t="s">
+        <v>71</v>
+      </c>
+      <c r="S41" s="65"/>
+      <c r="T41" s="65"/>
+      <c r="U41" s="65"/>
+      <c r="V41" s="65"/>
+      <c r="W41" s="66"/>
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A42" s="118"/>
-      <c r="B42" s="53"/>
-      <c r="C42" s="96" t="s">
+      <c r="A42" s="60"/>
+      <c r="B42" s="62"/>
+      <c r="C42" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="D42" s="113">
+      <c r="D42" s="58">
         <v>45.213999999999999</v>
       </c>
-      <c r="E42" s="114">
+      <c r="E42" s="52">
         <v>93.855999999999995</v>
       </c>
-      <c r="F42" s="114">
+      <c r="F42" s="52">
         <v>0.94850000000000001</v>
       </c>
-      <c r="G42" s="114">
+      <c r="G42" s="52">
         <v>0.94850000000000001</v>
       </c>
-      <c r="H42" s="92">
+      <c r="H42" s="53">
         <v>23.6</v>
       </c>
       <c r="I42" s="50">
         <v>21</v>
       </c>
-      <c r="J42" s="106">
+      <c r="J42">
         <v>562.19000000000005</v>
       </c>
-      <c r="K42" s="97">
-        <v>6</v>
-      </c>
-      <c r="L42" s="98" t="s">
-        <v>72</v>
-      </c>
-      <c r="M42" s="97">
-        <v>64</v>
-      </c>
-      <c r="N42" s="97">
+      <c r="K42">
+        <v>6</v>
+      </c>
+      <c r="L42" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="M42">
+        <v>64</v>
+      </c>
+      <c r="N42">
         <v>32</v>
       </c>
-      <c r="O42" s="98" t="s">
+      <c r="O42" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P42" s="97">
+      <c r="P42">
         <v>0.1</v>
       </c>
-      <c r="Q42" s="99">
+      <c r="Q42" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R42" s="58"/>
-      <c r="S42" s="107"/>
-      <c r="T42" s="107"/>
-      <c r="U42" s="107"/>
-      <c r="V42" s="107"/>
-      <c r="W42" s="60"/>
+      <c r="R42" s="67"/>
+      <c r="S42" s="68"/>
+      <c r="T42" s="68"/>
+      <c r="U42" s="68"/>
+      <c r="V42" s="68"/>
+      <c r="W42" s="69"/>
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A43" s="118"/>
-      <c r="B43" s="53"/>
-      <c r="C43" s="96" t="s">
+      <c r="A43" s="60"/>
+      <c r="B43" s="62"/>
+      <c r="C43" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="D43" s="100">
+      <c r="D43" s="1">
         <v>73.799000000000007</v>
       </c>
-      <c r="E43" s="97">
+      <c r="E43">
         <v>132.626</v>
       </c>
-      <c r="F43" s="97">
+      <c r="F43">
         <v>0.8972</v>
       </c>
-      <c r="G43" s="97">
+      <c r="G43">
         <v>0.89710000000000001</v>
       </c>
-      <c r="H43" s="99">
+      <c r="H43" s="8">
         <v>27</v>
       </c>
       <c r="I43" s="50">
         <v>21</v>
       </c>
-      <c r="J43" s="106">
+      <c r="J43">
         <v>690.97</v>
       </c>
-      <c r="K43" s="97">
-        <v>6</v>
-      </c>
-      <c r="L43" s="98" t="s">
+      <c r="K43">
+        <v>6</v>
+      </c>
+      <c r="L43" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="M43" s="97">
-        <v>64</v>
-      </c>
-      <c r="N43" s="108" t="s">
+      <c r="M43">
+        <v>64</v>
+      </c>
+      <c r="N43" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="O43" s="98" t="s">
+      <c r="O43" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P43" s="97">
+      <c r="P43">
         <v>0.1</v>
       </c>
-      <c r="Q43" s="99">
+      <c r="Q43" s="8">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R43" s="58"/>
-      <c r="S43" s="107"/>
-      <c r="T43" s="107"/>
-      <c r="U43" s="107"/>
-      <c r="V43" s="107"/>
-      <c r="W43" s="60"/>
+      <c r="R43" s="67"/>
+      <c r="S43" s="68"/>
+      <c r="T43" s="68"/>
+      <c r="U43" s="68"/>
+      <c r="V43" s="68"/>
+      <c r="W43" s="69"/>
     </row>
     <row r="44" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="118"/>
-      <c r="B44" s="54"/>
-      <c r="C44" s="101" t="s">
-        <v>70</v>
-      </c>
-      <c r="D44" s="109">
+      <c r="A44" s="60"/>
+      <c r="B44" s="63"/>
+      <c r="C44" s="31" t="s">
+        <v>67</v>
+      </c>
+      <c r="D44" s="2">
         <v>71.367000000000004</v>
       </c>
-      <c r="E44" s="110">
+      <c r="E44" s="3">
         <v>142.86600000000001</v>
       </c>
-      <c r="F44" s="110">
+      <c r="F44" s="3">
         <v>0.88070000000000004</v>
       </c>
-      <c r="G44" s="110">
+      <c r="G44" s="3">
         <v>0.88060000000000005</v>
       </c>
-      <c r="H44" s="111">
+      <c r="H44" s="4">
         <v>22</v>
       </c>
       <c r="I44" s="48">
@@ -3522,208 +3486,208 @@
       <c r="J44" s="3">
         <v>168.8</v>
       </c>
-      <c r="K44" s="110">
+      <c r="K44" s="3">
         <v>6</v>
       </c>
       <c r="L44" s="35" t="s">
         <v>49</v>
       </c>
-      <c r="M44" s="110">
-        <v>64</v>
-      </c>
-      <c r="N44" s="110">
+      <c r="M44" s="3">
+        <v>64</v>
+      </c>
+      <c r="N44" s="3">
         <v>32</v>
       </c>
-      <c r="O44" s="112" t="s">
+      <c r="O44" s="35" t="s">
         <v>39</v>
       </c>
       <c r="P44" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q44" s="111">
+        <v>68</v>
+      </c>
+      <c r="Q44" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R44" s="61"/>
-      <c r="S44" s="62"/>
-      <c r="T44" s="62"/>
-      <c r="U44" s="62"/>
-      <c r="V44" s="62"/>
-      <c r="W44" s="63"/>
+      <c r="R44" s="70"/>
+      <c r="S44" s="71"/>
+      <c r="T44" s="71"/>
+      <c r="U44" s="71"/>
+      <c r="V44" s="71"/>
+      <c r="W44" s="72"/>
     </row>
     <row r="45" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="118"/>
-      <c r="B45" s="52" t="s">
-        <v>75</v>
-      </c>
-      <c r="C45" s="96" t="s">
+      <c r="A45" s="60"/>
+      <c r="B45" s="61" t="s">
+        <v>55</v>
+      </c>
+      <c r="C45" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="D45" s="113">
+      <c r="D45" s="58">
         <v>47.497999999999998</v>
       </c>
-      <c r="E45" s="114">
+      <c r="E45" s="52">
         <v>98.091999999999999</v>
       </c>
-      <c r="F45" s="114">
+      <c r="F45" s="52">
         <v>0.94379999999999997</v>
       </c>
-      <c r="G45" s="114">
+      <c r="G45" s="52">
         <v>0.94369999999999998</v>
       </c>
-      <c r="H45" s="92">
+      <c r="H45" s="53">
         <v>22.9</v>
       </c>
       <c r="I45" s="50">
         <v>30</v>
       </c>
-      <c r="J45" s="97">
+      <c r="J45">
         <v>367.69</v>
       </c>
-      <c r="K45" s="103">
-        <v>6</v>
-      </c>
-      <c r="L45" s="98" t="s">
-        <v>78</v>
-      </c>
-      <c r="M45" s="103">
-        <v>64</v>
-      </c>
-      <c r="N45" s="116">
-        <v>64</v>
-      </c>
-      <c r="O45" s="98" t="s">
+      <c r="K45" s="9">
+        <v>6</v>
+      </c>
+      <c r="L45" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="M45" s="9">
+        <v>64</v>
+      </c>
+      <c r="N45" s="25">
+        <v>64</v>
+      </c>
+      <c r="O45" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P45" s="116">
+      <c r="P45" s="25">
         <v>0.1</v>
       </c>
-      <c r="Q45" s="104">
+      <c r="Q45" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R45" s="115" t="s">
-        <v>77</v>
-      </c>
-      <c r="S45" s="56"/>
-      <c r="T45" s="56"/>
-      <c r="U45" s="56"/>
-      <c r="V45" s="56"/>
-      <c r="W45" s="57"/>
+      <c r="R45" s="73" t="s">
+        <v>72</v>
+      </c>
+      <c r="S45" s="65"/>
+      <c r="T45" s="65"/>
+      <c r="U45" s="65"/>
+      <c r="V45" s="65"/>
+      <c r="W45" s="66"/>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A46" s="118"/>
-      <c r="B46" s="53"/>
-      <c r="C46" s="96" t="s">
+      <c r="A46" s="60"/>
+      <c r="B46" s="62"/>
+      <c r="C46" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="D46" s="113">
+      <c r="D46" s="58">
         <v>47.232999999999997</v>
       </c>
-      <c r="E46" s="114">
+      <c r="E46" s="52">
         <v>96.742000000000004</v>
       </c>
-      <c r="F46" s="114">
+      <c r="F46" s="52">
         <v>0.94530000000000003</v>
       </c>
-      <c r="G46" s="114">
+      <c r="G46" s="52">
         <v>0.94530000000000003</v>
       </c>
-      <c r="H46" s="92">
+      <c r="H46" s="53">
         <v>79.099999999999994</v>
       </c>
       <c r="I46" s="50">
         <v>30</v>
       </c>
-      <c r="J46" s="97">
+      <c r="J46">
         <v>671.14</v>
       </c>
-      <c r="K46" s="97">
-        <v>6</v>
-      </c>
-      <c r="L46" s="98" t="s">
-        <v>79</v>
-      </c>
-      <c r="M46" s="97">
-        <v>64</v>
-      </c>
-      <c r="N46" s="116">
+      <c r="K46">
+        <v>6</v>
+      </c>
+      <c r="L46" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="M46">
+        <v>64</v>
+      </c>
+      <c r="N46" s="25">
         <v>64</v>
       </c>
       <c r="O46" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P46" s="116">
+      <c r="P46" s="25">
         <v>0.1</v>
       </c>
-      <c r="Q46" s="99">
+      <c r="Q46" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R46" s="58"/>
-      <c r="S46" s="107"/>
-      <c r="T46" s="107"/>
-      <c r="U46" s="107"/>
-      <c r="V46" s="107"/>
-      <c r="W46" s="60"/>
+      <c r="R46" s="67"/>
+      <c r="S46" s="68"/>
+      <c r="T46" s="68"/>
+      <c r="U46" s="68"/>
+      <c r="V46" s="68"/>
+      <c r="W46" s="69"/>
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A47" s="118"/>
-      <c r="B47" s="53"/>
-      <c r="C47" s="96" t="s">
+      <c r="A47" s="60"/>
+      <c r="B47" s="62"/>
+      <c r="C47" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="D47" s="100">
+      <c r="D47" s="1">
         <v>65.77</v>
       </c>
-      <c r="E47" s="97">
+      <c r="E47">
         <v>126.881</v>
       </c>
-      <c r="F47" s="97">
+      <c r="F47">
         <v>0.90590000000000004</v>
       </c>
-      <c r="G47" s="97">
+      <c r="G47">
         <v>0.90580000000000005</v>
       </c>
-      <c r="H47" s="99">
+      <c r="H47" s="8">
         <v>61.1</v>
       </c>
       <c r="I47" s="50">
         <v>30</v>
       </c>
-      <c r="J47" s="97">
+      <c r="J47">
         <v>698.6</v>
       </c>
-      <c r="K47" s="97">
-        <v>6</v>
-      </c>
-      <c r="L47" s="98" t="s">
+      <c r="K47">
+        <v>6</v>
+      </c>
+      <c r="L47" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="M47" s="97">
-        <v>64</v>
-      </c>
-      <c r="N47" s="116">
-        <v>64</v>
-      </c>
-      <c r="O47" s="98" t="s">
+      <c r="M47">
+        <v>64</v>
+      </c>
+      <c r="N47" s="25">
+        <v>64</v>
+      </c>
+      <c r="O47" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P47" s="116">
+      <c r="P47" s="25">
         <v>0.1</v>
       </c>
-      <c r="Q47" s="99">
+      <c r="Q47" s="8">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R47" s="58"/>
-      <c r="S47" s="107"/>
-      <c r="T47" s="107"/>
-      <c r="U47" s="107"/>
-      <c r="V47" s="107"/>
-      <c r="W47" s="60"/>
+      <c r="R47" s="67"/>
+      <c r="S47" s="68"/>
+      <c r="T47" s="68"/>
+      <c r="U47" s="68"/>
+      <c r="V47" s="68"/>
+      <c r="W47" s="69"/>
     </row>
     <row r="48" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="118"/>
-      <c r="B48" s="54"/>
-      <c r="C48" s="101" t="s">
-        <v>70</v>
+      <c r="A48" s="60"/>
+      <c r="B48" s="63"/>
+      <c r="C48" s="31" t="s">
+        <v>67</v>
       </c>
       <c r="D48" s="2">
         <v>62.356000000000002</v>
@@ -3746,189 +3710,274 @@
       <c r="J48" s="3">
         <v>145.22999999999999</v>
       </c>
-      <c r="K48" s="110">
-        <v>6</v>
-      </c>
-      <c r="L48" s="98" t="s">
+      <c r="K48" s="3">
+        <v>6</v>
+      </c>
+      <c r="L48" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="M48" s="110">
+      <c r="M48" s="3">
         <v>64</v>
       </c>
       <c r="N48" s="28">
         <v>64</v>
       </c>
-      <c r="O48" s="112" t="s">
+      <c r="O48" s="35" t="s">
         <v>39</v>
       </c>
       <c r="P48" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q48" s="111">
+        <v>68</v>
+      </c>
+      <c r="Q48" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R48" s="61"/>
-      <c r="S48" s="62"/>
-      <c r="T48" s="62"/>
-      <c r="U48" s="62"/>
-      <c r="V48" s="62"/>
-      <c r="W48" s="63"/>
+      <c r="R48" s="70"/>
+      <c r="S48" s="71"/>
+      <c r="T48" s="71"/>
+      <c r="U48" s="71"/>
+      <c r="V48" s="71"/>
+      <c r="W48" s="72"/>
     </row>
     <row r="49" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="117"/>
-      <c r="B49" s="52" t="s">
-        <v>80</v>
-      </c>
-      <c r="C49" s="96" t="s">
+      <c r="A49" s="59"/>
+      <c r="B49" s="61" t="s">
+        <v>58</v>
+      </c>
+      <c r="C49" s="30" t="s">
         <v>13</v>
+      </c>
+      <c r="D49" s="58">
+        <v>45.665999999999997</v>
+      </c>
+      <c r="E49" s="104">
+        <v>100.13</v>
+      </c>
+      <c r="F49" s="104">
+        <v>0.94140000000000001</v>
+      </c>
+      <c r="G49" s="104">
+        <v>0.94130000000000003</v>
+      </c>
+      <c r="H49" s="53">
+        <v>22.9</v>
       </c>
       <c r="I49" s="50">
         <v>18</v>
       </c>
-      <c r="K49" s="103">
-        <v>6</v>
-      </c>
-      <c r="L49" s="9"/>
-      <c r="M49" s="103">
-        <v>64</v>
-      </c>
-      <c r="N49" s="97">
-        <v>64</v>
-      </c>
-      <c r="O49" s="98" t="s">
+      <c r="J49" s="101">
+        <v>245.39</v>
+      </c>
+      <c r="K49" s="9">
+        <v>6</v>
+      </c>
+      <c r="L49" s="40" t="s">
+        <v>75</v>
+      </c>
+      <c r="M49" s="9">
+        <v>64</v>
+      </c>
+      <c r="N49">
+        <v>64</v>
+      </c>
+      <c r="O49" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P49" s="116">
+      <c r="P49" s="25">
         <v>0.1</v>
       </c>
-      <c r="Q49" s="104">
+      <c r="Q49" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R49" s="55"/>
-      <c r="S49" s="56"/>
-      <c r="T49" s="56"/>
-      <c r="U49" s="56"/>
-      <c r="V49" s="56"/>
-      <c r="W49" s="57"/>
+      <c r="R49" s="64"/>
+      <c r="S49" s="65"/>
+      <c r="T49" s="65"/>
+      <c r="U49" s="65"/>
+      <c r="V49" s="65"/>
+      <c r="W49" s="66"/>
     </row>
     <row r="50" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A50" s="117"/>
-      <c r="B50" s="53"/>
-      <c r="C50" s="96" t="s">
+      <c r="A50" s="59"/>
+      <c r="B50" s="62"/>
+      <c r="C50" s="30" t="s">
         <v>12</v>
+      </c>
+      <c r="D50" s="58">
+        <v>47.45</v>
+      </c>
+      <c r="E50" s="104">
+        <v>97.483999999999995</v>
+      </c>
+      <c r="F50" s="104">
+        <v>0.94440000000000002</v>
+      </c>
+      <c r="G50" s="104">
+        <v>0.94440000000000002</v>
+      </c>
+      <c r="H50" s="53">
+        <v>79.099999999999994</v>
       </c>
       <c r="I50" s="50">
         <v>18</v>
       </c>
-      <c r="K50" s="97">
-        <v>6</v>
-      </c>
-      <c r="M50" s="97">
-        <v>64</v>
-      </c>
-      <c r="N50" s="97">
+      <c r="J50" s="101">
+        <v>819.18</v>
+      </c>
+      <c r="K50">
+        <v>6</v>
+      </c>
+      <c r="L50" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="M50">
+        <v>64</v>
+      </c>
+      <c r="N50">
         <v>64</v>
       </c>
       <c r="O50" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P50" s="116">
+      <c r="P50" s="25">
         <v>0.1</v>
       </c>
-      <c r="Q50" s="99">
+      <c r="Q50" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R50" s="58"/>
-      <c r="S50" s="107"/>
-      <c r="T50" s="107"/>
-      <c r="U50" s="107"/>
-      <c r="V50" s="107"/>
-      <c r="W50" s="60"/>
+      <c r="R50" s="67"/>
+      <c r="S50" s="68"/>
+      <c r="T50" s="68"/>
+      <c r="U50" s="68"/>
+      <c r="V50" s="68"/>
+      <c r="W50" s="69"/>
     </row>
     <row r="51" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A51" s="117"/>
-      <c r="B51" s="53"/>
-      <c r="C51" s="96" t="s">
+      <c r="A51" s="59"/>
+      <c r="B51" s="62"/>
+      <c r="C51" s="30" t="s">
         <v>14</v>
+      </c>
+      <c r="D51" s="102">
+        <v>74.283000000000001</v>
+      </c>
+      <c r="E51" s="101">
+        <v>130.41999999999999</v>
+      </c>
+      <c r="F51" s="101">
+        <v>0.90059999999999996</v>
+      </c>
+      <c r="G51" s="101">
+        <v>0.90049999999999997</v>
+      </c>
+      <c r="H51" s="103">
+        <v>61.1</v>
       </c>
       <c r="I51" s="50">
         <v>18</v>
       </c>
-      <c r="K51" s="97">
-        <v>6</v>
-      </c>
-      <c r="M51" s="97">
-        <v>64</v>
-      </c>
-      <c r="N51" s="97">
-        <v>64</v>
-      </c>
-      <c r="O51" s="98" t="s">
+      <c r="J51" s="101">
+        <v>450.04</v>
+      </c>
+      <c r="K51">
+        <v>6</v>
+      </c>
+      <c r="L51" s="32" t="s">
+        <v>49</v>
+      </c>
+      <c r="M51">
+        <v>64</v>
+      </c>
+      <c r="N51">
+        <v>64</v>
+      </c>
+      <c r="O51" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P51" s="116">
+      <c r="P51" s="25">
         <v>0.1</v>
       </c>
-      <c r="Q51" s="99">
+      <c r="Q51" s="8">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R51" s="58"/>
-      <c r="S51" s="107"/>
-      <c r="T51" s="107"/>
-      <c r="U51" s="107"/>
-      <c r="V51" s="107"/>
-      <c r="W51" s="60"/>
+      <c r="R51" s="67"/>
+      <c r="S51" s="68"/>
+      <c r="T51" s="68"/>
+      <c r="U51" s="68"/>
+      <c r="V51" s="68"/>
+      <c r="W51" s="69"/>
     </row>
     <row r="52" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="117"/>
-      <c r="B52" s="54"/>
-      <c r="C52" s="101" t="s">
-        <v>70</v>
-      </c>
-      <c r="D52" s="3"/>
-      <c r="E52" s="3"/>
-      <c r="F52" s="3"/>
-      <c r="G52" s="3"/>
-      <c r="H52" s="4"/>
+      <c r="A52" s="59"/>
+      <c r="B52" s="63"/>
+      <c r="C52" s="31" t="s">
+        <v>67</v>
+      </c>
+      <c r="D52" s="3">
+        <v>74.88</v>
+      </c>
+      <c r="E52" s="3">
+        <v>141.005</v>
+      </c>
+      <c r="F52" s="3">
+        <v>0.88380000000000003</v>
+      </c>
+      <c r="G52" s="3">
+        <v>0.88360000000000005</v>
+      </c>
+      <c r="H52" s="4">
+        <v>39.9</v>
+      </c>
       <c r="I52" s="48">
         <v>18</v>
       </c>
-      <c r="J52" s="3"/>
-      <c r="K52" s="110">
-        <v>6</v>
-      </c>
-      <c r="L52" s="3"/>
-      <c r="M52" s="110">
-        <v>64</v>
-      </c>
-      <c r="N52" s="110">
-        <v>64</v>
-      </c>
-      <c r="O52" s="112" t="s">
+      <c r="J52" s="3">
+        <v>170.66</v>
+      </c>
+      <c r="K52" s="3">
+        <v>6</v>
+      </c>
+      <c r="L52" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="M52" s="3">
+        <v>64</v>
+      </c>
+      <c r="N52" s="3">
+        <v>64</v>
+      </c>
+      <c r="O52" s="35" t="s">
         <v>39</v>
       </c>
       <c r="P52" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q52" s="111">
+        <v>68</v>
+      </c>
+      <c r="Q52" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R52" s="61"/>
-      <c r="S52" s="62"/>
-      <c r="T52" s="62"/>
-      <c r="U52" s="62"/>
-      <c r="V52" s="62"/>
-      <c r="W52" s="63"/>
+      <c r="R52" s="70"/>
+      <c r="S52" s="71"/>
+      <c r="T52" s="71"/>
+      <c r="U52" s="71"/>
+      <c r="V52" s="71"/>
+      <c r="W52" s="72"/>
     </row>
     <row r="53" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="B41:B44"/>
-    <mergeCell ref="R41:W44"/>
-    <mergeCell ref="R45:W48"/>
-    <mergeCell ref="B45:B48"/>
-    <mergeCell ref="R49:W52"/>
-    <mergeCell ref="B49:B52"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="R38:W40"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="R35:W37"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="R29:W31"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="R32:W34"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="I3:Q3"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="R3:W4"/>
+    <mergeCell ref="R5:W7"/>
+    <mergeCell ref="R8:W10"/>
     <mergeCell ref="B23:B25"/>
     <mergeCell ref="R23:W25"/>
     <mergeCell ref="B26:B28"/>
@@ -3941,21 +3990,12 @@
     <mergeCell ref="B20:B22"/>
     <mergeCell ref="R14:W16"/>
     <mergeCell ref="B14:B16"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="I3:Q3"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="R3:W4"/>
-    <mergeCell ref="R5:W7"/>
-    <mergeCell ref="R8:W10"/>
-    <mergeCell ref="B38:B40"/>
-    <mergeCell ref="R38:W40"/>
-    <mergeCell ref="B35:B37"/>
-    <mergeCell ref="R35:W37"/>
-    <mergeCell ref="B29:B31"/>
-    <mergeCell ref="R29:W31"/>
-    <mergeCell ref="B32:B34"/>
-    <mergeCell ref="R32:W34"/>
+    <mergeCell ref="B41:B44"/>
+    <mergeCell ref="R41:W44"/>
+    <mergeCell ref="R45:W48"/>
+    <mergeCell ref="B45:B48"/>
+    <mergeCell ref="R49:W52"/>
+    <mergeCell ref="B49:B52"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>

<commit_message>
Entrenamiento del modelo MLP con el resto de modelos
</commit_message>
<xml_diff>
--- a/modelos_tfg/MetricasValidacion.xlsx
+++ b/modelos_tfg/MetricasValidacion.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\modelos_tfg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0EDF74F-87BA-4A8C-AEC1-3579DC2DD54A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BA035B1-3EDA-48E9-B8C3-AFDF67D3C157}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="87">
   <si>
     <t>ID Train</t>
   </si>
@@ -285,12 +296,31 @@
 V_gen e I_gen. Además, he vuelto a las configuraciones de
 los modelos que mejores resultados han dado en todos
 los entrenamiento, con el droput de todas al 0,1</t>
+  </si>
+  <si>
+    <t>55 (ES)</t>
+  </si>
+  <si>
+    <t>MLP</t>
+  </si>
+  <si>
+    <t>V12</t>
+  </si>
+  <si>
+    <t>Entrenamiento equilibrado, sin V_gen e I_gen, modificando
+el lr del modelo GRU. Además he añadido el modelo
+MLP haciendo que el entrenamiento sea el mismo para todos.
+Falta entrenar al modelo MLP quitando filas con irradiancia
+muy muy baja.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.000"/>
+  </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -329,7 +359,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -393,12 +423,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -641,7 +665,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -737,153 +761,141 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -892,8 +904,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFFB7EC"/>
       <color rgb="FF35D33D"/>
-      <color rgb="FFFFB7EC"/>
       <color rgb="FF1B7B20"/>
       <color rgb="FF3366FF"/>
     </mruColors>
@@ -1232,7 +1244,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:W61"/>
+  <dimension ref="A2:W66"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.42578125" customWidth="1"/>
@@ -1251,32 +1263,32 @@
   <sheetData>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D3" s="83" t="s">
+      <c r="D3" s="89" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="84"/>
-      <c r="F3" s="84"/>
-      <c r="G3" s="84"/>
-      <c r="H3" s="85"/>
-      <c r="I3" s="86" t="s">
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="91"/>
+      <c r="I3" s="92" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="87"/>
-      <c r="K3" s="87"/>
-      <c r="L3" s="87"/>
-      <c r="M3" s="87"/>
-      <c r="N3" s="87"/>
-      <c r="O3" s="87"/>
-      <c r="P3" s="87"/>
-      <c r="Q3" s="88"/>
-      <c r="R3" s="93" t="s">
+      <c r="J3" s="93"/>
+      <c r="K3" s="93"/>
+      <c r="L3" s="93"/>
+      <c r="M3" s="93"/>
+      <c r="N3" s="93"/>
+      <c r="O3" s="93"/>
+      <c r="P3" s="93"/>
+      <c r="Q3" s="94"/>
+      <c r="R3" s="97" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="94"/>
-      <c r="T3" s="94"/>
-      <c r="U3" s="94"/>
-      <c r="V3" s="94"/>
-      <c r="W3" s="95"/>
+      <c r="S3" s="98"/>
+      <c r="T3" s="98"/>
+      <c r="U3" s="98"/>
+      <c r="V3" s="98"/>
+      <c r="W3" s="99"/>
     </row>
     <row r="4" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="20" t="s">
@@ -1327,16 +1339,16 @@
       <c r="Q4" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="96"/>
-      <c r="S4" s="97"/>
-      <c r="T4" s="97"/>
-      <c r="U4" s="97"/>
-      <c r="V4" s="97"/>
-      <c r="W4" s="98"/>
+      <c r="R4" s="100"/>
+      <c r="S4" s="101"/>
+      <c r="T4" s="101"/>
+      <c r="U4" s="101"/>
+      <c r="V4" s="101"/>
+      <c r="W4" s="102"/>
     </row>
     <row r="5" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
-      <c r="B5" s="89" t="s">
+      <c r="B5" s="95" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -1384,7 +1396,7 @@
       <c r="Q5" s="17">
         <v>1E-3</v>
       </c>
-      <c r="R5" s="82" t="s">
+      <c r="R5" s="64" t="s">
         <v>38</v>
       </c>
       <c r="S5" s="65"/>
@@ -1395,7 +1407,7 @@
     </row>
     <row r="6" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
-      <c r="B6" s="90"/>
+      <c r="B6" s="74"/>
       <c r="C6" s="5" t="s">
         <v>12</v>
       </c>
@@ -1450,7 +1462,7 @@
     </row>
     <row r="7" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8"/>
-      <c r="B7" s="91"/>
+      <c r="B7" s="96"/>
       <c r="C7" s="14" t="s">
         <v>14</v>
       </c>
@@ -1505,7 +1517,7 @@
     </row>
     <row r="8" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
-      <c r="B8" s="92" t="s">
+      <c r="B8" s="73" t="s">
         <v>24</v>
       </c>
       <c r="C8" s="5" t="s">
@@ -1553,7 +1565,7 @@
       <c r="Q8" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R8" s="82" t="s">
+      <c r="R8" s="64" t="s">
         <v>38</v>
       </c>
       <c r="S8" s="65"/>
@@ -1564,7 +1576,7 @@
     </row>
     <row r="9" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
-      <c r="B9" s="90"/>
+      <c r="B9" s="74"/>
       <c r="C9" s="5" t="s">
         <v>12</v>
       </c>
@@ -1619,7 +1631,7 @@
     </row>
     <row r="10" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8"/>
-      <c r="B10" s="91"/>
+      <c r="B10" s="96"/>
       <c r="C10" s="5" t="s">
         <v>14</v>
       </c>
@@ -1673,7 +1685,7 @@
       <c r="W10" s="72"/>
     </row>
     <row r="11" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="92" t="s">
+      <c r="B11" s="73" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="29" t="s">
@@ -1721,7 +1733,7 @@
       <c r="Q11" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R11" s="82" t="s">
+      <c r="R11" s="64" t="s">
         <v>38</v>
       </c>
       <c r="S11" s="65"/>
@@ -1731,7 +1743,7 @@
       <c r="W11" s="66"/>
     </row>
     <row r="12" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="90"/>
+      <c r="B12" s="74"/>
       <c r="C12" s="26" t="s">
         <v>12</v>
       </c>
@@ -1785,7 +1797,7 @@
       <c r="W12" s="69"/>
     </row>
     <row r="13" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="90"/>
+      <c r="B13" s="74"/>
       <c r="C13" s="27" t="s">
         <v>14</v>
       </c>
@@ -1839,7 +1851,7 @@
       <c r="W13" s="72"/>
     </row>
     <row r="14" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="92" t="s">
+      <c r="B14" s="73" t="s">
         <v>36</v>
       </c>
       <c r="C14" s="20" t="s">
@@ -1887,7 +1899,7 @@
       <c r="Q14" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R14" s="82" t="s">
+      <c r="R14" s="64" t="s">
         <v>37</v>
       </c>
       <c r="S14" s="65"/>
@@ -1897,7 +1909,7 @@
       <c r="W14" s="66"/>
     </row>
     <row r="15" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="90"/>
+      <c r="B15" s="74"/>
       <c r="C15" s="30" t="s">
         <v>12</v>
       </c>
@@ -1951,7 +1963,7 @@
       <c r="W15" s="69"/>
     </row>
     <row r="16" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="91"/>
+      <c r="B16" s="96"/>
       <c r="C16" s="31" t="s">
         <v>14</v>
       </c>
@@ -2006,7 +2018,7 @@
     </row>
     <row r="17" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
-      <c r="B17" s="95" t="s">
+      <c r="B17" s="99" t="s">
         <v>44</v>
       </c>
       <c r="C17" s="30" t="s">
@@ -2065,7 +2077,7 @@
     </row>
     <row r="18" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
-      <c r="B18" s="99"/>
+      <c r="B18" s="103"/>
       <c r="C18" s="30" t="s">
         <v>12</v>
       </c>
@@ -2120,7 +2132,7 @@
     </row>
     <row r="19" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8"/>
-      <c r="B19" s="98"/>
+      <c r="B19" s="102"/>
       <c r="C19" s="31" t="s">
         <v>14</v>
       </c>
@@ -2175,7 +2187,7 @@
     </row>
     <row r="20" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8"/>
-      <c r="B20" s="92" t="s">
+      <c r="B20" s="73" t="s">
         <v>46</v>
       </c>
       <c r="C20" s="30" t="s">
@@ -2223,7 +2235,7 @@
       <c r="Q20" s="36">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R20" s="64" t="s">
+      <c r="R20" s="78" t="s">
         <v>45</v>
       </c>
       <c r="S20" s="65"/>
@@ -2234,7 +2246,7 @@
     </row>
     <row r="21" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
-      <c r="B21" s="90"/>
+      <c r="B21" s="74"/>
       <c r="C21" s="30" t="s">
         <v>12</v>
       </c>
@@ -2289,7 +2301,7 @@
     </row>
     <row r="22" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="8"/>
-      <c r="B22" s="91"/>
+      <c r="B22" s="96"/>
       <c r="C22" s="31" t="s">
         <v>14</v>
       </c>
@@ -2342,9 +2354,9 @@
       <c r="V22" s="71"/>
       <c r="W22" s="72"/>
     </row>
-    <row r="23" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A23" s="59"/>
-      <c r="B23" s="61" t="s">
+      <c r="B23" s="75" t="s">
         <v>15</v>
       </c>
       <c r="C23" s="20" t="s">
@@ -2392,7 +2404,7 @@
       <c r="Q23" s="10">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R23" s="64" t="s">
+      <c r="R23" s="78" t="s">
         <v>53</v>
       </c>
       <c r="S23" s="65"/>
@@ -2401,9 +2413,9 @@
       <c r="V23" s="65"/>
       <c r="W23" s="66"/>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="59"/>
-      <c r="B24" s="62"/>
+      <c r="B24" s="76"/>
       <c r="C24" s="30" t="s">
         <v>12</v>
       </c>
@@ -2456,9 +2468,9 @@
       <c r="V24" s="68"/>
       <c r="W24" s="69"/>
     </row>
-    <row r="25" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="59"/>
-      <c r="B25" s="63"/>
+      <c r="B25" s="77"/>
       <c r="C25" s="31" t="s">
         <v>14</v>
       </c>
@@ -2511,9 +2523,9 @@
       <c r="V25" s="71"/>
       <c r="W25" s="72"/>
     </row>
-    <row r="26" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A26" s="59"/>
-      <c r="B26" s="61" t="s">
+      <c r="B26" s="75" t="s">
         <v>24</v>
       </c>
       <c r="C26" s="20" t="s">
@@ -2561,7 +2573,7 @@
       <c r="Q26" s="36">
         <v>1E-3</v>
       </c>
-      <c r="R26" s="82" t="s">
+      <c r="R26" s="64" t="s">
         <v>57</v>
       </c>
       <c r="S26" s="65"/>
@@ -2570,9 +2582,9 @@
       <c r="V26" s="65"/>
       <c r="W26" s="66"/>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="59"/>
-      <c r="B27" s="62"/>
+      <c r="B27" s="76"/>
       <c r="C27" s="30" t="s">
         <v>12</v>
       </c>
@@ -2625,9 +2637,9 @@
       <c r="V27" s="68"/>
       <c r="W27" s="69"/>
     </row>
-    <row r="28" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="59"/>
-      <c r="B28" s="63"/>
+      <c r="B28" s="77"/>
       <c r="C28" s="31" t="s">
         <v>14</v>
       </c>
@@ -2680,9 +2692,9 @@
       <c r="V28" s="71"/>
       <c r="W28" s="72"/>
     </row>
-    <row r="29" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A29" s="60"/>
-      <c r="B29" s="61" t="s">
+      <c r="B29" s="75" t="s">
         <v>34</v>
       </c>
       <c r="C29" s="29" t="s">
@@ -2730,7 +2742,7 @@
       <c r="Q29" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R29" s="64" t="s">
+      <c r="R29" s="78" t="s">
         <v>60</v>
       </c>
       <c r="S29" s="65"/>
@@ -2739,9 +2751,9 @@
       <c r="V29" s="65"/>
       <c r="W29" s="66"/>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="59"/>
-      <c r="B30" s="62"/>
+      <c r="B30" s="76"/>
       <c r="C30" s="26" t="s">
         <v>12</v>
       </c>
@@ -2794,9 +2806,9 @@
       <c r="V30" s="68"/>
       <c r="W30" s="69"/>
     </row>
-    <row r="31" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="59"/>
-      <c r="B31" s="63"/>
+      <c r="B31" s="77"/>
       <c r="C31" s="43" t="s">
         <v>14</v>
       </c>
@@ -2849,9 +2861,9 @@
       <c r="V31" s="71"/>
       <c r="W31" s="72"/>
     </row>
-    <row r="32" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A32" s="60"/>
-      <c r="B32" s="61" t="s">
+      <c r="B32" s="75" t="s">
         <v>36</v>
       </c>
       <c r="C32" s="29" t="s">
@@ -2899,7 +2911,7 @@
       <c r="Q32" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R32" s="82" t="s">
+      <c r="R32" s="64" t="s">
         <v>61</v>
       </c>
       <c r="S32" s="65"/>
@@ -2908,9 +2920,9 @@
       <c r="V32" s="65"/>
       <c r="W32" s="66"/>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="60"/>
-      <c r="B33" s="62"/>
+      <c r="B33" s="76"/>
       <c r="C33" s="26" t="s">
         <v>12</v>
       </c>
@@ -2963,9 +2975,9 @@
       <c r="V33" s="68"/>
       <c r="W33" s="69"/>
     </row>
-    <row r="34" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="60"/>
-      <c r="B34" s="63"/>
+      <c r="B34" s="77"/>
       <c r="C34" s="43" t="s">
         <v>14</v>
       </c>
@@ -3018,9 +3030,9 @@
       <c r="V34" s="71"/>
       <c r="W34" s="72"/>
     </row>
-    <row r="35" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A35" s="59"/>
-      <c r="B35" s="61" t="s">
+      <c r="B35" s="75" t="s">
         <v>44</v>
       </c>
       <c r="C35" s="26" t="s">
@@ -3068,7 +3080,7 @@
       <c r="Q35" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R35" s="64" t="s">
+      <c r="R35" s="78" t="s">
         <v>63</v>
       </c>
       <c r="S35" s="65"/>
@@ -3077,9 +3089,9 @@
       <c r="V35" s="65"/>
       <c r="W35" s="66"/>
     </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="59"/>
-      <c r="B36" s="62"/>
+      <c r="B36" s="76"/>
       <c r="C36" s="26" t="s">
         <v>12</v>
       </c>
@@ -3132,9 +3144,9 @@
       <c r="V36" s="68"/>
       <c r="W36" s="69"/>
     </row>
-    <row r="37" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="59"/>
-      <c r="B37" s="63"/>
+      <c r="B37" s="77"/>
       <c r="C37" s="31" t="s">
         <v>14</v>
       </c>
@@ -3187,9 +3199,9 @@
       <c r="V37" s="71"/>
       <c r="W37" s="72"/>
     </row>
-    <row r="38" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A38" s="60"/>
-      <c r="B38" s="61" t="s">
+      <c r="B38" s="75" t="s">
         <v>46</v>
       </c>
       <c r="C38" s="20" t="s">
@@ -3237,16 +3249,16 @@
       <c r="Q38" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R38" s="73"/>
-      <c r="S38" s="74"/>
-      <c r="T38" s="74"/>
-      <c r="U38" s="74"/>
-      <c r="V38" s="74"/>
-      <c r="W38" s="75"/>
-    </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="R38" s="79"/>
+      <c r="S38" s="80"/>
+      <c r="T38" s="80"/>
+      <c r="U38" s="80"/>
+      <c r="V38" s="80"/>
+      <c r="W38" s="81"/>
+    </row>
+    <row r="39" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="60"/>
-      <c r="B39" s="62"/>
+      <c r="B39" s="76"/>
       <c r="C39" s="30" t="s">
         <v>12</v>
       </c>
@@ -3292,16 +3304,16 @@
       <c r="Q39" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R39" s="76"/>
-      <c r="S39" s="77"/>
-      <c r="T39" s="77"/>
-      <c r="U39" s="77"/>
-      <c r="V39" s="77"/>
-      <c r="W39" s="78"/>
-    </row>
-    <row r="40" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R39" s="82"/>
+      <c r="S39" s="83"/>
+      <c r="T39" s="83"/>
+      <c r="U39" s="83"/>
+      <c r="V39" s="83"/>
+      <c r="W39" s="84"/>
+    </row>
+    <row r="40" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="60"/>
-      <c r="B40" s="63"/>
+      <c r="B40" s="77"/>
       <c r="C40" s="31" t="s">
         <v>14</v>
       </c>
@@ -3347,16 +3359,16 @@
       <c r="Q40" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R40" s="79"/>
-      <c r="S40" s="80"/>
-      <c r="T40" s="80"/>
-      <c r="U40" s="80"/>
-      <c r="V40" s="80"/>
-      <c r="W40" s="81"/>
-    </row>
-    <row r="41" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="R40" s="85"/>
+      <c r="S40" s="86"/>
+      <c r="T40" s="86"/>
+      <c r="U40" s="86"/>
+      <c r="V40" s="86"/>
+      <c r="W40" s="87"/>
+    </row>
+    <row r="41" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A41" s="60"/>
-      <c r="B41" s="61" t="s">
+      <c r="B41" s="75" t="s">
         <v>50</v>
       </c>
       <c r="C41" s="30" t="s">
@@ -3404,7 +3416,7 @@
       <c r="Q41" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R41" s="82" t="s">
+      <c r="R41" s="64" t="s">
         <v>71</v>
       </c>
       <c r="S41" s="65"/>
@@ -3413,9 +3425,9 @@
       <c r="V41" s="65"/>
       <c r="W41" s="66"/>
     </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="60"/>
-      <c r="B42" s="62"/>
+      <c r="B42" s="76"/>
       <c r="C42" s="30" t="s">
         <v>12</v>
       </c>
@@ -3468,9 +3480,9 @@
       <c r="V42" s="68"/>
       <c r="W42" s="69"/>
     </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="60"/>
-      <c r="B43" s="62"/>
+      <c r="B43" s="76"/>
       <c r="C43" s="30" t="s">
         <v>14</v>
       </c>
@@ -3523,9 +3535,9 @@
       <c r="V43" s="68"/>
       <c r="W43" s="69"/>
     </row>
-    <row r="44" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="60"/>
-      <c r="B44" s="63"/>
+      <c r="B44" s="77"/>
       <c r="C44" s="31" t="s">
         <v>67</v>
       </c>
@@ -3578,9 +3590,9 @@
       <c r="V44" s="71"/>
       <c r="W44" s="72"/>
     </row>
-    <row r="45" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A45" s="60"/>
-      <c r="B45" s="61" t="s">
+      <c r="B45" s="75" t="s">
         <v>55</v>
       </c>
       <c r="C45" s="30" t="s">
@@ -3628,18 +3640,18 @@
       <c r="Q45" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R45" s="100" t="s">
+      <c r="R45" s="88" t="s">
         <v>72</v>
       </c>
-      <c r="S45" s="74"/>
-      <c r="T45" s="74"/>
-      <c r="U45" s="74"/>
-      <c r="V45" s="74"/>
-      <c r="W45" s="75"/>
-    </row>
-    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="S45" s="80"/>
+      <c r="T45" s="80"/>
+      <c r="U45" s="80"/>
+      <c r="V45" s="80"/>
+      <c r="W45" s="81"/>
+    </row>
+    <row r="46" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="60"/>
-      <c r="B46" s="62"/>
+      <c r="B46" s="76"/>
       <c r="C46" s="30" t="s">
         <v>12</v>
       </c>
@@ -3685,16 +3697,16 @@
       <c r="Q46" s="8">
         <v>1E-3</v>
       </c>
-      <c r="R46" s="76"/>
-      <c r="S46" s="77"/>
-      <c r="T46" s="77"/>
-      <c r="U46" s="77"/>
-      <c r="V46" s="77"/>
-      <c r="W46" s="78"/>
-    </row>
-    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="R46" s="82"/>
+      <c r="S46" s="83"/>
+      <c r="T46" s="83"/>
+      <c r="U46" s="83"/>
+      <c r="V46" s="83"/>
+      <c r="W46" s="84"/>
+    </row>
+    <row r="47" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="60"/>
-      <c r="B47" s="62"/>
+      <c r="B47" s="76"/>
       <c r="C47" s="30" t="s">
         <v>14</v>
       </c>
@@ -3740,16 +3752,16 @@
       <c r="Q47" s="8">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R47" s="76"/>
-      <c r="S47" s="77"/>
-      <c r="T47" s="77"/>
-      <c r="U47" s="77"/>
-      <c r="V47" s="77"/>
-      <c r="W47" s="78"/>
-    </row>
-    <row r="48" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R47" s="82"/>
+      <c r="S47" s="83"/>
+      <c r="T47" s="83"/>
+      <c r="U47" s="83"/>
+      <c r="V47" s="83"/>
+      <c r="W47" s="84"/>
+    </row>
+    <row r="48" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="60"/>
-      <c r="B48" s="63"/>
+      <c r="B48" s="77"/>
       <c r="C48" s="31" t="s">
         <v>67</v>
       </c>
@@ -3795,16 +3807,16 @@
       <c r="Q48" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R48" s="79"/>
-      <c r="S48" s="80"/>
-      <c r="T48" s="80"/>
-      <c r="U48" s="80"/>
-      <c r="V48" s="80"/>
-      <c r="W48" s="81"/>
-    </row>
-    <row r="49" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="R48" s="85"/>
+      <c r="S48" s="86"/>
+      <c r="T48" s="86"/>
+      <c r="U48" s="86"/>
+      <c r="V48" s="86"/>
+      <c r="W48" s="87"/>
+    </row>
+    <row r="49" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A49" s="59"/>
-      <c r="B49" s="61" t="s">
+      <c r="B49" s="75" t="s">
         <v>58</v>
       </c>
       <c r="C49" s="30" t="s">
@@ -3852,7 +3864,7 @@
       <c r="Q49" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R49" s="64" t="s">
+      <c r="R49" s="78" t="s">
         <v>79</v>
       </c>
       <c r="S49" s="65"/>
@@ -3861,9 +3873,9 @@
       <c r="V49" s="65"/>
       <c r="W49" s="66"/>
     </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="59"/>
-      <c r="B50" s="62"/>
+      <c r="B50" s="76"/>
       <c r="C50" s="30" t="s">
         <v>12</v>
       </c>
@@ -3916,9 +3928,9 @@
       <c r="V50" s="68"/>
       <c r="W50" s="69"/>
     </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="59"/>
-      <c r="B51" s="62"/>
+      <c r="B51" s="76"/>
       <c r="C51" s="30" t="s">
         <v>14</v>
       </c>
@@ -3971,9 +3983,9 @@
       <c r="V51" s="68"/>
       <c r="W51" s="69"/>
     </row>
-    <row r="52" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="59"/>
-      <c r="B52" s="63"/>
+      <c r="B52" s="77"/>
       <c r="C52" s="31" t="s">
         <v>67</v>
       </c>
@@ -4027,8 +4039,8 @@
       <c r="W52" s="72"/>
     </row>
     <row r="53" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="120"/>
-      <c r="B53" s="61" t="s">
+      <c r="A53" s="60"/>
+      <c r="B53" s="75" t="s">
         <v>77</v>
       </c>
       <c r="C53" s="20" t="s">
@@ -4049,7 +4061,7 @@
       <c r="H53" s="53">
         <v>22.5</v>
       </c>
-      <c r="I53" s="117">
+      <c r="I53" s="9">
         <v>18</v>
       </c>
       <c r="J53" s="9">
@@ -4070,13 +4082,13 @@
       <c r="O53" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P53" s="101" t="s">
+      <c r="P53" s="61" t="s">
         <v>68</v>
       </c>
       <c r="Q53" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R53" s="64" t="s">
+      <c r="R53" s="78" t="s">
         <v>80</v>
       </c>
       <c r="S53" s="65"/>
@@ -4086,27 +4098,27 @@
       <c r="W53" s="66"/>
     </row>
     <row r="54" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A54" s="120"/>
-      <c r="B54" s="62"/>
+      <c r="A54" s="60"/>
+      <c r="B54" s="76"/>
       <c r="C54" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="D54" s="104">
+      <c r="D54">
         <v>270.029</v>
       </c>
-      <c r="E54" s="104">
+      <c r="E54">
         <v>498.339</v>
       </c>
-      <c r="F54" s="106">
+      <c r="F54" s="41">
         <v>-0.45190000000000002</v>
       </c>
-      <c r="G54" s="106">
+      <c r="G54" s="41">
         <v>-0.45300000000000001</v>
       </c>
       <c r="H54" s="8">
         <v>77.099999999999994</v>
       </c>
-      <c r="I54" s="118">
+      <c r="I54" s="1">
         <v>18</v>
       </c>
       <c r="J54">
@@ -4127,7 +4139,7 @@
       <c r="O54" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P54" s="102" t="s">
+      <c r="P54" s="62" t="s">
         <v>68</v>
       </c>
       <c r="Q54" s="8">
@@ -4141,27 +4153,27 @@
       <c r="W54" s="69"/>
     </row>
     <row r="55" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A55" s="120"/>
-      <c r="B55" s="62"/>
+      <c r="A55" s="60"/>
+      <c r="B55" s="76"/>
       <c r="C55" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="D55" s="104">
+      <c r="D55">
         <v>68.706999999999994</v>
       </c>
-      <c r="E55" s="104">
+      <c r="E55">
         <v>124.129</v>
       </c>
-      <c r="F55" s="104">
+      <c r="F55">
         <v>0.90990000000000004</v>
       </c>
-      <c r="G55" s="104">
+      <c r="G55">
         <v>0.90980000000000005</v>
       </c>
       <c r="H55" s="8">
         <v>59.6</v>
       </c>
-      <c r="I55" s="118">
+      <c r="I55" s="1">
         <v>18</v>
       </c>
       <c r="J55">
@@ -4182,7 +4194,7 @@
       <c r="O55" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P55" s="102" t="s">
+      <c r="P55" s="62" t="s">
         <v>68</v>
       </c>
       <c r="Q55" s="8">
@@ -4196,8 +4208,8 @@
       <c r="W55" s="69"/>
     </row>
     <row r="56" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="120"/>
-      <c r="B56" s="63"/>
+      <c r="A56" s="60"/>
+      <c r="B56" s="77"/>
       <c r="C56" s="31" t="s">
         <v>67</v>
       </c>
@@ -4213,10 +4225,10 @@
       <c r="G56" s="49">
         <v>-0.45300000000000001</v>
       </c>
-      <c r="H56" s="105">
+      <c r="H56" s="8">
         <v>38.4</v>
       </c>
-      <c r="I56" s="119">
+      <c r="I56" s="2">
         <v>18</v>
       </c>
       <c r="J56" s="3">
@@ -4237,7 +4249,7 @@
       <c r="O56" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="P56" s="103" t="s">
+      <c r="P56" s="63" t="s">
         <v>68</v>
       </c>
       <c r="Q56" s="4">
@@ -4251,11 +4263,11 @@
       <c r="W56" s="72"/>
     </row>
     <row r="57" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="121"/>
-      <c r="B57" s="61" t="s">
+      <c r="A57" s="59"/>
+      <c r="B57" s="75" t="s">
         <v>81</v>
       </c>
-      <c r="C57" s="109" t="s">
+      <c r="C57" s="20" t="s">
         <v>13</v>
       </c>
       <c r="D57" s="9">
@@ -4273,34 +4285,34 @@
       <c r="H57" s="10">
         <v>22.4</v>
       </c>
-      <c r="I57" s="118">
+      <c r="I57" s="1">
         <v>18</v>
       </c>
-      <c r="J57" s="104">
+      <c r="J57">
         <v>236</v>
       </c>
-      <c r="K57" s="104">
-        <v>6</v>
-      </c>
-      <c r="L57" s="107" t="s">
+      <c r="K57">
+        <v>6</v>
+      </c>
+      <c r="L57" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="M57" s="104">
-        <v>64</v>
-      </c>
-      <c r="N57" s="113">
-        <v>64</v>
-      </c>
-      <c r="O57" s="107" t="s">
+      <c r="M57">
+        <v>64</v>
+      </c>
+      <c r="N57" s="46">
+        <v>64</v>
+      </c>
+      <c r="O57" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P57" s="113">
+      <c r="P57" s="46">
         <v>0.1</v>
       </c>
       <c r="Q57" s="10">
         <v>1E-3</v>
       </c>
-      <c r="R57" s="64" t="s">
+      <c r="R57" s="78" t="s">
         <v>82</v>
       </c>
       <c r="S57" s="65"/>
@@ -4310,119 +4322,119 @@
       <c r="W57" s="66"/>
     </row>
     <row r="58" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A58" s="121"/>
-      <c r="B58" s="62"/>
-      <c r="C58" s="108" t="s">
+      <c r="A58" s="59"/>
+      <c r="B58" s="76"/>
+      <c r="C58" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="D58" s="115">
+      <c r="D58" s="104">
         <v>87.501999999999995</v>
       </c>
-      <c r="E58" s="115">
+      <c r="E58" s="104">
         <v>143.33000000000001</v>
       </c>
-      <c r="F58" s="116">
+      <c r="F58" s="105">
         <v>0.87990000000000002</v>
       </c>
-      <c r="G58" s="116">
+      <c r="G58" s="105">
         <v>0.87980000000000003</v>
       </c>
-      <c r="H58" s="53">
+      <c r="H58" s="106">
         <v>22.6</v>
       </c>
-      <c r="I58" s="118">
+      <c r="I58" s="1">
         <v>18</v>
       </c>
-      <c r="J58" s="104">
+      <c r="J58">
         <v>282.67</v>
       </c>
-      <c r="K58" s="104">
-        <v>6</v>
-      </c>
-      <c r="L58" s="107" t="s">
+      <c r="K58">
+        <v>6</v>
+      </c>
+      <c r="L58" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="M58" s="104">
-        <v>64</v>
-      </c>
-      <c r="N58" s="113">
+      <c r="M58">
+        <v>64</v>
+      </c>
+      <c r="N58" s="46">
         <v>32</v>
       </c>
-      <c r="O58" s="107" t="s">
+      <c r="O58" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P58" s="113">
+      <c r="P58" s="46">
         <v>0.1</v>
       </c>
       <c r="Q58" s="8">
         <v>1E-3</v>
       </c>
       <c r="R58" s="67"/>
-      <c r="S58" s="114"/>
-      <c r="T58" s="114"/>
-      <c r="U58" s="114"/>
-      <c r="V58" s="114"/>
+      <c r="S58" s="68"/>
+      <c r="T58" s="68"/>
+      <c r="U58" s="68"/>
+      <c r="V58" s="68"/>
       <c r="W58" s="69"/>
     </row>
     <row r="59" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A59" s="121"/>
-      <c r="B59" s="62"/>
-      <c r="C59" s="108" t="s">
+      <c r="A59" s="59"/>
+      <c r="B59" s="76"/>
+      <c r="C59" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="D59" s="104">
+      <c r="D59" s="52">
         <v>53.17</v>
       </c>
-      <c r="E59" s="104">
+      <c r="E59" s="52">
         <v>96.721999999999994</v>
       </c>
-      <c r="F59" s="104">
+      <c r="F59" s="52">
         <v>0.94530000000000003</v>
       </c>
-      <c r="G59" s="104">
+      <c r="G59" s="52">
         <v>0.94530000000000003</v>
       </c>
-      <c r="H59" s="8">
+      <c r="H59" s="53">
         <v>17.899999999999999</v>
       </c>
-      <c r="I59" s="118">
+      <c r="I59" s="1">
         <v>18</v>
       </c>
-      <c r="J59" s="104">
+      <c r="J59">
         <v>555.5</v>
       </c>
-      <c r="K59" s="104">
-        <v>6</v>
-      </c>
-      <c r="L59" s="107" t="s">
+      <c r="K59">
+        <v>6</v>
+      </c>
+      <c r="L59" s="32" t="s">
         <v>52</v>
       </c>
-      <c r="M59" s="104">
-        <v>64</v>
-      </c>
-      <c r="N59" s="113">
+      <c r="M59">
+        <v>64</v>
+      </c>
+      <c r="N59" s="46">
         <v>32</v>
       </c>
-      <c r="O59" s="107" t="s">
+      <c r="O59" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P59" s="113">
+      <c r="P59" s="46">
         <v>0.1</v>
       </c>
       <c r="Q59" s="8">
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="R59" s="67"/>
-      <c r="S59" s="114"/>
-      <c r="T59" s="114"/>
-      <c r="U59" s="114"/>
-      <c r="V59" s="114"/>
+      <c r="S59" s="68"/>
+      <c r="T59" s="68"/>
+      <c r="U59" s="68"/>
+      <c r="V59" s="68"/>
       <c r="W59" s="69"/>
     </row>
     <row r="60" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="121"/>
-      <c r="B60" s="63"/>
-      <c r="C60" s="110" t="s">
+      <c r="A60" s="59"/>
+      <c r="B60" s="77"/>
+      <c r="C60" s="31" t="s">
         <v>67</v>
       </c>
       <c r="D60" s="3">
@@ -4440,25 +4452,25 @@
       <c r="H60" s="4">
         <v>19.3</v>
       </c>
-      <c r="I60" s="119">
+      <c r="I60" s="2">
         <v>18</v>
       </c>
       <c r="J60" s="3">
         <v>155.08000000000001</v>
       </c>
-      <c r="K60" s="111">
-        <v>6</v>
-      </c>
-      <c r="L60" s="3" t="s">
+      <c r="K60" s="3">
+        <v>6</v>
+      </c>
+      <c r="L60" s="35" t="s">
         <v>49</v>
       </c>
-      <c r="M60" s="111">
+      <c r="M60" s="3">
         <v>64</v>
       </c>
       <c r="N60" s="47">
         <v>32</v>
       </c>
-      <c r="O60" s="112" t="s">
+      <c r="O60" s="35" t="s">
         <v>39</v>
       </c>
       <c r="P60" s="47">
@@ -4474,9 +4486,290 @@
       <c r="V60" s="71"/>
       <c r="W60" s="72"/>
     </row>
-    <row r="61" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="8"/>
+      <c r="B61" s="75" t="s">
+        <v>85</v>
+      </c>
+      <c r="C61" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61" s="112">
+        <v>54.145000000000003</v>
+      </c>
+      <c r="E61" s="108">
+        <v>102.96899999999999</v>
+      </c>
+      <c r="F61">
+        <v>0.93799999999999994</v>
+      </c>
+      <c r="G61">
+        <v>0.93799999999999994</v>
+      </c>
+      <c r="H61" s="106">
+        <v>22.4</v>
+      </c>
+      <c r="I61" s="107">
+        <v>18</v>
+      </c>
+      <c r="J61" s="108">
+        <v>339.69</v>
+      </c>
+      <c r="K61" s="108">
+        <v>6</v>
+      </c>
+      <c r="L61" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="M61" s="108">
+        <v>64</v>
+      </c>
+      <c r="N61" s="108">
+        <v>64</v>
+      </c>
+      <c r="O61" s="109" t="s">
+        <v>39</v>
+      </c>
+      <c r="P61" s="108">
+        <v>0.1</v>
+      </c>
+      <c r="Q61" s="106">
+        <v>1E-3</v>
+      </c>
+      <c r="R61" s="88" t="s">
+        <v>86</v>
+      </c>
+      <c r="S61" s="80"/>
+      <c r="T61" s="80"/>
+      <c r="U61" s="80"/>
+      <c r="V61" s="80"/>
+      <c r="W61" s="81"/>
+    </row>
+    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A62" s="8"/>
+      <c r="B62" s="76"/>
+      <c r="C62" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="D62" s="113">
+        <v>51.847000000000001</v>
+      </c>
+      <c r="E62" s="52">
+        <v>99.551000000000002</v>
+      </c>
+      <c r="F62" s="52">
+        <v>0.94210000000000005</v>
+      </c>
+      <c r="G62" s="52">
+        <v>0.94199999999999995</v>
+      </c>
+      <c r="H62" s="53">
+        <v>22.6</v>
+      </c>
+      <c r="I62" s="107">
+        <v>18</v>
+      </c>
+      <c r="J62" s="108">
+        <v>665.01</v>
+      </c>
+      <c r="K62" s="108">
+        <v>6</v>
+      </c>
+      <c r="L62" s="32" t="s">
+        <v>83</v>
+      </c>
+      <c r="M62" s="108">
+        <v>64</v>
+      </c>
+      <c r="N62" s="108">
+        <v>32</v>
+      </c>
+      <c r="O62" s="109" t="s">
+        <v>39</v>
+      </c>
+      <c r="P62" s="108">
+        <v>0.1</v>
+      </c>
+      <c r="Q62" s="106">
+        <v>1E-3</v>
+      </c>
+      <c r="R62" s="82"/>
+      <c r="S62" s="83"/>
+      <c r="T62" s="83"/>
+      <c r="U62" s="83"/>
+      <c r="V62" s="83"/>
+      <c r="W62" s="84"/>
+    </row>
+    <row r="63" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A63" s="8"/>
+      <c r="B63" s="76"/>
+      <c r="C63" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D63" s="108">
+        <v>105.566</v>
+      </c>
+      <c r="E63">
+        <v>149.756</v>
+      </c>
+      <c r="F63">
+        <v>0.86890000000000001</v>
+      </c>
+      <c r="G63">
+        <v>0.86880000000000002</v>
+      </c>
+      <c r="H63" s="106">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="I63" s="107">
+        <v>18</v>
+      </c>
+      <c r="J63" s="108">
+        <v>382.5</v>
+      </c>
+      <c r="K63" s="108">
+        <v>6</v>
+      </c>
+      <c r="L63" s="32" t="s">
+        <v>49</v>
+      </c>
+      <c r="M63" s="108">
+        <v>64</v>
+      </c>
+      <c r="N63" s="108">
+        <v>32</v>
+      </c>
+      <c r="O63" s="109" t="s">
+        <v>39</v>
+      </c>
+      <c r="P63" s="108">
+        <v>0.1</v>
+      </c>
+      <c r="Q63" s="111">
+        <v>1E-3</v>
+      </c>
+      <c r="R63" s="82"/>
+      <c r="S63" s="83"/>
+      <c r="T63" s="83"/>
+      <c r="U63" s="83"/>
+      <c r="V63" s="83"/>
+      <c r="W63" s="84"/>
+    </row>
+    <row r="64" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A64" s="8"/>
+      <c r="B64" s="76"/>
+      <c r="C64" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="D64" s="108">
+        <v>109.354</v>
+      </c>
+      <c r="E64">
+        <v>173.17099999999999</v>
+      </c>
+      <c r="F64">
+        <v>0.82469999999999999</v>
+      </c>
+      <c r="G64">
+        <v>0.82450000000000001</v>
+      </c>
+      <c r="H64" s="106">
+        <v>19.3</v>
+      </c>
+      <c r="I64" s="107">
+        <v>18</v>
+      </c>
+      <c r="J64" s="108">
+        <v>189.74</v>
+      </c>
+      <c r="K64" s="108">
+        <v>6</v>
+      </c>
+      <c r="L64" s="32" t="s">
+        <v>49</v>
+      </c>
+      <c r="M64" s="108">
+        <v>64</v>
+      </c>
+      <c r="N64" s="108">
+        <v>32</v>
+      </c>
+      <c r="O64" s="109" t="s">
+        <v>39</v>
+      </c>
+      <c r="P64" s="108">
+        <v>0.1</v>
+      </c>
+      <c r="Q64" s="8">
+        <v>1E-3</v>
+      </c>
+      <c r="R64" s="82"/>
+      <c r="S64" s="83"/>
+      <c r="T64" s="83"/>
+      <c r="U64" s="83"/>
+      <c r="V64" s="83"/>
+      <c r="W64" s="84"/>
+    </row>
+    <row r="65" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="8"/>
+      <c r="B65" s="77"/>
+      <c r="C65" s="31" t="s">
+        <v>84</v>
+      </c>
+      <c r="D65" s="3">
+        <v>122.208</v>
+      </c>
+      <c r="E65" s="3">
+        <v>174.66300000000001</v>
+      </c>
+      <c r="F65" s="3">
+        <v>0.8216</v>
+      </c>
+      <c r="G65" s="3">
+        <v>0.82150000000000001</v>
+      </c>
+      <c r="H65" s="4">
+        <v>20.3</v>
+      </c>
+      <c r="I65" s="2">
+        <v>18</v>
+      </c>
+      <c r="J65" s="3">
+        <v>132.01</v>
+      </c>
+      <c r="K65" s="3">
+        <v>6</v>
+      </c>
+      <c r="L65" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="M65" s="3">
+        <v>64</v>
+      </c>
+      <c r="N65" s="3">
+        <v>32</v>
+      </c>
+      <c r="O65" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="P65" s="110">
+        <v>0.1</v>
+      </c>
+      <c r="Q65" s="4">
+        <v>1E-3</v>
+      </c>
+      <c r="R65" s="85"/>
+      <c r="S65" s="86"/>
+      <c r="T65" s="86"/>
+      <c r="U65" s="86"/>
+      <c r="V65" s="86"/>
+      <c r="W65" s="87"/>
+    </row>
+    <row r="66" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="37">
+  <mergeCells count="39">
+    <mergeCell ref="B61:B65"/>
+    <mergeCell ref="R61:W65"/>
     <mergeCell ref="B57:B60"/>
     <mergeCell ref="R57:W60"/>
     <mergeCell ref="R11:W13"/>
@@ -4490,6 +4783,9 @@
     <mergeCell ref="R29:W31"/>
     <mergeCell ref="B32:B34"/>
     <mergeCell ref="R32:W34"/>
+    <mergeCell ref="B23:B25"/>
+    <mergeCell ref="R23:W25"/>
+    <mergeCell ref="B26:B28"/>
     <mergeCell ref="D3:H3"/>
     <mergeCell ref="I3:Q3"/>
     <mergeCell ref="B5:B7"/>
@@ -4497,9 +4793,6 @@
     <mergeCell ref="R3:W4"/>
     <mergeCell ref="R5:W7"/>
     <mergeCell ref="R8:W10"/>
-    <mergeCell ref="B23:B25"/>
-    <mergeCell ref="R23:W25"/>
-    <mergeCell ref="B26:B28"/>
     <mergeCell ref="R26:W28"/>
     <mergeCell ref="B11:B13"/>
     <mergeCell ref="B53:B56"/>

</xml_diff>

<commit_message>
Nuevo script para comparar datos diurnos vs. dia completo
</commit_message>
<xml_diff>
--- a/modelos_tfg/MetricasValidacion.xlsx
+++ b/modelos_tfg/MetricasValidacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\modelos_tfg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BA035B1-3EDA-48E9-B8C3-AFDF67D3C157}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13C9D6B3-DA7A-4650-A1CF-C1C0F2323CC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -427,7 +427,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -661,11 +661,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -673,9 +686,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
@@ -764,105 +774,108 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -884,18 +897,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1281,23 +1285,23 @@
       <c r="O3" s="93"/>
       <c r="P3" s="93"/>
       <c r="Q3" s="94"/>
-      <c r="R3" s="97" t="s">
+      <c r="R3" s="99" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="98"/>
-      <c r="T3" s="98"/>
-      <c r="U3" s="98"/>
-      <c r="V3" s="98"/>
-      <c r="W3" s="99"/>
+      <c r="S3" s="100"/>
+      <c r="T3" s="100"/>
+      <c r="U3" s="100"/>
+      <c r="V3" s="100"/>
+      <c r="W3" s="101"/>
     </row>
     <row r="4" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="15" t="s">
+      <c r="C4" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="14" t="s">
         <v>22</v>
       </c>
       <c r="E4" s="6" t="s">
@@ -1309,45 +1313,45 @@
       <c r="G4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="106" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="11" t="s">
+      <c r="I4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="J4" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="K4" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="12" t="s">
+      <c r="L4" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="M4" s="12" t="s">
+      <c r="M4" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="N4" s="12" t="s">
+      <c r="N4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="O4" s="12" t="s">
+      <c r="O4" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="P4" s="12" t="s">
+      <c r="P4" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="Q4" s="13" t="s">
+      <c r="Q4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="100"/>
-      <c r="S4" s="101"/>
-      <c r="T4" s="101"/>
-      <c r="U4" s="101"/>
-      <c r="V4" s="101"/>
-      <c r="W4" s="102"/>
-    </row>
-    <row r="5" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
+      <c r="R4" s="102"/>
+      <c r="S4" s="103"/>
+      <c r="T4" s="103"/>
+      <c r="U4" s="103"/>
+      <c r="V4" s="103"/>
+      <c r="W4" s="104"/>
+    </row>
+    <row r="5" spans="1:23" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="7"/>
       <c r="B5" s="95" t="s">
         <v>15</v>
       </c>
@@ -1357,57 +1361,57 @@
       <c r="D5" s="1">
         <v>154.94499999999999</v>
       </c>
-      <c r="E5" s="16">
+      <c r="E5" s="15">
         <v>449.51100000000002</v>
       </c>
-      <c r="F5" s="16">
+      <c r="F5" s="15">
         <v>0.79569999999999996</v>
       </c>
-      <c r="G5" s="16">
+      <c r="G5" s="15">
         <v>0.79520000000000002</v>
       </c>
-      <c r="H5" s="17">
+      <c r="H5" s="7">
         <v>30</v>
       </c>
-      <c r="I5" s="18">
+      <c r="I5" s="17">
         <v>18</v>
       </c>
-      <c r="J5" s="24">
+      <c r="J5" s="23">
         <v>105.81</v>
       </c>
-      <c r="K5" s="16">
-        <v>6</v>
-      </c>
-      <c r="L5" s="24" t="s">
+      <c r="K5" s="15">
+        <v>6</v>
+      </c>
+      <c r="L5" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="M5" s="16">
+      <c r="M5" s="15">
         <v>32</v>
       </c>
-      <c r="N5" s="16">
-        <v>64</v>
-      </c>
-      <c r="O5" s="21" t="s">
+      <c r="N5" s="15">
+        <v>64</v>
+      </c>
+      <c r="O5" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="P5" s="16">
+      <c r="P5" s="15">
         <v>0.2</v>
       </c>
-      <c r="Q5" s="17">
+      <c r="Q5" s="16">
         <v>1E-3</v>
       </c>
-      <c r="R5" s="64" t="s">
+      <c r="R5" s="87" t="s">
         <v>38</v>
       </c>
-      <c r="S5" s="65"/>
-      <c r="T5" s="65"/>
-      <c r="U5" s="65"/>
-      <c r="V5" s="65"/>
-      <c r="W5" s="66"/>
+      <c r="S5" s="70"/>
+      <c r="T5" s="70"/>
+      <c r="U5" s="70"/>
+      <c r="V5" s="70"/>
+      <c r="W5" s="71"/>
     </row>
     <row r="6" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8"/>
-      <c r="B6" s="74"/>
+      <c r="A6" s="7"/>
+      <c r="B6" s="96"/>
       <c r="C6" s="5" t="s">
         <v>12</v>
       </c>
@@ -1423,7 +1427,7 @@
       <c r="G6">
         <v>0.80389999999999995</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="7">
         <v>87.8</v>
       </c>
       <c r="I6" s="1">
@@ -1435,7 +1439,7 @@
       <c r="K6">
         <v>6</v>
       </c>
-      <c r="L6" s="32" t="s">
+      <c r="L6" s="31" t="s">
         <v>27</v>
       </c>
       <c r="M6">
@@ -1444,26 +1448,26 @@
       <c r="N6">
         <v>64</v>
       </c>
-      <c r="O6" s="22" t="s">
+      <c r="O6" s="21" t="s">
         <v>19</v>
       </c>
       <c r="P6">
         <v>0.2</v>
       </c>
-      <c r="Q6" s="8">
+      <c r="Q6" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R6" s="67"/>
-      <c r="S6" s="68"/>
-      <c r="T6" s="68"/>
-      <c r="U6" s="68"/>
-      <c r="V6" s="68"/>
-      <c r="W6" s="69"/>
+      <c r="R6" s="72"/>
+      <c r="S6" s="73"/>
+      <c r="T6" s="73"/>
+      <c r="U6" s="73"/>
+      <c r="V6" s="73"/>
+      <c r="W6" s="74"/>
     </row>
     <row r="7" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="8"/>
-      <c r="B7" s="96"/>
-      <c r="C7" s="14" t="s">
+      <c r="A7" s="7"/>
+      <c r="B7" s="97"/>
+      <c r="C7" s="13" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="2">
@@ -1490,7 +1494,7 @@
       <c r="K7" s="3">
         <v>6</v>
       </c>
-      <c r="L7" s="35" t="s">
+      <c r="L7" s="34" t="s">
         <v>28</v>
       </c>
       <c r="M7" s="3">
@@ -1499,7 +1503,7 @@
       <c r="N7" s="3">
         <v>64</v>
       </c>
-      <c r="O7" s="23" t="s">
+      <c r="O7" s="22" t="s">
         <v>19</v>
       </c>
       <c r="P7" s="3">
@@ -1508,16 +1512,16 @@
       <c r="Q7" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R7" s="70"/>
-      <c r="S7" s="71"/>
-      <c r="T7" s="71"/>
-      <c r="U7" s="71"/>
-      <c r="V7" s="71"/>
-      <c r="W7" s="72"/>
+      <c r="R7" s="75"/>
+      <c r="S7" s="76"/>
+      <c r="T7" s="76"/>
+      <c r="U7" s="76"/>
+      <c r="V7" s="76"/>
+      <c r="W7" s="77"/>
     </row>
     <row r="8" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
-      <c r="B8" s="73" t="s">
+      <c r="A8" s="7"/>
+      <c r="B8" s="98" t="s">
         <v>24</v>
       </c>
       <c r="C8" s="5" t="s">
@@ -1526,16 +1530,16 @@
       <c r="D8" s="1">
         <v>175.917</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="8">
         <v>453.26499999999999</v>
       </c>
-      <c r="F8" s="9">
+      <c r="F8" s="8">
         <v>0.79220000000000002</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="8">
         <v>0.79179999999999995</v>
       </c>
-      <c r="H8" s="10">
+      <c r="H8" s="9">
         <v>30</v>
       </c>
       <c r="I8" s="1">
@@ -1547,7 +1551,7 @@
       <c r="K8">
         <v>6</v>
       </c>
-      <c r="L8" s="32" t="s">
+      <c r="L8" s="31" t="s">
         <v>29</v>
       </c>
       <c r="M8">
@@ -1556,27 +1560,27 @@
       <c r="N8">
         <v>64</v>
       </c>
-      <c r="O8" s="22" t="s">
+      <c r="O8" s="21" t="s">
         <v>19</v>
       </c>
       <c r="P8">
         <v>0.2</v>
       </c>
-      <c r="Q8" s="8">
+      <c r="Q8" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R8" s="64" t="s">
+      <c r="R8" s="87" t="s">
         <v>38</v>
       </c>
-      <c r="S8" s="65"/>
-      <c r="T8" s="65"/>
-      <c r="U8" s="65"/>
-      <c r="V8" s="65"/>
-      <c r="W8" s="66"/>
+      <c r="S8" s="70"/>
+      <c r="T8" s="70"/>
+      <c r="U8" s="70"/>
+      <c r="V8" s="70"/>
+      <c r="W8" s="71"/>
     </row>
     <row r="9" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
-      <c r="B9" s="74"/>
+      <c r="A9" s="7"/>
+      <c r="B9" s="96"/>
       <c r="C9" s="5" t="s">
         <v>12</v>
       </c>
@@ -1592,7 +1596,7 @@
       <c r="G9">
         <v>0.80049999999999999</v>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="7">
         <v>87.8</v>
       </c>
       <c r="I9" s="1">
@@ -1604,7 +1608,7 @@
       <c r="K9">
         <v>6</v>
       </c>
-      <c r="L9" s="32" t="s">
+      <c r="L9" s="31" t="s">
         <v>30</v>
       </c>
       <c r="M9">
@@ -1613,25 +1617,25 @@
       <c r="N9">
         <v>64</v>
       </c>
-      <c r="O9" s="22" t="s">
+      <c r="O9" s="21" t="s">
         <v>25</v>
       </c>
       <c r="P9">
         <v>0.2</v>
       </c>
-      <c r="Q9" s="8">
+      <c r="Q9" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R9" s="67"/>
-      <c r="S9" s="68"/>
-      <c r="T9" s="68"/>
-      <c r="U9" s="68"/>
-      <c r="V9" s="68"/>
-      <c r="W9" s="69"/>
+      <c r="R9" s="72"/>
+      <c r="S9" s="73"/>
+      <c r="T9" s="73"/>
+      <c r="U9" s="73"/>
+      <c r="V9" s="73"/>
+      <c r="W9" s="74"/>
     </row>
     <row r="10" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="8"/>
-      <c r="B10" s="96"/>
+      <c r="A10" s="7"/>
+      <c r="B10" s="97"/>
       <c r="C10" s="5" t="s">
         <v>14</v>
       </c>
@@ -1659,7 +1663,7 @@
       <c r="K10" s="3">
         <v>6</v>
       </c>
-      <c r="L10" s="35" t="s">
+      <c r="L10" s="34" t="s">
         <v>29</v>
       </c>
       <c r="M10" s="3">
@@ -1668,7 +1672,7 @@
       <c r="N10" s="3">
         <v>64</v>
       </c>
-      <c r="O10" s="23" t="s">
+      <c r="O10" s="22" t="s">
         <v>19</v>
       </c>
       <c r="P10" s="3">
@@ -1677,18 +1681,18 @@
       <c r="Q10" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R10" s="70"/>
-      <c r="S10" s="71"/>
-      <c r="T10" s="71"/>
-      <c r="U10" s="71"/>
-      <c r="V10" s="71"/>
-      <c r="W10" s="72"/>
+      <c r="R10" s="75"/>
+      <c r="S10" s="76"/>
+      <c r="T10" s="76"/>
+      <c r="U10" s="76"/>
+      <c r="V10" s="76"/>
+      <c r="W10" s="77"/>
     </row>
     <row r="11" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="73" t="s">
+      <c r="B11" s="98" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="29" t="s">
+      <c r="C11" s="28" t="s">
         <v>13</v>
       </c>
       <c r="D11" s="1">
@@ -1703,7 +1707,7 @@
       <c r="G11">
         <v>0.80469999999999997</v>
       </c>
-      <c r="H11" s="8">
+      <c r="H11" s="7">
         <v>30</v>
       </c>
       <c r="I11" s="1">
@@ -1715,36 +1719,36 @@
       <c r="K11">
         <v>6</v>
       </c>
-      <c r="L11" s="32" t="s">
+      <c r="L11" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="M11" s="25">
+      <c r="M11" s="24">
         <v>64</v>
       </c>
       <c r="N11">
         <v>64</v>
       </c>
-      <c r="O11" s="22" t="s">
+      <c r="O11" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="P11" s="25">
+      <c r="P11" s="24">
         <v>0.3</v>
       </c>
-      <c r="Q11" s="8">
+      <c r="Q11" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R11" s="64" t="s">
+      <c r="R11" s="87" t="s">
         <v>38</v>
       </c>
-      <c r="S11" s="65"/>
-      <c r="T11" s="65"/>
-      <c r="U11" s="65"/>
-      <c r="V11" s="65"/>
-      <c r="W11" s="66"/>
+      <c r="S11" s="70"/>
+      <c r="T11" s="70"/>
+      <c r="U11" s="70"/>
+      <c r="V11" s="70"/>
+      <c r="W11" s="71"/>
     </row>
     <row r="12" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="74"/>
-      <c r="C12" s="26" t="s">
+      <c r="B12" s="96"/>
+      <c r="C12" s="25" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="1">
@@ -1759,7 +1763,7 @@
       <c r="G12">
         <v>0.71819999999999995</v>
       </c>
-      <c r="H12" s="8">
+      <c r="H12" s="7">
         <v>87.8</v>
       </c>
       <c r="I12" s="1">
@@ -1771,34 +1775,34 @@
       <c r="K12">
         <v>6</v>
       </c>
-      <c r="L12" s="32" t="s">
+      <c r="L12" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="M12" s="25">
+      <c r="M12" s="24">
         <v>64</v>
       </c>
       <c r="N12">
         <v>64</v>
       </c>
-      <c r="O12" s="22" t="s">
+      <c r="O12" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="P12" s="25">
+      <c r="P12" s="24">
         <v>0.3</v>
       </c>
-      <c r="Q12" s="8">
+      <c r="Q12" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R12" s="67"/>
-      <c r="S12" s="68"/>
-      <c r="T12" s="68"/>
-      <c r="U12" s="68"/>
-      <c r="V12" s="68"/>
-      <c r="W12" s="69"/>
+      <c r="R12" s="72"/>
+      <c r="S12" s="73"/>
+      <c r="T12" s="73"/>
+      <c r="U12" s="73"/>
+      <c r="V12" s="73"/>
+      <c r="W12" s="74"/>
     </row>
     <row r="13" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="74"/>
-      <c r="C13" s="27" t="s">
+      <c r="B13" s="96"/>
+      <c r="C13" s="26" t="s">
         <v>14</v>
       </c>
       <c r="D13" s="2">
@@ -1825,36 +1829,36 @@
       <c r="K13" s="3">
         <v>6</v>
       </c>
-      <c r="L13" s="35" t="s">
+      <c r="L13" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="M13" s="28">
+      <c r="M13" s="27">
         <v>64</v>
       </c>
       <c r="N13" s="3">
         <v>64</v>
       </c>
-      <c r="O13" s="23" t="s">
+      <c r="O13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="P13" s="28">
+      <c r="P13" s="27">
         <v>0.3</v>
       </c>
       <c r="Q13" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R13" s="70"/>
-      <c r="S13" s="71"/>
-      <c r="T13" s="71"/>
-      <c r="U13" s="71"/>
-      <c r="V13" s="71"/>
-      <c r="W13" s="72"/>
+      <c r="R13" s="75"/>
+      <c r="S13" s="76"/>
+      <c r="T13" s="76"/>
+      <c r="U13" s="76"/>
+      <c r="V13" s="76"/>
+      <c r="W13" s="77"/>
     </row>
     <row r="14" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="73" t="s">
+      <c r="B14" s="98" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="19" t="s">
         <v>13</v>
       </c>
       <c r="D14" s="1">
@@ -1869,7 +1873,7 @@
       <c r="G14">
         <v>0.94030000000000002</v>
       </c>
-      <c r="H14" s="8">
+      <c r="H14" s="7">
         <v>30</v>
       </c>
       <c r="I14" s="1">
@@ -1881,7 +1885,7 @@
       <c r="K14">
         <v>6</v>
       </c>
-      <c r="L14" s="32" t="s">
+      <c r="L14" s="31" t="s">
         <v>35</v>
       </c>
       <c r="M14">
@@ -1890,27 +1894,27 @@
       <c r="N14">
         <v>64</v>
       </c>
-      <c r="O14" s="22" t="s">
+      <c r="O14" s="21" t="s">
         <v>19</v>
       </c>
       <c r="P14">
         <v>0.3</v>
       </c>
-      <c r="Q14" s="8">
+      <c r="Q14" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R14" s="64" t="s">
+      <c r="R14" s="87" t="s">
         <v>37</v>
       </c>
-      <c r="S14" s="65"/>
-      <c r="T14" s="65"/>
-      <c r="U14" s="65"/>
-      <c r="V14" s="65"/>
-      <c r="W14" s="66"/>
+      <c r="S14" s="70"/>
+      <c r="T14" s="70"/>
+      <c r="U14" s="70"/>
+      <c r="V14" s="70"/>
+      <c r="W14" s="71"/>
     </row>
     <row r="15" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="74"/>
-      <c r="C15" s="30" t="s">
+      <c r="B15" s="96"/>
+      <c r="C15" s="29" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="1">
@@ -1925,7 +1929,7 @@
       <c r="G15">
         <v>0.90280000000000005</v>
       </c>
-      <c r="H15" s="8">
+      <c r="H15" s="7">
         <v>87.8</v>
       </c>
       <c r="I15" s="1">
@@ -1937,7 +1941,7 @@
       <c r="K15">
         <v>6</v>
       </c>
-      <c r="L15" s="32" t="s">
+      <c r="L15" s="31" t="s">
         <v>32</v>
       </c>
       <c r="M15">
@@ -1946,25 +1950,25 @@
       <c r="N15">
         <v>64</v>
       </c>
-      <c r="O15" s="22" t="s">
+      <c r="O15" s="21" t="s">
         <v>19</v>
       </c>
       <c r="P15">
         <v>0.3</v>
       </c>
-      <c r="Q15" s="8">
+      <c r="Q15" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R15" s="67"/>
-      <c r="S15" s="68"/>
-      <c r="T15" s="68"/>
-      <c r="U15" s="68"/>
-      <c r="V15" s="68"/>
-      <c r="W15" s="69"/>
+      <c r="R15" s="72"/>
+      <c r="S15" s="73"/>
+      <c r="T15" s="73"/>
+      <c r="U15" s="73"/>
+      <c r="V15" s="73"/>
+      <c r="W15" s="74"/>
     </row>
     <row r="16" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="96"/>
-      <c r="C16" s="31" t="s">
+      <c r="B16" s="97"/>
+      <c r="C16" s="30" t="s">
         <v>14</v>
       </c>
       <c r="D16" s="3">
@@ -1991,7 +1995,7 @@
       <c r="K16" s="3">
         <v>6</v>
       </c>
-      <c r="L16" s="32" t="s">
+      <c r="L16" s="31" t="s">
         <v>32</v>
       </c>
       <c r="M16" s="3">
@@ -2000,7 +2004,7 @@
       <c r="N16" s="3">
         <v>64</v>
       </c>
-      <c r="O16" s="23" t="s">
+      <c r="O16" s="22" t="s">
         <v>19</v>
       </c>
       <c r="P16" s="3">
@@ -2009,19 +2013,19 @@
       <c r="Q16" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R16" s="70"/>
-      <c r="S16" s="71"/>
-      <c r="T16" s="71"/>
-      <c r="U16" s="71"/>
-      <c r="V16" s="71"/>
-      <c r="W16" s="72"/>
+      <c r="R16" s="75"/>
+      <c r="S16" s="76"/>
+      <c r="T16" s="76"/>
+      <c r="U16" s="76"/>
+      <c r="V16" s="76"/>
+      <c r="W16" s="77"/>
     </row>
     <row r="17" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="8"/>
-      <c r="B17" s="99" t="s">
+      <c r="A17" s="7"/>
+      <c r="B17" s="101" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="30" t="s">
+      <c r="C17" s="29" t="s">
         <v>13</v>
       </c>
       <c r="D17">
@@ -2036,49 +2040,49 @@
       <c r="G17">
         <v>0.93659999999999999</v>
       </c>
-      <c r="H17" s="8">
+      <c r="H17" s="7">
         <v>23.1</v>
       </c>
       <c r="I17" s="1">
         <v>18</v>
       </c>
-      <c r="J17" s="9">
+      <c r="J17" s="8">
         <v>142.66</v>
       </c>
       <c r="K17">
         <v>6</v>
       </c>
-      <c r="L17" s="40" t="s">
+      <c r="L17" s="39" t="s">
         <v>41</v>
       </c>
       <c r="M17">
         <v>64</v>
       </c>
-      <c r="N17" s="25">
-        <v>64</v>
-      </c>
-      <c r="O17" s="33" t="s">
+      <c r="N17" s="24">
+        <v>64</v>
+      </c>
+      <c r="O17" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P17" s="25">
+      <c r="P17" s="24">
         <v>0.2</v>
       </c>
-      <c r="Q17" s="10">
+      <c r="Q17" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R17" s="65" t="s">
+      <c r="R17" s="70" t="s">
         <v>43</v>
       </c>
-      <c r="S17" s="65"/>
-      <c r="T17" s="65"/>
-      <c r="U17" s="65"/>
-      <c r="V17" s="65"/>
-      <c r="W17" s="66"/>
+      <c r="S17" s="70"/>
+      <c r="T17" s="70"/>
+      <c r="U17" s="70"/>
+      <c r="V17" s="70"/>
+      <c r="W17" s="71"/>
     </row>
     <row r="18" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="8"/>
-      <c r="B18" s="103"/>
-      <c r="C18" s="30" t="s">
+      <c r="A18" s="7"/>
+      <c r="B18" s="105"/>
+      <c r="C18" s="29" t="s">
         <v>12</v>
       </c>
       <c r="D18">
@@ -2093,7 +2097,7 @@
       <c r="G18">
         <v>0.80179999999999996</v>
       </c>
-      <c r="H18" s="8">
+      <c r="H18" s="7">
         <v>126.6</v>
       </c>
       <c r="I18" s="1">
@@ -2105,35 +2109,35 @@
       <c r="K18">
         <v>6</v>
       </c>
-      <c r="L18" s="32" t="s">
+      <c r="L18" s="31" t="s">
         <v>42</v>
       </c>
       <c r="M18">
         <v>64</v>
       </c>
-      <c r="N18" s="33" t="s">
+      <c r="N18" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="O18" s="33" t="s">
+      <c r="O18" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="P18" s="25">
+      <c r="P18" s="24">
         <v>0.15</v>
       </c>
-      <c r="Q18" s="8">
+      <c r="Q18" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R18" s="68"/>
-      <c r="S18" s="68"/>
-      <c r="T18" s="68"/>
-      <c r="U18" s="68"/>
-      <c r="V18" s="68"/>
-      <c r="W18" s="69"/>
+      <c r="R18" s="73"/>
+      <c r="S18" s="73"/>
+      <c r="T18" s="73"/>
+      <c r="U18" s="73"/>
+      <c r="V18" s="73"/>
+      <c r="W18" s="74"/>
     </row>
     <row r="19" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="8"/>
-      <c r="B19" s="102"/>
-      <c r="C19" s="31" t="s">
+      <c r="A19" s="7"/>
+      <c r="B19" s="104"/>
+      <c r="C19" s="30" t="s">
         <v>14</v>
       </c>
       <c r="D19" s="3">
@@ -2160,37 +2164,37 @@
       <c r="K19" s="3">
         <v>6</v>
       </c>
-      <c r="L19" s="35" t="s">
+      <c r="L19" s="34" t="s">
         <v>42</v>
       </c>
       <c r="M19" s="3">
         <v>64</v>
       </c>
-      <c r="N19" s="34" t="s">
+      <c r="N19" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="O19" s="34" t="s">
+      <c r="O19" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="P19" s="28">
+      <c r="P19" s="27">
         <v>0.15</v>
       </c>
       <c r="Q19" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R19" s="71"/>
-      <c r="S19" s="71"/>
-      <c r="T19" s="71"/>
-      <c r="U19" s="71"/>
-      <c r="V19" s="71"/>
-      <c r="W19" s="72"/>
+      <c r="R19" s="76"/>
+      <c r="S19" s="76"/>
+      <c r="T19" s="76"/>
+      <c r="U19" s="76"/>
+      <c r="V19" s="76"/>
+      <c r="W19" s="77"/>
     </row>
     <row r="20" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="8"/>
-      <c r="B20" s="73" t="s">
+      <c r="A20" s="7"/>
+      <c r="B20" s="98" t="s">
         <v>46</v>
       </c>
-      <c r="C20" s="30" t="s">
+      <c r="C20" s="29" t="s">
         <v>13</v>
       </c>
       <c r="D20">
@@ -2205,7 +2209,7 @@
       <c r="G20">
         <v>0.93149999999999999</v>
       </c>
-      <c r="H20" s="8">
+      <c r="H20" s="7">
         <v>23.1</v>
       </c>
       <c r="I20">
@@ -2217,37 +2221,37 @@
       <c r="K20">
         <v>6</v>
       </c>
-      <c r="L20" s="32" t="s">
+      <c r="L20" s="31" t="s">
         <v>47</v>
       </c>
       <c r="M20">
         <v>64</v>
       </c>
-      <c r="N20" s="32">
-        <v>64</v>
-      </c>
-      <c r="O20" s="32" t="s">
+      <c r="N20" s="31">
+        <v>64</v>
+      </c>
+      <c r="O20" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P20" s="25">
+      <c r="P20" s="24">
         <v>0.2</v>
       </c>
-      <c r="Q20" s="36">
+      <c r="Q20" s="35">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R20" s="78" t="s">
+      <c r="R20" s="69" t="s">
         <v>45</v>
       </c>
-      <c r="S20" s="65"/>
-      <c r="T20" s="65"/>
-      <c r="U20" s="65"/>
-      <c r="V20" s="65"/>
-      <c r="W20" s="66"/>
+      <c r="S20" s="70"/>
+      <c r="T20" s="70"/>
+      <c r="U20" s="70"/>
+      <c r="V20" s="70"/>
+      <c r="W20" s="71"/>
     </row>
     <row r="21" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="8"/>
-      <c r="B21" s="74"/>
-      <c r="C21" s="30" t="s">
+      <c r="A21" s="7"/>
+      <c r="B21" s="96"/>
+      <c r="C21" s="29" t="s">
         <v>12</v>
       </c>
       <c r="D21">
@@ -2256,13 +2260,13 @@
       <c r="E21">
         <v>495.26499999999999</v>
       </c>
-      <c r="F21" s="41">
+      <c r="F21" s="40">
         <v>-0.45350000000000001</v>
       </c>
-      <c r="G21" s="41">
+      <c r="G21" s="40">
         <v>-0.4551</v>
       </c>
-      <c r="H21" s="8">
+      <c r="H21" s="7">
         <v>35.4</v>
       </c>
       <c r="I21">
@@ -2274,35 +2278,35 @@
       <c r="K21">
         <v>6</v>
       </c>
-      <c r="L21" s="32" t="s">
+      <c r="L21" s="31" t="s">
         <v>49</v>
       </c>
       <c r="M21">
         <v>64</v>
       </c>
-      <c r="N21" s="33" t="s">
+      <c r="N21" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="O21" s="32" t="s">
+      <c r="O21" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P21" s="25">
+      <c r="P21" s="24">
         <v>0.1</v>
       </c>
-      <c r="Q21" s="37">
+      <c r="Q21" s="36">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R21" s="67"/>
-      <c r="S21" s="68"/>
-      <c r="T21" s="68"/>
-      <c r="U21" s="68"/>
-      <c r="V21" s="68"/>
-      <c r="W21" s="69"/>
+      <c r="R21" s="72"/>
+      <c r="S21" s="73"/>
+      <c r="T21" s="73"/>
+      <c r="U21" s="73"/>
+      <c r="V21" s="73"/>
+      <c r="W21" s="74"/>
     </row>
     <row r="22" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="8"/>
-      <c r="B22" s="96"/>
-      <c r="C22" s="31" t="s">
+      <c r="A22" s="7"/>
+      <c r="B22" s="97"/>
+      <c r="C22" s="30" t="s">
         <v>14</v>
       </c>
       <c r="D22" s="3">
@@ -2329,109 +2333,109 @@
       <c r="K22" s="3">
         <v>6</v>
       </c>
-      <c r="L22" s="35" t="s">
+      <c r="L22" s="34" t="s">
         <v>49</v>
       </c>
       <c r="M22" s="3">
         <v>64</v>
       </c>
-      <c r="N22" s="34" t="s">
+      <c r="N22" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="O22" s="35" t="s">
+      <c r="O22" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="P22" s="28">
+      <c r="P22" s="27">
         <v>0.1</v>
       </c>
-      <c r="Q22" s="38">
+      <c r="Q22" s="37">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R22" s="70"/>
-      <c r="S22" s="71"/>
-      <c r="T22" s="71"/>
-      <c r="U22" s="71"/>
-      <c r="V22" s="71"/>
-      <c r="W22" s="72"/>
+      <c r="R22" s="75"/>
+      <c r="S22" s="76"/>
+      <c r="T22" s="76"/>
+      <c r="U22" s="76"/>
+      <c r="V22" s="76"/>
+      <c r="W22" s="77"/>
     </row>
     <row r="23" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="59"/>
-      <c r="B23" s="75" t="s">
+      <c r="A23" s="58"/>
+      <c r="B23" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="C23" s="20" t="s">
+      <c r="C23" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D23" s="9">
+      <c r="D23" s="8">
         <v>276.649</v>
       </c>
-      <c r="E23" s="39">
+      <c r="E23" s="38">
         <v>495265</v>
       </c>
-      <c r="F23" s="42">
+      <c r="F23" s="41">
         <v>-0.45350000000000001</v>
       </c>
-      <c r="G23" s="42">
+      <c r="G23" s="41">
         <v>-0.4551</v>
       </c>
-      <c r="H23" s="10">
+      <c r="H23" s="9">
         <v>23.1</v>
       </c>
-      <c r="I23" s="9">
+      <c r="I23" s="8">
         <v>18</v>
       </c>
-      <c r="J23" s="9">
+      <c r="J23" s="8">
         <v>219.42</v>
       </c>
-      <c r="K23" s="9">
-        <v>6</v>
-      </c>
-      <c r="L23" s="40" t="s">
+      <c r="K23" s="8">
+        <v>6</v>
+      </c>
+      <c r="L23" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="M23" s="9">
-        <v>64</v>
-      </c>
-      <c r="N23" s="40">
-        <v>64</v>
-      </c>
-      <c r="O23" s="40" t="s">
+      <c r="M23" s="8">
+        <v>64</v>
+      </c>
+      <c r="N23" s="39">
+        <v>64</v>
+      </c>
+      <c r="O23" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="P23" s="9">
+      <c r="P23" s="8">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="10">
+      <c r="Q23" s="9">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R23" s="78" t="s">
+      <c r="R23" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="S23" s="65"/>
-      <c r="T23" s="65"/>
-      <c r="U23" s="65"/>
-      <c r="V23" s="65"/>
-      <c r="W23" s="66"/>
+      <c r="S23" s="70"/>
+      <c r="T23" s="70"/>
+      <c r="U23" s="70"/>
+      <c r="V23" s="70"/>
+      <c r="W23" s="71"/>
     </row>
     <row r="24" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="59"/>
-      <c r="B24" s="76"/>
-      <c r="C24" s="30" t="s">
+      <c r="A24" s="58"/>
+      <c r="B24" s="67"/>
+      <c r="C24" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="52">
+      <c r="D24" s="51">
         <v>51.393000000000001</v>
       </c>
-      <c r="E24" s="52">
+      <c r="E24" s="51">
         <v>110.699</v>
       </c>
-      <c r="F24" s="52">
+      <c r="F24" s="51">
         <v>0.9274</v>
       </c>
-      <c r="G24" s="52">
+      <c r="G24" s="51">
         <v>0.92730000000000001</v>
       </c>
-      <c r="H24" s="53">
+      <c r="H24" s="52">
         <v>35.4</v>
       </c>
       <c r="I24">
@@ -2443,35 +2447,35 @@
       <c r="K24">
         <v>6</v>
       </c>
-      <c r="L24" s="32" t="s">
+      <c r="L24" s="31" t="s">
         <v>52</v>
       </c>
       <c r="M24">
         <v>64</v>
       </c>
-      <c r="N24" s="32" t="s">
+      <c r="N24" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="O24" s="32" t="s">
+      <c r="O24" s="31" t="s">
         <v>39</v>
       </c>
       <c r="P24">
         <v>0.1</v>
       </c>
-      <c r="Q24" s="8">
+      <c r="Q24" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R24" s="67"/>
-      <c r="S24" s="68"/>
-      <c r="T24" s="68"/>
-      <c r="U24" s="68"/>
-      <c r="V24" s="68"/>
-      <c r="W24" s="69"/>
+      <c r="R24" s="72"/>
+      <c r="S24" s="73"/>
+      <c r="T24" s="73"/>
+      <c r="U24" s="73"/>
+      <c r="V24" s="73"/>
+      <c r="W24" s="74"/>
     </row>
     <row r="25" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="59"/>
-      <c r="B25" s="77"/>
-      <c r="C25" s="31" t="s">
+      <c r="A25" s="58"/>
+      <c r="B25" s="68"/>
+      <c r="C25" s="30" t="s">
         <v>14</v>
       </c>
       <c r="D25" s="3">
@@ -2498,16 +2502,16 @@
       <c r="K25" s="3">
         <v>6</v>
       </c>
-      <c r="L25" s="35" t="s">
+      <c r="L25" s="34" t="s">
         <v>49</v>
       </c>
       <c r="M25" s="3">
         <v>64</v>
       </c>
-      <c r="N25" s="35" t="s">
+      <c r="N25" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="O25" s="35" t="s">
+      <c r="O25" s="34" t="s">
         <v>39</v>
       </c>
       <c r="P25" s="3">
@@ -2516,76 +2520,76 @@
       <c r="Q25" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R25" s="70"/>
-      <c r="S25" s="71"/>
-      <c r="T25" s="71"/>
-      <c r="U25" s="71"/>
-      <c r="V25" s="71"/>
-      <c r="W25" s="72"/>
+      <c r="R25" s="75"/>
+      <c r="S25" s="76"/>
+      <c r="T25" s="76"/>
+      <c r="U25" s="76"/>
+      <c r="V25" s="76"/>
+      <c r="W25" s="77"/>
     </row>
     <row r="26" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="59"/>
-      <c r="B26" s="75" t="s">
+      <c r="A26" s="58"/>
+      <c r="B26" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="C26" s="20" t="s">
+      <c r="C26" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D26" s="54">
+      <c r="D26" s="53">
         <v>47.706000000000003</v>
       </c>
-      <c r="E26" s="54">
+      <c r="E26" s="53">
         <v>101.812</v>
       </c>
-      <c r="F26" s="54">
+      <c r="F26" s="53">
         <v>0.93859999999999999</v>
       </c>
-      <c r="G26" s="54">
+      <c r="G26" s="53">
         <v>0.9385</v>
       </c>
-      <c r="H26" s="55">
+      <c r="H26" s="54">
         <v>29.3</v>
       </c>
-      <c r="I26" s="9">
+      <c r="I26" s="8">
         <v>18</v>
       </c>
-      <c r="J26" s="9">
+      <c r="J26" s="8">
         <v>360.29</v>
       </c>
-      <c r="K26" s="9">
-        <v>6</v>
-      </c>
-      <c r="L26" s="40" t="s">
+      <c r="K26" s="8">
+        <v>6</v>
+      </c>
+      <c r="L26" s="39" t="s">
         <v>56</v>
       </c>
-      <c r="M26" s="9">
-        <v>64</v>
-      </c>
-      <c r="N26" s="9">
-        <v>64</v>
-      </c>
-      <c r="O26" s="44" t="s">
+      <c r="M26" s="8">
+        <v>64</v>
+      </c>
+      <c r="N26" s="8">
+        <v>64</v>
+      </c>
+      <c r="O26" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="P26" s="9">
+      <c r="P26" s="8">
         <v>0.2</v>
       </c>
-      <c r="Q26" s="36">
+      <c r="Q26" s="35">
         <v>1E-3</v>
       </c>
-      <c r="R26" s="64" t="s">
+      <c r="R26" s="87" t="s">
         <v>57</v>
       </c>
-      <c r="S26" s="65"/>
-      <c r="T26" s="65"/>
-      <c r="U26" s="65"/>
-      <c r="V26" s="65"/>
-      <c r="W26" s="66"/>
+      <c r="S26" s="70"/>
+      <c r="T26" s="70"/>
+      <c r="U26" s="70"/>
+      <c r="V26" s="70"/>
+      <c r="W26" s="71"/>
     </row>
     <row r="27" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="59"/>
-      <c r="B27" s="76"/>
-      <c r="C27" s="30" t="s">
+      <c r="A27" s="58"/>
+      <c r="B27" s="67"/>
+      <c r="C27" s="29" t="s">
         <v>12</v>
       </c>
       <c r="D27">
@@ -2594,13 +2598,13 @@
       <c r="E27">
         <v>495.26499999999999</v>
       </c>
-      <c r="F27" s="41">
+      <c r="F27" s="40">
         <v>-0.45350000000000001</v>
       </c>
-      <c r="G27" s="41">
+      <c r="G27" s="40">
         <v>-0.4551</v>
       </c>
-      <c r="H27" s="8">
+      <c r="H27" s="7">
         <v>126.6</v>
       </c>
       <c r="I27">
@@ -2612,35 +2616,35 @@
       <c r="K27">
         <v>6</v>
       </c>
-      <c r="L27" s="32" t="s">
+      <c r="L27" s="31" t="s">
         <v>49</v>
       </c>
       <c r="M27">
         <v>64</v>
       </c>
-      <c r="N27" s="33" t="s">
+      <c r="N27" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="O27" s="32" t="s">
+      <c r="O27" s="31" t="s">
         <v>39</v>
       </c>
       <c r="P27">
         <v>0.1</v>
       </c>
-      <c r="Q27" s="37">
+      <c r="Q27" s="36">
         <v>1E-3</v>
       </c>
-      <c r="R27" s="67"/>
-      <c r="S27" s="68"/>
-      <c r="T27" s="68"/>
-      <c r="U27" s="68"/>
-      <c r="V27" s="68"/>
-      <c r="W27" s="69"/>
+      <c r="R27" s="72"/>
+      <c r="S27" s="73"/>
+      <c r="T27" s="73"/>
+      <c r="U27" s="73"/>
+      <c r="V27" s="73"/>
+      <c r="W27" s="74"/>
     </row>
     <row r="28" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="59"/>
-      <c r="B28" s="77"/>
-      <c r="C28" s="31" t="s">
+      <c r="A28" s="58"/>
+      <c r="B28" s="68"/>
+      <c r="C28" s="30" t="s">
         <v>14</v>
       </c>
       <c r="D28" s="3">
@@ -2667,94 +2671,94 @@
       <c r="K28" s="3">
         <v>6</v>
       </c>
-      <c r="L28" s="35" t="s">
+      <c r="L28" s="34" t="s">
         <v>49</v>
       </c>
       <c r="M28" s="3">
         <v>64</v>
       </c>
-      <c r="N28" s="34" t="s">
+      <c r="N28" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="O28" s="35" t="s">
+      <c r="O28" s="34" t="s">
         <v>39</v>
       </c>
       <c r="P28" s="3">
         <v>0.1</v>
       </c>
-      <c r="Q28" s="38">
+      <c r="Q28" s="37">
         <v>1E-3</v>
       </c>
-      <c r="R28" s="70"/>
-      <c r="S28" s="71"/>
-      <c r="T28" s="71"/>
-      <c r="U28" s="71"/>
-      <c r="V28" s="71"/>
-      <c r="W28" s="72"/>
+      <c r="R28" s="75"/>
+      <c r="S28" s="76"/>
+      <c r="T28" s="76"/>
+      <c r="U28" s="76"/>
+      <c r="V28" s="76"/>
+      <c r="W28" s="77"/>
     </row>
     <row r="29" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="60"/>
-      <c r="B29" s="75" t="s">
+      <c r="A29" s="59"/>
+      <c r="B29" s="66" t="s">
         <v>34</v>
       </c>
-      <c r="C29" s="29" t="s">
+      <c r="C29" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="D29" s="54">
+      <c r="D29" s="53">
         <v>49.481000000000002</v>
       </c>
-      <c r="E29" s="54">
+      <c r="E29" s="53">
         <v>104.151</v>
       </c>
-      <c r="F29" s="54">
+      <c r="F29" s="53">
         <v>0.93569999999999998</v>
       </c>
-      <c r="G29" s="54">
+      <c r="G29" s="53">
         <v>0.93569999999999998</v>
       </c>
-      <c r="H29" s="55">
+      <c r="H29" s="54">
         <v>23.1</v>
       </c>
-      <c r="I29" s="9">
+      <c r="I29" s="8">
         <v>18</v>
       </c>
-      <c r="J29" s="9">
+      <c r="J29" s="8">
         <v>222.14</v>
       </c>
-      <c r="K29" s="9">
-        <v>6</v>
-      </c>
-      <c r="L29" s="40" t="s">
+      <c r="K29" s="8">
+        <v>6</v>
+      </c>
+      <c r="L29" s="39" t="s">
         <v>59</v>
       </c>
-      <c r="M29" s="9">
-        <v>64</v>
-      </c>
-      <c r="N29" s="9">
-        <v>64</v>
-      </c>
-      <c r="O29" s="44" t="s">
+      <c r="M29" s="8">
+        <v>64</v>
+      </c>
+      <c r="N29" s="8">
+        <v>64</v>
+      </c>
+      <c r="O29" s="43" t="s">
         <v>39</v>
       </c>
-      <c r="P29" s="9">
+      <c r="P29" s="8">
         <v>0.2</v>
       </c>
-      <c r="Q29" s="10">
+      <c r="Q29" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R29" s="78" t="s">
+      <c r="R29" s="69" t="s">
         <v>60</v>
       </c>
-      <c r="S29" s="65"/>
-      <c r="T29" s="65"/>
-      <c r="U29" s="65"/>
-      <c r="V29" s="65"/>
-      <c r="W29" s="66"/>
+      <c r="S29" s="70"/>
+      <c r="T29" s="70"/>
+      <c r="U29" s="70"/>
+      <c r="V29" s="70"/>
+      <c r="W29" s="71"/>
     </row>
     <row r="30" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="59"/>
-      <c r="B30" s="76"/>
-      <c r="C30" s="26" t="s">
+      <c r="A30" s="58"/>
+      <c r="B30" s="67"/>
+      <c r="C30" s="25" t="s">
         <v>12</v>
       </c>
       <c r="D30">
@@ -2769,7 +2773,7 @@
       <c r="G30">
         <v>0.87609999999999999</v>
       </c>
-      <c r="H30" s="8">
+      <c r="H30" s="7">
         <v>35.4</v>
       </c>
       <c r="I30">
@@ -2781,35 +2785,35 @@
       <c r="K30">
         <v>6</v>
       </c>
-      <c r="L30" s="32" t="s">
+      <c r="L30" s="31" t="s">
         <v>49</v>
       </c>
       <c r="M30">
         <v>64</v>
       </c>
-      <c r="N30" s="33" t="s">
+      <c r="N30" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="O30" s="32" t="s">
+      <c r="O30" s="31" t="s">
         <v>39</v>
       </c>
       <c r="P30">
         <v>0.1</v>
       </c>
-      <c r="Q30" s="8">
+      <c r="Q30" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R30" s="67"/>
-      <c r="S30" s="68"/>
-      <c r="T30" s="68"/>
-      <c r="U30" s="68"/>
-      <c r="V30" s="68"/>
-      <c r="W30" s="69"/>
+      <c r="R30" s="72"/>
+      <c r="S30" s="73"/>
+      <c r="T30" s="73"/>
+      <c r="U30" s="73"/>
+      <c r="V30" s="73"/>
+      <c r="W30" s="74"/>
     </row>
     <row r="31" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="59"/>
-      <c r="B31" s="77"/>
-      <c r="C31" s="43" t="s">
+      <c r="A31" s="58"/>
+      <c r="B31" s="68"/>
+      <c r="C31" s="42" t="s">
         <v>14</v>
       </c>
       <c r="D31" s="3">
@@ -2836,16 +2840,16 @@
       <c r="K31" s="3">
         <v>6</v>
       </c>
-      <c r="L31" s="35" t="s">
+      <c r="L31" s="34" t="s">
         <v>49</v>
       </c>
       <c r="M31" s="3">
         <v>64</v>
       </c>
-      <c r="N31" s="34" t="s">
+      <c r="N31" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="O31" s="35" t="s">
+      <c r="O31" s="34" t="s">
         <v>39</v>
       </c>
       <c r="P31" s="3">
@@ -2854,76 +2858,76 @@
       <c r="Q31" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R31" s="70"/>
-      <c r="S31" s="71"/>
-      <c r="T31" s="71"/>
-      <c r="U31" s="71"/>
-      <c r="V31" s="71"/>
-      <c r="W31" s="72"/>
+      <c r="R31" s="75"/>
+      <c r="S31" s="76"/>
+      <c r="T31" s="76"/>
+      <c r="U31" s="76"/>
+      <c r="V31" s="76"/>
+      <c r="W31" s="77"/>
     </row>
     <row r="32" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="60"/>
-      <c r="B32" s="75" t="s">
+      <c r="A32" s="59"/>
+      <c r="B32" s="66" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="29" t="s">
+      <c r="C32" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="D32" s="54">
+      <c r="D32" s="53">
         <v>46.76</v>
       </c>
-      <c r="E32" s="54">
+      <c r="E32" s="53">
         <v>95.427999999999997</v>
       </c>
-      <c r="F32" s="54">
+      <c r="F32" s="53">
         <v>0.94679999999999997</v>
       </c>
-      <c r="G32" s="54">
+      <c r="G32" s="53">
         <v>0.94669999999999999</v>
       </c>
-      <c r="H32" s="55">
+      <c r="H32" s="54">
         <v>23.1</v>
       </c>
-      <c r="I32" s="45">
+      <c r="I32" s="44">
         <v>30</v>
       </c>
-      <c r="J32" s="9">
+      <c r="J32" s="8">
         <v>260.20999999999998</v>
       </c>
-      <c r="K32" s="9">
-        <v>6</v>
-      </c>
-      <c r="L32" s="40" t="s">
+      <c r="K32" s="8">
+        <v>6</v>
+      </c>
+      <c r="L32" s="39" t="s">
         <v>59</v>
       </c>
-      <c r="M32" s="9">
-        <v>64</v>
-      </c>
-      <c r="N32" s="9">
-        <v>64</v>
-      </c>
-      <c r="O32" s="40" t="s">
+      <c r="M32" s="8">
+        <v>64</v>
+      </c>
+      <c r="N32" s="8">
+        <v>64</v>
+      </c>
+      <c r="O32" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="P32" s="9">
+      <c r="P32" s="8">
         <v>0.2</v>
       </c>
-      <c r="Q32" s="10">
+      <c r="Q32" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R32" s="64" t="s">
+      <c r="R32" s="87" t="s">
         <v>61</v>
       </c>
-      <c r="S32" s="65"/>
-      <c r="T32" s="65"/>
-      <c r="U32" s="65"/>
-      <c r="V32" s="65"/>
-      <c r="W32" s="66"/>
+      <c r="S32" s="70"/>
+      <c r="T32" s="70"/>
+      <c r="U32" s="70"/>
+      <c r="V32" s="70"/>
+      <c r="W32" s="71"/>
     </row>
     <row r="33" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="60"/>
-      <c r="B33" s="76"/>
-      <c r="C33" s="26" t="s">
+      <c r="A33" s="59"/>
+      <c r="B33" s="67"/>
+      <c r="C33" s="25" t="s">
         <v>12</v>
       </c>
       <c r="D33">
@@ -2938,10 +2942,10 @@
       <c r="G33">
         <v>0.69969999999999999</v>
       </c>
-      <c r="H33" s="8">
+      <c r="H33" s="7">
         <v>35.4</v>
       </c>
-      <c r="I33" s="46">
+      <c r="I33" s="45">
         <v>30</v>
       </c>
       <c r="J33">
@@ -2950,35 +2954,35 @@
       <c r="K33">
         <v>6</v>
       </c>
-      <c r="L33" s="32" t="s">
+      <c r="L33" s="31" t="s">
         <v>49</v>
       </c>
       <c r="M33">
         <v>64</v>
       </c>
-      <c r="N33" s="32" t="s">
+      <c r="N33" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="O33" s="32" t="s">
+      <c r="O33" s="31" t="s">
         <v>39</v>
       </c>
       <c r="P33">
         <v>0.1</v>
       </c>
-      <c r="Q33" s="8">
+      <c r="Q33" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R33" s="67"/>
-      <c r="S33" s="68"/>
-      <c r="T33" s="68"/>
-      <c r="U33" s="68"/>
-      <c r="V33" s="68"/>
-      <c r="W33" s="69"/>
+      <c r="R33" s="72"/>
+      <c r="S33" s="73"/>
+      <c r="T33" s="73"/>
+      <c r="U33" s="73"/>
+      <c r="V33" s="73"/>
+      <c r="W33" s="74"/>
     </row>
     <row r="34" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="60"/>
-      <c r="B34" s="77"/>
-      <c r="C34" s="43" t="s">
+      <c r="A34" s="59"/>
+      <c r="B34" s="68"/>
+      <c r="C34" s="42" t="s">
         <v>14</v>
       </c>
       <c r="D34" s="3">
@@ -2996,7 +3000,7 @@
       <c r="H34" s="4">
         <v>27.4</v>
       </c>
-      <c r="I34" s="47">
+      <c r="I34" s="46">
         <v>30</v>
       </c>
       <c r="J34" s="3">
@@ -3005,16 +3009,16 @@
       <c r="K34" s="3">
         <v>6</v>
       </c>
-      <c r="L34" s="35" t="s">
+      <c r="L34" s="34" t="s">
         <v>49</v>
       </c>
       <c r="M34" s="3">
         <v>64</v>
       </c>
-      <c r="N34" s="35" t="s">
+      <c r="N34" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="O34" s="35" t="s">
+      <c r="O34" s="34" t="s">
         <v>39</v>
       </c>
       <c r="P34" s="3">
@@ -3023,37 +3027,37 @@
       <c r="Q34" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R34" s="70"/>
-      <c r="S34" s="71"/>
-      <c r="T34" s="71"/>
-      <c r="U34" s="71"/>
-      <c r="V34" s="71"/>
-      <c r="W34" s="72"/>
+      <c r="R34" s="75"/>
+      <c r="S34" s="76"/>
+      <c r="T34" s="76"/>
+      <c r="U34" s="76"/>
+      <c r="V34" s="76"/>
+      <c r="W34" s="77"/>
     </row>
     <row r="35" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="59"/>
-      <c r="B35" s="75" t="s">
+      <c r="A35" s="58"/>
+      <c r="B35" s="66" t="s">
         <v>44</v>
       </c>
-      <c r="C35" s="26" t="s">
+      <c r="C35" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="D35" s="56">
+      <c r="D35" s="55">
         <v>48.41</v>
       </c>
-      <c r="E35" s="54">
+      <c r="E35" s="53">
         <v>101.381</v>
       </c>
-      <c r="F35" s="54">
+      <c r="F35" s="53">
         <v>0.93989999999999996</v>
       </c>
-      <c r="G35" s="54">
+      <c r="G35" s="53">
         <v>0.93979999999999997</v>
       </c>
-      <c r="H35" s="55">
+      <c r="H35" s="54">
         <v>22.9</v>
       </c>
-      <c r="I35" s="46">
+      <c r="I35" s="45">
         <v>9</v>
       </c>
       <c r="J35">
@@ -3062,7 +3066,7 @@
       <c r="K35">
         <v>6</v>
       </c>
-      <c r="L35" s="32" t="s">
+      <c r="L35" s="31" t="s">
         <v>62</v>
       </c>
       <c r="M35">
@@ -3071,28 +3075,28 @@
       <c r="N35">
         <v>64</v>
       </c>
-      <c r="O35" s="32" t="s">
+      <c r="O35" s="31" t="s">
         <v>39</v>
       </c>
       <c r="P35">
         <v>0.2</v>
       </c>
-      <c r="Q35" s="8">
+      <c r="Q35" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R35" s="78" t="s">
+      <c r="R35" s="69" t="s">
         <v>63</v>
       </c>
-      <c r="S35" s="65"/>
-      <c r="T35" s="65"/>
-      <c r="U35" s="65"/>
-      <c r="V35" s="65"/>
-      <c r="W35" s="66"/>
+      <c r="S35" s="70"/>
+      <c r="T35" s="70"/>
+      <c r="U35" s="70"/>
+      <c r="V35" s="70"/>
+      <c r="W35" s="71"/>
     </row>
     <row r="36" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="59"/>
-      <c r="B36" s="76"/>
-      <c r="C36" s="26" t="s">
+      <c r="A36" s="58"/>
+      <c r="B36" s="67"/>
+      <c r="C36" s="25" t="s">
         <v>12</v>
       </c>
       <c r="D36" s="1">
@@ -3107,10 +3111,10 @@
       <c r="G36">
         <v>0.86439999999999995</v>
       </c>
-      <c r="H36" s="8">
+      <c r="H36" s="7">
         <v>23.6</v>
       </c>
-      <c r="I36" s="46">
+      <c r="I36" s="45">
         <v>9</v>
       </c>
       <c r="J36">
@@ -3119,35 +3123,35 @@
       <c r="K36">
         <v>6</v>
       </c>
-      <c r="L36" s="32" t="s">
+      <c r="L36" s="31" t="s">
         <v>49</v>
       </c>
       <c r="M36">
         <v>64</v>
       </c>
-      <c r="N36" s="25">
+      <c r="N36" s="24">
         <v>32</v>
       </c>
-      <c r="O36" s="32" t="s">
+      <c r="O36" s="31" t="s">
         <v>39</v>
       </c>
       <c r="P36">
         <v>0.1</v>
       </c>
-      <c r="Q36" s="37">
+      <c r="Q36" s="36">
         <v>1E-3</v>
       </c>
-      <c r="R36" s="67"/>
-      <c r="S36" s="68"/>
-      <c r="T36" s="68"/>
-      <c r="U36" s="68"/>
-      <c r="V36" s="68"/>
-      <c r="W36" s="69"/>
+      <c r="R36" s="72"/>
+      <c r="S36" s="73"/>
+      <c r="T36" s="73"/>
+      <c r="U36" s="73"/>
+      <c r="V36" s="73"/>
+      <c r="W36" s="74"/>
     </row>
     <row r="37" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="59"/>
-      <c r="B37" s="77"/>
-      <c r="C37" s="31" t="s">
+      <c r="A37" s="58"/>
+      <c r="B37" s="68"/>
+      <c r="C37" s="30" t="s">
         <v>14</v>
       </c>
       <c r="D37" s="2">
@@ -3156,16 +3160,16 @@
       <c r="E37" s="3">
         <v>498.125</v>
       </c>
-      <c r="F37" s="49">
+      <c r="F37" s="48">
         <v>-0.45140000000000002</v>
       </c>
-      <c r="G37" s="49">
+      <c r="G37" s="48">
         <v>-0.45279999999999998</v>
       </c>
       <c r="H37" s="4">
         <v>27</v>
       </c>
-      <c r="I37" s="48">
+      <c r="I37" s="47">
         <v>9</v>
       </c>
       <c r="J37" s="3">
@@ -3174,16 +3178,16 @@
       <c r="K37" s="3">
         <v>6</v>
       </c>
-      <c r="L37" s="35" t="s">
+      <c r="L37" s="34" t="s">
         <v>49</v>
       </c>
       <c r="M37" s="3">
         <v>64</v>
       </c>
-      <c r="N37" s="35" t="s">
+      <c r="N37" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="O37" s="35" t="s">
+      <c r="O37" s="34" t="s">
         <v>39</v>
       </c>
       <c r="P37" s="3">
@@ -3192,74 +3196,74 @@
       <c r="Q37" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R37" s="70"/>
-      <c r="S37" s="71"/>
-      <c r="T37" s="71"/>
-      <c r="U37" s="71"/>
-      <c r="V37" s="71"/>
-      <c r="W37" s="72"/>
+      <c r="R37" s="75"/>
+      <c r="S37" s="76"/>
+      <c r="T37" s="76"/>
+      <c r="U37" s="76"/>
+      <c r="V37" s="76"/>
+      <c r="W37" s="77"/>
     </row>
     <row r="38" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="60"/>
-      <c r="B38" s="75" t="s">
+      <c r="A38" s="59"/>
+      <c r="B38" s="66" t="s">
         <v>46</v>
       </c>
-      <c r="C38" s="20" t="s">
+      <c r="C38" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D38" s="56">
+      <c r="D38" s="55">
         <v>42.213999999999999</v>
       </c>
-      <c r="E38" s="54">
+      <c r="E38" s="53">
         <v>92.585999999999999</v>
       </c>
-      <c r="F38" s="54">
+      <c r="F38" s="53">
         <v>0.94740000000000002</v>
       </c>
-      <c r="G38" s="54">
+      <c r="G38" s="53">
         <v>0.94730000000000003</v>
       </c>
-      <c r="H38" s="55">
+      <c r="H38" s="54">
         <v>22.9</v>
       </c>
-      <c r="I38" s="51">
+      <c r="I38" s="50">
         <v>240</v>
       </c>
-      <c r="J38" s="9">
+      <c r="J38" s="8">
         <v>729.62</v>
       </c>
-      <c r="K38" s="9">
-        <v>6</v>
-      </c>
-      <c r="L38" s="40" t="s">
-        <v>64</v>
-      </c>
-      <c r="M38" s="9">
-        <v>64</v>
-      </c>
-      <c r="N38" s="9">
-        <v>64</v>
-      </c>
-      <c r="O38" s="40" t="s">
+      <c r="K38" s="8">
+        <v>6</v>
+      </c>
+      <c r="L38" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="M38" s="8">
+        <v>64</v>
+      </c>
+      <c r="N38" s="8">
+        <v>64</v>
+      </c>
+      <c r="O38" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="P38" s="9">
+      <c r="P38" s="8">
         <v>0.2</v>
       </c>
-      <c r="Q38" s="10">
+      <c r="Q38" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R38" s="79"/>
-      <c r="S38" s="80"/>
-      <c r="T38" s="80"/>
-      <c r="U38" s="80"/>
-      <c r="V38" s="80"/>
-      <c r="W38" s="81"/>
+      <c r="R38" s="78"/>
+      <c r="S38" s="79"/>
+      <c r="T38" s="79"/>
+      <c r="U38" s="79"/>
+      <c r="V38" s="79"/>
+      <c r="W38" s="80"/>
     </row>
     <row r="39" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="60"/>
-      <c r="B39" s="76"/>
-      <c r="C39" s="30" t="s">
+      <c r="A39" s="59"/>
+      <c r="B39" s="67"/>
+      <c r="C39" s="29" t="s">
         <v>12</v>
       </c>
       <c r="D39" s="1">
@@ -3274,10 +3278,10 @@
       <c r="G39">
         <v>0.94210000000000005</v>
       </c>
-      <c r="H39" s="8">
+      <c r="H39" s="7">
         <v>23.6</v>
       </c>
-      <c r="I39" s="50">
+      <c r="I39" s="49">
         <v>240</v>
       </c>
       <c r="J39">
@@ -3286,7 +3290,7 @@
       <c r="K39">
         <v>6</v>
       </c>
-      <c r="L39" s="32" t="s">
+      <c r="L39" s="31" t="s">
         <v>65</v>
       </c>
       <c r="M39">
@@ -3295,26 +3299,26 @@
       <c r="N39">
         <v>32</v>
       </c>
-      <c r="O39" s="32" t="s">
+      <c r="O39" s="31" t="s">
         <v>39</v>
       </c>
       <c r="P39">
         <v>0.1</v>
       </c>
-      <c r="Q39" s="8">
+      <c r="Q39" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R39" s="82"/>
-      <c r="S39" s="83"/>
-      <c r="T39" s="83"/>
-      <c r="U39" s="83"/>
-      <c r="V39" s="83"/>
-      <c r="W39" s="84"/>
+      <c r="R39" s="81"/>
+      <c r="S39" s="82"/>
+      <c r="T39" s="82"/>
+      <c r="U39" s="82"/>
+      <c r="V39" s="82"/>
+      <c r="W39" s="83"/>
     </row>
     <row r="40" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="60"/>
-      <c r="B40" s="77"/>
-      <c r="C40" s="31" t="s">
+      <c r="A40" s="59"/>
+      <c r="B40" s="68"/>
+      <c r="C40" s="30" t="s">
         <v>14</v>
       </c>
       <c r="D40" s="2">
@@ -3332,7 +3336,7 @@
       <c r="H40" s="4">
         <v>27</v>
       </c>
-      <c r="I40" s="48">
+      <c r="I40" s="47">
         <v>240</v>
       </c>
       <c r="J40" s="3">
@@ -3341,16 +3345,16 @@
       <c r="K40" s="3">
         <v>6</v>
       </c>
-      <c r="L40" s="35" t="s">
+      <c r="L40" s="34" t="s">
         <v>66</v>
       </c>
       <c r="M40" s="3">
         <v>64</v>
       </c>
-      <c r="N40" s="35" t="s">
+      <c r="N40" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="O40" s="35" t="s">
+      <c r="O40" s="34" t="s">
         <v>39</v>
       </c>
       <c r="P40" s="3">
@@ -3359,94 +3363,94 @@
       <c r="Q40" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R40" s="85"/>
-      <c r="S40" s="86"/>
-      <c r="T40" s="86"/>
-      <c r="U40" s="86"/>
-      <c r="V40" s="86"/>
-      <c r="W40" s="87"/>
+      <c r="R40" s="84"/>
+      <c r="S40" s="85"/>
+      <c r="T40" s="85"/>
+      <c r="U40" s="85"/>
+      <c r="V40" s="85"/>
+      <c r="W40" s="86"/>
     </row>
     <row r="41" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="60"/>
-      <c r="B41" s="75" t="s">
+      <c r="A41" s="59"/>
+      <c r="B41" s="66" t="s">
         <v>50</v>
       </c>
-      <c r="C41" s="30" t="s">
+      <c r="C41" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="D41" s="57">
+      <c r="D41" s="56">
         <v>48614</v>
       </c>
-      <c r="E41" s="9">
+      <c r="E41" s="8">
         <v>99.918999999999997</v>
       </c>
-      <c r="F41" s="9">
+      <c r="F41" s="8">
         <v>0.94159999999999999</v>
       </c>
-      <c r="G41" s="9">
+      <c r="G41" s="8">
         <v>0.94159999999999999</v>
       </c>
-      <c r="H41" s="10">
+      <c r="H41" s="9">
         <v>22.9</v>
       </c>
-      <c r="I41" s="51">
+      <c r="I41" s="50">
         <v>21</v>
       </c>
-      <c r="J41" s="9">
+      <c r="J41" s="8">
         <v>232.8</v>
       </c>
-      <c r="K41" s="9">
-        <v>6</v>
-      </c>
-      <c r="L41" s="40" t="s">
+      <c r="K41" s="8">
+        <v>6</v>
+      </c>
+      <c r="L41" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="M41" s="9">
-        <v>64</v>
-      </c>
-      <c r="N41" s="9">
-        <v>64</v>
-      </c>
-      <c r="O41" s="40" t="s">
+      <c r="M41" s="8">
+        <v>64</v>
+      </c>
+      <c r="N41" s="8">
+        <v>64</v>
+      </c>
+      <c r="O41" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="P41" s="9">
+      <c r="P41" s="8">
         <v>0.2</v>
       </c>
-      <c r="Q41" s="10">
+      <c r="Q41" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R41" s="64" t="s">
+      <c r="R41" s="87" t="s">
         <v>71</v>
       </c>
-      <c r="S41" s="65"/>
-      <c r="T41" s="65"/>
-      <c r="U41" s="65"/>
-      <c r="V41" s="65"/>
-      <c r="W41" s="66"/>
+      <c r="S41" s="70"/>
+      <c r="T41" s="70"/>
+      <c r="U41" s="70"/>
+      <c r="V41" s="70"/>
+      <c r="W41" s="71"/>
     </row>
     <row r="42" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="60"/>
-      <c r="B42" s="76"/>
-      <c r="C42" s="30" t="s">
+      <c r="A42" s="59"/>
+      <c r="B42" s="67"/>
+      <c r="C42" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="D42" s="58">
+      <c r="D42" s="57">
         <v>45.213999999999999</v>
       </c>
-      <c r="E42" s="52">
+      <c r="E42" s="51">
         <v>93.855999999999995</v>
       </c>
-      <c r="F42" s="52">
+      <c r="F42" s="51">
         <v>0.94850000000000001</v>
       </c>
-      <c r="G42" s="52">
+      <c r="G42" s="51">
         <v>0.94850000000000001</v>
       </c>
-      <c r="H42" s="53">
+      <c r="H42" s="52">
         <v>23.6</v>
       </c>
-      <c r="I42" s="50">
+      <c r="I42" s="49">
         <v>21</v>
       </c>
       <c r="J42">
@@ -3455,7 +3459,7 @@
       <c r="K42">
         <v>6</v>
       </c>
-      <c r="L42" s="32" t="s">
+      <c r="L42" s="31" t="s">
         <v>69</v>
       </c>
       <c r="M42">
@@ -3464,26 +3468,26 @@
       <c r="N42">
         <v>32</v>
       </c>
-      <c r="O42" s="32" t="s">
+      <c r="O42" s="31" t="s">
         <v>39</v>
       </c>
       <c r="P42">
         <v>0.1</v>
       </c>
-      <c r="Q42" s="8">
+      <c r="Q42" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R42" s="67"/>
-      <c r="S42" s="68"/>
-      <c r="T42" s="68"/>
-      <c r="U42" s="68"/>
-      <c r="V42" s="68"/>
-      <c r="W42" s="69"/>
+      <c r="R42" s="72"/>
+      <c r="S42" s="73"/>
+      <c r="T42" s="73"/>
+      <c r="U42" s="73"/>
+      <c r="V42" s="73"/>
+      <c r="W42" s="74"/>
     </row>
     <row r="43" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="60"/>
-      <c r="B43" s="76"/>
-      <c r="C43" s="30" t="s">
+      <c r="A43" s="59"/>
+      <c r="B43" s="67"/>
+      <c r="C43" s="29" t="s">
         <v>14</v>
       </c>
       <c r="D43" s="1">
@@ -3498,10 +3502,10 @@
       <c r="G43">
         <v>0.89710000000000001</v>
       </c>
-      <c r="H43" s="8">
+      <c r="H43" s="7">
         <v>27</v>
       </c>
-      <c r="I43" s="50">
+      <c r="I43" s="49">
         <v>21</v>
       </c>
       <c r="J43">
@@ -3510,35 +3514,35 @@
       <c r="K43">
         <v>6</v>
       </c>
-      <c r="L43" s="32" t="s">
+      <c r="L43" s="31" t="s">
         <v>49</v>
       </c>
       <c r="M43">
         <v>64</v>
       </c>
-      <c r="N43" s="32" t="s">
+      <c r="N43" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="O43" s="32" t="s">
+      <c r="O43" s="31" t="s">
         <v>39</v>
       </c>
       <c r="P43">
         <v>0.1</v>
       </c>
-      <c r="Q43" s="8">
+      <c r="Q43" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R43" s="67"/>
-      <c r="S43" s="68"/>
-      <c r="T43" s="68"/>
-      <c r="U43" s="68"/>
-      <c r="V43" s="68"/>
-      <c r="W43" s="69"/>
+      <c r="R43" s="72"/>
+      <c r="S43" s="73"/>
+      <c r="T43" s="73"/>
+      <c r="U43" s="73"/>
+      <c r="V43" s="73"/>
+      <c r="W43" s="74"/>
     </row>
     <row r="44" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="60"/>
-      <c r="B44" s="77"/>
-      <c r="C44" s="31" t="s">
+      <c r="A44" s="59"/>
+      <c r="B44" s="68"/>
+      <c r="C44" s="30" t="s">
         <v>67</v>
       </c>
       <c r="D44" s="2">
@@ -3556,7 +3560,7 @@
       <c r="H44" s="4">
         <v>22</v>
       </c>
-      <c r="I44" s="48">
+      <c r="I44" s="47">
         <v>21</v>
       </c>
       <c r="J44" s="3">
@@ -3565,7 +3569,7 @@
       <c r="K44" s="3">
         <v>6</v>
       </c>
-      <c r="L44" s="35" t="s">
+      <c r="L44" s="34" t="s">
         <v>49</v>
       </c>
       <c r="M44" s="3">
@@ -3574,7 +3578,7 @@
       <c r="N44" s="3">
         <v>32</v>
       </c>
-      <c r="O44" s="35" t="s">
+      <c r="O44" s="34" t="s">
         <v>39</v>
       </c>
       <c r="P44" s="3" t="s">
@@ -3583,94 +3587,94 @@
       <c r="Q44" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R44" s="70"/>
-      <c r="S44" s="71"/>
-      <c r="T44" s="71"/>
-      <c r="U44" s="71"/>
-      <c r="V44" s="71"/>
-      <c r="W44" s="72"/>
+      <c r="R44" s="75"/>
+      <c r="S44" s="76"/>
+      <c r="T44" s="76"/>
+      <c r="U44" s="76"/>
+      <c r="V44" s="76"/>
+      <c r="W44" s="77"/>
     </row>
     <row r="45" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="60"/>
-      <c r="B45" s="75" t="s">
+      <c r="A45" s="59"/>
+      <c r="B45" s="66" t="s">
         <v>55</v>
       </c>
-      <c r="C45" s="30" t="s">
+      <c r="C45" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="D45" s="58">
+      <c r="D45" s="57">
         <v>47.497999999999998</v>
       </c>
-      <c r="E45" s="52">
+      <c r="E45" s="51">
         <v>98.091999999999999</v>
       </c>
-      <c r="F45" s="52">
+      <c r="F45" s="51">
         <v>0.94379999999999997</v>
       </c>
-      <c r="G45" s="52">
+      <c r="G45" s="51">
         <v>0.94369999999999998</v>
       </c>
-      <c r="H45" s="53">
+      <c r="H45" s="52">
         <v>22.9</v>
       </c>
-      <c r="I45" s="50">
+      <c r="I45" s="49">
         <v>30</v>
       </c>
       <c r="J45">
         <v>367.69</v>
       </c>
-      <c r="K45" s="9">
-        <v>6</v>
-      </c>
-      <c r="L45" s="32" t="s">
+      <c r="K45" s="8">
+        <v>6</v>
+      </c>
+      <c r="L45" s="31" t="s">
         <v>73</v>
       </c>
-      <c r="M45" s="9">
-        <v>64</v>
-      </c>
-      <c r="N45" s="25">
-        <v>64</v>
-      </c>
-      <c r="O45" s="32" t="s">
+      <c r="M45" s="8">
+        <v>64</v>
+      </c>
+      <c r="N45" s="24">
+        <v>64</v>
+      </c>
+      <c r="O45" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P45" s="25">
+      <c r="P45" s="24">
         <v>0.1</v>
       </c>
-      <c r="Q45" s="10">
+      <c r="Q45" s="9">
         <v>1E-3</v>
       </c>
       <c r="R45" s="88" t="s">
         <v>72</v>
       </c>
-      <c r="S45" s="80"/>
-      <c r="T45" s="80"/>
-      <c r="U45" s="80"/>
-      <c r="V45" s="80"/>
-      <c r="W45" s="81"/>
+      <c r="S45" s="79"/>
+      <c r="T45" s="79"/>
+      <c r="U45" s="79"/>
+      <c r="V45" s="79"/>
+      <c r="W45" s="80"/>
     </row>
     <row r="46" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="60"/>
-      <c r="B46" s="76"/>
-      <c r="C46" s="30" t="s">
+      <c r="A46" s="59"/>
+      <c r="B46" s="67"/>
+      <c r="C46" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="D46" s="58">
+      <c r="D46" s="57">
         <v>47.232999999999997</v>
       </c>
-      <c r="E46" s="52">
+      <c r="E46" s="51">
         <v>96.742000000000004</v>
       </c>
-      <c r="F46" s="52">
+      <c r="F46" s="51">
         <v>0.94530000000000003</v>
       </c>
-      <c r="G46" s="52">
+      <c r="G46" s="51">
         <v>0.94530000000000003</v>
       </c>
-      <c r="H46" s="53">
+      <c r="H46" s="52">
         <v>79.099999999999994</v>
       </c>
-      <c r="I46" s="50">
+      <c r="I46" s="49">
         <v>30</v>
       </c>
       <c r="J46">
@@ -3679,35 +3683,35 @@
       <c r="K46">
         <v>6</v>
       </c>
-      <c r="L46" s="32" t="s">
+      <c r="L46" s="31" t="s">
         <v>74</v>
       </c>
       <c r="M46">
         <v>64</v>
       </c>
-      <c r="N46" s="25">
-        <v>64</v>
-      </c>
-      <c r="O46" s="32" t="s">
+      <c r="N46" s="24">
+        <v>64</v>
+      </c>
+      <c r="O46" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P46" s="25">
+      <c r="P46" s="24">
         <v>0.1</v>
       </c>
-      <c r="Q46" s="8">
+      <c r="Q46" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R46" s="82"/>
-      <c r="S46" s="83"/>
-      <c r="T46" s="83"/>
-      <c r="U46" s="83"/>
-      <c r="V46" s="83"/>
-      <c r="W46" s="84"/>
+      <c r="R46" s="81"/>
+      <c r="S46" s="82"/>
+      <c r="T46" s="82"/>
+      <c r="U46" s="82"/>
+      <c r="V46" s="82"/>
+      <c r="W46" s="83"/>
     </row>
     <row r="47" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="60"/>
-      <c r="B47" s="76"/>
-      <c r="C47" s="30" t="s">
+      <c r="A47" s="59"/>
+      <c r="B47" s="67"/>
+      <c r="C47" s="29" t="s">
         <v>14</v>
       </c>
       <c r="D47" s="1">
@@ -3722,10 +3726,10 @@
       <c r="G47">
         <v>0.90580000000000005</v>
       </c>
-      <c r="H47" s="8">
+      <c r="H47" s="7">
         <v>61.1</v>
       </c>
-      <c r="I47" s="50">
+      <c r="I47" s="49">
         <v>30</v>
       </c>
       <c r="J47">
@@ -3734,35 +3738,35 @@
       <c r="K47">
         <v>6</v>
       </c>
-      <c r="L47" s="32" t="s">
+      <c r="L47" s="31" t="s">
         <v>49</v>
       </c>
       <c r="M47">
         <v>64</v>
       </c>
-      <c r="N47" s="25">
-        <v>64</v>
-      </c>
-      <c r="O47" s="32" t="s">
+      <c r="N47" s="24">
+        <v>64</v>
+      </c>
+      <c r="O47" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P47" s="25">
+      <c r="P47" s="24">
         <v>0.1</v>
       </c>
-      <c r="Q47" s="8">
+      <c r="Q47" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R47" s="82"/>
-      <c r="S47" s="83"/>
-      <c r="T47" s="83"/>
-      <c r="U47" s="83"/>
-      <c r="V47" s="83"/>
-      <c r="W47" s="84"/>
+      <c r="R47" s="81"/>
+      <c r="S47" s="82"/>
+      <c r="T47" s="82"/>
+      <c r="U47" s="82"/>
+      <c r="V47" s="82"/>
+      <c r="W47" s="83"/>
     </row>
     <row r="48" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="60"/>
-      <c r="B48" s="77"/>
-      <c r="C48" s="31" t="s">
+      <c r="A48" s="59"/>
+      <c r="B48" s="68"/>
+      <c r="C48" s="30" t="s">
         <v>67</v>
       </c>
       <c r="D48" s="2">
@@ -3780,7 +3784,7 @@
       <c r="H48" s="4">
         <v>63.9</v>
       </c>
-      <c r="I48" s="48">
+      <c r="I48" s="47">
         <v>30</v>
       </c>
       <c r="J48" s="3">
@@ -3789,16 +3793,16 @@
       <c r="K48" s="3">
         <v>6</v>
       </c>
-      <c r="L48" s="32" t="s">
+      <c r="L48" s="31" t="s">
         <v>49</v>
       </c>
       <c r="M48" s="3">
         <v>64</v>
       </c>
-      <c r="N48" s="28">
-        <v>64</v>
-      </c>
-      <c r="O48" s="35" t="s">
+      <c r="N48" s="27">
+        <v>64</v>
+      </c>
+      <c r="O48" s="34" t="s">
         <v>39</v>
       </c>
       <c r="P48" s="3" t="s">
@@ -3807,94 +3811,94 @@
       <c r="Q48" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R48" s="85"/>
-      <c r="S48" s="86"/>
-      <c r="T48" s="86"/>
-      <c r="U48" s="86"/>
-      <c r="V48" s="86"/>
-      <c r="W48" s="87"/>
+      <c r="R48" s="84"/>
+      <c r="S48" s="85"/>
+      <c r="T48" s="85"/>
+      <c r="U48" s="85"/>
+      <c r="V48" s="85"/>
+      <c r="W48" s="86"/>
     </row>
     <row r="49" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="59"/>
-      <c r="B49" s="75" t="s">
+      <c r="A49" s="58"/>
+      <c r="B49" s="66" t="s">
         <v>58</v>
       </c>
-      <c r="C49" s="30" t="s">
+      <c r="C49" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="D49" s="58">
+      <c r="D49" s="57">
         <v>45.665999999999997</v>
       </c>
-      <c r="E49" s="52">
+      <c r="E49" s="51">
         <v>100.13</v>
       </c>
-      <c r="F49" s="52">
+      <c r="F49" s="51">
         <v>0.94140000000000001</v>
       </c>
-      <c r="G49" s="52">
+      <c r="G49" s="51">
         <v>0.94130000000000003</v>
       </c>
-      <c r="H49" s="53">
+      <c r="H49" s="52">
         <v>22.9</v>
       </c>
-      <c r="I49" s="50">
+      <c r="I49" s="49">
         <v>18</v>
       </c>
       <c r="J49">
         <v>245.39</v>
       </c>
-      <c r="K49" s="9">
-        <v>6</v>
-      </c>
-      <c r="L49" s="40" t="s">
+      <c r="K49" s="8">
+        <v>6</v>
+      </c>
+      <c r="L49" s="39" t="s">
         <v>75</v>
       </c>
-      <c r="M49" s="9">
+      <c r="M49" s="8">
         <v>64</v>
       </c>
       <c r="N49">
         <v>64</v>
       </c>
-      <c r="O49" s="32" t="s">
+      <c r="O49" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P49" s="25">
+      <c r="P49" s="24">
         <v>0.1</v>
       </c>
-      <c r="Q49" s="10">
+      <c r="Q49" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R49" s="78" t="s">
+      <c r="R49" s="69" t="s">
         <v>79</v>
       </c>
-      <c r="S49" s="65"/>
-      <c r="T49" s="65"/>
-      <c r="U49" s="65"/>
-      <c r="V49" s="65"/>
-      <c r="W49" s="66"/>
+      <c r="S49" s="70"/>
+      <c r="T49" s="70"/>
+      <c r="U49" s="70"/>
+      <c r="V49" s="70"/>
+      <c r="W49" s="71"/>
     </row>
     <row r="50" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="59"/>
-      <c r="B50" s="76"/>
-      <c r="C50" s="30" t="s">
+      <c r="A50" s="58"/>
+      <c r="B50" s="67"/>
+      <c r="C50" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="D50" s="58">
+      <c r="D50" s="57">
         <v>47.45</v>
       </c>
-      <c r="E50" s="52">
+      <c r="E50" s="51">
         <v>97.483999999999995</v>
       </c>
-      <c r="F50" s="52">
+      <c r="F50" s="51">
         <v>0.94440000000000002</v>
       </c>
-      <c r="G50" s="52">
+      <c r="G50" s="51">
         <v>0.94440000000000002</v>
       </c>
-      <c r="H50" s="53">
+      <c r="H50" s="52">
         <v>79.099999999999994</v>
       </c>
-      <c r="I50" s="50">
+      <c r="I50" s="49">
         <v>18</v>
       </c>
       <c r="J50">
@@ -3903,7 +3907,7 @@
       <c r="K50">
         <v>6</v>
       </c>
-      <c r="L50" s="32" t="s">
+      <c r="L50" s="31" t="s">
         <v>76</v>
       </c>
       <c r="M50">
@@ -3912,26 +3916,26 @@
       <c r="N50">
         <v>64</v>
       </c>
-      <c r="O50" s="32" t="s">
+      <c r="O50" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P50" s="25">
+      <c r="P50" s="24">
         <v>0.1</v>
       </c>
-      <c r="Q50" s="8">
+      <c r="Q50" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R50" s="67"/>
-      <c r="S50" s="68"/>
-      <c r="T50" s="68"/>
-      <c r="U50" s="68"/>
-      <c r="V50" s="68"/>
-      <c r="W50" s="69"/>
+      <c r="R50" s="72"/>
+      <c r="S50" s="73"/>
+      <c r="T50" s="73"/>
+      <c r="U50" s="73"/>
+      <c r="V50" s="73"/>
+      <c r="W50" s="74"/>
     </row>
     <row r="51" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="59"/>
-      <c r="B51" s="76"/>
-      <c r="C51" s="30" t="s">
+      <c r="A51" s="58"/>
+      <c r="B51" s="67"/>
+      <c r="C51" s="29" t="s">
         <v>14</v>
       </c>
       <c r="D51" s="1">
@@ -3946,10 +3950,10 @@
       <c r="G51">
         <v>0.90049999999999997</v>
       </c>
-      <c r="H51" s="8">
+      <c r="H51" s="7">
         <v>61.1</v>
       </c>
-      <c r="I51" s="50">
+      <c r="I51" s="49">
         <v>18</v>
       </c>
       <c r="J51">
@@ -3958,7 +3962,7 @@
       <c r="K51">
         <v>6</v>
       </c>
-      <c r="L51" s="32" t="s">
+      <c r="L51" s="31" t="s">
         <v>49</v>
       </c>
       <c r="M51">
@@ -3967,26 +3971,26 @@
       <c r="N51">
         <v>64</v>
       </c>
-      <c r="O51" s="32" t="s">
+      <c r="O51" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P51" s="25">
+      <c r="P51" s="24">
         <v>0.1</v>
       </c>
-      <c r="Q51" s="8">
+      <c r="Q51" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R51" s="67"/>
-      <c r="S51" s="68"/>
-      <c r="T51" s="68"/>
-      <c r="U51" s="68"/>
-      <c r="V51" s="68"/>
-      <c r="W51" s="69"/>
+      <c r="R51" s="72"/>
+      <c r="S51" s="73"/>
+      <c r="T51" s="73"/>
+      <c r="U51" s="73"/>
+      <c r="V51" s="73"/>
+      <c r="W51" s="74"/>
     </row>
     <row r="52" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="59"/>
-      <c r="B52" s="77"/>
-      <c r="C52" s="31" t="s">
+      <c r="A52" s="58"/>
+      <c r="B52" s="68"/>
+      <c r="C52" s="30" t="s">
         <v>67</v>
       </c>
       <c r="D52" s="3">
@@ -4004,7 +4008,7 @@
       <c r="H52" s="4">
         <v>39.9</v>
       </c>
-      <c r="I52" s="48">
+      <c r="I52" s="47">
         <v>18</v>
       </c>
       <c r="J52" s="3">
@@ -4013,7 +4017,7 @@
       <c r="K52" s="3">
         <v>6</v>
       </c>
-      <c r="L52" s="35" t="s">
+      <c r="L52" s="34" t="s">
         <v>49</v>
       </c>
       <c r="M52" s="3">
@@ -4022,7 +4026,7 @@
       <c r="N52" s="3">
         <v>64</v>
       </c>
-      <c r="O52" s="35" t="s">
+      <c r="O52" s="34" t="s">
         <v>39</v>
       </c>
       <c r="P52" s="3" t="s">
@@ -4031,76 +4035,76 @@
       <c r="Q52" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R52" s="70"/>
-      <c r="S52" s="71"/>
-      <c r="T52" s="71"/>
-      <c r="U52" s="71"/>
-      <c r="V52" s="71"/>
-      <c r="W52" s="72"/>
+      <c r="R52" s="75"/>
+      <c r="S52" s="76"/>
+      <c r="T52" s="76"/>
+      <c r="U52" s="76"/>
+      <c r="V52" s="76"/>
+      <c r="W52" s="77"/>
     </row>
     <row r="53" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="60"/>
-      <c r="B53" s="75" t="s">
+      <c r="A53" s="59"/>
+      <c r="B53" s="66" t="s">
         <v>77</v>
       </c>
-      <c r="C53" s="20" t="s">
+      <c r="C53" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D53" s="54">
+      <c r="D53" s="53">
         <v>46.415999999999997</v>
       </c>
-      <c r="E53" s="54">
+      <c r="E53" s="53">
         <v>96.207999999999998</v>
       </c>
-      <c r="F53" s="54">
+      <c r="F53" s="53">
         <v>0.94589999999999996</v>
       </c>
-      <c r="G53" s="54">
+      <c r="G53" s="53">
         <v>0.94579999999999997</v>
       </c>
-      <c r="H53" s="53">
+      <c r="H53" s="52">
         <v>22.5</v>
       </c>
-      <c r="I53" s="9">
+      <c r="I53" s="8">
         <v>18</v>
       </c>
-      <c r="J53" s="9">
+      <c r="J53" s="8">
         <v>217.61</v>
       </c>
-      <c r="K53" s="9">
-        <v>6</v>
-      </c>
-      <c r="L53" s="40" t="s">
+      <c r="K53" s="8">
+        <v>6</v>
+      </c>
+      <c r="L53" s="39" t="s">
         <v>78</v>
       </c>
-      <c r="M53" s="9">
-        <v>64</v>
-      </c>
-      <c r="N53" s="9">
-        <v>64</v>
-      </c>
-      <c r="O53" s="32" t="s">
+      <c r="M53" s="8">
+        <v>64</v>
+      </c>
+      <c r="N53" s="8">
+        <v>64</v>
+      </c>
+      <c r="O53" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="P53" s="61" t="s">
+      <c r="P53" s="60" t="s">
         <v>68</v>
       </c>
-      <c r="Q53" s="10">
+      <c r="Q53" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R53" s="78" t="s">
+      <c r="R53" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="S53" s="65"/>
-      <c r="T53" s="65"/>
-      <c r="U53" s="65"/>
-      <c r="V53" s="65"/>
-      <c r="W53" s="66"/>
+      <c r="S53" s="70"/>
+      <c r="T53" s="70"/>
+      <c r="U53" s="70"/>
+      <c r="V53" s="70"/>
+      <c r="W53" s="71"/>
     </row>
     <row r="54" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A54" s="60"/>
-      <c r="B54" s="76"/>
-      <c r="C54" s="30" t="s">
+      <c r="A54" s="59"/>
+      <c r="B54" s="67"/>
+      <c r="C54" s="29" t="s">
         <v>12</v>
       </c>
       <c r="D54">
@@ -4109,13 +4113,13 @@
       <c r="E54">
         <v>498.339</v>
       </c>
-      <c r="F54" s="41">
+      <c r="F54" s="40">
         <v>-0.45190000000000002</v>
       </c>
-      <c r="G54" s="41">
+      <c r="G54" s="40">
         <v>-0.45300000000000001</v>
       </c>
-      <c r="H54" s="8">
+      <c r="H54" s="7">
         <v>77.099999999999994</v>
       </c>
       <c r="I54" s="1">
@@ -4127,7 +4131,7 @@
       <c r="K54">
         <v>6</v>
       </c>
-      <c r="L54" s="32" t="s">
+      <c r="L54" s="31" t="s">
         <v>49</v>
       </c>
       <c r="M54">
@@ -4136,26 +4140,26 @@
       <c r="N54">
         <v>64</v>
       </c>
-      <c r="O54" s="32" t="s">
+      <c r="O54" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P54" s="62" t="s">
+      <c r="P54" s="61" t="s">
         <v>68</v>
       </c>
-      <c r="Q54" s="8">
+      <c r="Q54" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R54" s="67"/>
-      <c r="S54" s="68"/>
-      <c r="T54" s="68"/>
-      <c r="U54" s="68"/>
-      <c r="V54" s="68"/>
-      <c r="W54" s="69"/>
+      <c r="R54" s="72"/>
+      <c r="S54" s="73"/>
+      <c r="T54" s="73"/>
+      <c r="U54" s="73"/>
+      <c r="V54" s="73"/>
+      <c r="W54" s="74"/>
     </row>
     <row r="55" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A55" s="60"/>
-      <c r="B55" s="76"/>
-      <c r="C55" s="30" t="s">
+      <c r="A55" s="59"/>
+      <c r="B55" s="67"/>
+      <c r="C55" s="29" t="s">
         <v>14</v>
       </c>
       <c r="D55">
@@ -4170,7 +4174,7 @@
       <c r="G55">
         <v>0.90980000000000005</v>
       </c>
-      <c r="H55" s="8">
+      <c r="H55" s="7">
         <v>59.6</v>
       </c>
       <c r="I55" s="1">
@@ -4182,7 +4186,7 @@
       <c r="K55">
         <v>6</v>
       </c>
-      <c r="L55" s="32" t="s">
+      <c r="L55" s="31" t="s">
         <v>49</v>
       </c>
       <c r="M55">
@@ -4191,26 +4195,26 @@
       <c r="N55">
         <v>64</v>
       </c>
-      <c r="O55" s="32" t="s">
+      <c r="O55" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P55" s="62" t="s">
+      <c r="P55" s="61" t="s">
         <v>68</v>
       </c>
-      <c r="Q55" s="8">
+      <c r="Q55" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R55" s="67"/>
-      <c r="S55" s="68"/>
-      <c r="T55" s="68"/>
-      <c r="U55" s="68"/>
-      <c r="V55" s="68"/>
-      <c r="W55" s="69"/>
+      <c r="R55" s="72"/>
+      <c r="S55" s="73"/>
+      <c r="T55" s="73"/>
+      <c r="U55" s="73"/>
+      <c r="V55" s="73"/>
+      <c r="W55" s="74"/>
     </row>
     <row r="56" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="60"/>
-      <c r="B56" s="77"/>
-      <c r="C56" s="31" t="s">
+      <c r="A56" s="59"/>
+      <c r="B56" s="68"/>
+      <c r="C56" s="30" t="s">
         <v>67</v>
       </c>
       <c r="D56" s="3">
@@ -4219,13 +4223,13 @@
       <c r="E56" s="3">
         <v>498.339</v>
       </c>
-      <c r="F56" s="49">
+      <c r="F56" s="48">
         <v>-0.45190000000000002</v>
       </c>
-      <c r="G56" s="49">
+      <c r="G56" s="48">
         <v>-0.45300000000000001</v>
       </c>
-      <c r="H56" s="8">
+      <c r="H56" s="7">
         <v>38.4</v>
       </c>
       <c r="I56" s="2">
@@ -4237,7 +4241,7 @@
       <c r="K56" s="3">
         <v>6</v>
       </c>
-      <c r="L56" s="35" t="s">
+      <c r="L56" s="34" t="s">
         <v>49</v>
       </c>
       <c r="M56" s="3">
@@ -4246,43 +4250,43 @@
       <c r="N56" s="3">
         <v>64</v>
       </c>
-      <c r="O56" s="35" t="s">
+      <c r="O56" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="P56" s="63" t="s">
+      <c r="P56" s="62" t="s">
         <v>68</v>
       </c>
       <c r="Q56" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R56" s="70"/>
-      <c r="S56" s="71"/>
-      <c r="T56" s="71"/>
-      <c r="U56" s="71"/>
-      <c r="V56" s="71"/>
-      <c r="W56" s="72"/>
+      <c r="R56" s="75"/>
+      <c r="S56" s="76"/>
+      <c r="T56" s="76"/>
+      <c r="U56" s="76"/>
+      <c r="V56" s="76"/>
+      <c r="W56" s="77"/>
     </row>
     <row r="57" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="59"/>
-      <c r="B57" s="75" t="s">
+      <c r="A57" s="58"/>
+      <c r="B57" s="66" t="s">
         <v>81</v>
       </c>
-      <c r="C57" s="20" t="s">
+      <c r="C57" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D57" s="9">
+      <c r="D57" s="8">
         <v>56.648000000000003</v>
       </c>
-      <c r="E57" s="9">
+      <c r="E57" s="8">
         <v>98.847999999999999</v>
       </c>
-      <c r="F57" s="9">
+      <c r="F57" s="8">
         <v>0.94289999999999996</v>
       </c>
-      <c r="G57" s="9">
+      <c r="G57" s="8">
         <v>0.94279999999999997</v>
       </c>
-      <c r="H57" s="10">
+      <c r="H57" s="9">
         <v>22.4</v>
       </c>
       <c r="I57" s="1">
@@ -4294,52 +4298,52 @@
       <c r="K57">
         <v>6</v>
       </c>
-      <c r="L57" s="32" t="s">
+      <c r="L57" s="31" t="s">
         <v>74</v>
       </c>
       <c r="M57">
         <v>64</v>
       </c>
-      <c r="N57" s="46">
-        <v>64</v>
-      </c>
-      <c r="O57" s="32" t="s">
+      <c r="N57" s="45">
+        <v>64</v>
+      </c>
+      <c r="O57" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P57" s="46">
+      <c r="P57" s="45">
         <v>0.1</v>
       </c>
-      <c r="Q57" s="10">
+      <c r="Q57" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R57" s="78" t="s">
+      <c r="R57" s="69" t="s">
         <v>82</v>
       </c>
-      <c r="S57" s="65"/>
-      <c r="T57" s="65"/>
-      <c r="U57" s="65"/>
-      <c r="V57" s="65"/>
-      <c r="W57" s="66"/>
+      <c r="S57" s="70"/>
+      <c r="T57" s="70"/>
+      <c r="U57" s="70"/>
+      <c r="V57" s="70"/>
+      <c r="W57" s="71"/>
     </row>
     <row r="58" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A58" s="59"/>
-      <c r="B58" s="76"/>
-      <c r="C58" s="30" t="s">
+      <c r="A58" s="58"/>
+      <c r="B58" s="67"/>
+      <c r="C58" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="D58" s="104">
+      <c r="D58">
         <v>87.501999999999995</v>
       </c>
-      <c r="E58" s="104">
+      <c r="E58">
         <v>143.33000000000001</v>
       </c>
-      <c r="F58" s="105">
+      <c r="F58" s="63">
         <v>0.87990000000000002</v>
       </c>
-      <c r="G58" s="105">
+      <c r="G58" s="63">
         <v>0.87980000000000003</v>
       </c>
-      <c r="H58" s="106">
+      <c r="H58" s="7">
         <v>22.6</v>
       </c>
       <c r="I58" s="1">
@@ -4351,50 +4355,50 @@
       <c r="K58">
         <v>6</v>
       </c>
-      <c r="L58" s="32" t="s">
+      <c r="L58" s="31" t="s">
         <v>49</v>
       </c>
       <c r="M58">
         <v>64</v>
       </c>
-      <c r="N58" s="46">
+      <c r="N58" s="45">
         <v>32</v>
       </c>
-      <c r="O58" s="32" t="s">
+      <c r="O58" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P58" s="46">
+      <c r="P58" s="45">
         <v>0.1</v>
       </c>
-      <c r="Q58" s="8">
+      <c r="Q58" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R58" s="67"/>
-      <c r="S58" s="68"/>
-      <c r="T58" s="68"/>
-      <c r="U58" s="68"/>
-      <c r="V58" s="68"/>
-      <c r="W58" s="69"/>
+      <c r="R58" s="72"/>
+      <c r="S58" s="73"/>
+      <c r="T58" s="73"/>
+      <c r="U58" s="73"/>
+      <c r="V58" s="73"/>
+      <c r="W58" s="74"/>
     </row>
     <row r="59" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A59" s="59"/>
-      <c r="B59" s="76"/>
-      <c r="C59" s="30" t="s">
+      <c r="A59" s="58"/>
+      <c r="B59" s="67"/>
+      <c r="C59" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="D59" s="52">
+      <c r="D59" s="51">
         <v>53.17</v>
       </c>
-      <c r="E59" s="52">
+      <c r="E59" s="51">
         <v>96.721999999999994</v>
       </c>
-      <c r="F59" s="52">
+      <c r="F59" s="51">
         <v>0.94530000000000003</v>
       </c>
-      <c r="G59" s="52">
+      <c r="G59" s="51">
         <v>0.94530000000000003</v>
       </c>
-      <c r="H59" s="53">
+      <c r="H59" s="52">
         <v>17.899999999999999</v>
       </c>
       <c r="I59" s="1">
@@ -4406,35 +4410,35 @@
       <c r="K59">
         <v>6</v>
       </c>
-      <c r="L59" s="32" t="s">
+      <c r="L59" s="31" t="s">
         <v>52</v>
       </c>
       <c r="M59">
         <v>64</v>
       </c>
-      <c r="N59" s="46">
+      <c r="N59" s="45">
         <v>32</v>
       </c>
-      <c r="O59" s="32" t="s">
+      <c r="O59" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P59" s="46">
+      <c r="P59" s="45">
         <v>0.1</v>
       </c>
-      <c r="Q59" s="8">
+      <c r="Q59" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R59" s="67"/>
-      <c r="S59" s="68"/>
-      <c r="T59" s="68"/>
-      <c r="U59" s="68"/>
-      <c r="V59" s="68"/>
-      <c r="W59" s="69"/>
+      <c r="R59" s="72"/>
+      <c r="S59" s="73"/>
+      <c r="T59" s="73"/>
+      <c r="U59" s="73"/>
+      <c r="V59" s="73"/>
+      <c r="W59" s="74"/>
     </row>
     <row r="60" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="59"/>
-      <c r="B60" s="77"/>
-      <c r="C60" s="31" t="s">
+      <c r="A60" s="58"/>
+      <c r="B60" s="68"/>
+      <c r="C60" s="30" t="s">
         <v>67</v>
       </c>
       <c r="D60" s="3">
@@ -4461,43 +4465,43 @@
       <c r="K60" s="3">
         <v>6</v>
       </c>
-      <c r="L60" s="35" t="s">
+      <c r="L60" s="34" t="s">
         <v>49</v>
       </c>
       <c r="M60" s="3">
         <v>64</v>
       </c>
-      <c r="N60" s="47">
+      <c r="N60" s="46">
         <v>32</v>
       </c>
-      <c r="O60" s="35" t="s">
+      <c r="O60" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="P60" s="47">
+      <c r="P60" s="46">
         <v>0.1</v>
       </c>
       <c r="Q60" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R60" s="70"/>
-      <c r="S60" s="71"/>
-      <c r="T60" s="71"/>
-      <c r="U60" s="71"/>
-      <c r="V60" s="71"/>
-      <c r="W60" s="72"/>
+      <c r="R60" s="75"/>
+      <c r="S60" s="76"/>
+      <c r="T60" s="76"/>
+      <c r="U60" s="76"/>
+      <c r="V60" s="76"/>
+      <c r="W60" s="77"/>
     </row>
     <row r="61" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="8"/>
-      <c r="B61" s="75" t="s">
+      <c r="A61" s="7"/>
+      <c r="B61" s="66" t="s">
         <v>85</v>
       </c>
-      <c r="C61" s="29" t="s">
+      <c r="C61" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="D61" s="112">
+      <c r="D61" s="65">
         <v>54.145000000000003</v>
       </c>
-      <c r="E61" s="108">
+      <c r="E61">
         <v>102.96899999999999</v>
       </c>
       <c r="F61">
@@ -4506,107 +4510,107 @@
       <c r="G61">
         <v>0.93799999999999994</v>
       </c>
-      <c r="H61" s="106">
+      <c r="H61" s="7">
         <v>22.4</v>
       </c>
-      <c r="I61" s="107">
+      <c r="I61" s="1">
         <v>18</v>
       </c>
-      <c r="J61" s="108">
+      <c r="J61">
         <v>339.69</v>
       </c>
-      <c r="K61" s="108">
-        <v>6</v>
-      </c>
-      <c r="L61" s="32" t="s">
-        <v>64</v>
-      </c>
-      <c r="M61" s="108">
-        <v>64</v>
-      </c>
-      <c r="N61" s="108">
-        <v>64</v>
-      </c>
-      <c r="O61" s="109" t="s">
+      <c r="K61">
+        <v>6</v>
+      </c>
+      <c r="L61" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="M61">
+        <v>64</v>
+      </c>
+      <c r="N61">
+        <v>64</v>
+      </c>
+      <c r="O61" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P61" s="108">
+      <c r="P61">
         <v>0.1</v>
       </c>
-      <c r="Q61" s="106">
+      <c r="Q61" s="7">
         <v>1E-3</v>
       </c>
       <c r="R61" s="88" t="s">
         <v>86</v>
       </c>
-      <c r="S61" s="80"/>
-      <c r="T61" s="80"/>
-      <c r="U61" s="80"/>
-      <c r="V61" s="80"/>
-      <c r="W61" s="81"/>
+      <c r="S61" s="79"/>
+      <c r="T61" s="79"/>
+      <c r="U61" s="79"/>
+      <c r="V61" s="79"/>
+      <c r="W61" s="80"/>
     </row>
     <row r="62" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A62" s="8"/>
-      <c r="B62" s="76"/>
-      <c r="C62" s="26" t="s">
+      <c r="A62" s="7"/>
+      <c r="B62" s="67"/>
+      <c r="C62" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="D62" s="113">
+      <c r="D62" s="51">
         <v>51.847000000000001</v>
       </c>
-      <c r="E62" s="52">
+      <c r="E62" s="51">
         <v>99.551000000000002</v>
       </c>
-      <c r="F62" s="52">
+      <c r="F62" s="51">
         <v>0.94210000000000005</v>
       </c>
-      <c r="G62" s="52">
+      <c r="G62" s="51">
         <v>0.94199999999999995</v>
       </c>
-      <c r="H62" s="53">
+      <c r="H62" s="52">
         <v>22.6</v>
       </c>
-      <c r="I62" s="107">
+      <c r="I62" s="1">
         <v>18</v>
       </c>
-      <c r="J62" s="108">
+      <c r="J62">
         <v>665.01</v>
       </c>
-      <c r="K62" s="108">
-        <v>6</v>
-      </c>
-      <c r="L62" s="32" t="s">
+      <c r="K62">
+        <v>6</v>
+      </c>
+      <c r="L62" s="31" t="s">
         <v>83</v>
       </c>
-      <c r="M62" s="108">
-        <v>64</v>
-      </c>
-      <c r="N62" s="108">
+      <c r="M62">
+        <v>64</v>
+      </c>
+      <c r="N62">
         <v>32</v>
       </c>
-      <c r="O62" s="109" t="s">
+      <c r="O62" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P62" s="108">
+      <c r="P62">
         <v>0.1</v>
       </c>
-      <c r="Q62" s="106">
+      <c r="Q62" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R62" s="82"/>
-      <c r="S62" s="83"/>
-      <c r="T62" s="83"/>
-      <c r="U62" s="83"/>
-      <c r="V62" s="83"/>
-      <c r="W62" s="84"/>
+      <c r="R62" s="81"/>
+      <c r="S62" s="82"/>
+      <c r="T62" s="82"/>
+      <c r="U62" s="82"/>
+      <c r="V62" s="82"/>
+      <c r="W62" s="83"/>
     </row>
     <row r="63" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A63" s="8"/>
-      <c r="B63" s="76"/>
-      <c r="C63" s="26" t="s">
+      <c r="A63" s="7"/>
+      <c r="B63" s="67"/>
+      <c r="C63" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="D63" s="108">
+      <c r="D63">
         <v>105.566</v>
       </c>
       <c r="E63">
@@ -4618,50 +4622,50 @@
       <c r="G63">
         <v>0.86880000000000002</v>
       </c>
-      <c r="H63" s="106">
+      <c r="H63" s="7">
         <v>17.899999999999999</v>
       </c>
-      <c r="I63" s="107">
+      <c r="I63" s="1">
         <v>18</v>
       </c>
-      <c r="J63" s="108">
+      <c r="J63">
         <v>382.5</v>
       </c>
-      <c r="K63" s="108">
-        <v>6</v>
-      </c>
-      <c r="L63" s="32" t="s">
+      <c r="K63">
+        <v>6</v>
+      </c>
+      <c r="L63" s="31" t="s">
         <v>49</v>
       </c>
-      <c r="M63" s="108">
-        <v>64</v>
-      </c>
-      <c r="N63" s="108">
+      <c r="M63">
+        <v>64</v>
+      </c>
+      <c r="N63">
         <v>32</v>
       </c>
-      <c r="O63" s="109" t="s">
+      <c r="O63" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P63" s="108">
+      <c r="P63">
         <v>0.1</v>
       </c>
-      <c r="Q63" s="111">
+      <c r="Q63" s="64">
         <v>1E-3</v>
       </c>
-      <c r="R63" s="82"/>
-      <c r="S63" s="83"/>
-      <c r="T63" s="83"/>
-      <c r="U63" s="83"/>
-      <c r="V63" s="83"/>
-      <c r="W63" s="84"/>
+      <c r="R63" s="81"/>
+      <c r="S63" s="82"/>
+      <c r="T63" s="82"/>
+      <c r="U63" s="82"/>
+      <c r="V63" s="82"/>
+      <c r="W63" s="83"/>
     </row>
     <row r="64" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A64" s="8"/>
-      <c r="B64" s="76"/>
-      <c r="C64" s="26" t="s">
+      <c r="A64" s="7"/>
+      <c r="B64" s="67"/>
+      <c r="C64" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="D64" s="108">
+      <c r="D64">
         <v>109.354</v>
       </c>
       <c r="E64">
@@ -4673,47 +4677,47 @@
       <c r="G64">
         <v>0.82450000000000001</v>
       </c>
-      <c r="H64" s="106">
+      <c r="H64" s="7">
         <v>19.3</v>
       </c>
-      <c r="I64" s="107">
+      <c r="I64" s="1">
         <v>18</v>
       </c>
-      <c r="J64" s="108">
+      <c r="J64">
         <v>189.74</v>
       </c>
-      <c r="K64" s="108">
-        <v>6</v>
-      </c>
-      <c r="L64" s="32" t="s">
+      <c r="K64">
+        <v>6</v>
+      </c>
+      <c r="L64" s="31" t="s">
         <v>49</v>
       </c>
-      <c r="M64" s="108">
-        <v>64</v>
-      </c>
-      <c r="N64" s="108">
+      <c r="M64">
+        <v>64</v>
+      </c>
+      <c r="N64">
         <v>32</v>
       </c>
-      <c r="O64" s="109" t="s">
+      <c r="O64" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="P64" s="108">
+      <c r="P64">
         <v>0.1</v>
       </c>
-      <c r="Q64" s="8">
+      <c r="Q64" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R64" s="82"/>
-      <c r="S64" s="83"/>
-      <c r="T64" s="83"/>
-      <c r="U64" s="83"/>
-      <c r="V64" s="83"/>
-      <c r="W64" s="84"/>
+      <c r="R64" s="81"/>
+      <c r="S64" s="82"/>
+      <c r="T64" s="82"/>
+      <c r="U64" s="82"/>
+      <c r="V64" s="82"/>
+      <c r="W64" s="83"/>
     </row>
     <row r="65" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="8"/>
-      <c r="B65" s="77"/>
-      <c r="C65" s="31" t="s">
+      <c r="A65" s="7"/>
+      <c r="B65" s="68"/>
+      <c r="C65" s="30" t="s">
         <v>84</v>
       </c>
       <c r="D65" s="3">
@@ -4740,7 +4744,7 @@
       <c r="K65" s="3">
         <v>6</v>
       </c>
-      <c r="L65" s="35" t="s">
+      <c r="L65" s="34" t="s">
         <v>49</v>
       </c>
       <c r="M65" s="3">
@@ -4749,21 +4753,21 @@
       <c r="N65" s="3">
         <v>32</v>
       </c>
-      <c r="O65" s="35" t="s">
+      <c r="O65" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="P65" s="110">
+      <c r="P65" s="3">
         <v>0.1</v>
       </c>
       <c r="Q65" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R65" s="85"/>
-      <c r="S65" s="86"/>
-      <c r="T65" s="86"/>
-      <c r="U65" s="86"/>
-      <c r="V65" s="86"/>
-      <c r="W65" s="87"/>
+      <c r="R65" s="84"/>
+      <c r="S65" s="85"/>
+      <c r="T65" s="85"/>
+      <c r="U65" s="85"/>
+      <c r="V65" s="85"/>
+      <c r="W65" s="86"/>
     </row>
     <row r="66" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>

</xml_diff>

<commit_message>
{V13}: entrenamiento con datos diurnos completado.
</commit_message>
<xml_diff>
--- a/modelos_tfg/MetricasValidacion.xlsx
+++ b/modelos_tfg/MetricasValidacion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\modelos_tfg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13C9D6B3-DA7A-4650-A1CF-C1C0F2323CC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8956D507-7938-49F9-BD9B-2C7A665916C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="0" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="91">
   <si>
     <t>ID Train</t>
   </si>
@@ -290,12 +290,6 @@
   </si>
   <si>
     <t>V11</t>
-  </si>
-  <si>
-    <t>Este entrenamiento ha vuelto a ser sin los inputs de P_gen,
-V_gen e I_gen. Además, he vuelto a las configuraciones de
-los modelos que mejores resultados han dado en todos
-los entrenamiento, con el droput de todas al 0,1</t>
   </si>
   <si>
     <t>55 (ES)</t>
@@ -312,6 +306,25 @@
 MLP haciendo que el entrenamiento sea el mismo para todos.
 Falta entrenar al modelo MLP quitando filas con irradiancia
 muy muy baja.</t>
+  </si>
+  <si>
+    <t>V13</t>
+  </si>
+  <si>
+    <t>Este entrenamiento ha vuelto a ser sin los inputs de P_gen, V_gen e I_gen. Además, he vuelto a las configuraciones de los modelos que mejores resultados han dado en todos los entrenamiento, con el droput de todas al 0,1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Este entrenamiento es el más completo porque es una comparativa del entrenamiento de modelos comparando días completos (teniendo en cuenta las noches) y días con irradiancia superior a 10 W/m^2. 
+Los modelos tienes los hiperparámetros óptimos, es decir en las versiones que mejor
+han salido. </t>
+  </si>
+  <si>
+    <t>V13
+-
+diurnos</t>
+  </si>
+  <si>
+    <t>Datos diurnos para G &gt; 10 W/m^2</t>
   </si>
 </sst>
 </file>
@@ -359,7 +372,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -426,8 +439,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="22">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -674,11 +693,55 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="136">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -777,6 +840,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -787,6 +853,33 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -814,37 +907,25 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -867,39 +948,72 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1248,7 +1362,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:W66"/>
+  <dimension ref="A2:W74"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.42578125" customWidth="1"/>
@@ -1263,36 +1377,37 @@
     <col min="11" max="11" width="12.42578125" customWidth="1"/>
     <col min="13" max="13" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="14" max="15" width="11.7109375" customWidth="1"/>
+    <col min="18" max="23" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D3" s="89" t="s">
+      <c r="D3" s="95" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="91"/>
-      <c r="I3" s="92" t="s">
+      <c r="E3" s="96"/>
+      <c r="F3" s="96"/>
+      <c r="G3" s="96"/>
+      <c r="H3" s="97"/>
+      <c r="I3" s="98" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="93"/>
-      <c r="K3" s="93"/>
-      <c r="L3" s="93"/>
-      <c r="M3" s="93"/>
-      <c r="N3" s="93"/>
-      <c r="O3" s="93"/>
-      <c r="P3" s="93"/>
-      <c r="Q3" s="94"/>
-      <c r="R3" s="99" t="s">
+      <c r="J3" s="99"/>
+      <c r="K3" s="99"/>
+      <c r="L3" s="99"/>
+      <c r="M3" s="99"/>
+      <c r="N3" s="99"/>
+      <c r="O3" s="99"/>
+      <c r="P3" s="99"/>
+      <c r="Q3" s="100"/>
+      <c r="R3" s="102" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="100"/>
-      <c r="T3" s="100"/>
-      <c r="U3" s="100"/>
-      <c r="V3" s="100"/>
-      <c r="W3" s="101"/>
+      <c r="S3" s="103"/>
+      <c r="T3" s="103"/>
+      <c r="U3" s="103"/>
+      <c r="V3" s="103"/>
+      <c r="W3" s="89"/>
     </row>
     <row r="4" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="19" t="s">
@@ -1313,7 +1428,7 @@
       <c r="G4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="106" t="s">
+      <c r="H4" s="66" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="10" t="s">
@@ -1343,16 +1458,16 @@
       <c r="Q4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="102"/>
-      <c r="S4" s="103"/>
-      <c r="T4" s="103"/>
-      <c r="U4" s="103"/>
-      <c r="V4" s="103"/>
-      <c r="W4" s="104"/>
-    </row>
-    <row r="5" spans="1:23" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R4" s="104"/>
+      <c r="S4" s="105"/>
+      <c r="T4" s="105"/>
+      <c r="U4" s="105"/>
+      <c r="V4" s="105"/>
+      <c r="W4" s="91"/>
+    </row>
+    <row r="5" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
-      <c r="B5" s="95" t="s">
+      <c r="B5" s="101" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -1400,18 +1515,18 @@
       <c r="Q5" s="16">
         <v>1E-3</v>
       </c>
-      <c r="R5" s="87" t="s">
+      <c r="R5" s="88" t="s">
         <v>38</v>
       </c>
-      <c r="S5" s="70"/>
-      <c r="T5" s="70"/>
-      <c r="U5" s="70"/>
-      <c r="V5" s="70"/>
-      <c r="W5" s="71"/>
+      <c r="S5" s="80"/>
+      <c r="T5" s="80"/>
+      <c r="U5" s="80"/>
+      <c r="V5" s="80"/>
+      <c r="W5" s="81"/>
     </row>
     <row r="6" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7"/>
-      <c r="B6" s="96"/>
+      <c r="B6" s="93"/>
       <c r="C6" s="5" t="s">
         <v>12</v>
       </c>
@@ -1457,16 +1572,16 @@
       <c r="Q6" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R6" s="72"/>
-      <c r="S6" s="73"/>
-      <c r="T6" s="73"/>
-      <c r="U6" s="73"/>
-      <c r="V6" s="73"/>
-      <c r="W6" s="74"/>
+      <c r="R6" s="82"/>
+      <c r="S6" s="83"/>
+      <c r="T6" s="83"/>
+      <c r="U6" s="83"/>
+      <c r="V6" s="83"/>
+      <c r="W6" s="84"/>
     </row>
     <row r="7" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7"/>
-      <c r="B7" s="97"/>
+      <c r="B7" s="94"/>
       <c r="C7" s="13" t="s">
         <v>14</v>
       </c>
@@ -1512,16 +1627,16 @@
       <c r="Q7" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R7" s="75"/>
-      <c r="S7" s="76"/>
-      <c r="T7" s="76"/>
-      <c r="U7" s="76"/>
-      <c r="V7" s="76"/>
-      <c r="W7" s="77"/>
+      <c r="R7" s="85"/>
+      <c r="S7" s="86"/>
+      <c r="T7" s="86"/>
+      <c r="U7" s="86"/>
+      <c r="V7" s="86"/>
+      <c r="W7" s="87"/>
     </row>
     <row r="8" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
-      <c r="B8" s="98" t="s">
+      <c r="B8" s="92" t="s">
         <v>24</v>
       </c>
       <c r="C8" s="5" t="s">
@@ -1569,18 +1684,18 @@
       <c r="Q8" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R8" s="87" t="s">
+      <c r="R8" s="88" t="s">
         <v>38</v>
       </c>
-      <c r="S8" s="70"/>
-      <c r="T8" s="70"/>
-      <c r="U8" s="70"/>
-      <c r="V8" s="70"/>
-      <c r="W8" s="71"/>
+      <c r="S8" s="80"/>
+      <c r="T8" s="80"/>
+      <c r="U8" s="80"/>
+      <c r="V8" s="80"/>
+      <c r="W8" s="81"/>
     </row>
     <row r="9" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
-      <c r="B9" s="96"/>
+      <c r="B9" s="93"/>
       <c r="C9" s="5" t="s">
         <v>12</v>
       </c>
@@ -1626,16 +1741,16 @@
       <c r="Q9" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R9" s="72"/>
-      <c r="S9" s="73"/>
-      <c r="T9" s="73"/>
-      <c r="U9" s="73"/>
-      <c r="V9" s="73"/>
-      <c r="W9" s="74"/>
+      <c r="R9" s="82"/>
+      <c r="S9" s="83"/>
+      <c r="T9" s="83"/>
+      <c r="U9" s="83"/>
+      <c r="V9" s="83"/>
+      <c r="W9" s="84"/>
     </row>
     <row r="10" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7"/>
-      <c r="B10" s="97"/>
+      <c r="B10" s="94"/>
       <c r="C10" s="5" t="s">
         <v>14</v>
       </c>
@@ -1681,15 +1796,15 @@
       <c r="Q10" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R10" s="75"/>
-      <c r="S10" s="76"/>
-      <c r="T10" s="76"/>
-      <c r="U10" s="76"/>
-      <c r="V10" s="76"/>
-      <c r="W10" s="77"/>
+      <c r="R10" s="85"/>
+      <c r="S10" s="86"/>
+      <c r="T10" s="86"/>
+      <c r="U10" s="86"/>
+      <c r="V10" s="86"/>
+      <c r="W10" s="87"/>
     </row>
     <row r="11" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="98" t="s">
+      <c r="B11" s="92" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="28" t="s">
@@ -1737,17 +1852,17 @@
       <c r="Q11" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R11" s="87" t="s">
+      <c r="R11" s="88" t="s">
         <v>38</v>
       </c>
-      <c r="S11" s="70"/>
-      <c r="T11" s="70"/>
-      <c r="U11" s="70"/>
-      <c r="V11" s="70"/>
-      <c r="W11" s="71"/>
+      <c r="S11" s="80"/>
+      <c r="T11" s="80"/>
+      <c r="U11" s="80"/>
+      <c r="V11" s="80"/>
+      <c r="W11" s="81"/>
     </row>
     <row r="12" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="96"/>
+      <c r="B12" s="93"/>
       <c r="C12" s="25" t="s">
         <v>12</v>
       </c>
@@ -1793,15 +1908,15 @@
       <c r="Q12" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R12" s="72"/>
-      <c r="S12" s="73"/>
-      <c r="T12" s="73"/>
-      <c r="U12" s="73"/>
-      <c r="V12" s="73"/>
-      <c r="W12" s="74"/>
+      <c r="R12" s="82"/>
+      <c r="S12" s="83"/>
+      <c r="T12" s="83"/>
+      <c r="U12" s="83"/>
+      <c r="V12" s="83"/>
+      <c r="W12" s="84"/>
     </row>
     <row r="13" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="96"/>
+      <c r="B13" s="93"/>
       <c r="C13" s="26" t="s">
         <v>14</v>
       </c>
@@ -1847,15 +1962,15 @@
       <c r="Q13" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R13" s="75"/>
-      <c r="S13" s="76"/>
-      <c r="T13" s="76"/>
-      <c r="U13" s="76"/>
-      <c r="V13" s="76"/>
-      <c r="W13" s="77"/>
+      <c r="R13" s="85"/>
+      <c r="S13" s="86"/>
+      <c r="T13" s="86"/>
+      <c r="U13" s="86"/>
+      <c r="V13" s="86"/>
+      <c r="W13" s="87"/>
     </row>
     <row r="14" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="98" t="s">
+      <c r="B14" s="92" t="s">
         <v>36</v>
       </c>
       <c r="C14" s="19" t="s">
@@ -1903,17 +2018,17 @@
       <c r="Q14" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R14" s="87" t="s">
+      <c r="R14" s="88" t="s">
         <v>37</v>
       </c>
-      <c r="S14" s="70"/>
-      <c r="T14" s="70"/>
-      <c r="U14" s="70"/>
-      <c r="V14" s="70"/>
-      <c r="W14" s="71"/>
+      <c r="S14" s="80"/>
+      <c r="T14" s="80"/>
+      <c r="U14" s="80"/>
+      <c r="V14" s="80"/>
+      <c r="W14" s="81"/>
     </row>
     <row r="15" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="96"/>
+      <c r="B15" s="93"/>
       <c r="C15" s="29" t="s">
         <v>12</v>
       </c>
@@ -1959,15 +2074,15 @@
       <c r="Q15" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R15" s="72"/>
-      <c r="S15" s="73"/>
-      <c r="T15" s="73"/>
-      <c r="U15" s="73"/>
-      <c r="V15" s="73"/>
-      <c r="W15" s="74"/>
+      <c r="R15" s="82"/>
+      <c r="S15" s="83"/>
+      <c r="T15" s="83"/>
+      <c r="U15" s="83"/>
+      <c r="V15" s="83"/>
+      <c r="W15" s="84"/>
     </row>
     <row r="16" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="97"/>
+      <c r="B16" s="94"/>
       <c r="C16" s="30" t="s">
         <v>14</v>
       </c>
@@ -2013,16 +2128,16 @@
       <c r="Q16" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R16" s="75"/>
-      <c r="S16" s="76"/>
-      <c r="T16" s="76"/>
-      <c r="U16" s="76"/>
-      <c r="V16" s="76"/>
-      <c r="W16" s="77"/>
+      <c r="R16" s="85"/>
+      <c r="S16" s="86"/>
+      <c r="T16" s="86"/>
+      <c r="U16" s="86"/>
+      <c r="V16" s="86"/>
+      <c r="W16" s="87"/>
     </row>
     <row r="17" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7"/>
-      <c r="B17" s="101" t="s">
+      <c r="B17" s="89" t="s">
         <v>44</v>
       </c>
       <c r="C17" s="29" t="s">
@@ -2070,18 +2185,18 @@
       <c r="Q17" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R17" s="70" t="s">
+      <c r="R17" s="80" t="s">
         <v>43</v>
       </c>
-      <c r="S17" s="70"/>
-      <c r="T17" s="70"/>
-      <c r="U17" s="70"/>
-      <c r="V17" s="70"/>
-      <c r="W17" s="71"/>
+      <c r="S17" s="80"/>
+      <c r="T17" s="80"/>
+      <c r="U17" s="80"/>
+      <c r="V17" s="80"/>
+      <c r="W17" s="81"/>
     </row>
     <row r="18" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
-      <c r="B18" s="105"/>
+      <c r="B18" s="90"/>
       <c r="C18" s="29" t="s">
         <v>12</v>
       </c>
@@ -2127,16 +2242,16 @@
       <c r="Q18" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R18" s="73"/>
-      <c r="S18" s="73"/>
-      <c r="T18" s="73"/>
-      <c r="U18" s="73"/>
-      <c r="V18" s="73"/>
-      <c r="W18" s="74"/>
+      <c r="R18" s="83"/>
+      <c r="S18" s="83"/>
+      <c r="T18" s="83"/>
+      <c r="U18" s="83"/>
+      <c r="V18" s="83"/>
+      <c r="W18" s="84"/>
     </row>
     <row r="19" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7"/>
-      <c r="B19" s="104"/>
+      <c r="B19" s="91"/>
       <c r="C19" s="30" t="s">
         <v>14</v>
       </c>
@@ -2182,16 +2297,16 @@
       <c r="Q19" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R19" s="76"/>
-      <c r="S19" s="76"/>
-      <c r="T19" s="76"/>
-      <c r="U19" s="76"/>
-      <c r="V19" s="76"/>
-      <c r="W19" s="77"/>
+      <c r="R19" s="86"/>
+      <c r="S19" s="86"/>
+      <c r="T19" s="86"/>
+      <c r="U19" s="86"/>
+      <c r="V19" s="86"/>
+      <c r="W19" s="87"/>
     </row>
     <row r="20" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7"/>
-      <c r="B20" s="98" t="s">
+      <c r="B20" s="92" t="s">
         <v>46</v>
       </c>
       <c r="C20" s="29" t="s">
@@ -2239,18 +2354,18 @@
       <c r="Q20" s="35">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R20" s="69" t="s">
+      <c r="R20" s="79" t="s">
         <v>45</v>
       </c>
-      <c r="S20" s="70"/>
-      <c r="T20" s="70"/>
-      <c r="U20" s="70"/>
-      <c r="V20" s="70"/>
-      <c r="W20" s="71"/>
+      <c r="S20" s="80"/>
+      <c r="T20" s="80"/>
+      <c r="U20" s="80"/>
+      <c r="V20" s="80"/>
+      <c r="W20" s="81"/>
     </row>
     <row r="21" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
-      <c r="B21" s="96"/>
+      <c r="B21" s="93"/>
       <c r="C21" s="29" t="s">
         <v>12</v>
       </c>
@@ -2296,16 +2411,16 @@
       <c r="Q21" s="36">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R21" s="72"/>
-      <c r="S21" s="73"/>
-      <c r="T21" s="73"/>
-      <c r="U21" s="73"/>
-      <c r="V21" s="73"/>
-      <c r="W21" s="74"/>
+      <c r="R21" s="82"/>
+      <c r="S21" s="83"/>
+      <c r="T21" s="83"/>
+      <c r="U21" s="83"/>
+      <c r="V21" s="83"/>
+      <c r="W21" s="84"/>
     </row>
     <row r="22" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="7"/>
-      <c r="B22" s="97"/>
+      <c r="B22" s="94"/>
       <c r="C22" s="30" t="s">
         <v>14</v>
       </c>
@@ -2351,16 +2466,16 @@
       <c r="Q22" s="37">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R22" s="75"/>
-      <c r="S22" s="76"/>
-      <c r="T22" s="76"/>
-      <c r="U22" s="76"/>
-      <c r="V22" s="76"/>
-      <c r="W22" s="77"/>
+      <c r="R22" s="85"/>
+      <c r="S22" s="86"/>
+      <c r="T22" s="86"/>
+      <c r="U22" s="86"/>
+      <c r="V22" s="86"/>
+      <c r="W22" s="87"/>
     </row>
     <row r="23" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A23" s="58"/>
-      <c r="B23" s="66" t="s">
+      <c r="B23" s="67" t="s">
         <v>15</v>
       </c>
       <c r="C23" s="19" t="s">
@@ -2408,18 +2523,18 @@
       <c r="Q23" s="9">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R23" s="69" t="s">
+      <c r="R23" s="79" t="s">
         <v>53</v>
       </c>
-      <c r="S23" s="70"/>
-      <c r="T23" s="70"/>
-      <c r="U23" s="70"/>
-      <c r="V23" s="70"/>
-      <c r="W23" s="71"/>
+      <c r="S23" s="80"/>
+      <c r="T23" s="80"/>
+      <c r="U23" s="80"/>
+      <c r="V23" s="80"/>
+      <c r="W23" s="81"/>
     </row>
     <row r="24" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="58"/>
-      <c r="B24" s="67"/>
+      <c r="B24" s="68"/>
       <c r="C24" s="29" t="s">
         <v>12</v>
       </c>
@@ -2465,16 +2580,16 @@
       <c r="Q24" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R24" s="72"/>
-      <c r="S24" s="73"/>
-      <c r="T24" s="73"/>
-      <c r="U24" s="73"/>
-      <c r="V24" s="73"/>
-      <c r="W24" s="74"/>
+      <c r="R24" s="82"/>
+      <c r="S24" s="83"/>
+      <c r="T24" s="83"/>
+      <c r="U24" s="83"/>
+      <c r="V24" s="83"/>
+      <c r="W24" s="84"/>
     </row>
     <row r="25" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="58"/>
-      <c r="B25" s="68"/>
+      <c r="B25" s="69"/>
       <c r="C25" s="30" t="s">
         <v>14</v>
       </c>
@@ -2520,16 +2635,16 @@
       <c r="Q25" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R25" s="75"/>
-      <c r="S25" s="76"/>
-      <c r="T25" s="76"/>
-      <c r="U25" s="76"/>
-      <c r="V25" s="76"/>
-      <c r="W25" s="77"/>
+      <c r="R25" s="85"/>
+      <c r="S25" s="86"/>
+      <c r="T25" s="86"/>
+      <c r="U25" s="86"/>
+      <c r="V25" s="86"/>
+      <c r="W25" s="87"/>
     </row>
     <row r="26" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A26" s="58"/>
-      <c r="B26" s="66" t="s">
+      <c r="B26" s="67" t="s">
         <v>24</v>
       </c>
       <c r="C26" s="19" t="s">
@@ -2577,18 +2692,18 @@
       <c r="Q26" s="35">
         <v>1E-3</v>
       </c>
-      <c r="R26" s="87" t="s">
+      <c r="R26" s="88" t="s">
         <v>57</v>
       </c>
-      <c r="S26" s="70"/>
-      <c r="T26" s="70"/>
-      <c r="U26" s="70"/>
-      <c r="V26" s="70"/>
-      <c r="W26" s="71"/>
+      <c r="S26" s="80"/>
+      <c r="T26" s="80"/>
+      <c r="U26" s="80"/>
+      <c r="V26" s="80"/>
+      <c r="W26" s="81"/>
     </row>
     <row r="27" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="58"/>
-      <c r="B27" s="67"/>
+      <c r="B27" s="68"/>
       <c r="C27" s="29" t="s">
         <v>12</v>
       </c>
@@ -2634,16 +2749,16 @@
       <c r="Q27" s="36">
         <v>1E-3</v>
       </c>
-      <c r="R27" s="72"/>
-      <c r="S27" s="73"/>
-      <c r="T27" s="73"/>
-      <c r="U27" s="73"/>
-      <c r="V27" s="73"/>
-      <c r="W27" s="74"/>
+      <c r="R27" s="82"/>
+      <c r="S27" s="83"/>
+      <c r="T27" s="83"/>
+      <c r="U27" s="83"/>
+      <c r="V27" s="83"/>
+      <c r="W27" s="84"/>
     </row>
     <row r="28" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="58"/>
-      <c r="B28" s="68"/>
+      <c r="B28" s="69"/>
       <c r="C28" s="30" t="s">
         <v>14</v>
       </c>
@@ -2689,16 +2804,16 @@
       <c r="Q28" s="37">
         <v>1E-3</v>
       </c>
-      <c r="R28" s="75"/>
-      <c r="S28" s="76"/>
-      <c r="T28" s="76"/>
-      <c r="U28" s="76"/>
-      <c r="V28" s="76"/>
-      <c r="W28" s="77"/>
+      <c r="R28" s="85"/>
+      <c r="S28" s="86"/>
+      <c r="T28" s="86"/>
+      <c r="U28" s="86"/>
+      <c r="V28" s="86"/>
+      <c r="W28" s="87"/>
     </row>
     <row r="29" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A29" s="59"/>
-      <c r="B29" s="66" t="s">
+      <c r="B29" s="67" t="s">
         <v>34</v>
       </c>
       <c r="C29" s="28" t="s">
@@ -2746,18 +2861,18 @@
       <c r="Q29" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R29" s="69" t="s">
+      <c r="R29" s="79" t="s">
         <v>60</v>
       </c>
-      <c r="S29" s="70"/>
-      <c r="T29" s="70"/>
-      <c r="U29" s="70"/>
-      <c r="V29" s="70"/>
-      <c r="W29" s="71"/>
+      <c r="S29" s="80"/>
+      <c r="T29" s="80"/>
+      <c r="U29" s="80"/>
+      <c r="V29" s="80"/>
+      <c r="W29" s="81"/>
     </row>
     <row r="30" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="58"/>
-      <c r="B30" s="67"/>
+      <c r="B30" s="68"/>
       <c r="C30" s="25" t="s">
         <v>12</v>
       </c>
@@ -2803,16 +2918,16 @@
       <c r="Q30" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R30" s="72"/>
-      <c r="S30" s="73"/>
-      <c r="T30" s="73"/>
-      <c r="U30" s="73"/>
-      <c r="V30" s="73"/>
-      <c r="W30" s="74"/>
+      <c r="R30" s="82"/>
+      <c r="S30" s="83"/>
+      <c r="T30" s="83"/>
+      <c r="U30" s="83"/>
+      <c r="V30" s="83"/>
+      <c r="W30" s="84"/>
     </row>
     <row r="31" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="58"/>
-      <c r="B31" s="68"/>
+      <c r="B31" s="69"/>
       <c r="C31" s="42" t="s">
         <v>14</v>
       </c>
@@ -2858,16 +2973,16 @@
       <c r="Q31" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R31" s="75"/>
-      <c r="S31" s="76"/>
-      <c r="T31" s="76"/>
-      <c r="U31" s="76"/>
-      <c r="V31" s="76"/>
-      <c r="W31" s="77"/>
+      <c r="R31" s="85"/>
+      <c r="S31" s="86"/>
+      <c r="T31" s="86"/>
+      <c r="U31" s="86"/>
+      <c r="V31" s="86"/>
+      <c r="W31" s="87"/>
     </row>
     <row r="32" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A32" s="59"/>
-      <c r="B32" s="66" t="s">
+      <c r="B32" s="67" t="s">
         <v>36</v>
       </c>
       <c r="C32" s="28" t="s">
@@ -2915,18 +3030,18 @@
       <c r="Q32" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R32" s="87" t="s">
+      <c r="R32" s="88" t="s">
         <v>61</v>
       </c>
-      <c r="S32" s="70"/>
-      <c r="T32" s="70"/>
-      <c r="U32" s="70"/>
-      <c r="V32" s="70"/>
-      <c r="W32" s="71"/>
+      <c r="S32" s="80"/>
+      <c r="T32" s="80"/>
+      <c r="U32" s="80"/>
+      <c r="V32" s="80"/>
+      <c r="W32" s="81"/>
     </row>
     <row r="33" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="59"/>
-      <c r="B33" s="67"/>
+      <c r="B33" s="68"/>
       <c r="C33" s="25" t="s">
         <v>12</v>
       </c>
@@ -2972,16 +3087,16 @@
       <c r="Q33" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R33" s="72"/>
-      <c r="S33" s="73"/>
-      <c r="T33" s="73"/>
-      <c r="U33" s="73"/>
-      <c r="V33" s="73"/>
-      <c r="W33" s="74"/>
+      <c r="R33" s="82"/>
+      <c r="S33" s="83"/>
+      <c r="T33" s="83"/>
+      <c r="U33" s="83"/>
+      <c r="V33" s="83"/>
+      <c r="W33" s="84"/>
     </row>
     <row r="34" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="59"/>
-      <c r="B34" s="68"/>
+      <c r="B34" s="69"/>
       <c r="C34" s="42" t="s">
         <v>14</v>
       </c>
@@ -3027,16 +3142,16 @@
       <c r="Q34" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R34" s="75"/>
-      <c r="S34" s="76"/>
-      <c r="T34" s="76"/>
-      <c r="U34" s="76"/>
-      <c r="V34" s="76"/>
-      <c r="W34" s="77"/>
+      <c r="R34" s="85"/>
+      <c r="S34" s="86"/>
+      <c r="T34" s="86"/>
+      <c r="U34" s="86"/>
+      <c r="V34" s="86"/>
+      <c r="W34" s="87"/>
     </row>
     <row r="35" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A35" s="58"/>
-      <c r="B35" s="66" t="s">
+      <c r="B35" s="67" t="s">
         <v>44</v>
       </c>
       <c r="C35" s="25" t="s">
@@ -3084,18 +3199,18 @@
       <c r="Q35" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R35" s="69" t="s">
+      <c r="R35" s="79" t="s">
         <v>63</v>
       </c>
-      <c r="S35" s="70"/>
-      <c r="T35" s="70"/>
-      <c r="U35" s="70"/>
-      <c r="V35" s="70"/>
-      <c r="W35" s="71"/>
+      <c r="S35" s="80"/>
+      <c r="T35" s="80"/>
+      <c r="U35" s="80"/>
+      <c r="V35" s="80"/>
+      <c r="W35" s="81"/>
     </row>
     <row r="36" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="58"/>
-      <c r="B36" s="67"/>
+      <c r="B36" s="68"/>
       <c r="C36" s="25" t="s">
         <v>12</v>
       </c>
@@ -3141,16 +3256,16 @@
       <c r="Q36" s="36">
         <v>1E-3</v>
       </c>
-      <c r="R36" s="72"/>
-      <c r="S36" s="73"/>
-      <c r="T36" s="73"/>
-      <c r="U36" s="73"/>
-      <c r="V36" s="73"/>
-      <c r="W36" s="74"/>
+      <c r="R36" s="82"/>
+      <c r="S36" s="83"/>
+      <c r="T36" s="83"/>
+      <c r="U36" s="83"/>
+      <c r="V36" s="83"/>
+      <c r="W36" s="84"/>
     </row>
     <row r="37" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="58"/>
-      <c r="B37" s="68"/>
+      <c r="B37" s="69"/>
       <c r="C37" s="30" t="s">
         <v>14</v>
       </c>
@@ -3196,16 +3311,16 @@
       <c r="Q37" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R37" s="75"/>
-      <c r="S37" s="76"/>
-      <c r="T37" s="76"/>
-      <c r="U37" s="76"/>
-      <c r="V37" s="76"/>
-      <c r="W37" s="77"/>
+      <c r="R37" s="85"/>
+      <c r="S37" s="86"/>
+      <c r="T37" s="86"/>
+      <c r="U37" s="86"/>
+      <c r="V37" s="86"/>
+      <c r="W37" s="87"/>
     </row>
     <row r="38" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A38" s="59"/>
-      <c r="B38" s="66" t="s">
+      <c r="B38" s="67" t="s">
         <v>46</v>
       </c>
       <c r="C38" s="19" t="s">
@@ -3253,16 +3368,16 @@
       <c r="Q38" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R38" s="78"/>
-      <c r="S38" s="79"/>
-      <c r="T38" s="79"/>
-      <c r="U38" s="79"/>
-      <c r="V38" s="79"/>
-      <c r="W38" s="80"/>
+      <c r="R38" s="106"/>
+      <c r="S38" s="71"/>
+      <c r="T38" s="71"/>
+      <c r="U38" s="71"/>
+      <c r="V38" s="71"/>
+      <c r="W38" s="72"/>
     </row>
     <row r="39" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="59"/>
-      <c r="B39" s="67"/>
+      <c r="B39" s="68"/>
       <c r="C39" s="29" t="s">
         <v>12</v>
       </c>
@@ -3308,16 +3423,16 @@
       <c r="Q39" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R39" s="81"/>
-      <c r="S39" s="82"/>
-      <c r="T39" s="82"/>
-      <c r="U39" s="82"/>
-      <c r="V39" s="82"/>
-      <c r="W39" s="83"/>
+      <c r="R39" s="73"/>
+      <c r="S39" s="74"/>
+      <c r="T39" s="74"/>
+      <c r="U39" s="74"/>
+      <c r="V39" s="74"/>
+      <c r="W39" s="75"/>
     </row>
     <row r="40" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="59"/>
-      <c r="B40" s="68"/>
+      <c r="B40" s="69"/>
       <c r="C40" s="30" t="s">
         <v>14</v>
       </c>
@@ -3363,16 +3478,16 @@
       <c r="Q40" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R40" s="84"/>
-      <c r="S40" s="85"/>
-      <c r="T40" s="85"/>
-      <c r="U40" s="85"/>
-      <c r="V40" s="85"/>
-      <c r="W40" s="86"/>
+      <c r="R40" s="76"/>
+      <c r="S40" s="77"/>
+      <c r="T40" s="77"/>
+      <c r="U40" s="77"/>
+      <c r="V40" s="77"/>
+      <c r="W40" s="78"/>
     </row>
     <row r="41" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A41" s="59"/>
-      <c r="B41" s="66" t="s">
+      <c r="B41" s="67" t="s">
         <v>50</v>
       </c>
       <c r="C41" s="29" t="s">
@@ -3420,18 +3535,18 @@
       <c r="Q41" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R41" s="87" t="s">
+      <c r="R41" s="88" t="s">
         <v>71</v>
       </c>
-      <c r="S41" s="70"/>
-      <c r="T41" s="70"/>
-      <c r="U41" s="70"/>
-      <c r="V41" s="70"/>
-      <c r="W41" s="71"/>
+      <c r="S41" s="80"/>
+      <c r="T41" s="80"/>
+      <c r="U41" s="80"/>
+      <c r="V41" s="80"/>
+      <c r="W41" s="81"/>
     </row>
     <row r="42" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="59"/>
-      <c r="B42" s="67"/>
+      <c r="B42" s="68"/>
       <c r="C42" s="29" t="s">
         <v>12</v>
       </c>
@@ -3477,16 +3592,16 @@
       <c r="Q42" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R42" s="72"/>
-      <c r="S42" s="73"/>
-      <c r="T42" s="73"/>
-      <c r="U42" s="73"/>
-      <c r="V42" s="73"/>
-      <c r="W42" s="74"/>
+      <c r="R42" s="82"/>
+      <c r="S42" s="83"/>
+      <c r="T42" s="83"/>
+      <c r="U42" s="83"/>
+      <c r="V42" s="83"/>
+      <c r="W42" s="84"/>
     </row>
     <row r="43" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="59"/>
-      <c r="B43" s="67"/>
+      <c r="B43" s="68"/>
       <c r="C43" s="29" t="s">
         <v>14</v>
       </c>
@@ -3532,16 +3647,16 @@
       <c r="Q43" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R43" s="72"/>
-      <c r="S43" s="73"/>
-      <c r="T43" s="73"/>
-      <c r="U43" s="73"/>
-      <c r="V43" s="73"/>
-      <c r="W43" s="74"/>
+      <c r="R43" s="82"/>
+      <c r="S43" s="83"/>
+      <c r="T43" s="83"/>
+      <c r="U43" s="83"/>
+      <c r="V43" s="83"/>
+      <c r="W43" s="84"/>
     </row>
     <row r="44" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="59"/>
-      <c r="B44" s="68"/>
+      <c r="B44" s="69"/>
       <c r="C44" s="30" t="s">
         <v>67</v>
       </c>
@@ -3587,16 +3702,16 @@
       <c r="Q44" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R44" s="75"/>
-      <c r="S44" s="76"/>
-      <c r="T44" s="76"/>
-      <c r="U44" s="76"/>
-      <c r="V44" s="76"/>
-      <c r="W44" s="77"/>
+      <c r="R44" s="85"/>
+      <c r="S44" s="86"/>
+      <c r="T44" s="86"/>
+      <c r="U44" s="86"/>
+      <c r="V44" s="86"/>
+      <c r="W44" s="87"/>
     </row>
     <row r="45" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A45" s="59"/>
-      <c r="B45" s="66" t="s">
+      <c r="B45" s="67" t="s">
         <v>55</v>
       </c>
       <c r="C45" s="29" t="s">
@@ -3644,18 +3759,18 @@
       <c r="Q45" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R45" s="88" t="s">
+      <c r="R45" s="70" t="s">
         <v>72</v>
       </c>
-      <c r="S45" s="79"/>
-      <c r="T45" s="79"/>
-      <c r="U45" s="79"/>
-      <c r="V45" s="79"/>
-      <c r="W45" s="80"/>
+      <c r="S45" s="71"/>
+      <c r="T45" s="71"/>
+      <c r="U45" s="71"/>
+      <c r="V45" s="71"/>
+      <c r="W45" s="72"/>
     </row>
     <row r="46" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="59"/>
-      <c r="B46" s="67"/>
+      <c r="B46" s="68"/>
       <c r="C46" s="29" t="s">
         <v>12</v>
       </c>
@@ -3701,16 +3816,16 @@
       <c r="Q46" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R46" s="81"/>
-      <c r="S46" s="82"/>
-      <c r="T46" s="82"/>
-      <c r="U46" s="82"/>
-      <c r="V46" s="82"/>
-      <c r="W46" s="83"/>
+      <c r="R46" s="73"/>
+      <c r="S46" s="74"/>
+      <c r="T46" s="74"/>
+      <c r="U46" s="74"/>
+      <c r="V46" s="74"/>
+      <c r="W46" s="75"/>
     </row>
     <row r="47" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="59"/>
-      <c r="B47" s="67"/>
+      <c r="B47" s="68"/>
       <c r="C47" s="29" t="s">
         <v>14</v>
       </c>
@@ -3756,16 +3871,16 @@
       <c r="Q47" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R47" s="81"/>
-      <c r="S47" s="82"/>
-      <c r="T47" s="82"/>
-      <c r="U47" s="82"/>
-      <c r="V47" s="82"/>
-      <c r="W47" s="83"/>
+      <c r="R47" s="73"/>
+      <c r="S47" s="74"/>
+      <c r="T47" s="74"/>
+      <c r="U47" s="74"/>
+      <c r="V47" s="74"/>
+      <c r="W47" s="75"/>
     </row>
     <row r="48" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="59"/>
-      <c r="B48" s="68"/>
+      <c r="B48" s="69"/>
       <c r="C48" s="30" t="s">
         <v>67</v>
       </c>
@@ -3811,16 +3926,16 @@
       <c r="Q48" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R48" s="84"/>
-      <c r="S48" s="85"/>
-      <c r="T48" s="85"/>
-      <c r="U48" s="85"/>
-      <c r="V48" s="85"/>
-      <c r="W48" s="86"/>
+      <c r="R48" s="76"/>
+      <c r="S48" s="77"/>
+      <c r="T48" s="77"/>
+      <c r="U48" s="77"/>
+      <c r="V48" s="77"/>
+      <c r="W48" s="78"/>
     </row>
     <row r="49" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A49" s="58"/>
-      <c r="B49" s="66" t="s">
+      <c r="B49" s="67" t="s">
         <v>58</v>
       </c>
       <c r="C49" s="29" t="s">
@@ -3868,18 +3983,18 @@
       <c r="Q49" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R49" s="69" t="s">
+      <c r="R49" s="79" t="s">
         <v>79</v>
       </c>
-      <c r="S49" s="70"/>
-      <c r="T49" s="70"/>
-      <c r="U49" s="70"/>
-      <c r="V49" s="70"/>
-      <c r="W49" s="71"/>
+      <c r="S49" s="80"/>
+      <c r="T49" s="80"/>
+      <c r="U49" s="80"/>
+      <c r="V49" s="80"/>
+      <c r="W49" s="81"/>
     </row>
     <row r="50" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="58"/>
-      <c r="B50" s="67"/>
+      <c r="B50" s="68"/>
       <c r="C50" s="29" t="s">
         <v>12</v>
       </c>
@@ -3925,16 +4040,16 @@
       <c r="Q50" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R50" s="72"/>
-      <c r="S50" s="73"/>
-      <c r="T50" s="73"/>
-      <c r="U50" s="73"/>
-      <c r="V50" s="73"/>
-      <c r="W50" s="74"/>
+      <c r="R50" s="82"/>
+      <c r="S50" s="83"/>
+      <c r="T50" s="83"/>
+      <c r="U50" s="83"/>
+      <c r="V50" s="83"/>
+      <c r="W50" s="84"/>
     </row>
     <row r="51" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="58"/>
-      <c r="B51" s="67"/>
+      <c r="B51" s="68"/>
       <c r="C51" s="29" t="s">
         <v>14</v>
       </c>
@@ -3980,16 +4095,16 @@
       <c r="Q51" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R51" s="72"/>
-      <c r="S51" s="73"/>
-      <c r="T51" s="73"/>
-      <c r="U51" s="73"/>
-      <c r="V51" s="73"/>
-      <c r="W51" s="74"/>
+      <c r="R51" s="82"/>
+      <c r="S51" s="83"/>
+      <c r="T51" s="83"/>
+      <c r="U51" s="83"/>
+      <c r="V51" s="83"/>
+      <c r="W51" s="84"/>
     </row>
     <row r="52" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="58"/>
-      <c r="B52" s="68"/>
+      <c r="B52" s="69"/>
       <c r="C52" s="30" t="s">
         <v>67</v>
       </c>
@@ -4035,16 +4150,16 @@
       <c r="Q52" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R52" s="75"/>
-      <c r="S52" s="76"/>
-      <c r="T52" s="76"/>
-      <c r="U52" s="76"/>
-      <c r="V52" s="76"/>
-      <c r="W52" s="77"/>
-    </row>
-    <row r="53" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="R52" s="85"/>
+      <c r="S52" s="86"/>
+      <c r="T52" s="86"/>
+      <c r="U52" s="86"/>
+      <c r="V52" s="86"/>
+      <c r="W52" s="87"/>
+    </row>
+    <row r="53" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A53" s="59"/>
-      <c r="B53" s="66" t="s">
+      <c r="B53" s="67" t="s">
         <v>77</v>
       </c>
       <c r="C53" s="19" t="s">
@@ -4092,18 +4207,18 @@
       <c r="Q53" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R53" s="69" t="s">
+      <c r="R53" s="79" t="s">
         <v>80</v>
       </c>
-      <c r="S53" s="70"/>
-      <c r="T53" s="70"/>
-      <c r="U53" s="70"/>
-      <c r="V53" s="70"/>
-      <c r="W53" s="71"/>
-    </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="S53" s="80"/>
+      <c r="T53" s="80"/>
+      <c r="U53" s="80"/>
+      <c r="V53" s="80"/>
+      <c r="W53" s="81"/>
+    </row>
+    <row r="54" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="59"/>
-      <c r="B54" s="67"/>
+      <c r="B54" s="68"/>
       <c r="C54" s="29" t="s">
         <v>12</v>
       </c>
@@ -4149,16 +4264,16 @@
       <c r="Q54" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R54" s="72"/>
-      <c r="S54" s="73"/>
-      <c r="T54" s="73"/>
-      <c r="U54" s="73"/>
-      <c r="V54" s="73"/>
-      <c r="W54" s="74"/>
-    </row>
-    <row r="55" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="R54" s="82"/>
+      <c r="S54" s="83"/>
+      <c r="T54" s="83"/>
+      <c r="U54" s="83"/>
+      <c r="V54" s="83"/>
+      <c r="W54" s="84"/>
+    </row>
+    <row r="55" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="59"/>
-      <c r="B55" s="67"/>
+      <c r="B55" s="68"/>
       <c r="C55" s="29" t="s">
         <v>14</v>
       </c>
@@ -4204,16 +4319,16 @@
       <c r="Q55" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R55" s="72"/>
-      <c r="S55" s="73"/>
-      <c r="T55" s="73"/>
-      <c r="U55" s="73"/>
-      <c r="V55" s="73"/>
-      <c r="W55" s="74"/>
-    </row>
-    <row r="56" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R55" s="82"/>
+      <c r="S55" s="83"/>
+      <c r="T55" s="83"/>
+      <c r="U55" s="83"/>
+      <c r="V55" s="83"/>
+      <c r="W55" s="84"/>
+    </row>
+    <row r="56" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="59"/>
-      <c r="B56" s="68"/>
+      <c r="B56" s="69"/>
       <c r="C56" s="30" t="s">
         <v>67</v>
       </c>
@@ -4259,16 +4374,16 @@
       <c r="Q56" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R56" s="75"/>
-      <c r="S56" s="76"/>
-      <c r="T56" s="76"/>
-      <c r="U56" s="76"/>
-      <c r="V56" s="76"/>
-      <c r="W56" s="77"/>
-    </row>
-    <row r="57" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="R56" s="85"/>
+      <c r="S56" s="86"/>
+      <c r="T56" s="86"/>
+      <c r="U56" s="86"/>
+      <c r="V56" s="86"/>
+      <c r="W56" s="87"/>
+    </row>
+    <row r="57" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A57" s="58"/>
-      <c r="B57" s="66" t="s">
+      <c r="B57" s="67" t="s">
         <v>81</v>
       </c>
       <c r="C57" s="19" t="s">
@@ -4316,18 +4431,18 @@
       <c r="Q57" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R57" s="69" t="s">
-        <v>82</v>
-      </c>
-      <c r="S57" s="70"/>
-      <c r="T57" s="70"/>
-      <c r="U57" s="70"/>
-      <c r="V57" s="70"/>
-      <c r="W57" s="71"/>
-    </row>
-    <row r="58" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="R57" s="79" t="s">
+        <v>87</v>
+      </c>
+      <c r="S57" s="80"/>
+      <c r="T57" s="80"/>
+      <c r="U57" s="80"/>
+      <c r="V57" s="80"/>
+      <c r="W57" s="81"/>
+    </row>
+    <row r="58" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="58"/>
-      <c r="B58" s="67"/>
+      <c r="B58" s="68"/>
       <c r="C58" s="29" t="s">
         <v>12</v>
       </c>
@@ -4373,16 +4488,16 @@
       <c r="Q58" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R58" s="72"/>
-      <c r="S58" s="73"/>
-      <c r="T58" s="73"/>
-      <c r="U58" s="73"/>
-      <c r="V58" s="73"/>
-      <c r="W58" s="74"/>
-    </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="R58" s="82"/>
+      <c r="S58" s="83"/>
+      <c r="T58" s="83"/>
+      <c r="U58" s="83"/>
+      <c r="V58" s="83"/>
+      <c r="W58" s="84"/>
+    </row>
+    <row r="59" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="58"/>
-      <c r="B59" s="67"/>
+      <c r="B59" s="68"/>
       <c r="C59" s="29" t="s">
         <v>14</v>
       </c>
@@ -4428,16 +4543,16 @@
       <c r="Q59" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R59" s="72"/>
-      <c r="S59" s="73"/>
-      <c r="T59" s="73"/>
-      <c r="U59" s="73"/>
-      <c r="V59" s="73"/>
-      <c r="W59" s="74"/>
-    </row>
-    <row r="60" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R59" s="82"/>
+      <c r="S59" s="83"/>
+      <c r="T59" s="83"/>
+      <c r="U59" s="83"/>
+      <c r="V59" s="83"/>
+      <c r="W59" s="84"/>
+    </row>
+    <row r="60" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="58"/>
-      <c r="B60" s="68"/>
+      <c r="B60" s="69"/>
       <c r="C60" s="30" t="s">
         <v>67</v>
       </c>
@@ -4483,17 +4598,17 @@
       <c r="Q60" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R60" s="75"/>
-      <c r="S60" s="76"/>
-      <c r="T60" s="76"/>
-      <c r="U60" s="76"/>
-      <c r="V60" s="76"/>
-      <c r="W60" s="77"/>
-    </row>
-    <row r="61" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="R60" s="85"/>
+      <c r="S60" s="86"/>
+      <c r="T60" s="86"/>
+      <c r="U60" s="86"/>
+      <c r="V60" s="86"/>
+      <c r="W60" s="87"/>
+    </row>
+    <row r="61" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A61" s="7"/>
-      <c r="B61" s="66" t="s">
-        <v>85</v>
+      <c r="B61" s="67" t="s">
+        <v>84</v>
       </c>
       <c r="C61" s="28" t="s">
         <v>13</v>
@@ -4540,18 +4655,18 @@
       <c r="Q61" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R61" s="88" t="s">
-        <v>86</v>
-      </c>
-      <c r="S61" s="79"/>
-      <c r="T61" s="79"/>
-      <c r="U61" s="79"/>
-      <c r="V61" s="79"/>
-      <c r="W61" s="80"/>
-    </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="R61" s="70" t="s">
+        <v>85</v>
+      </c>
+      <c r="S61" s="71"/>
+      <c r="T61" s="71"/>
+      <c r="U61" s="71"/>
+      <c r="V61" s="71"/>
+      <c r="W61" s="72"/>
+    </row>
+    <row r="62" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="7"/>
-      <c r="B62" s="67"/>
+      <c r="B62" s="68"/>
       <c r="C62" s="25" t="s">
         <v>12</v>
       </c>
@@ -4580,7 +4695,7 @@
         <v>6</v>
       </c>
       <c r="L62" s="31" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="M62">
         <v>64</v>
@@ -4597,16 +4712,16 @@
       <c r="Q62" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R62" s="81"/>
-      <c r="S62" s="82"/>
-      <c r="T62" s="82"/>
-      <c r="U62" s="82"/>
-      <c r="V62" s="82"/>
-      <c r="W62" s="83"/>
-    </row>
-    <row r="63" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="R62" s="73"/>
+      <c r="S62" s="74"/>
+      <c r="T62" s="74"/>
+      <c r="U62" s="74"/>
+      <c r="V62" s="74"/>
+      <c r="W62" s="75"/>
+    </row>
+    <row r="63" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="67"/>
+      <c r="B63" s="68"/>
       <c r="C63" s="25" t="s">
         <v>14</v>
       </c>
@@ -4652,16 +4767,16 @@
       <c r="Q63" s="64">
         <v>1E-3</v>
       </c>
-      <c r="R63" s="81"/>
-      <c r="S63" s="82"/>
-      <c r="T63" s="82"/>
-      <c r="U63" s="82"/>
-      <c r="V63" s="82"/>
-      <c r="W63" s="83"/>
-    </row>
-    <row r="64" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="R63" s="73"/>
+      <c r="S63" s="74"/>
+      <c r="T63" s="74"/>
+      <c r="U63" s="74"/>
+      <c r="V63" s="74"/>
+      <c r="W63" s="75"/>
+    </row>
+    <row r="64" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="67"/>
+      <c r="B64" s="68"/>
       <c r="C64" s="25" t="s">
         <v>67</v>
       </c>
@@ -4707,71 +4822,538 @@
       <c r="Q64" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R64" s="81"/>
-      <c r="S64" s="82"/>
-      <c r="T64" s="82"/>
-      <c r="U64" s="82"/>
-      <c r="V64" s="82"/>
-      <c r="W64" s="83"/>
-    </row>
-    <row r="65" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R64" s="73"/>
+      <c r="S64" s="74"/>
+      <c r="T64" s="74"/>
+      <c r="U64" s="74"/>
+      <c r="V64" s="74"/>
+      <c r="W64" s="75"/>
+    </row>
+    <row r="65" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="7"/>
-      <c r="B65" s="68"/>
-      <c r="C65" s="30" t="s">
-        <v>84</v>
-      </c>
-      <c r="D65" s="3">
+      <c r="B65" s="69"/>
+      <c r="C65" s="107" t="s">
+        <v>83</v>
+      </c>
+      <c r="D65" s="108">
         <v>122.208</v>
       </c>
-      <c r="E65" s="3">
+      <c r="E65" s="108">
         <v>174.66300000000001</v>
       </c>
-      <c r="F65" s="3">
+      <c r="F65" s="108">
         <v>0.8216</v>
       </c>
-      <c r="G65" s="3">
+      <c r="G65" s="108">
         <v>0.82150000000000001</v>
       </c>
-      <c r="H65" s="4">
+      <c r="H65" s="109">
         <v>20.3</v>
       </c>
-      <c r="I65" s="2">
+      <c r="I65" s="110">
         <v>18</v>
       </c>
-      <c r="J65" s="3">
+      <c r="J65" s="108">
         <v>132.01</v>
       </c>
-      <c r="K65" s="3">
-        <v>6</v>
-      </c>
-      <c r="L65" s="34" t="s">
+      <c r="K65" s="108">
+        <v>6</v>
+      </c>
+      <c r="L65" s="111" t="s">
         <v>49</v>
       </c>
-      <c r="M65" s="3">
-        <v>64</v>
-      </c>
-      <c r="N65" s="3">
+      <c r="M65" s="108">
+        <v>64</v>
+      </c>
+      <c r="N65" s="108">
         <v>32</v>
       </c>
-      <c r="O65" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="P65" s="3">
+      <c r="O65" s="111" t="s">
+        <v>39</v>
+      </c>
+      <c r="P65" s="108">
         <v>0.1</v>
       </c>
-      <c r="Q65" s="4">
+      <c r="Q65" s="109">
         <v>1E-3</v>
       </c>
-      <c r="R65" s="84"/>
-      <c r="S65" s="85"/>
-      <c r="T65" s="85"/>
-      <c r="U65" s="85"/>
-      <c r="V65" s="85"/>
-      <c r="W65" s="86"/>
-    </row>
-    <row r="66" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+      <c r="R65" s="76"/>
+      <c r="S65" s="77"/>
+      <c r="T65" s="77"/>
+      <c r="U65" s="77"/>
+      <c r="V65" s="77"/>
+      <c r="W65" s="78"/>
+    </row>
+    <row r="66" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B66" s="67" t="s">
+        <v>86</v>
+      </c>
+      <c r="C66" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D66" s="134">
+        <v>48.537999999999997</v>
+      </c>
+      <c r="E66" s="134">
+        <v>96.697000000000003</v>
+      </c>
+      <c r="F66" s="134">
+        <v>0.94530000000000003</v>
+      </c>
+      <c r="G66" s="134">
+        <v>0.94530000000000003</v>
+      </c>
+      <c r="H66" s="135">
+        <v>22.4</v>
+      </c>
+      <c r="I66" s="8">
+        <v>18</v>
+      </c>
+      <c r="J66" s="8">
+        <v>196.4</v>
+      </c>
+      <c r="K66" s="8">
+        <v>6</v>
+      </c>
+      <c r="L66" s="39">
+        <v>60</v>
+      </c>
+      <c r="M66" s="8">
+        <v>64</v>
+      </c>
+      <c r="N66" s="8">
+        <v>64</v>
+      </c>
+      <c r="O66" s="39" t="s">
+        <v>39</v>
+      </c>
+      <c r="P66" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="Q66" s="9">
+        <v>1E-3</v>
+      </c>
+      <c r="R66" s="117" t="s">
+        <v>88</v>
+      </c>
+      <c r="S66" s="71"/>
+      <c r="T66" s="71"/>
+      <c r="U66" s="71"/>
+      <c r="V66" s="71"/>
+      <c r="W66" s="72"/>
+    </row>
+    <row r="67" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B67" s="68"/>
+      <c r="C67" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="D67" s="114">
+        <v>51.738</v>
+      </c>
+      <c r="E67" s="114">
+        <v>92.930999999999997</v>
+      </c>
+      <c r="F67" s="114">
+        <v>0.94950000000000001</v>
+      </c>
+      <c r="G67" s="114">
+        <v>0.94950000000000001</v>
+      </c>
+      <c r="H67" s="7">
+        <v>22.6</v>
+      </c>
+      <c r="I67" s="114">
+        <v>18</v>
+      </c>
+      <c r="J67" s="114">
+        <v>332.8</v>
+      </c>
+      <c r="K67" s="114">
+        <v>6</v>
+      </c>
+      <c r="L67" s="116">
+        <v>71</v>
+      </c>
+      <c r="M67" s="114">
+        <v>64</v>
+      </c>
+      <c r="N67" s="114">
+        <v>32</v>
+      </c>
+      <c r="O67" s="115" t="s">
+        <v>39</v>
+      </c>
+      <c r="P67" s="114">
+        <v>0.1</v>
+      </c>
+      <c r="Q67" s="7">
+        <v>1E-3</v>
+      </c>
+      <c r="R67" s="73"/>
+      <c r="S67" s="113"/>
+      <c r="T67" s="113"/>
+      <c r="U67" s="113"/>
+      <c r="V67" s="113"/>
+      <c r="W67" s="75"/>
+    </row>
+    <row r="68" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B68" s="68"/>
+      <c r="C68" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="D68" s="114">
+        <v>48.079000000000001</v>
+      </c>
+      <c r="E68" s="114">
+        <v>102.464</v>
+      </c>
+      <c r="F68" s="114">
+        <v>0.93859999999999999</v>
+      </c>
+      <c r="G68" s="114">
+        <v>0.93859999999999999</v>
+      </c>
+      <c r="H68" s="7">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="I68" s="114">
+        <v>18</v>
+      </c>
+      <c r="J68" s="114">
+        <v>546.79999999999995</v>
+      </c>
+      <c r="K68" s="114">
+        <v>6</v>
+      </c>
+      <c r="L68" s="116">
+        <v>106</v>
+      </c>
+      <c r="M68" s="114">
+        <v>64</v>
+      </c>
+      <c r="N68" s="114">
+        <v>32</v>
+      </c>
+      <c r="O68" s="116" t="s">
+        <v>39</v>
+      </c>
+      <c r="P68" s="114">
+        <v>0.1</v>
+      </c>
+      <c r="Q68" s="7">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R68" s="73"/>
+      <c r="S68" s="113"/>
+      <c r="T68" s="113"/>
+      <c r="U68" s="113"/>
+      <c r="V68" s="113"/>
+      <c r="W68" s="75"/>
+    </row>
+    <row r="69" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B69" s="119"/>
+      <c r="C69" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="D69" s="114">
+        <v>63.225000000000001</v>
+      </c>
+      <c r="E69" s="114">
+        <v>123.163</v>
+      </c>
+      <c r="F69" s="114">
+        <v>0.9113</v>
+      </c>
+      <c r="G69" s="121">
+        <v>0.91120000000000001</v>
+      </c>
+      <c r="H69" s="122">
+        <v>38.4</v>
+      </c>
+      <c r="I69" s="123">
+        <v>18</v>
+      </c>
+      <c r="J69" s="114">
+        <v>152.30000000000001</v>
+      </c>
+      <c r="K69" s="121">
+        <v>6</v>
+      </c>
+      <c r="L69" s="115">
+        <v>59</v>
+      </c>
+      <c r="M69" s="112">
+        <v>64</v>
+      </c>
+      <c r="N69" s="112">
+        <v>32</v>
+      </c>
+      <c r="O69" s="115" t="s">
+        <v>39</v>
+      </c>
+      <c r="P69" s="112">
+        <v>0.1</v>
+      </c>
+      <c r="Q69" s="7">
+        <v>1E-3</v>
+      </c>
+      <c r="R69" s="126"/>
+      <c r="S69" s="127"/>
+      <c r="T69" s="127"/>
+      <c r="U69" s="127"/>
+      <c r="V69" s="127"/>
+      <c r="W69" s="128"/>
+    </row>
+    <row r="70" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B70" s="118" t="s">
+        <v>89</v>
+      </c>
+      <c r="C70" s="120" t="s">
+        <v>13</v>
+      </c>
+      <c r="D70" s="129">
+        <v>117.86</v>
+      </c>
+      <c r="E70" s="130">
+        <v>155.45699999999999</v>
+      </c>
+      <c r="F70" s="130">
+        <v>0.78659999999999997</v>
+      </c>
+      <c r="G70" s="114">
+        <v>0.78620000000000001</v>
+      </c>
+      <c r="H70" s="131">
+        <v>22.4</v>
+      </c>
+      <c r="I70" s="112">
+        <v>18</v>
+      </c>
+      <c r="J70" s="15">
+        <v>196.4</v>
+      </c>
+      <c r="K70" s="112">
+        <v>6</v>
+      </c>
+      <c r="L70" s="23">
+        <v>60</v>
+      </c>
+      <c r="M70" s="15">
+        <v>64</v>
+      </c>
+      <c r="N70" s="15">
+        <v>64</v>
+      </c>
+      <c r="O70" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="P70" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="Q70" s="16">
+        <v>1E-3</v>
+      </c>
+      <c r="R70" s="82" t="s">
+        <v>90</v>
+      </c>
+      <c r="S70" s="125"/>
+      <c r="T70" s="125"/>
+      <c r="U70" s="125"/>
+      <c r="V70" s="125"/>
+      <c r="W70" s="84"/>
+    </row>
+    <row r="71" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B71" s="68"/>
+      <c r="C71" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="D71" s="124">
+        <v>118.28</v>
+      </c>
+      <c r="E71" s="114">
+        <v>149.739</v>
+      </c>
+      <c r="F71" s="114">
+        <v>0.80200000000000005</v>
+      </c>
+      <c r="G71" s="114">
+        <v>0.80159999999999998</v>
+      </c>
+      <c r="H71" s="131">
+        <v>22.6</v>
+      </c>
+      <c r="I71" s="112">
+        <v>18</v>
+      </c>
+      <c r="J71" s="112">
+        <v>332.8</v>
+      </c>
+      <c r="K71" s="112">
+        <v>6</v>
+      </c>
+      <c r="L71" s="115">
+        <v>71</v>
+      </c>
+      <c r="M71" s="112">
+        <v>64</v>
+      </c>
+      <c r="N71" s="112">
+        <v>32</v>
+      </c>
+      <c r="O71" s="115" t="s">
+        <v>39</v>
+      </c>
+      <c r="P71" s="112">
+        <v>0.1</v>
+      </c>
+      <c r="Q71" s="7">
+        <v>1E-3</v>
+      </c>
+      <c r="R71" s="82"/>
+      <c r="S71" s="125"/>
+      <c r="T71" s="125"/>
+      <c r="U71" s="125"/>
+      <c r="V71" s="125"/>
+      <c r="W71" s="84"/>
+    </row>
+    <row r="72" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B72" s="68"/>
+      <c r="C72" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="D72" s="124">
+        <v>125.658</v>
+      </c>
+      <c r="E72" s="114">
+        <v>166.56800000000001</v>
+      </c>
+      <c r="F72" s="114">
+        <v>0.755</v>
+      </c>
+      <c r="G72" s="114">
+        <v>0.75449999999999995</v>
+      </c>
+      <c r="H72" s="131">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="I72" s="112">
+        <v>18</v>
+      </c>
+      <c r="J72" s="112">
+        <v>546.79999999999995</v>
+      </c>
+      <c r="K72" s="112">
+        <v>6</v>
+      </c>
+      <c r="L72" s="115">
+        <v>106</v>
+      </c>
+      <c r="M72" s="112">
+        <v>64</v>
+      </c>
+      <c r="N72" s="112">
+        <v>32</v>
+      </c>
+      <c r="O72" s="115" t="s">
+        <v>39</v>
+      </c>
+      <c r="P72" s="112">
+        <v>0.1</v>
+      </c>
+      <c r="Q72" s="7">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="R72" s="82"/>
+      <c r="S72" s="125"/>
+      <c r="T72" s="125"/>
+      <c r="U72" s="125"/>
+      <c r="V72" s="125"/>
+      <c r="W72" s="84"/>
+    </row>
+    <row r="73" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B73" s="69"/>
+      <c r="C73" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="D73" s="132">
+        <v>155.00899999999999</v>
+      </c>
+      <c r="E73" s="132">
+        <v>196.97300000000001</v>
+      </c>
+      <c r="F73" s="132">
+        <v>0.65739999999999998</v>
+      </c>
+      <c r="G73" s="132">
+        <v>0.67669999999999997</v>
+      </c>
+      <c r="H73" s="133">
+        <v>38.4</v>
+      </c>
+      <c r="I73" s="3">
+        <v>18</v>
+      </c>
+      <c r="J73" s="3">
+        <v>152.30000000000001</v>
+      </c>
+      <c r="K73" s="3">
+        <v>6</v>
+      </c>
+      <c r="L73" s="34">
+        <v>59</v>
+      </c>
+      <c r="M73" s="3">
+        <v>64</v>
+      </c>
+      <c r="N73" s="3">
+        <v>32</v>
+      </c>
+      <c r="O73" s="34" t="s">
+        <v>39</v>
+      </c>
+      <c r="P73" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="Q73" s="4">
+        <v>1E-3</v>
+      </c>
+      <c r="R73" s="85"/>
+      <c r="S73" s="86"/>
+      <c r="T73" s="86"/>
+      <c r="U73" s="86"/>
+      <c r="V73" s="86"/>
+      <c r="W73" s="87"/>
+    </row>
+    <row r="74" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="39">
+  <mergeCells count="43">
+    <mergeCell ref="R66:W69"/>
+    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="R70:W73"/>
+    <mergeCell ref="B53:B56"/>
+    <mergeCell ref="R53:W56"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="R38:W40"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="R35:W37"/>
+    <mergeCell ref="B41:B44"/>
+    <mergeCell ref="R41:W44"/>
+    <mergeCell ref="R45:W48"/>
+    <mergeCell ref="B45:B48"/>
+    <mergeCell ref="R49:W52"/>
+    <mergeCell ref="B49:B52"/>
+    <mergeCell ref="R23:W25"/>
+    <mergeCell ref="B26:B28"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="I3:Q3"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="R3:W4"/>
+    <mergeCell ref="R5:W7"/>
+    <mergeCell ref="R8:W10"/>
+    <mergeCell ref="R26:W28"/>
+    <mergeCell ref="B11:B13"/>
     <mergeCell ref="B61:B65"/>
     <mergeCell ref="R61:W65"/>
     <mergeCell ref="B57:B60"/>
@@ -4788,29 +5370,6 @@
     <mergeCell ref="B32:B34"/>
     <mergeCell ref="R32:W34"/>
     <mergeCell ref="B23:B25"/>
-    <mergeCell ref="R23:W25"/>
-    <mergeCell ref="B26:B28"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="I3:Q3"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="R3:W4"/>
-    <mergeCell ref="R5:W7"/>
-    <mergeCell ref="R8:W10"/>
-    <mergeCell ref="R26:W28"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B53:B56"/>
-    <mergeCell ref="R53:W56"/>
-    <mergeCell ref="B38:B40"/>
-    <mergeCell ref="R38:W40"/>
-    <mergeCell ref="B35:B37"/>
-    <mergeCell ref="R35:W37"/>
-    <mergeCell ref="B41:B44"/>
-    <mergeCell ref="R41:W44"/>
-    <mergeCell ref="R45:W48"/>
-    <mergeCell ref="B45:B48"/>
-    <mergeCell ref="R49:W52"/>
-    <mergeCell ref="B49:B52"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>

<commit_message>
Actualizo repo. He hecho la sección del entrenamiento del MLP
</commit_message>
<xml_diff>
--- a/modelos_tfg/MetricasValidacion.xlsx
+++ b/modelos_tfg/MetricasValidacion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\modelos_tfg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8956D507-7938-49F9-BD9B-2C7A665916C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3A2EFEB-C37A-4309-88CE-986D7C64F31B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="0" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="0" windowWidth="29040" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -741,7 +741,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="136">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -843,126 +843,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
@@ -970,33 +850,129 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1007,13 +983,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1382,32 +1357,32 @@
   <sheetData>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D3" s="95" t="s">
+      <c r="D3" s="104" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="97"/>
-      <c r="I3" s="98" t="s">
+      <c r="E3" s="105"/>
+      <c r="F3" s="105"/>
+      <c r="G3" s="105"/>
+      <c r="H3" s="106"/>
+      <c r="I3" s="107" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="99"/>
-      <c r="K3" s="99"/>
-      <c r="L3" s="99"/>
-      <c r="M3" s="99"/>
-      <c r="N3" s="99"/>
-      <c r="O3" s="99"/>
-      <c r="P3" s="99"/>
-      <c r="Q3" s="100"/>
-      <c r="R3" s="102" t="s">
+      <c r="J3" s="108"/>
+      <c r="K3" s="108"/>
+      <c r="L3" s="108"/>
+      <c r="M3" s="108"/>
+      <c r="N3" s="108"/>
+      <c r="O3" s="108"/>
+      <c r="P3" s="108"/>
+      <c r="Q3" s="109"/>
+      <c r="R3" s="111" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="103"/>
-      <c r="T3" s="103"/>
-      <c r="U3" s="103"/>
-      <c r="V3" s="103"/>
-      <c r="W3" s="89"/>
+      <c r="S3" s="112"/>
+      <c r="T3" s="112"/>
+      <c r="U3" s="112"/>
+      <c r="V3" s="112"/>
+      <c r="W3" s="100"/>
     </row>
     <row r="4" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="19" t="s">
@@ -1458,16 +1433,16 @@
       <c r="Q4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="104"/>
-      <c r="S4" s="105"/>
-      <c r="T4" s="105"/>
-      <c r="U4" s="105"/>
-      <c r="V4" s="105"/>
-      <c r="W4" s="91"/>
+      <c r="R4" s="113"/>
+      <c r="S4" s="114"/>
+      <c r="T4" s="114"/>
+      <c r="U4" s="114"/>
+      <c r="V4" s="114"/>
+      <c r="W4" s="102"/>
     </row>
     <row r="5" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
-      <c r="B5" s="101" t="s">
+      <c r="B5" s="110" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -1515,18 +1490,18 @@
       <c r="Q5" s="16">
         <v>1E-3</v>
       </c>
-      <c r="R5" s="88" t="s">
+      <c r="R5" s="99" t="s">
         <v>38</v>
       </c>
-      <c r="S5" s="80"/>
-      <c r="T5" s="80"/>
-      <c r="U5" s="80"/>
-      <c r="V5" s="80"/>
-      <c r="W5" s="81"/>
+      <c r="S5" s="91"/>
+      <c r="T5" s="91"/>
+      <c r="U5" s="91"/>
+      <c r="V5" s="91"/>
+      <c r="W5" s="92"/>
     </row>
     <row r="6" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7"/>
-      <c r="B6" s="93"/>
+      <c r="B6" s="77"/>
       <c r="C6" s="5" t="s">
         <v>12</v>
       </c>
@@ -1572,16 +1547,16 @@
       <c r="Q6" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R6" s="82"/>
-      <c r="S6" s="83"/>
-      <c r="T6" s="83"/>
-      <c r="U6" s="83"/>
-      <c r="V6" s="83"/>
-      <c r="W6" s="84"/>
+      <c r="R6" s="93"/>
+      <c r="S6" s="94"/>
+      <c r="T6" s="94"/>
+      <c r="U6" s="94"/>
+      <c r="V6" s="94"/>
+      <c r="W6" s="95"/>
     </row>
     <row r="7" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7"/>
-      <c r="B7" s="94"/>
+      <c r="B7" s="103"/>
       <c r="C7" s="13" t="s">
         <v>14</v>
       </c>
@@ -1627,16 +1602,16 @@
       <c r="Q7" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R7" s="85"/>
-      <c r="S7" s="86"/>
-      <c r="T7" s="86"/>
-      <c r="U7" s="86"/>
-      <c r="V7" s="86"/>
-      <c r="W7" s="87"/>
+      <c r="R7" s="96"/>
+      <c r="S7" s="97"/>
+      <c r="T7" s="97"/>
+      <c r="U7" s="97"/>
+      <c r="V7" s="97"/>
+      <c r="W7" s="98"/>
     </row>
     <row r="8" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
-      <c r="B8" s="92" t="s">
+      <c r="B8" s="76" t="s">
         <v>24</v>
       </c>
       <c r="C8" s="5" t="s">
@@ -1684,18 +1659,18 @@
       <c r="Q8" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R8" s="88" t="s">
+      <c r="R8" s="99" t="s">
         <v>38</v>
       </c>
-      <c r="S8" s="80"/>
-      <c r="T8" s="80"/>
-      <c r="U8" s="80"/>
-      <c r="V8" s="80"/>
-      <c r="W8" s="81"/>
+      <c r="S8" s="91"/>
+      <c r="T8" s="91"/>
+      <c r="U8" s="91"/>
+      <c r="V8" s="91"/>
+      <c r="W8" s="92"/>
     </row>
     <row r="9" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
-      <c r="B9" s="93"/>
+      <c r="B9" s="77"/>
       <c r="C9" s="5" t="s">
         <v>12</v>
       </c>
@@ -1741,16 +1716,16 @@
       <c r="Q9" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R9" s="82"/>
-      <c r="S9" s="83"/>
-      <c r="T9" s="83"/>
-      <c r="U9" s="83"/>
-      <c r="V9" s="83"/>
-      <c r="W9" s="84"/>
+      <c r="R9" s="93"/>
+      <c r="S9" s="94"/>
+      <c r="T9" s="94"/>
+      <c r="U9" s="94"/>
+      <c r="V9" s="94"/>
+      <c r="W9" s="95"/>
     </row>
     <row r="10" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7"/>
-      <c r="B10" s="94"/>
+      <c r="B10" s="103"/>
       <c r="C10" s="5" t="s">
         <v>14</v>
       </c>
@@ -1796,15 +1771,15 @@
       <c r="Q10" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R10" s="85"/>
-      <c r="S10" s="86"/>
-      <c r="T10" s="86"/>
-      <c r="U10" s="86"/>
-      <c r="V10" s="86"/>
-      <c r="W10" s="87"/>
+      <c r="R10" s="96"/>
+      <c r="S10" s="97"/>
+      <c r="T10" s="97"/>
+      <c r="U10" s="97"/>
+      <c r="V10" s="97"/>
+      <c r="W10" s="98"/>
     </row>
     <row r="11" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="92" t="s">
+      <c r="B11" s="76" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="28" t="s">
@@ -1852,17 +1827,17 @@
       <c r="Q11" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R11" s="88" t="s">
+      <c r="R11" s="99" t="s">
         <v>38</v>
       </c>
-      <c r="S11" s="80"/>
-      <c r="T11" s="80"/>
-      <c r="U11" s="80"/>
-      <c r="V11" s="80"/>
-      <c r="W11" s="81"/>
+      <c r="S11" s="91"/>
+      <c r="T11" s="91"/>
+      <c r="U11" s="91"/>
+      <c r="V11" s="91"/>
+      <c r="W11" s="92"/>
     </row>
     <row r="12" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="93"/>
+      <c r="B12" s="77"/>
       <c r="C12" s="25" t="s">
         <v>12</v>
       </c>
@@ -1908,15 +1883,15 @@
       <c r="Q12" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R12" s="82"/>
-      <c r="S12" s="83"/>
-      <c r="T12" s="83"/>
-      <c r="U12" s="83"/>
-      <c r="V12" s="83"/>
-      <c r="W12" s="84"/>
+      <c r="R12" s="93"/>
+      <c r="S12" s="94"/>
+      <c r="T12" s="94"/>
+      <c r="U12" s="94"/>
+      <c r="V12" s="94"/>
+      <c r="W12" s="95"/>
     </row>
     <row r="13" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="93"/>
+      <c r="B13" s="77"/>
       <c r="C13" s="26" t="s">
         <v>14</v>
       </c>
@@ -1962,15 +1937,15 @@
       <c r="Q13" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R13" s="85"/>
-      <c r="S13" s="86"/>
-      <c r="T13" s="86"/>
-      <c r="U13" s="86"/>
-      <c r="V13" s="86"/>
-      <c r="W13" s="87"/>
+      <c r="R13" s="96"/>
+      <c r="S13" s="97"/>
+      <c r="T13" s="97"/>
+      <c r="U13" s="97"/>
+      <c r="V13" s="97"/>
+      <c r="W13" s="98"/>
     </row>
     <row r="14" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="92" t="s">
+      <c r="B14" s="76" t="s">
         <v>36</v>
       </c>
       <c r="C14" s="19" t="s">
@@ -2018,17 +1993,17 @@
       <c r="Q14" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R14" s="88" t="s">
+      <c r="R14" s="99" t="s">
         <v>37</v>
       </c>
-      <c r="S14" s="80"/>
-      <c r="T14" s="80"/>
-      <c r="U14" s="80"/>
-      <c r="V14" s="80"/>
-      <c r="W14" s="81"/>
+      <c r="S14" s="91"/>
+      <c r="T14" s="91"/>
+      <c r="U14" s="91"/>
+      <c r="V14" s="91"/>
+      <c r="W14" s="92"/>
     </row>
     <row r="15" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="93"/>
+      <c r="B15" s="77"/>
       <c r="C15" s="29" t="s">
         <v>12</v>
       </c>
@@ -2074,15 +2049,15 @@
       <c r="Q15" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R15" s="82"/>
-      <c r="S15" s="83"/>
-      <c r="T15" s="83"/>
-      <c r="U15" s="83"/>
-      <c r="V15" s="83"/>
-      <c r="W15" s="84"/>
+      <c r="R15" s="93"/>
+      <c r="S15" s="94"/>
+      <c r="T15" s="94"/>
+      <c r="U15" s="94"/>
+      <c r="V15" s="94"/>
+      <c r="W15" s="95"/>
     </row>
     <row r="16" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="94"/>
+      <c r="B16" s="103"/>
       <c r="C16" s="30" t="s">
         <v>14</v>
       </c>
@@ -2128,16 +2103,16 @@
       <c r="Q16" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R16" s="85"/>
-      <c r="S16" s="86"/>
-      <c r="T16" s="86"/>
-      <c r="U16" s="86"/>
-      <c r="V16" s="86"/>
-      <c r="W16" s="87"/>
+      <c r="R16" s="96"/>
+      <c r="S16" s="97"/>
+      <c r="T16" s="97"/>
+      <c r="U16" s="97"/>
+      <c r="V16" s="97"/>
+      <c r="W16" s="98"/>
     </row>
     <row r="17" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7"/>
-      <c r="B17" s="89" t="s">
+      <c r="B17" s="100" t="s">
         <v>44</v>
       </c>
       <c r="C17" s="29" t="s">
@@ -2185,18 +2160,18 @@
       <c r="Q17" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R17" s="80" t="s">
+      <c r="R17" s="91" t="s">
         <v>43</v>
       </c>
-      <c r="S17" s="80"/>
-      <c r="T17" s="80"/>
-      <c r="U17" s="80"/>
-      <c r="V17" s="80"/>
-      <c r="W17" s="81"/>
+      <c r="S17" s="91"/>
+      <c r="T17" s="91"/>
+      <c r="U17" s="91"/>
+      <c r="V17" s="91"/>
+      <c r="W17" s="92"/>
     </row>
     <row r="18" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
-      <c r="B18" s="90"/>
+      <c r="B18" s="101"/>
       <c r="C18" s="29" t="s">
         <v>12</v>
       </c>
@@ -2242,16 +2217,16 @@
       <c r="Q18" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R18" s="83"/>
-      <c r="S18" s="83"/>
-      <c r="T18" s="83"/>
-      <c r="U18" s="83"/>
-      <c r="V18" s="83"/>
-      <c r="W18" s="84"/>
+      <c r="R18" s="94"/>
+      <c r="S18" s="94"/>
+      <c r="T18" s="94"/>
+      <c r="U18" s="94"/>
+      <c r="V18" s="94"/>
+      <c r="W18" s="95"/>
     </row>
     <row r="19" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7"/>
-      <c r="B19" s="91"/>
+      <c r="B19" s="102"/>
       <c r="C19" s="30" t="s">
         <v>14</v>
       </c>
@@ -2297,16 +2272,16 @@
       <c r="Q19" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R19" s="86"/>
-      <c r="S19" s="86"/>
-      <c r="T19" s="86"/>
-      <c r="U19" s="86"/>
-      <c r="V19" s="86"/>
-      <c r="W19" s="87"/>
+      <c r="R19" s="97"/>
+      <c r="S19" s="97"/>
+      <c r="T19" s="97"/>
+      <c r="U19" s="97"/>
+      <c r="V19" s="97"/>
+      <c r="W19" s="98"/>
     </row>
     <row r="20" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7"/>
-      <c r="B20" s="92" t="s">
+      <c r="B20" s="76" t="s">
         <v>46</v>
       </c>
       <c r="C20" s="29" t="s">
@@ -2354,18 +2329,18 @@
       <c r="Q20" s="35">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R20" s="79" t="s">
+      <c r="R20" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="S20" s="80"/>
-      <c r="T20" s="80"/>
-      <c r="U20" s="80"/>
-      <c r="V20" s="80"/>
-      <c r="W20" s="81"/>
+      <c r="S20" s="91"/>
+      <c r="T20" s="91"/>
+      <c r="U20" s="91"/>
+      <c r="V20" s="91"/>
+      <c r="W20" s="92"/>
     </row>
     <row r="21" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
-      <c r="B21" s="93"/>
+      <c r="B21" s="77"/>
       <c r="C21" s="29" t="s">
         <v>12</v>
       </c>
@@ -2411,16 +2386,16 @@
       <c r="Q21" s="36">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R21" s="82"/>
-      <c r="S21" s="83"/>
-      <c r="T21" s="83"/>
-      <c r="U21" s="83"/>
-      <c r="V21" s="83"/>
-      <c r="W21" s="84"/>
+      <c r="R21" s="93"/>
+      <c r="S21" s="94"/>
+      <c r="T21" s="94"/>
+      <c r="U21" s="94"/>
+      <c r="V21" s="94"/>
+      <c r="W21" s="95"/>
     </row>
     <row r="22" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="7"/>
-      <c r="B22" s="94"/>
+      <c r="B22" s="103"/>
       <c r="C22" s="30" t="s">
         <v>14</v>
       </c>
@@ -2466,16 +2441,16 @@
       <c r="Q22" s="37">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R22" s="85"/>
-      <c r="S22" s="86"/>
-      <c r="T22" s="86"/>
-      <c r="U22" s="86"/>
-      <c r="V22" s="86"/>
-      <c r="W22" s="87"/>
+      <c r="R22" s="96"/>
+      <c r="S22" s="97"/>
+      <c r="T22" s="97"/>
+      <c r="U22" s="97"/>
+      <c r="V22" s="97"/>
+      <c r="W22" s="98"/>
     </row>
     <row r="23" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A23" s="58"/>
-      <c r="B23" s="67" t="s">
+      <c r="B23" s="78" t="s">
         <v>15</v>
       </c>
       <c r="C23" s="19" t="s">
@@ -2523,18 +2498,18 @@
       <c r="Q23" s="9">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R23" s="79" t="s">
+      <c r="R23" s="90" t="s">
         <v>53</v>
       </c>
-      <c r="S23" s="80"/>
-      <c r="T23" s="80"/>
-      <c r="U23" s="80"/>
-      <c r="V23" s="80"/>
-      <c r="W23" s="81"/>
+      <c r="S23" s="91"/>
+      <c r="T23" s="91"/>
+      <c r="U23" s="91"/>
+      <c r="V23" s="91"/>
+      <c r="W23" s="92"/>
     </row>
     <row r="24" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="58"/>
-      <c r="B24" s="68"/>
+      <c r="B24" s="79"/>
       <c r="C24" s="29" t="s">
         <v>12</v>
       </c>
@@ -2580,16 +2555,16 @@
       <c r="Q24" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R24" s="82"/>
-      <c r="S24" s="83"/>
-      <c r="T24" s="83"/>
-      <c r="U24" s="83"/>
-      <c r="V24" s="83"/>
-      <c r="W24" s="84"/>
+      <c r="R24" s="93"/>
+      <c r="S24" s="94"/>
+      <c r="T24" s="94"/>
+      <c r="U24" s="94"/>
+      <c r="V24" s="94"/>
+      <c r="W24" s="95"/>
     </row>
     <row r="25" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="58"/>
-      <c r="B25" s="69"/>
+      <c r="B25" s="80"/>
       <c r="C25" s="30" t="s">
         <v>14</v>
       </c>
@@ -2635,16 +2610,16 @@
       <c r="Q25" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R25" s="85"/>
-      <c r="S25" s="86"/>
-      <c r="T25" s="86"/>
-      <c r="U25" s="86"/>
-      <c r="V25" s="86"/>
-      <c r="W25" s="87"/>
+      <c r="R25" s="96"/>
+      <c r="S25" s="97"/>
+      <c r="T25" s="97"/>
+      <c r="U25" s="97"/>
+      <c r="V25" s="97"/>
+      <c r="W25" s="98"/>
     </row>
     <row r="26" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A26" s="58"/>
-      <c r="B26" s="67" t="s">
+      <c r="B26" s="78" t="s">
         <v>24</v>
       </c>
       <c r="C26" s="19" t="s">
@@ -2692,18 +2667,18 @@
       <c r="Q26" s="35">
         <v>1E-3</v>
       </c>
-      <c r="R26" s="88" t="s">
+      <c r="R26" s="99" t="s">
         <v>57</v>
       </c>
-      <c r="S26" s="80"/>
-      <c r="T26" s="80"/>
-      <c r="U26" s="80"/>
-      <c r="V26" s="80"/>
-      <c r="W26" s="81"/>
+      <c r="S26" s="91"/>
+      <c r="T26" s="91"/>
+      <c r="U26" s="91"/>
+      <c r="V26" s="91"/>
+      <c r="W26" s="92"/>
     </row>
     <row r="27" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="58"/>
-      <c r="B27" s="68"/>
+      <c r="B27" s="79"/>
       <c r="C27" s="29" t="s">
         <v>12</v>
       </c>
@@ -2749,16 +2724,16 @@
       <c r="Q27" s="36">
         <v>1E-3</v>
       </c>
-      <c r="R27" s="82"/>
-      <c r="S27" s="83"/>
-      <c r="T27" s="83"/>
-      <c r="U27" s="83"/>
-      <c r="V27" s="83"/>
-      <c r="W27" s="84"/>
+      <c r="R27" s="93"/>
+      <c r="S27" s="94"/>
+      <c r="T27" s="94"/>
+      <c r="U27" s="94"/>
+      <c r="V27" s="94"/>
+      <c r="W27" s="95"/>
     </row>
     <row r="28" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="58"/>
-      <c r="B28" s="69"/>
+      <c r="B28" s="80"/>
       <c r="C28" s="30" t="s">
         <v>14</v>
       </c>
@@ -2804,16 +2779,16 @@
       <c r="Q28" s="37">
         <v>1E-3</v>
       </c>
-      <c r="R28" s="85"/>
-      <c r="S28" s="86"/>
-      <c r="T28" s="86"/>
-      <c r="U28" s="86"/>
-      <c r="V28" s="86"/>
-      <c r="W28" s="87"/>
+      <c r="R28" s="96"/>
+      <c r="S28" s="97"/>
+      <c r="T28" s="97"/>
+      <c r="U28" s="97"/>
+      <c r="V28" s="97"/>
+      <c r="W28" s="98"/>
     </row>
     <row r="29" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A29" s="59"/>
-      <c r="B29" s="67" t="s">
+      <c r="B29" s="78" t="s">
         <v>34</v>
       </c>
       <c r="C29" s="28" t="s">
@@ -2861,18 +2836,18 @@
       <c r="Q29" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R29" s="79" t="s">
+      <c r="R29" s="90" t="s">
         <v>60</v>
       </c>
-      <c r="S29" s="80"/>
-      <c r="T29" s="80"/>
-      <c r="U29" s="80"/>
-      <c r="V29" s="80"/>
-      <c r="W29" s="81"/>
+      <c r="S29" s="91"/>
+      <c r="T29" s="91"/>
+      <c r="U29" s="91"/>
+      <c r="V29" s="91"/>
+      <c r="W29" s="92"/>
     </row>
     <row r="30" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="58"/>
-      <c r="B30" s="68"/>
+      <c r="B30" s="79"/>
       <c r="C30" s="25" t="s">
         <v>12</v>
       </c>
@@ -2918,16 +2893,16 @@
       <c r="Q30" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R30" s="82"/>
-      <c r="S30" s="83"/>
-      <c r="T30" s="83"/>
-      <c r="U30" s="83"/>
-      <c r="V30" s="83"/>
-      <c r="W30" s="84"/>
+      <c r="R30" s="93"/>
+      <c r="S30" s="94"/>
+      <c r="T30" s="94"/>
+      <c r="U30" s="94"/>
+      <c r="V30" s="94"/>
+      <c r="W30" s="95"/>
     </row>
     <row r="31" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="58"/>
-      <c r="B31" s="69"/>
+      <c r="B31" s="80"/>
       <c r="C31" s="42" t="s">
         <v>14</v>
       </c>
@@ -2973,16 +2948,16 @@
       <c r="Q31" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R31" s="85"/>
-      <c r="S31" s="86"/>
-      <c r="T31" s="86"/>
-      <c r="U31" s="86"/>
-      <c r="V31" s="86"/>
-      <c r="W31" s="87"/>
+      <c r="R31" s="96"/>
+      <c r="S31" s="97"/>
+      <c r="T31" s="97"/>
+      <c r="U31" s="97"/>
+      <c r="V31" s="97"/>
+      <c r="W31" s="98"/>
     </row>
     <row r="32" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A32" s="59"/>
-      <c r="B32" s="67" t="s">
+      <c r="B32" s="78" t="s">
         <v>36</v>
       </c>
       <c r="C32" s="28" t="s">
@@ -3030,18 +3005,18 @@
       <c r="Q32" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R32" s="88" t="s">
+      <c r="R32" s="99" t="s">
         <v>61</v>
       </c>
-      <c r="S32" s="80"/>
-      <c r="T32" s="80"/>
-      <c r="U32" s="80"/>
-      <c r="V32" s="80"/>
-      <c r="W32" s="81"/>
+      <c r="S32" s="91"/>
+      <c r="T32" s="91"/>
+      <c r="U32" s="91"/>
+      <c r="V32" s="91"/>
+      <c r="W32" s="92"/>
     </row>
     <row r="33" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="59"/>
-      <c r="B33" s="68"/>
+      <c r="B33" s="79"/>
       <c r="C33" s="25" t="s">
         <v>12</v>
       </c>
@@ -3087,16 +3062,16 @@
       <c r="Q33" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R33" s="82"/>
-      <c r="S33" s="83"/>
-      <c r="T33" s="83"/>
-      <c r="U33" s="83"/>
-      <c r="V33" s="83"/>
-      <c r="W33" s="84"/>
+      <c r="R33" s="93"/>
+      <c r="S33" s="94"/>
+      <c r="T33" s="94"/>
+      <c r="U33" s="94"/>
+      <c r="V33" s="94"/>
+      <c r="W33" s="95"/>
     </row>
     <row r="34" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="59"/>
-      <c r="B34" s="69"/>
+      <c r="B34" s="80"/>
       <c r="C34" s="42" t="s">
         <v>14</v>
       </c>
@@ -3142,16 +3117,16 @@
       <c r="Q34" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R34" s="85"/>
-      <c r="S34" s="86"/>
-      <c r="T34" s="86"/>
-      <c r="U34" s="86"/>
-      <c r="V34" s="86"/>
-      <c r="W34" s="87"/>
+      <c r="R34" s="96"/>
+      <c r="S34" s="97"/>
+      <c r="T34" s="97"/>
+      <c r="U34" s="97"/>
+      <c r="V34" s="97"/>
+      <c r="W34" s="98"/>
     </row>
     <row r="35" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A35" s="58"/>
-      <c r="B35" s="67" t="s">
+      <c r="B35" s="78" t="s">
         <v>44</v>
       </c>
       <c r="C35" s="25" t="s">
@@ -3199,18 +3174,18 @@
       <c r="Q35" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R35" s="79" t="s">
+      <c r="R35" s="90" t="s">
         <v>63</v>
       </c>
-      <c r="S35" s="80"/>
-      <c r="T35" s="80"/>
-      <c r="U35" s="80"/>
-      <c r="V35" s="80"/>
-      <c r="W35" s="81"/>
+      <c r="S35" s="91"/>
+      <c r="T35" s="91"/>
+      <c r="U35" s="91"/>
+      <c r="V35" s="91"/>
+      <c r="W35" s="92"/>
     </row>
     <row r="36" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="58"/>
-      <c r="B36" s="68"/>
+      <c r="B36" s="79"/>
       <c r="C36" s="25" t="s">
         <v>12</v>
       </c>
@@ -3256,16 +3231,16 @@
       <c r="Q36" s="36">
         <v>1E-3</v>
       </c>
-      <c r="R36" s="82"/>
-      <c r="S36" s="83"/>
-      <c r="T36" s="83"/>
-      <c r="U36" s="83"/>
-      <c r="V36" s="83"/>
-      <c r="W36" s="84"/>
+      <c r="R36" s="93"/>
+      <c r="S36" s="94"/>
+      <c r="T36" s="94"/>
+      <c r="U36" s="94"/>
+      <c r="V36" s="94"/>
+      <c r="W36" s="95"/>
     </row>
     <row r="37" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="58"/>
-      <c r="B37" s="69"/>
+      <c r="B37" s="80"/>
       <c r="C37" s="30" t="s">
         <v>14</v>
       </c>
@@ -3311,16 +3286,16 @@
       <c r="Q37" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R37" s="85"/>
-      <c r="S37" s="86"/>
-      <c r="T37" s="86"/>
-      <c r="U37" s="86"/>
-      <c r="V37" s="86"/>
-      <c r="W37" s="87"/>
+      <c r="R37" s="96"/>
+      <c r="S37" s="97"/>
+      <c r="T37" s="97"/>
+      <c r="U37" s="97"/>
+      <c r="V37" s="97"/>
+      <c r="W37" s="98"/>
     </row>
     <row r="38" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A38" s="59"/>
-      <c r="B38" s="67" t="s">
+      <c r="B38" s="78" t="s">
         <v>46</v>
       </c>
       <c r="C38" s="19" t="s">
@@ -3368,16 +3343,16 @@
       <c r="Q38" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R38" s="106"/>
-      <c r="S38" s="71"/>
-      <c r="T38" s="71"/>
-      <c r="U38" s="71"/>
-      <c r="V38" s="71"/>
-      <c r="W38" s="72"/>
+      <c r="R38" s="115"/>
+      <c r="S38" s="82"/>
+      <c r="T38" s="82"/>
+      <c r="U38" s="82"/>
+      <c r="V38" s="82"/>
+      <c r="W38" s="83"/>
     </row>
     <row r="39" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="59"/>
-      <c r="B39" s="68"/>
+      <c r="B39" s="79"/>
       <c r="C39" s="29" t="s">
         <v>12</v>
       </c>
@@ -3423,16 +3398,16 @@
       <c r="Q39" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R39" s="73"/>
-      <c r="S39" s="74"/>
-      <c r="T39" s="74"/>
-      <c r="U39" s="74"/>
-      <c r="V39" s="74"/>
-      <c r="W39" s="75"/>
+      <c r="R39" s="84"/>
+      <c r="S39" s="85"/>
+      <c r="T39" s="85"/>
+      <c r="U39" s="85"/>
+      <c r="V39" s="85"/>
+      <c r="W39" s="86"/>
     </row>
     <row r="40" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="59"/>
-      <c r="B40" s="69"/>
+      <c r="B40" s="80"/>
       <c r="C40" s="30" t="s">
         <v>14</v>
       </c>
@@ -3478,16 +3453,16 @@
       <c r="Q40" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R40" s="76"/>
-      <c r="S40" s="77"/>
-      <c r="T40" s="77"/>
-      <c r="U40" s="77"/>
-      <c r="V40" s="77"/>
-      <c r="W40" s="78"/>
+      <c r="R40" s="87"/>
+      <c r="S40" s="88"/>
+      <c r="T40" s="88"/>
+      <c r="U40" s="88"/>
+      <c r="V40" s="88"/>
+      <c r="W40" s="89"/>
     </row>
     <row r="41" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A41" s="59"/>
-      <c r="B41" s="67" t="s">
+      <c r="B41" s="78" t="s">
         <v>50</v>
       </c>
       <c r="C41" s="29" t="s">
@@ -3535,18 +3510,18 @@
       <c r="Q41" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R41" s="88" t="s">
+      <c r="R41" s="99" t="s">
         <v>71</v>
       </c>
-      <c r="S41" s="80"/>
-      <c r="T41" s="80"/>
-      <c r="U41" s="80"/>
-      <c r="V41" s="80"/>
-      <c r="W41" s="81"/>
+      <c r="S41" s="91"/>
+      <c r="T41" s="91"/>
+      <c r="U41" s="91"/>
+      <c r="V41" s="91"/>
+      <c r="W41" s="92"/>
     </row>
     <row r="42" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="59"/>
-      <c r="B42" s="68"/>
+      <c r="B42" s="79"/>
       <c r="C42" s="29" t="s">
         <v>12</v>
       </c>
@@ -3592,16 +3567,16 @@
       <c r="Q42" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R42" s="82"/>
-      <c r="S42" s="83"/>
-      <c r="T42" s="83"/>
-      <c r="U42" s="83"/>
-      <c r="V42" s="83"/>
-      <c r="W42" s="84"/>
+      <c r="R42" s="93"/>
+      <c r="S42" s="94"/>
+      <c r="T42" s="94"/>
+      <c r="U42" s="94"/>
+      <c r="V42" s="94"/>
+      <c r="W42" s="95"/>
     </row>
     <row r="43" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="59"/>
-      <c r="B43" s="68"/>
+      <c r="B43" s="79"/>
       <c r="C43" s="29" t="s">
         <v>14</v>
       </c>
@@ -3647,16 +3622,16 @@
       <c r="Q43" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R43" s="82"/>
-      <c r="S43" s="83"/>
-      <c r="T43" s="83"/>
-      <c r="U43" s="83"/>
-      <c r="V43" s="83"/>
-      <c r="W43" s="84"/>
+      <c r="R43" s="93"/>
+      <c r="S43" s="94"/>
+      <c r="T43" s="94"/>
+      <c r="U43" s="94"/>
+      <c r="V43" s="94"/>
+      <c r="W43" s="95"/>
     </row>
     <row r="44" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="59"/>
-      <c r="B44" s="69"/>
+      <c r="B44" s="80"/>
       <c r="C44" s="30" t="s">
         <v>67</v>
       </c>
@@ -3702,16 +3677,16 @@
       <c r="Q44" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R44" s="85"/>
-      <c r="S44" s="86"/>
-      <c r="T44" s="86"/>
-      <c r="U44" s="86"/>
-      <c r="V44" s="86"/>
-      <c r="W44" s="87"/>
+      <c r="R44" s="96"/>
+      <c r="S44" s="97"/>
+      <c r="T44" s="97"/>
+      <c r="U44" s="97"/>
+      <c r="V44" s="97"/>
+      <c r="W44" s="98"/>
     </row>
     <row r="45" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A45" s="59"/>
-      <c r="B45" s="67" t="s">
+      <c r="B45" s="78" t="s">
         <v>55</v>
       </c>
       <c r="C45" s="29" t="s">
@@ -3759,18 +3734,18 @@
       <c r="Q45" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R45" s="70" t="s">
+      <c r="R45" s="81" t="s">
         <v>72</v>
       </c>
-      <c r="S45" s="71"/>
-      <c r="T45" s="71"/>
-      <c r="U45" s="71"/>
-      <c r="V45" s="71"/>
-      <c r="W45" s="72"/>
+      <c r="S45" s="82"/>
+      <c r="T45" s="82"/>
+      <c r="U45" s="82"/>
+      <c r="V45" s="82"/>
+      <c r="W45" s="83"/>
     </row>
     <row r="46" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="59"/>
-      <c r="B46" s="68"/>
+      <c r="B46" s="79"/>
       <c r="C46" s="29" t="s">
         <v>12</v>
       </c>
@@ -3816,16 +3791,16 @@
       <c r="Q46" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R46" s="73"/>
-      <c r="S46" s="74"/>
-      <c r="T46" s="74"/>
-      <c r="U46" s="74"/>
-      <c r="V46" s="74"/>
-      <c r="W46" s="75"/>
+      <c r="R46" s="84"/>
+      <c r="S46" s="85"/>
+      <c r="T46" s="85"/>
+      <c r="U46" s="85"/>
+      <c r="V46" s="85"/>
+      <c r="W46" s="86"/>
     </row>
     <row r="47" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="59"/>
-      <c r="B47" s="68"/>
+      <c r="B47" s="79"/>
       <c r="C47" s="29" t="s">
         <v>14</v>
       </c>
@@ -3871,16 +3846,16 @@
       <c r="Q47" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R47" s="73"/>
-      <c r="S47" s="74"/>
-      <c r="T47" s="74"/>
-      <c r="U47" s="74"/>
-      <c r="V47" s="74"/>
-      <c r="W47" s="75"/>
+      <c r="R47" s="84"/>
+      <c r="S47" s="85"/>
+      <c r="T47" s="85"/>
+      <c r="U47" s="85"/>
+      <c r="V47" s="85"/>
+      <c r="W47" s="86"/>
     </row>
     <row r="48" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="59"/>
-      <c r="B48" s="69"/>
+      <c r="B48" s="80"/>
       <c r="C48" s="30" t="s">
         <v>67</v>
       </c>
@@ -3926,16 +3901,16 @@
       <c r="Q48" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R48" s="76"/>
-      <c r="S48" s="77"/>
-      <c r="T48" s="77"/>
-      <c r="U48" s="77"/>
-      <c r="V48" s="77"/>
-      <c r="W48" s="78"/>
+      <c r="R48" s="87"/>
+      <c r="S48" s="88"/>
+      <c r="T48" s="88"/>
+      <c r="U48" s="88"/>
+      <c r="V48" s="88"/>
+      <c r="W48" s="89"/>
     </row>
     <row r="49" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A49" s="58"/>
-      <c r="B49" s="67" t="s">
+      <c r="B49" s="78" t="s">
         <v>58</v>
       </c>
       <c r="C49" s="29" t="s">
@@ -3983,18 +3958,18 @@
       <c r="Q49" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R49" s="79" t="s">
+      <c r="R49" s="90" t="s">
         <v>79</v>
       </c>
-      <c r="S49" s="80"/>
-      <c r="T49" s="80"/>
-      <c r="U49" s="80"/>
-      <c r="V49" s="80"/>
-      <c r="W49" s="81"/>
+      <c r="S49" s="91"/>
+      <c r="T49" s="91"/>
+      <c r="U49" s="91"/>
+      <c r="V49" s="91"/>
+      <c r="W49" s="92"/>
     </row>
     <row r="50" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="58"/>
-      <c r="B50" s="68"/>
+      <c r="B50" s="79"/>
       <c r="C50" s="29" t="s">
         <v>12</v>
       </c>
@@ -4040,16 +4015,16 @@
       <c r="Q50" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R50" s="82"/>
-      <c r="S50" s="83"/>
-      <c r="T50" s="83"/>
-      <c r="U50" s="83"/>
-      <c r="V50" s="83"/>
-      <c r="W50" s="84"/>
+      <c r="R50" s="93"/>
+      <c r="S50" s="94"/>
+      <c r="T50" s="94"/>
+      <c r="U50" s="94"/>
+      <c r="V50" s="94"/>
+      <c r="W50" s="95"/>
     </row>
     <row r="51" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="58"/>
-      <c r="B51" s="68"/>
+      <c r="B51" s="79"/>
       <c r="C51" s="29" t="s">
         <v>14</v>
       </c>
@@ -4095,16 +4070,16 @@
       <c r="Q51" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R51" s="82"/>
-      <c r="S51" s="83"/>
-      <c r="T51" s="83"/>
-      <c r="U51" s="83"/>
-      <c r="V51" s="83"/>
-      <c r="W51" s="84"/>
+      <c r="R51" s="93"/>
+      <c r="S51" s="94"/>
+      <c r="T51" s="94"/>
+      <c r="U51" s="94"/>
+      <c r="V51" s="94"/>
+      <c r="W51" s="95"/>
     </row>
     <row r="52" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="58"/>
-      <c r="B52" s="69"/>
+      <c r="B52" s="80"/>
       <c r="C52" s="30" t="s">
         <v>67</v>
       </c>
@@ -4150,16 +4125,16 @@
       <c r="Q52" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R52" s="85"/>
-      <c r="S52" s="86"/>
-      <c r="T52" s="86"/>
-      <c r="U52" s="86"/>
-      <c r="V52" s="86"/>
-      <c r="W52" s="87"/>
+      <c r="R52" s="96"/>
+      <c r="S52" s="97"/>
+      <c r="T52" s="97"/>
+      <c r="U52" s="97"/>
+      <c r="V52" s="97"/>
+      <c r="W52" s="98"/>
     </row>
     <row r="53" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A53" s="59"/>
-      <c r="B53" s="67" t="s">
+      <c r="B53" s="78" t="s">
         <v>77</v>
       </c>
       <c r="C53" s="19" t="s">
@@ -4207,18 +4182,18 @@
       <c r="Q53" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R53" s="79" t="s">
+      <c r="R53" s="90" t="s">
         <v>80</v>
       </c>
-      <c r="S53" s="80"/>
-      <c r="T53" s="80"/>
-      <c r="U53" s="80"/>
-      <c r="V53" s="80"/>
-      <c r="W53" s="81"/>
+      <c r="S53" s="91"/>
+      <c r="T53" s="91"/>
+      <c r="U53" s="91"/>
+      <c r="V53" s="91"/>
+      <c r="W53" s="92"/>
     </row>
     <row r="54" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="59"/>
-      <c r="B54" s="68"/>
+      <c r="B54" s="79"/>
       <c r="C54" s="29" t="s">
         <v>12</v>
       </c>
@@ -4264,16 +4239,16 @@
       <c r="Q54" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R54" s="82"/>
-      <c r="S54" s="83"/>
-      <c r="T54" s="83"/>
-      <c r="U54" s="83"/>
-      <c r="V54" s="83"/>
-      <c r="W54" s="84"/>
+      <c r="R54" s="93"/>
+      <c r="S54" s="94"/>
+      <c r="T54" s="94"/>
+      <c r="U54" s="94"/>
+      <c r="V54" s="94"/>
+      <c r="W54" s="95"/>
     </row>
     <row r="55" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="59"/>
-      <c r="B55" s="68"/>
+      <c r="B55" s="79"/>
       <c r="C55" s="29" t="s">
         <v>14</v>
       </c>
@@ -4319,16 +4294,16 @@
       <c r="Q55" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R55" s="82"/>
-      <c r="S55" s="83"/>
-      <c r="T55" s="83"/>
-      <c r="U55" s="83"/>
-      <c r="V55" s="83"/>
-      <c r="W55" s="84"/>
+      <c r="R55" s="93"/>
+      <c r="S55" s="94"/>
+      <c r="T55" s="94"/>
+      <c r="U55" s="94"/>
+      <c r="V55" s="94"/>
+      <c r="W55" s="95"/>
     </row>
     <row r="56" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="59"/>
-      <c r="B56" s="69"/>
+      <c r="B56" s="80"/>
       <c r="C56" s="30" t="s">
         <v>67</v>
       </c>
@@ -4374,16 +4349,16 @@
       <c r="Q56" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R56" s="85"/>
-      <c r="S56" s="86"/>
-      <c r="T56" s="86"/>
-      <c r="U56" s="86"/>
-      <c r="V56" s="86"/>
-      <c r="W56" s="87"/>
+      <c r="R56" s="96"/>
+      <c r="S56" s="97"/>
+      <c r="T56" s="97"/>
+      <c r="U56" s="97"/>
+      <c r="V56" s="97"/>
+      <c r="W56" s="98"/>
     </row>
     <row r="57" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A57" s="58"/>
-      <c r="B57" s="67" t="s">
+      <c r="B57" s="78" t="s">
         <v>81</v>
       </c>
       <c r="C57" s="19" t="s">
@@ -4431,18 +4406,18 @@
       <c r="Q57" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R57" s="79" t="s">
+      <c r="R57" s="90" t="s">
         <v>87</v>
       </c>
-      <c r="S57" s="80"/>
-      <c r="T57" s="80"/>
-      <c r="U57" s="80"/>
-      <c r="V57" s="80"/>
-      <c r="W57" s="81"/>
+      <c r="S57" s="91"/>
+      <c r="T57" s="91"/>
+      <c r="U57" s="91"/>
+      <c r="V57" s="91"/>
+      <c r="W57" s="92"/>
     </row>
     <row r="58" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="58"/>
-      <c r="B58" s="68"/>
+      <c r="B58" s="79"/>
       <c r="C58" s="29" t="s">
         <v>12</v>
       </c>
@@ -4488,16 +4463,16 @@
       <c r="Q58" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R58" s="82"/>
-      <c r="S58" s="83"/>
-      <c r="T58" s="83"/>
-      <c r="U58" s="83"/>
-      <c r="V58" s="83"/>
-      <c r="W58" s="84"/>
+      <c r="R58" s="93"/>
+      <c r="S58" s="94"/>
+      <c r="T58" s="94"/>
+      <c r="U58" s="94"/>
+      <c r="V58" s="94"/>
+      <c r="W58" s="95"/>
     </row>
     <row r="59" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="58"/>
-      <c r="B59" s="68"/>
+      <c r="B59" s="79"/>
       <c r="C59" s="29" t="s">
         <v>14</v>
       </c>
@@ -4543,16 +4518,16 @@
       <c r="Q59" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R59" s="82"/>
-      <c r="S59" s="83"/>
-      <c r="T59" s="83"/>
-      <c r="U59" s="83"/>
-      <c r="V59" s="83"/>
-      <c r="W59" s="84"/>
+      <c r="R59" s="93"/>
+      <c r="S59" s="94"/>
+      <c r="T59" s="94"/>
+      <c r="U59" s="94"/>
+      <c r="V59" s="94"/>
+      <c r="W59" s="95"/>
     </row>
     <row r="60" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="58"/>
-      <c r="B60" s="69"/>
+      <c r="B60" s="80"/>
       <c r="C60" s="30" t="s">
         <v>67</v>
       </c>
@@ -4598,16 +4573,16 @@
       <c r="Q60" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R60" s="85"/>
-      <c r="S60" s="86"/>
-      <c r="T60" s="86"/>
-      <c r="U60" s="86"/>
-      <c r="V60" s="86"/>
-      <c r="W60" s="87"/>
-    </row>
-    <row r="61" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="R60" s="96"/>
+      <c r="S60" s="97"/>
+      <c r="T60" s="97"/>
+      <c r="U60" s="97"/>
+      <c r="V60" s="97"/>
+      <c r="W60" s="98"/>
+    </row>
+    <row r="61" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A61" s="7"/>
-      <c r="B61" s="67" t="s">
+      <c r="B61" s="78" t="s">
         <v>84</v>
       </c>
       <c r="C61" s="28" t="s">
@@ -4655,18 +4630,18 @@
       <c r="Q61" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R61" s="70" t="s">
+      <c r="R61" s="81" t="s">
         <v>85</v>
       </c>
-      <c r="S61" s="71"/>
-      <c r="T61" s="71"/>
-      <c r="U61" s="71"/>
-      <c r="V61" s="71"/>
-      <c r="W61" s="72"/>
-    </row>
-    <row r="62" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+      <c r="S61" s="82"/>
+      <c r="T61" s="82"/>
+      <c r="U61" s="82"/>
+      <c r="V61" s="82"/>
+      <c r="W61" s="83"/>
+    </row>
+    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A62" s="7"/>
-      <c r="B62" s="68"/>
+      <c r="B62" s="79"/>
       <c r="C62" s="25" t="s">
         <v>12</v>
       </c>
@@ -4712,16 +4687,16 @@
       <c r="Q62" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R62" s="73"/>
-      <c r="S62" s="74"/>
-      <c r="T62" s="74"/>
-      <c r="U62" s="74"/>
-      <c r="V62" s="74"/>
-      <c r="W62" s="75"/>
-    </row>
-    <row r="63" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+      <c r="R62" s="84"/>
+      <c r="S62" s="85"/>
+      <c r="T62" s="85"/>
+      <c r="U62" s="85"/>
+      <c r="V62" s="85"/>
+      <c r="W62" s="86"/>
+    </row>
+    <row r="63" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="68"/>
+      <c r="B63" s="79"/>
       <c r="C63" s="25" t="s">
         <v>14</v>
       </c>
@@ -4767,16 +4742,16 @@
       <c r="Q63" s="64">
         <v>1E-3</v>
       </c>
-      <c r="R63" s="73"/>
-      <c r="S63" s="74"/>
-      <c r="T63" s="74"/>
-      <c r="U63" s="74"/>
-      <c r="V63" s="74"/>
-      <c r="W63" s="75"/>
-    </row>
-    <row r="64" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+      <c r="R63" s="84"/>
+      <c r="S63" s="85"/>
+      <c r="T63" s="85"/>
+      <c r="U63" s="85"/>
+      <c r="V63" s="85"/>
+      <c r="W63" s="86"/>
+    </row>
+    <row r="64" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="68"/>
+      <c r="B64" s="79"/>
       <c r="C64" s="25" t="s">
         <v>67</v>
       </c>
@@ -4822,88 +4797,88 @@
       <c r="Q64" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R64" s="73"/>
-      <c r="S64" s="74"/>
-      <c r="T64" s="74"/>
-      <c r="U64" s="74"/>
-      <c r="V64" s="74"/>
-      <c r="W64" s="75"/>
-    </row>
-    <row r="65" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R64" s="84"/>
+      <c r="S64" s="85"/>
+      <c r="T64" s="85"/>
+      <c r="U64" s="85"/>
+      <c r="V64" s="85"/>
+      <c r="W64" s="86"/>
+    </row>
+    <row r="65" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="7"/>
-      <c r="B65" s="69"/>
-      <c r="C65" s="107" t="s">
+      <c r="B65" s="80"/>
+      <c r="C65" s="67" t="s">
         <v>83</v>
       </c>
-      <c r="D65" s="108">
+      <c r="D65" s="68">
         <v>122.208</v>
       </c>
-      <c r="E65" s="108">
+      <c r="E65" s="68">
         <v>174.66300000000001</v>
       </c>
-      <c r="F65" s="108">
+      <c r="F65" s="68">
         <v>0.8216</v>
       </c>
-      <c r="G65" s="108">
+      <c r="G65" s="68">
         <v>0.82150000000000001</v>
       </c>
-      <c r="H65" s="109">
+      <c r="H65" s="69">
         <v>20.3</v>
       </c>
-      <c r="I65" s="110">
+      <c r="I65" s="70">
         <v>18</v>
       </c>
-      <c r="J65" s="108">
+      <c r="J65" s="68">
         <v>132.01</v>
       </c>
-      <c r="K65" s="108">
-        <v>6</v>
-      </c>
-      <c r="L65" s="111" t="s">
+      <c r="K65" s="68">
+        <v>6</v>
+      </c>
+      <c r="L65" s="71" t="s">
         <v>49</v>
       </c>
-      <c r="M65" s="108">
-        <v>64</v>
-      </c>
-      <c r="N65" s="108">
+      <c r="M65" s="68">
+        <v>64</v>
+      </c>
+      <c r="N65" s="68">
         <v>32</v>
       </c>
-      <c r="O65" s="111" t="s">
-        <v>39</v>
-      </c>
-      <c r="P65" s="108">
+      <c r="O65" s="71" t="s">
+        <v>39</v>
+      </c>
+      <c r="P65" s="68">
         <v>0.1</v>
       </c>
-      <c r="Q65" s="109">
+      <c r="Q65" s="69">
         <v>1E-3</v>
       </c>
-      <c r="R65" s="76"/>
-      <c r="S65" s="77"/>
-      <c r="T65" s="77"/>
-      <c r="U65" s="77"/>
-      <c r="V65" s="77"/>
-      <c r="W65" s="78"/>
+      <c r="R65" s="87"/>
+      <c r="S65" s="88"/>
+      <c r="T65" s="88"/>
+      <c r="U65" s="88"/>
+      <c r="V65" s="88"/>
+      <c r="W65" s="89"/>
     </row>
     <row r="66" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="67" t="s">
+      <c r="B66" s="78" t="s">
         <v>86</v>
       </c>
       <c r="C66" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D66" s="134">
+      <c r="D66" s="8">
         <v>48.537999999999997</v>
       </c>
-      <c r="E66" s="134">
+      <c r="E66" s="8">
         <v>96.697000000000003</v>
       </c>
-      <c r="F66" s="134">
+      <c r="F66" s="8">
         <v>0.94530000000000003</v>
       </c>
-      <c r="G66" s="134">
+      <c r="G66" s="8">
         <v>0.94530000000000003</v>
       </c>
-      <c r="H66" s="135">
+      <c r="H66" s="9">
         <v>22.4</v>
       </c>
       <c r="I66" s="8">
@@ -4933,206 +4908,206 @@
       <c r="Q66" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R66" s="117" t="s">
+      <c r="R66" s="81" t="s">
         <v>88</v>
       </c>
-      <c r="S66" s="71"/>
-      <c r="T66" s="71"/>
-      <c r="U66" s="71"/>
-      <c r="V66" s="71"/>
-      <c r="W66" s="72"/>
+      <c r="S66" s="82"/>
+      <c r="T66" s="82"/>
+      <c r="U66" s="82"/>
+      <c r="V66" s="82"/>
+      <c r="W66" s="83"/>
     </row>
     <row r="67" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B67" s="68"/>
+      <c r="B67" s="79"/>
       <c r="C67" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="D67" s="114">
+      <c r="D67">
         <v>51.738</v>
       </c>
-      <c r="E67" s="114">
+      <c r="E67">
         <v>92.930999999999997</v>
       </c>
-      <c r="F67" s="114">
+      <c r="F67">
         <v>0.94950000000000001</v>
       </c>
-      <c r="G67" s="114">
+      <c r="G67">
         <v>0.94950000000000001</v>
       </c>
       <c r="H67" s="7">
         <v>22.6</v>
       </c>
-      <c r="I67" s="114">
+      <c r="I67">
         <v>18</v>
       </c>
-      <c r="J67" s="114">
+      <c r="J67">
         <v>332.8</v>
       </c>
-      <c r="K67" s="114">
-        <v>6</v>
-      </c>
-      <c r="L67" s="116">
+      <c r="K67">
+        <v>6</v>
+      </c>
+      <c r="L67" s="31">
         <v>71</v>
       </c>
-      <c r="M67" s="114">
-        <v>64</v>
-      </c>
-      <c r="N67" s="114">
+      <c r="M67">
+        <v>64</v>
+      </c>
+      <c r="N67">
         <v>32</v>
       </c>
-      <c r="O67" s="115" t="s">
-        <v>39</v>
-      </c>
-      <c r="P67" s="114">
+      <c r="O67" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="P67">
         <v>0.1</v>
       </c>
       <c r="Q67" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R67" s="73"/>
-      <c r="S67" s="113"/>
-      <c r="T67" s="113"/>
-      <c r="U67" s="113"/>
-      <c r="V67" s="113"/>
-      <c r="W67" s="75"/>
+      <c r="R67" s="84"/>
+      <c r="S67" s="85"/>
+      <c r="T67" s="85"/>
+      <c r="U67" s="85"/>
+      <c r="V67" s="85"/>
+      <c r="W67" s="86"/>
     </row>
     <row r="68" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B68" s="68"/>
+      <c r="B68" s="79"/>
       <c r="C68" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="D68" s="114">
+      <c r="D68">
         <v>48.079000000000001</v>
       </c>
-      <c r="E68" s="114">
+      <c r="E68">
         <v>102.464</v>
       </c>
-      <c r="F68" s="114">
+      <c r="F68">
         <v>0.93859999999999999</v>
       </c>
-      <c r="G68" s="114">
+      <c r="G68">
         <v>0.93859999999999999</v>
       </c>
       <c r="H68" s="7">
         <v>17.899999999999999</v>
       </c>
-      <c r="I68" s="114">
+      <c r="I68">
         <v>18</v>
       </c>
-      <c r="J68" s="114">
+      <c r="J68">
         <v>546.79999999999995</v>
       </c>
-      <c r="K68" s="114">
-        <v>6</v>
-      </c>
-      <c r="L68" s="116">
+      <c r="K68">
+        <v>6</v>
+      </c>
+      <c r="L68" s="31">
         <v>106</v>
       </c>
-      <c r="M68" s="114">
-        <v>64</v>
-      </c>
-      <c r="N68" s="114">
+      <c r="M68">
+        <v>64</v>
+      </c>
+      <c r="N68">
         <v>32</v>
       </c>
-      <c r="O68" s="116" t="s">
-        <v>39</v>
-      </c>
-      <c r="P68" s="114">
+      <c r="O68" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="P68">
         <v>0.1</v>
       </c>
       <c r="Q68" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R68" s="73"/>
-      <c r="S68" s="113"/>
-      <c r="T68" s="113"/>
-      <c r="U68" s="113"/>
-      <c r="V68" s="113"/>
-      <c r="W68" s="75"/>
+      <c r="R68" s="84"/>
+      <c r="S68" s="85"/>
+      <c r="T68" s="85"/>
+      <c r="U68" s="85"/>
+      <c r="V68" s="85"/>
+      <c r="W68" s="86"/>
     </row>
     <row r="69" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B69" s="119"/>
       <c r="C69" s="29" t="s">
         <v>67</v>
       </c>
-      <c r="D69" s="114">
+      <c r="D69">
         <v>63.225000000000001</v>
       </c>
-      <c r="E69" s="114">
+      <c r="E69">
         <v>123.163</v>
       </c>
-      <c r="F69" s="114">
+      <c r="F69">
         <v>0.9113</v>
       </c>
-      <c r="G69" s="121">
+      <c r="G69" s="73">
         <v>0.91120000000000001</v>
       </c>
-      <c r="H69" s="122">
+      <c r="H69" s="74">
         <v>38.4</v>
       </c>
-      <c r="I69" s="123">
+      <c r="I69" s="75">
         <v>18</v>
       </c>
-      <c r="J69" s="114">
+      <c r="J69">
         <v>152.30000000000001</v>
       </c>
-      <c r="K69" s="121">
-        <v>6</v>
-      </c>
-      <c r="L69" s="115">
+      <c r="K69" s="73">
+        <v>6</v>
+      </c>
+      <c r="L69" s="31">
         <v>59</v>
       </c>
-      <c r="M69" s="112">
-        <v>64</v>
-      </c>
-      <c r="N69" s="112">
+      <c r="M69">
+        <v>64</v>
+      </c>
+      <c r="N69">
         <v>32</v>
       </c>
-      <c r="O69" s="115" t="s">
-        <v>39</v>
-      </c>
-      <c r="P69" s="112">
+      <c r="O69" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="P69">
         <v>0.1</v>
       </c>
       <c r="Q69" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R69" s="126"/>
-      <c r="S69" s="127"/>
-      <c r="T69" s="127"/>
-      <c r="U69" s="127"/>
-      <c r="V69" s="127"/>
-      <c r="W69" s="128"/>
+      <c r="R69" s="116"/>
+      <c r="S69" s="117"/>
+      <c r="T69" s="117"/>
+      <c r="U69" s="117"/>
+      <c r="V69" s="117"/>
+      <c r="W69" s="118"/>
     </row>
     <row r="70" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B70" s="118" t="s">
+      <c r="B70" s="120" t="s">
         <v>89</v>
       </c>
-      <c r="C70" s="120" t="s">
+      <c r="C70" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="D70" s="129">
+      <c r="D70" s="17">
         <v>117.86</v>
       </c>
-      <c r="E70" s="130">
+      <c r="E70" s="15">
         <v>155.45699999999999</v>
       </c>
-      <c r="F70" s="130">
+      <c r="F70" s="15">
         <v>0.78659999999999997</v>
       </c>
-      <c r="G70" s="114">
+      <c r="G70">
         <v>0.78620000000000001</v>
       </c>
-      <c r="H70" s="131">
+      <c r="H70" s="7">
         <v>22.4</v>
       </c>
-      <c r="I70" s="112">
+      <c r="I70">
         <v>18</v>
       </c>
       <c r="J70" s="15">
         <v>196.4</v>
       </c>
-      <c r="K70" s="112">
+      <c r="K70">
         <v>6</v>
       </c>
       <c r="L70" s="23">
@@ -5153,141 +5128,141 @@
       <c r="Q70" s="16">
         <v>1E-3</v>
       </c>
-      <c r="R70" s="82" t="s">
+      <c r="R70" s="93" t="s">
         <v>90</v>
       </c>
-      <c r="S70" s="125"/>
-      <c r="T70" s="125"/>
-      <c r="U70" s="125"/>
-      <c r="V70" s="125"/>
-      <c r="W70" s="84"/>
+      <c r="S70" s="94"/>
+      <c r="T70" s="94"/>
+      <c r="U70" s="94"/>
+      <c r="V70" s="94"/>
+      <c r="W70" s="95"/>
     </row>
     <row r="71" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B71" s="68"/>
+      <c r="B71" s="79"/>
       <c r="C71" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="D71" s="124">
+      <c r="D71" s="1">
         <v>118.28</v>
       </c>
-      <c r="E71" s="114">
+      <c r="E71">
         <v>149.739</v>
       </c>
-      <c r="F71" s="114">
+      <c r="F71">
         <v>0.80200000000000005</v>
       </c>
-      <c r="G71" s="114">
+      <c r="G71">
         <v>0.80159999999999998</v>
       </c>
-      <c r="H71" s="131">
+      <c r="H71" s="7">
         <v>22.6</v>
       </c>
-      <c r="I71" s="112">
+      <c r="I71">
         <v>18</v>
       </c>
-      <c r="J71" s="112">
+      <c r="J71">
         <v>332.8</v>
       </c>
-      <c r="K71" s="112">
-        <v>6</v>
-      </c>
-      <c r="L71" s="115">
+      <c r="K71">
+        <v>6</v>
+      </c>
+      <c r="L71" s="31">
         <v>71</v>
       </c>
-      <c r="M71" s="112">
-        <v>64</v>
-      </c>
-      <c r="N71" s="112">
+      <c r="M71">
+        <v>64</v>
+      </c>
+      <c r="N71">
         <v>32</v>
       </c>
-      <c r="O71" s="115" t="s">
-        <v>39</v>
-      </c>
-      <c r="P71" s="112">
+      <c r="O71" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="P71">
         <v>0.1</v>
       </c>
       <c r="Q71" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R71" s="82"/>
-      <c r="S71" s="125"/>
-      <c r="T71" s="125"/>
-      <c r="U71" s="125"/>
-      <c r="V71" s="125"/>
-      <c r="W71" s="84"/>
+      <c r="R71" s="93"/>
+      <c r="S71" s="94"/>
+      <c r="T71" s="94"/>
+      <c r="U71" s="94"/>
+      <c r="V71" s="94"/>
+      <c r="W71" s="95"/>
     </row>
     <row r="72" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B72" s="68"/>
+      <c r="B72" s="79"/>
       <c r="C72" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="D72" s="124">
+      <c r="D72" s="1">
         <v>125.658</v>
       </c>
-      <c r="E72" s="114">
+      <c r="E72">
         <v>166.56800000000001</v>
       </c>
-      <c r="F72" s="114">
+      <c r="F72">
         <v>0.755</v>
       </c>
-      <c r="G72" s="114">
+      <c r="G72">
         <v>0.75449999999999995</v>
       </c>
-      <c r="H72" s="131">
+      <c r="H72" s="7">
         <v>17.899999999999999</v>
       </c>
-      <c r="I72" s="112">
+      <c r="I72">
         <v>18</v>
       </c>
-      <c r="J72" s="112">
+      <c r="J72">
         <v>546.79999999999995</v>
       </c>
-      <c r="K72" s="112">
-        <v>6</v>
-      </c>
-      <c r="L72" s="115">
+      <c r="K72">
+        <v>6</v>
+      </c>
+      <c r="L72" s="31">
         <v>106</v>
       </c>
-      <c r="M72" s="112">
-        <v>64</v>
-      </c>
-      <c r="N72" s="112">
+      <c r="M72">
+        <v>64</v>
+      </c>
+      <c r="N72">
         <v>32</v>
       </c>
-      <c r="O72" s="115" t="s">
-        <v>39</v>
-      </c>
-      <c r="P72" s="112">
+      <c r="O72" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="P72">
         <v>0.1</v>
       </c>
       <c r="Q72" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R72" s="82"/>
-      <c r="S72" s="125"/>
-      <c r="T72" s="125"/>
-      <c r="U72" s="125"/>
-      <c r="V72" s="125"/>
-      <c r="W72" s="84"/>
+      <c r="R72" s="93"/>
+      <c r="S72" s="94"/>
+      <c r="T72" s="94"/>
+      <c r="U72" s="94"/>
+      <c r="V72" s="94"/>
+      <c r="W72" s="95"/>
     </row>
     <row r="73" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="69"/>
+      <c r="B73" s="80"/>
       <c r="C73" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="D73" s="132">
+      <c r="D73" s="3">
         <v>155.00899999999999</v>
       </c>
-      <c r="E73" s="132">
+      <c r="E73" s="3">
         <v>196.97300000000001</v>
       </c>
-      <c r="F73" s="132">
+      <c r="F73" s="3">
         <v>0.65739999999999998</v>
       </c>
-      <c r="G73" s="132">
+      <c r="G73" s="3">
         <v>0.67669999999999997</v>
       </c>
-      <c r="H73" s="133">
+      <c r="H73" s="4">
         <v>38.4</v>
       </c>
       <c r="I73" s="3">
@@ -5317,12 +5292,12 @@
       <c r="Q73" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R73" s="85"/>
-      <c r="S73" s="86"/>
-      <c r="T73" s="86"/>
-      <c r="U73" s="86"/>
-      <c r="V73" s="86"/>
-      <c r="W73" s="87"/>
+      <c r="R73" s="96"/>
+      <c r="S73" s="97"/>
+      <c r="T73" s="97"/>
+      <c r="U73" s="97"/>
+      <c r="V73" s="97"/>
+      <c r="W73" s="98"/>
     </row>
     <row r="74" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
@@ -5333,18 +5308,20 @@
     <mergeCell ref="R70:W73"/>
     <mergeCell ref="B53:B56"/>
     <mergeCell ref="R53:W56"/>
+    <mergeCell ref="R45:W48"/>
+    <mergeCell ref="B45:B48"/>
+    <mergeCell ref="R49:W52"/>
+    <mergeCell ref="B49:B52"/>
+    <mergeCell ref="R23:W25"/>
+    <mergeCell ref="B26:B28"/>
+    <mergeCell ref="R26:W28"/>
+    <mergeCell ref="B23:B25"/>
     <mergeCell ref="B38:B40"/>
     <mergeCell ref="R38:W40"/>
     <mergeCell ref="B35:B37"/>
     <mergeCell ref="R35:W37"/>
     <mergeCell ref="B41:B44"/>
     <mergeCell ref="R41:W44"/>
-    <mergeCell ref="R45:W48"/>
-    <mergeCell ref="B45:B48"/>
-    <mergeCell ref="R49:W52"/>
-    <mergeCell ref="B49:B52"/>
-    <mergeCell ref="R23:W25"/>
-    <mergeCell ref="B26:B28"/>
     <mergeCell ref="D3:H3"/>
     <mergeCell ref="I3:Q3"/>
     <mergeCell ref="B5:B7"/>
@@ -5352,7 +5329,6 @@
     <mergeCell ref="R3:W4"/>
     <mergeCell ref="R5:W7"/>
     <mergeCell ref="R8:W10"/>
-    <mergeCell ref="R26:W28"/>
     <mergeCell ref="B11:B13"/>
     <mergeCell ref="B61:B65"/>
     <mergeCell ref="R61:W65"/>
@@ -5369,7 +5345,6 @@
     <mergeCell ref="R29:W31"/>
     <mergeCell ref="B32:B34"/>
     <mergeCell ref="R32:W34"/>
-    <mergeCell ref="B23:B25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>

<commit_message>
Mini test para comunicar ordenador con ESP32 por pyserial
</commit_message>
<xml_diff>
--- a/modelos_tfg/MetricasValidacion.xlsx
+++ b/modelos_tfg/MetricasValidacion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\modelos_tfg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3A2EFEB-C37A-4309-88CE-986D7C64F31B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C30969A-68B7-4012-B837-2103EE9EDC06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="0" windowWidth="29040" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1440,7 +1440,7 @@
       <c r="V4" s="114"/>
       <c r="W4" s="102"/>
     </row>
-    <row r="5" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
       <c r="B5" s="110" t="s">
         <v>15</v>
@@ -1499,7 +1499,7 @@
       <c r="V5" s="91"/>
       <c r="W5" s="92"/>
     </row>
-    <row r="6" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="7"/>
       <c r="B6" s="77"/>
       <c r="C6" s="5" t="s">
@@ -1554,7 +1554,7 @@
       <c r="V6" s="94"/>
       <c r="W6" s="95"/>
     </row>
-    <row r="7" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7"/>
       <c r="B7" s="103"/>
       <c r="C7" s="13" t="s">
@@ -1609,7 +1609,7 @@
       <c r="V7" s="97"/>
       <c r="W7" s="98"/>
     </row>
-    <row r="8" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
       <c r="B8" s="76" t="s">
         <v>24</v>
@@ -1668,7 +1668,7 @@
       <c r="V8" s="91"/>
       <c r="W8" s="92"/>
     </row>
-    <row r="9" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
       <c r="B9" s="77"/>
       <c r="C9" s="5" t="s">
@@ -1723,7 +1723,7 @@
       <c r="V9" s="94"/>
       <c r="W9" s="95"/>
     </row>
-    <row r="10" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7"/>
       <c r="B10" s="103"/>
       <c r="C10" s="5" t="s">
@@ -1778,7 +1778,7 @@
       <c r="V10" s="97"/>
       <c r="W10" s="98"/>
     </row>
-    <row r="11" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B11" s="76" t="s">
         <v>34</v>
       </c>
@@ -1836,7 +1836,7 @@
       <c r="V11" s="91"/>
       <c r="W11" s="92"/>
     </row>
-    <row r="12" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B12" s="77"/>
       <c r="C12" s="25" t="s">
         <v>12</v>
@@ -1890,7 +1890,7 @@
       <c r="V12" s="94"/>
       <c r="W12" s="95"/>
     </row>
-    <row r="13" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="77"/>
       <c r="C13" s="26" t="s">
         <v>14</v>
@@ -1944,7 +1944,7 @@
       <c r="V13" s="97"/>
       <c r="W13" s="98"/>
     </row>
-    <row r="14" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B14" s="76" t="s">
         <v>36</v>
       </c>
@@ -2002,7 +2002,7 @@
       <c r="V14" s="91"/>
       <c r="W14" s="92"/>
     </row>
-    <row r="15" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B15" s="77"/>
       <c r="C15" s="29" t="s">
         <v>12</v>
@@ -2056,7 +2056,7 @@
       <c r="V15" s="94"/>
       <c r="W15" s="95"/>
     </row>
-    <row r="16" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="103"/>
       <c r="C16" s="30" t="s">
         <v>14</v>
@@ -2110,7 +2110,7 @@
       <c r="V16" s="97"/>
       <c r="W16" s="98"/>
     </row>
-    <row r="17" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7"/>
       <c r="B17" s="100" t="s">
         <v>44</v>
@@ -2169,7 +2169,7 @@
       <c r="V17" s="91"/>
       <c r="W17" s="92"/>
     </row>
-    <row r="18" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
       <c r="B18" s="101"/>
       <c r="C18" s="29" t="s">
@@ -2224,7 +2224,7 @@
       <c r="V18" s="94"/>
       <c r="W18" s="95"/>
     </row>
-    <row r="19" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7"/>
       <c r="B19" s="102"/>
       <c r="C19" s="30" t="s">
@@ -2279,7 +2279,7 @@
       <c r="V19" s="97"/>
       <c r="W19" s="98"/>
     </row>
-    <row r="20" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7"/>
       <c r="B20" s="76" t="s">
         <v>46</v>
@@ -2338,7 +2338,7 @@
       <c r="V20" s="91"/>
       <c r="W20" s="92"/>
     </row>
-    <row r="21" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
       <c r="B21" s="77"/>
       <c r="C21" s="29" t="s">
@@ -2393,7 +2393,7 @@
       <c r="V21" s="94"/>
       <c r="W21" s="95"/>
     </row>
-    <row r="22" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="7"/>
       <c r="B22" s="103"/>
       <c r="C22" s="30" t="s">
@@ -2448,7 +2448,7 @@
       <c r="V22" s="97"/>
       <c r="W22" s="98"/>
     </row>
-    <row r="23" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A23" s="58"/>
       <c r="B23" s="78" t="s">
         <v>15</v>
@@ -2507,7 +2507,7 @@
       <c r="V23" s="91"/>
       <c r="W23" s="92"/>
     </row>
-    <row r="24" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A24" s="58"/>
       <c r="B24" s="79"/>
       <c r="C24" s="29" t="s">
@@ -2562,7 +2562,7 @@
       <c r="V24" s="94"/>
       <c r="W24" s="95"/>
     </row>
-    <row r="25" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="58"/>
       <c r="B25" s="80"/>
       <c r="C25" s="30" t="s">
@@ -2617,7 +2617,7 @@
       <c r="V25" s="97"/>
       <c r="W25" s="98"/>
     </row>
-    <row r="26" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A26" s="58"/>
       <c r="B26" s="78" t="s">
         <v>24</v>
@@ -2676,7 +2676,7 @@
       <c r="V26" s="91"/>
       <c r="W26" s="92"/>
     </row>
-    <row r="27" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" s="58"/>
       <c r="B27" s="79"/>
       <c r="C27" s="29" t="s">
@@ -2731,7 +2731,7 @@
       <c r="V27" s="94"/>
       <c r="W27" s="95"/>
     </row>
-    <row r="28" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="58"/>
       <c r="B28" s="80"/>
       <c r="C28" s="30" t="s">
@@ -2786,7 +2786,7 @@
       <c r="V28" s="97"/>
       <c r="W28" s="98"/>
     </row>
-    <row r="29" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A29" s="59"/>
       <c r="B29" s="78" t="s">
         <v>34</v>
@@ -2845,7 +2845,7 @@
       <c r="V29" s="91"/>
       <c r="W29" s="92"/>
     </row>
-    <row r="30" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" s="58"/>
       <c r="B30" s="79"/>
       <c r="C30" s="25" t="s">
@@ -2900,7 +2900,7 @@
       <c r="V30" s="94"/>
       <c r="W30" s="95"/>
     </row>
-    <row r="31" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="58"/>
       <c r="B31" s="80"/>
       <c r="C31" s="42" t="s">
@@ -2955,7 +2955,7 @@
       <c r="V31" s="97"/>
       <c r="W31" s="98"/>
     </row>
-    <row r="32" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A32" s="59"/>
       <c r="B32" s="78" t="s">
         <v>36</v>
@@ -3014,7 +3014,7 @@
       <c r="V32" s="91"/>
       <c r="W32" s="92"/>
     </row>
-    <row r="33" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A33" s="59"/>
       <c r="B33" s="79"/>
       <c r="C33" s="25" t="s">
@@ -3069,7 +3069,7 @@
       <c r="V33" s="94"/>
       <c r="W33" s="95"/>
     </row>
-    <row r="34" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="59"/>
       <c r="B34" s="80"/>
       <c r="C34" s="42" t="s">
@@ -3124,7 +3124,7 @@
       <c r="V34" s="97"/>
       <c r="W34" s="98"/>
     </row>
-    <row r="35" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A35" s="58"/>
       <c r="B35" s="78" t="s">
         <v>44</v>
@@ -3183,7 +3183,7 @@
       <c r="V35" s="91"/>
       <c r="W35" s="92"/>
     </row>
-    <row r="36" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A36" s="58"/>
       <c r="B36" s="79"/>
       <c r="C36" s="25" t="s">
@@ -3238,7 +3238,7 @@
       <c r="V36" s="94"/>
       <c r="W36" s="95"/>
     </row>
-    <row r="37" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="58"/>
       <c r="B37" s="80"/>
       <c r="C37" s="30" t="s">
@@ -3293,7 +3293,7 @@
       <c r="V37" s="97"/>
       <c r="W37" s="98"/>
     </row>
-    <row r="38" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A38" s="59"/>
       <c r="B38" s="78" t="s">
         <v>46</v>
@@ -3350,7 +3350,7 @@
       <c r="V38" s="82"/>
       <c r="W38" s="83"/>
     </row>
-    <row r="39" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A39" s="59"/>
       <c r="B39" s="79"/>
       <c r="C39" s="29" t="s">
@@ -3405,7 +3405,7 @@
       <c r="V39" s="85"/>
       <c r="W39" s="86"/>
     </row>
-    <row r="40" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="59"/>
       <c r="B40" s="80"/>
       <c r="C40" s="30" t="s">
@@ -3460,7 +3460,7 @@
       <c r="V40" s="88"/>
       <c r="W40" s="89"/>
     </row>
-    <row r="41" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A41" s="59"/>
       <c r="B41" s="78" t="s">
         <v>50</v>
@@ -3519,7 +3519,7 @@
       <c r="V41" s="91"/>
       <c r="W41" s="92"/>
     </row>
-    <row r="42" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A42" s="59"/>
       <c r="B42" s="79"/>
       <c r="C42" s="29" t="s">
@@ -3574,7 +3574,7 @@
       <c r="V42" s="94"/>
       <c r="W42" s="95"/>
     </row>
-    <row r="43" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A43" s="59"/>
       <c r="B43" s="79"/>
       <c r="C43" s="29" t="s">
@@ -3629,7 +3629,7 @@
       <c r="V43" s="94"/>
       <c r="W43" s="95"/>
     </row>
-    <row r="44" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="59"/>
       <c r="B44" s="80"/>
       <c r="C44" s="30" t="s">
@@ -3684,7 +3684,7 @@
       <c r="V44" s="97"/>
       <c r="W44" s="98"/>
     </row>
-    <row r="45" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A45" s="59"/>
       <c r="B45" s="78" t="s">
         <v>55</v>
@@ -3743,7 +3743,7 @@
       <c r="V45" s="82"/>
       <c r="W45" s="83"/>
     </row>
-    <row r="46" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A46" s="59"/>
       <c r="B46" s="79"/>
       <c r="C46" s="29" t="s">
@@ -3798,7 +3798,7 @@
       <c r="V46" s="85"/>
       <c r="W46" s="86"/>
     </row>
-    <row r="47" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A47" s="59"/>
       <c r="B47" s="79"/>
       <c r="C47" s="29" t="s">
@@ -3853,7 +3853,7 @@
       <c r="V47" s="85"/>
       <c r="W47" s="86"/>
     </row>
-    <row r="48" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="59"/>
       <c r="B48" s="80"/>
       <c r="C48" s="30" t="s">
@@ -3908,7 +3908,7 @@
       <c r="V48" s="88"/>
       <c r="W48" s="89"/>
     </row>
-    <row r="49" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A49" s="58"/>
       <c r="B49" s="78" t="s">
         <v>58</v>
@@ -3967,7 +3967,7 @@
       <c r="V49" s="91"/>
       <c r="W49" s="92"/>
     </row>
-    <row r="50" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A50" s="58"/>
       <c r="B50" s="79"/>
       <c r="C50" s="29" t="s">
@@ -4022,7 +4022,7 @@
       <c r="V50" s="94"/>
       <c r="W50" s="95"/>
     </row>
-    <row r="51" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A51" s="58"/>
       <c r="B51" s="79"/>
       <c r="C51" s="29" t="s">
@@ -4077,7 +4077,7 @@
       <c r="V51" s="94"/>
       <c r="W51" s="95"/>
     </row>
-    <row r="52" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="58"/>
       <c r="B52" s="80"/>
       <c r="C52" s="30" t="s">
@@ -4132,7 +4132,7 @@
       <c r="V52" s="97"/>
       <c r="W52" s="98"/>
     </row>
-    <row r="53" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A53" s="59"/>
       <c r="B53" s="78" t="s">
         <v>77</v>
@@ -4191,7 +4191,7 @@
       <c r="V53" s="91"/>
       <c r="W53" s="92"/>
     </row>
-    <row r="54" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A54" s="59"/>
       <c r="B54" s="79"/>
       <c r="C54" s="29" t="s">
@@ -4246,7 +4246,7 @@
       <c r="V54" s="94"/>
       <c r="W54" s="95"/>
     </row>
-    <row r="55" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A55" s="59"/>
       <c r="B55" s="79"/>
       <c r="C55" s="29" t="s">
@@ -4301,7 +4301,7 @@
       <c r="V55" s="94"/>
       <c r="W55" s="95"/>
     </row>
-    <row r="56" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="59"/>
       <c r="B56" s="80"/>
       <c r="C56" s="30" t="s">
@@ -4356,7 +4356,7 @@
       <c r="V56" s="97"/>
       <c r="W56" s="98"/>
     </row>
-    <row r="57" spans="1:23" ht="15.75" hidden="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A57" s="58"/>
       <c r="B57" s="78" t="s">
         <v>81</v>
@@ -4415,7 +4415,7 @@
       <c r="V57" s="91"/>
       <c r="W57" s="92"/>
     </row>
-    <row r="58" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A58" s="58"/>
       <c r="B58" s="79"/>
       <c r="C58" s="29" t="s">
@@ -4470,7 +4470,7 @@
       <c r="V58" s="94"/>
       <c r="W58" s="95"/>
     </row>
-    <row r="59" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A59" s="58"/>
       <c r="B59" s="79"/>
       <c r="C59" s="29" t="s">
@@ -4525,7 +4525,7 @@
       <c r="V59" s="94"/>
       <c r="W59" s="95"/>
     </row>
-    <row r="60" spans="1:23" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="58"/>
       <c r="B60" s="80"/>
       <c r="C60" s="30" t="s">
@@ -4922,19 +4922,19 @@
       <c r="C67" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="D67">
+      <c r="D67" s="51">
         <v>51.738</v>
       </c>
-      <c r="E67">
+      <c r="E67" s="51">
         <v>92.930999999999997</v>
       </c>
-      <c r="F67">
+      <c r="F67" s="51">
         <v>0.94950000000000001</v>
       </c>
-      <c r="G67">
+      <c r="G67" s="51">
         <v>0.94950000000000001</v>
       </c>
-      <c r="H67" s="7">
+      <c r="H67" s="52">
         <v>22.6</v>
       </c>
       <c r="I67">
@@ -4976,19 +4976,19 @@
       <c r="C68" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="D68">
+      <c r="D68" s="51">
         <v>48.079000000000001</v>
       </c>
-      <c r="E68">
+      <c r="E68" s="51">
         <v>102.464</v>
       </c>
-      <c r="F68">
+      <c r="F68" s="51">
         <v>0.93859999999999999</v>
       </c>
-      <c r="G68">
+      <c r="G68" s="51">
         <v>0.93859999999999999</v>
       </c>
-      <c r="H68" s="7">
+      <c r="H68" s="52">
         <v>17.899999999999999</v>
       </c>
       <c r="I68">

</xml_diff>